<commit_message>
added delta of absolute speed after ВНА
</commit_message>
<xml_diff>
--- a/results/Поступенчатый_расчет_ступеней.xlsx
+++ b/results/Поступенчатый_расчет_ступеней.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P82"/>
+  <dimension ref="A1:P83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -667,15 +667,17 @@
     <row r="7" ht="15" customHeight="1">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>a_кр_1_i_СА</t>
+          <t>delta_c_abs_ВНА</t>
         </is>
       </c>
       <c r="B7" s="1" t="inlineStr">
         <is>
-          <t>СА: Критическая скорость на входе</t>
-        </is>
-      </c>
-      <c r="C7" s="1" t="inlineStr"/>
+          <t>Изменение скорости абсолютной в ВНА</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="n">
+        <v>9.714170190180937</v>
+      </c>
       <c r="D7" s="1" t="inlineStr"/>
       <c r="E7" s="1" t="inlineStr"/>
       <c r="F7" s="1" t="inlineStr"/>
@@ -688,19 +690,17 @@
       <c r="M7" s="1" t="inlineStr"/>
       <c r="N7" s="1" t="inlineStr"/>
       <c r="O7" s="1" t="inlineStr"/>
-      <c r="P7" s="2" t="n">
-        <v>477.1612274741949</v>
-      </c>
+      <c r="P7" s="1" t="inlineStr"/>
     </row>
     <row r="8" ht="15" customHeight="1">
       <c r="A8" s="1" t="inlineStr">
         <is>
-          <t>r_ср1_отн_i_СА</t>
+          <t>a_кр_1_i_СА</t>
         </is>
       </c>
       <c r="B8" s="1" t="inlineStr">
         <is>
-          <t>СА: Относительный средний радиус на входе</t>
+          <t>СА: Критическая скорость на входе</t>
         </is>
       </c>
       <c r="C8" s="1" t="inlineStr"/>
@@ -717,18 +717,18 @@
       <c r="N8" s="1" t="inlineStr"/>
       <c r="O8" s="1" t="inlineStr"/>
       <c r="P8" s="2" t="n">
-        <v>0.9595531619480527</v>
+        <v>477.1612274741949</v>
       </c>
     </row>
     <row r="9" ht="15" customHeight="1">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>c_a2_i_СА</t>
+          <t>r_ср1_отн_i_СА</t>
         </is>
       </c>
       <c r="B9" s="1" t="inlineStr">
         <is>
-          <t>СА: Осевая скорость на входе</t>
+          <t>СА: Относительный средний радиус на входе</t>
         </is>
       </c>
       <c r="C9" s="1" t="inlineStr"/>
@@ -745,18 +745,18 @@
       <c r="N9" s="1" t="inlineStr"/>
       <c r="O9" s="1" t="inlineStr"/>
       <c r="P9" s="2" t="n">
-        <v>106.3166261739218</v>
+        <v>0.9595531619480527</v>
       </c>
     </row>
     <row r="10" ht="15" customHeight="1">
       <c r="A10" s="1" t="inlineStr">
         <is>
-          <t>q_1_i_СА</t>
+          <t>c_a2_i_СА</t>
         </is>
       </c>
       <c r="B10" s="1" t="inlineStr">
         <is>
-          <t>СА: ГДФ расхода на входе</t>
+          <t>СА: Осевая скорость на входе</t>
         </is>
       </c>
       <c r="C10" s="1" t="inlineStr"/>
@@ -773,18 +773,18 @@
       <c r="N10" s="1" t="inlineStr"/>
       <c r="O10" s="1" t="inlineStr"/>
       <c r="P10" s="2" t="n">
-        <v>0.4537118711400231</v>
+        <v>106.3166261739218</v>
       </c>
     </row>
     <row r="11" ht="15" customHeight="1">
       <c r="A11" s="1" t="inlineStr">
         <is>
-          <t>F_1_i_СА</t>
+          <t>q_1_i_СА</t>
         </is>
       </c>
       <c r="B11" s="1" t="inlineStr">
         <is>
-          <t>СА: Кольцевая площадь на входе</t>
+          <t>СА: ГДФ расхода на входе</t>
         </is>
       </c>
       <c r="C11" s="1" t="inlineStr"/>
@@ -801,18 +801,18 @@
       <c r="N11" s="1" t="inlineStr"/>
       <c r="O11" s="1" t="inlineStr"/>
       <c r="P11" s="2" t="n">
-        <v>0.05555276895854432</v>
+        <v>0.4537118711400231</v>
       </c>
     </row>
     <row r="12" ht="15" customHeight="1">
       <c r="A12" s="1" t="inlineStr">
         <is>
-          <t>α_3_i_СА</t>
+          <t>F_1_i_СА</t>
         </is>
       </c>
       <c r="B12" s="1" t="inlineStr">
         <is>
-          <t>СА: Угол абсолютной скорости на выходе</t>
+          <t>СА: Кольцевая площадь на входе</t>
         </is>
       </c>
       <c r="C12" s="1" t="inlineStr"/>
@@ -829,18 +829,18 @@
       <c r="N12" s="1" t="inlineStr"/>
       <c r="O12" s="1" t="inlineStr"/>
       <c r="P12" s="2" t="n">
-        <v>1.570796326794897</v>
-      </c>
-    </row>
-    <row r="13" ht="30" customHeight="1">
+        <v>0.05555276895854432</v>
+      </c>
+    </row>
+    <row r="13" ht="15" customHeight="1">
       <c r="A13" s="1" t="inlineStr">
         <is>
-          <t>F_3_i_СА</t>
+          <t>α_3_i_СА</t>
         </is>
       </c>
       <c r="B13" s="1" t="inlineStr">
         <is>
-          <t>СА: Действительная кольцевая площадь на выходе</t>
+          <t>СА: Угол абсолютной скорости на выходе</t>
         </is>
       </c>
       <c r="C13" s="1" t="inlineStr"/>
@@ -857,18 +857,18 @@
       <c r="N13" s="1" t="inlineStr"/>
       <c r="O13" s="1" t="inlineStr"/>
       <c r="P13" s="2" t="n">
-        <v>0.05555276895854432</v>
-      </c>
-    </row>
-    <row r="14" ht="15" customHeight="1">
+        <v>1.570796326794897</v>
+      </c>
+    </row>
+    <row r="14" ht="30" customHeight="1">
       <c r="A14" s="1" t="inlineStr">
         <is>
-          <t>D_вт3_i_СА</t>
+          <t>F_3_i_СА</t>
         </is>
       </c>
       <c r="B14" s="1" t="inlineStr">
         <is>
-          <t>СА: Втулочный диаметр на выходе</t>
+          <t>СА: Действительная кольцевая площадь на выходе</t>
         </is>
       </c>
       <c r="C14" s="1" t="inlineStr"/>
@@ -885,18 +885,18 @@
       <c r="N14" s="1" t="inlineStr"/>
       <c r="O14" s="1" t="inlineStr"/>
       <c r="P14" s="2" t="n">
-        <v>0.3421954010820806</v>
+        <v>0.05555276895854432</v>
       </c>
     </row>
     <row r="15" ht="15" customHeight="1">
       <c r="A15" s="1" t="inlineStr">
         <is>
-          <t>d3_отн_i_СА</t>
+          <t>D_вт3_i_СА</t>
         </is>
       </c>
       <c r="B15" s="1" t="inlineStr">
         <is>
-          <t>СА: Относительный диаметр втулки на выходе</t>
+          <t>СА: Втулочный диаметр на выходе</t>
         </is>
       </c>
       <c r="C15" s="1" t="inlineStr"/>
@@ -913,18 +913,18 @@
       <c r="N15" s="1" t="inlineStr"/>
       <c r="O15" s="1" t="inlineStr"/>
       <c r="P15" s="2" t="n">
-        <v>0.5026572059935642</v>
+        <v>0.3421954010820806</v>
       </c>
     </row>
     <row r="16" ht="15" customHeight="1">
       <c r="A16" s="1" t="inlineStr">
         <is>
-          <t>r_ср3_отн_i_СА</t>
+          <t>d3_отн_i_СА</t>
         </is>
       </c>
       <c r="B16" s="1" t="inlineStr">
         <is>
-          <t>СА: Относительный средний радиус на выходе</t>
+          <t>СА: Относительный диаметр втулки на выходе</t>
         </is>
       </c>
       <c r="C16" s="1" t="inlineStr"/>
@@ -941,18 +941,18 @@
       <c r="N16" s="1" t="inlineStr"/>
       <c r="O16" s="1" t="inlineStr"/>
       <c r="P16" s="2" t="n">
-        <v>0.7914114817012881</v>
+        <v>0.5026572059935642</v>
       </c>
     </row>
     <row r="17" ht="15" customHeight="1">
       <c r="A17" s="1" t="inlineStr">
         <is>
-          <t>α_2_i_СА</t>
+          <t>r_ср3_отн_i_СА</t>
         </is>
       </c>
       <c r="B17" s="1" t="inlineStr">
         <is>
-          <t>СА: Угол абсолютной скорости на входе</t>
+          <t>СА: Относительный средний радиус на выходе</t>
         </is>
       </c>
       <c r="C17" s="1" t="inlineStr"/>
@@ -969,18 +969,18 @@
       <c r="N17" s="1" t="inlineStr"/>
       <c r="O17" s="1" t="inlineStr"/>
       <c r="P17" s="2" t="n">
-        <v>0.8521100845146086</v>
+        <v>0.7914114817012881</v>
       </c>
     </row>
     <row r="18" ht="15" customHeight="1">
       <c r="A18" s="1" t="inlineStr">
         <is>
-          <t>ε_на_i_СА</t>
+          <t>α_2_i_СА</t>
         </is>
       </c>
       <c r="B18" s="1" t="inlineStr">
         <is>
-          <t>СА: Диффузность решетки</t>
+          <t>СА: Угол абсолютной скорости на входе</t>
         </is>
       </c>
       <c r="C18" s="1" t="inlineStr"/>
@@ -997,18 +997,18 @@
       <c r="N18" s="1" t="inlineStr"/>
       <c r="O18" s="1" t="inlineStr"/>
       <c r="P18" s="2" t="n">
-        <v>0.718686242280288</v>
+        <v>0.8521100845146086</v>
       </c>
     </row>
     <row r="19" ht="15" customHeight="1">
       <c r="A19" s="1" t="inlineStr">
         <is>
-          <t>c_2_i_СА</t>
+          <t>ε_на_i_СА</t>
         </is>
       </c>
       <c r="B19" s="1" t="inlineStr">
         <is>
-          <t>СА: Абсолютная скорость на входе</t>
+          <t>СА: Диффузность решетки</t>
         </is>
       </c>
       <c r="C19" s="1" t="inlineStr"/>
@@ -1025,18 +1025,18 @@
       <c r="N19" s="1" t="inlineStr"/>
       <c r="O19" s="1" t="inlineStr"/>
       <c r="P19" s="2" t="n">
-        <v>141.2523884686373</v>
-      </c>
-    </row>
-    <row r="20" ht="30" customHeight="1">
+        <v>0.718686242280288</v>
+      </c>
+    </row>
+    <row r="20" ht="15" customHeight="1">
       <c r="A20" s="1" t="inlineStr">
         <is>
-          <t>d2_отн_i_СА</t>
+          <t>c_2_i_СА</t>
         </is>
       </c>
       <c r="B20" s="1" t="inlineStr">
         <is>
-          <t>СА: Относительный диаметр втулки на выходе РК</t>
+          <t>СА: Абсолютная скорость на входе</t>
         </is>
       </c>
       <c r="C20" s="1" t="inlineStr"/>
@@ -1053,18 +1053,18 @@
       <c r="N20" s="1" t="inlineStr"/>
       <c r="O20" s="1" t="inlineStr"/>
       <c r="P20" s="2" t="n">
-        <v>0.9189293312859016</v>
-      </c>
-    </row>
-    <row r="21" ht="15" customHeight="1">
+        <v>141.2523884686373</v>
+      </c>
+    </row>
+    <row r="21" ht="30" customHeight="1">
       <c r="A21" s="1" t="inlineStr">
         <is>
-          <t>D_вт2_i_СА</t>
+          <t>d2_отн_i_СА</t>
         </is>
       </c>
       <c r="B21" s="1" t="inlineStr">
         <is>
-          <t>СА: Втулочный диаметр на выходе РК</t>
+          <t>СА: Относительный диаметр втулки на выходе РК</t>
         </is>
       </c>
       <c r="C21" s="1" t="inlineStr"/>
@@ -1081,18 +1081,18 @@
       <c r="N21" s="1" t="inlineStr"/>
       <c r="O21" s="1" t="inlineStr"/>
       <c r="P21" s="2" t="n">
-        <v>0.6255821807307252</v>
+        <v>0.9189293312859016</v>
       </c>
     </row>
     <row r="22" ht="15" customHeight="1">
       <c r="A22" s="1" t="inlineStr">
         <is>
-          <t>h_на_i_СА</t>
+          <t>D_вт2_i_СА</t>
         </is>
       </c>
       <c r="B22" s="1" t="inlineStr">
         <is>
-          <t>СА: Высота лопаток на входе</t>
+          <t>СА: Втулочный диаметр на выходе РК</t>
         </is>
       </c>
       <c r="C22" s="1" t="inlineStr"/>
@@ -1109,18 +1109,18 @@
       <c r="N22" s="1" t="inlineStr"/>
       <c r="O22" s="1" t="inlineStr"/>
       <c r="P22" s="2" t="n">
-        <v>0.02759535690110904</v>
+        <v>0.6255821807307252</v>
       </c>
     </row>
     <row r="23" ht="15" customHeight="1">
       <c r="A23" s="1" t="inlineStr">
         <is>
-          <t>h_на_3_i_СА</t>
+          <t>h_на_i_СА</t>
         </is>
       </c>
       <c r="B23" s="1" t="inlineStr">
         <is>
-          <t>СА: Высота лопаток на выходе</t>
+          <t>СА: Высота лопаток на входе</t>
         </is>
       </c>
       <c r="C23" s="1" t="inlineStr"/>
@@ -1137,618 +1137,596 @@
       <c r="N23" s="1" t="inlineStr"/>
       <c r="O23" s="1" t="inlineStr"/>
       <c r="P23" s="2" t="n">
+        <v>0.02759535690110904</v>
+      </c>
+    </row>
+    <row r="24" ht="15" customHeight="1">
+      <c r="A24" s="1" t="inlineStr">
+        <is>
+          <t>h_на_3_i_СА</t>
+        </is>
+      </c>
+      <c r="B24" s="1" t="inlineStr">
+        <is>
+          <t>СА: Высота лопаток на выходе</t>
+        </is>
+      </c>
+      <c r="C24" s="1" t="inlineStr"/>
+      <c r="D24" s="1" t="inlineStr"/>
+      <c r="E24" s="1" t="inlineStr"/>
+      <c r="F24" s="1" t="inlineStr"/>
+      <c r="G24" s="1" t="inlineStr"/>
+      <c r="H24" s="1" t="inlineStr"/>
+      <c r="I24" s="1" t="inlineStr"/>
+      <c r="J24" s="1" t="inlineStr"/>
+      <c r="K24" s="1" t="inlineStr"/>
+      <c r="L24" s="1" t="inlineStr"/>
+      <c r="M24" s="1" t="inlineStr"/>
+      <c r="N24" s="1" t="inlineStr"/>
+      <c r="O24" s="1" t="inlineStr"/>
+      <c r="P24" s="2" t="n">
         <v>0.1692887467254313</v>
       </c>
     </row>
-    <row r="24" ht="30" customHeight="1">
-      <c r="A24" s="1" t="inlineStr">
+    <row r="25" ht="30" customHeight="1">
+      <c r="A25" s="1" t="inlineStr">
         <is>
           <t>k_i</t>
         </is>
       </c>
-      <c r="B24" s="1" t="inlineStr">
+      <c r="B25" s="1" t="inlineStr">
         <is>
           <t>Показатель адиабаты по длине компрессора перед РК</t>
-        </is>
-      </c>
-      <c r="C24" s="1" t="inlineStr"/>
-      <c r="D24" s="2" t="n">
-        <v>1.399944336209296</v>
-      </c>
-      <c r="E24" s="2" t="n">
-        <v>1.397730417935234</v>
-      </c>
-      <c r="F24" s="2" t="n">
-        <v>1.394860425858321</v>
-      </c>
-      <c r="G24" s="2" t="n">
-        <v>1.393519592252976</v>
-      </c>
-      <c r="H24" s="2" t="n">
-        <v>1.390731081206798</v>
-      </c>
-      <c r="I24" s="2" t="n">
-        <v>1.388035570101426</v>
-      </c>
-      <c r="J24" s="2" t="n">
-        <v>1.384399004818129</v>
-      </c>
-      <c r="K24" s="2" t="n">
-        <v>1.38071062867211</v>
-      </c>
-      <c r="L24" s="2" t="n">
-        <v>1.37610539882691</v>
-      </c>
-      <c r="M24" s="2" t="n">
-        <v>1.372438981258499</v>
-      </c>
-      <c r="N24" s="2" t="n">
-        <v>1.368632710893606</v>
-      </c>
-      <c r="O24" s="2" t="n">
-        <v>1.364566577433034</v>
-      </c>
-      <c r="P24" s="1" t="inlineStr"/>
-    </row>
-    <row r="25" ht="15" customHeight="1">
-      <c r="A25" s="1" t="inlineStr">
-        <is>
-          <t>c_a_i_отн</t>
-        </is>
-      </c>
-      <c r="B25" s="1" t="inlineStr">
-        <is>
-          <t>Коэффициент расхода на входе в ступень</t>
         </is>
       </c>
       <c r="C25" s="1" t="inlineStr"/>
       <c r="D25" s="2" t="n">
-        <v>0.65</v>
+        <v>1.399944336209296</v>
       </c>
       <c r="E25" s="2" t="n">
-        <v>0.6236363636363637</v>
+        <v>1.397730417935234</v>
       </c>
       <c r="F25" s="2" t="n">
-        <v>0.5972727272727273</v>
+        <v>1.394860425858321</v>
       </c>
       <c r="G25" s="2" t="n">
-        <v>0.5709090909090909</v>
+        <v>1.393519592252976</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>0.5445454545454546</v>
+        <v>1.390731081206798</v>
       </c>
       <c r="I25" s="2" t="n">
-        <v>0.5181818181818182</v>
+        <v>1.388035570101426</v>
       </c>
       <c r="J25" s="2" t="n">
-        <v>0.4918181818181818</v>
+        <v>1.384399004818129</v>
       </c>
       <c r="K25" s="2" t="n">
-        <v>0.4654545454545455</v>
+        <v>1.38071062867211</v>
       </c>
       <c r="L25" s="2" t="n">
-        <v>0.4390909090909091</v>
+        <v>1.37610539882691</v>
       </c>
       <c r="M25" s="2" t="n">
-        <v>0.4127272727272727</v>
+        <v>1.372438981258499</v>
       </c>
       <c r="N25" s="2" t="n">
-        <v>0.3863636363636364</v>
+        <v>1.368632710893606</v>
       </c>
       <c r="O25" s="2" t="n">
-        <v>0.36</v>
+        <v>1.364566577433034</v>
       </c>
       <c r="P25" s="1" t="inlineStr"/>
     </row>
     <row r="26" ht="15" customHeight="1">
       <c r="A26" s="1" t="inlineStr">
         <is>
-          <t>c_a_i_отн_plus_1</t>
+          <t>c_a_i_отн</t>
         </is>
       </c>
       <c r="B26" s="1" t="inlineStr">
         <is>
-          <t>Коэффициент расхода на выходе из ступени</t>
+          <t>Коэффициент расхода на входе в ступень</t>
         </is>
       </c>
       <c r="C26" s="1" t="inlineStr"/>
       <c r="D26" s="2" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="E26" s="2" t="n">
         <v>0.6236363636363637</v>
       </c>
-      <c r="E26" s="2" t="n">
+      <c r="F26" s="2" t="n">
         <v>0.5972727272727273</v>
       </c>
-      <c r="F26" s="2" t="n">
+      <c r="G26" s="2" t="n">
         <v>0.5709090909090909</v>
       </c>
-      <c r="G26" s="2" t="n">
+      <c r="H26" s="2" t="n">
         <v>0.5445454545454546</v>
       </c>
-      <c r="H26" s="2" t="n">
+      <c r="I26" s="2" t="n">
         <v>0.5181818181818182</v>
       </c>
-      <c r="I26" s="2" t="n">
+      <c r="J26" s="2" t="n">
         <v>0.4918181818181818</v>
       </c>
-      <c r="J26" s="2" t="n">
+      <c r="K26" s="2" t="n">
         <v>0.4654545454545455</v>
       </c>
-      <c r="K26" s="2" t="n">
+      <c r="L26" s="2" t="n">
         <v>0.4390909090909091</v>
       </c>
-      <c r="L26" s="2" t="n">
+      <c r="M26" s="2" t="n">
         <v>0.4127272727272727</v>
       </c>
-      <c r="M26" s="2" t="n">
+      <c r="N26" s="2" t="n">
         <v>0.3863636363636364</v>
       </c>
-      <c r="N26" s="2" t="n">
+      <c r="O26" s="2" t="n">
         <v>0.36</v>
-      </c>
-      <c r="O26" s="2" t="n">
-        <v>0.3336363636363636</v>
       </c>
       <c r="P26" s="1" t="inlineStr"/>
     </row>
     <row r="27" ht="15" customHeight="1">
       <c r="A27" s="1" t="inlineStr">
         <is>
-          <t>P1_полн_i</t>
+          <t>c_a_i_отн_plus_1</t>
         </is>
       </c>
       <c r="B27" s="1" t="inlineStr">
         <is>
-          <t>Полное давление перед ступенью</t>
+          <t>Коэффициент расхода на выходе из ступени</t>
         </is>
       </c>
       <c r="C27" s="1" t="inlineStr"/>
       <c r="D27" s="2" t="n">
-        <v>100292.8790575521</v>
+        <v>0.6236363636363637</v>
       </c>
       <c r="E27" s="2" t="n">
-        <v>259542.8799520527</v>
+        <v>0.5972727272727273</v>
       </c>
       <c r="F27" s="2" t="n">
-        <v>418792.8808465532</v>
+        <v>0.5709090909090909</v>
       </c>
       <c r="G27" s="2" t="n">
-        <v>578042.8817410537</v>
+        <v>0.5445454545454546</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>737292.8826355543</v>
+        <v>0.5181818181818182</v>
       </c>
       <c r="I27" s="2" t="n">
-        <v>896542.8835300547</v>
+        <v>0.4918181818181818</v>
       </c>
       <c r="J27" s="2" t="n">
-        <v>1055792.884424555</v>
+        <v>0.4654545454545455</v>
       </c>
       <c r="K27" s="2" t="n">
-        <v>1215042.885319056</v>
+        <v>0.4390909090909091</v>
       </c>
       <c r="L27" s="2" t="n">
-        <v>1374292.886213556</v>
+        <v>0.4127272727272727</v>
       </c>
       <c r="M27" s="2" t="n">
-        <v>1533542.887108057</v>
+        <v>0.3863636363636364</v>
       </c>
       <c r="N27" s="2" t="n">
-        <v>1692792.888002557</v>
+        <v>0.36</v>
       </c>
       <c r="O27" s="2" t="n">
-        <v>1852042.888897058</v>
+        <v>0.3336363636363636</v>
       </c>
       <c r="P27" s="1" t="inlineStr"/>
     </row>
     <row r="28" ht="15" customHeight="1">
       <c r="A28" s="1" t="inlineStr">
         <is>
-          <t>T1_полн_i</t>
+          <t>P1_полн_i</t>
         </is>
       </c>
       <c r="B28" s="1" t="inlineStr">
         <is>
-          <t>Полная температура перед ступенью</t>
+          <t>Полное давление перед ступенью</t>
         </is>
       </c>
       <c r="C28" s="1" t="inlineStr"/>
       <c r="D28" s="2" t="n">
-        <v>288</v>
+        <v>100292.8790575521</v>
       </c>
       <c r="E28" s="2" t="n">
-        <v>324.2171870844151</v>
+        <v>259542.8799520527</v>
       </c>
       <c r="F28" s="2" t="n">
-        <v>360.4343741688301</v>
+        <v>418792.8808465532</v>
       </c>
       <c r="G28" s="2" t="n">
-        <v>396.6515612532452</v>
+        <v>578042.8817410537</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>432.8687483376602</v>
+        <v>737292.8826355543</v>
       </c>
       <c r="I28" s="2" t="n">
-        <v>469.0859354220753</v>
+        <v>896542.8835300547</v>
       </c>
       <c r="J28" s="2" t="n">
-        <v>505.3031225064903</v>
+        <v>1055792.884424555</v>
       </c>
       <c r="K28" s="2" t="n">
-        <v>541.5203095909053</v>
+        <v>1215042.885319056</v>
       </c>
       <c r="L28" s="2" t="n">
-        <v>577.7374966753205</v>
+        <v>1374292.886213556</v>
       </c>
       <c r="M28" s="2" t="n">
-        <v>613.9546837597354</v>
+        <v>1533542.887108057</v>
       </c>
       <c r="N28" s="2" t="n">
-        <v>650.1718708441506</v>
+        <v>1692792.888002557</v>
       </c>
       <c r="O28" s="2" t="n">
-        <v>686.3890579285655</v>
+        <v>1852042.888897058</v>
       </c>
       <c r="P28" s="1" t="inlineStr"/>
     </row>
-    <row r="29" ht="30" customHeight="1">
+    <row r="29" ht="15" customHeight="1">
       <c r="A29" s="1" t="inlineStr">
         <is>
-          <t>d1_отн_i</t>
+          <t>T1_полн_i</t>
         </is>
       </c>
       <c r="B29" s="1" t="inlineStr">
         <is>
-          <t>Относительный диаметр втулки на входе в ступень</t>
+          <t>Полная температура перед ступенью</t>
         </is>
       </c>
       <c r="C29" s="1" t="inlineStr"/>
       <c r="D29" s="2" t="n">
-        <v>0.43</v>
+        <v>288</v>
       </c>
       <c r="E29" s="2" t="n">
-        <v>0.4743022422822237</v>
+        <v>324.2171870844151</v>
       </c>
       <c r="F29" s="2" t="n">
-        <v>0.5186044845644475</v>
+        <v>360.4343741688301</v>
       </c>
       <c r="G29" s="2" t="n">
-        <v>0.5629067268466712</v>
+        <v>396.6515612532452</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>0.6072089691288949</v>
+        <v>432.8687483376602</v>
       </c>
       <c r="I29" s="2" t="n">
-        <v>0.6515112114111187</v>
+        <v>469.0859354220753</v>
       </c>
       <c r="J29" s="2" t="n">
-        <v>0.6958134536933425</v>
+        <v>505.3031225064903</v>
       </c>
       <c r="K29" s="2" t="n">
-        <v>0.7401156959755661</v>
+        <v>541.5203095909053</v>
       </c>
       <c r="L29" s="2" t="n">
-        <v>0.7844179382577898</v>
+        <v>577.7374966753205</v>
       </c>
       <c r="M29" s="2" t="n">
-        <v>0.8287201805400136</v>
+        <v>613.9546837597354</v>
       </c>
       <c r="N29" s="2" t="n">
-        <v>0.8730224228222374</v>
+        <v>650.1718708441506</v>
       </c>
       <c r="O29" s="2" t="n">
-        <v>0.9173246651044611</v>
+        <v>686.3890579285655</v>
       </c>
       <c r="P29" s="1" t="inlineStr"/>
     </row>
     <row r="30" ht="30" customHeight="1">
       <c r="A30" s="1" t="inlineStr">
         <is>
-          <t>U_k_i</t>
+          <t>d1_отн_i</t>
         </is>
       </c>
       <c r="B30" s="1" t="inlineStr">
         <is>
-          <t>Окружная скорость концов рабочих лопаток ступени</t>
+          <t>Относительный диаметр втулки на входе в ступень</t>
         </is>
       </c>
       <c r="C30" s="1" t="inlineStr"/>
       <c r="D30" s="2" t="n">
-        <v>306.5485944726447</v>
+        <v>0.43</v>
       </c>
       <c r="E30" s="2" t="n">
-        <v>306.5485944726447</v>
+        <v>0.4743022422822237</v>
       </c>
       <c r="F30" s="2" t="n">
-        <v>306.5485944726447</v>
+        <v>0.5186044845644475</v>
       </c>
       <c r="G30" s="2" t="n">
-        <v>306.5485944726447</v>
+        <v>0.5629067268466712</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>306.5485944726447</v>
+        <v>0.6072089691288949</v>
       </c>
       <c r="I30" s="2" t="n">
-        <v>306.5485944726447</v>
+        <v>0.6515112114111187</v>
       </c>
       <c r="J30" s="2" t="n">
-        <v>306.5485944726447</v>
+        <v>0.6958134536933425</v>
       </c>
       <c r="K30" s="2" t="n">
-        <v>306.5485944726447</v>
+        <v>0.7401156959755661</v>
       </c>
       <c r="L30" s="2" t="n">
-        <v>306.5485944726447</v>
+        <v>0.7844179382577898</v>
       </c>
       <c r="M30" s="2" t="n">
-        <v>306.5485944726447</v>
+        <v>0.8287201805400136</v>
       </c>
       <c r="N30" s="2" t="n">
-        <v>306.5485944726447</v>
+        <v>0.8730224228222374</v>
       </c>
       <c r="O30" s="2" t="n">
-        <v>306.5485944726447</v>
+        <v>0.9173246651044611</v>
       </c>
       <c r="P30" s="1" t="inlineStr"/>
     </row>
-    <row r="31" ht="15" customHeight="1">
+    <row r="31" ht="30" customHeight="1">
       <c r="A31" s="1" t="inlineStr">
         <is>
-          <t>Hт_i</t>
+          <t>U_k_i</t>
         </is>
       </c>
       <c r="B31" s="1" t="inlineStr">
         <is>
-          <t>Теоретический напор i-й ступени</t>
+          <t>Окружная скорость концов рабочих лопаток ступени</t>
         </is>
       </c>
       <c r="C31" s="1" t="inlineStr"/>
       <c r="D31" s="2" t="n">
-        <v>16967.12604306373</v>
+        <v>306.5485944726447</v>
       </c>
       <c r="E31" s="2" t="n">
-        <v>19070.88223528092</v>
+        <v>306.5485944726447</v>
       </c>
       <c r="F31" s="2" t="n">
-        <v>21057.52246874931</v>
+        <v>306.5485944726447</v>
       </c>
       <c r="G31" s="2" t="n">
-        <v>22950.09410526995</v>
+        <v>306.5485944726447</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>24759.14168894694</v>
+        <v>306.5485944726447</v>
       </c>
       <c r="I31" s="2" t="n">
-        <v>26487.00632294096</v>
+        <v>306.5485944726447</v>
       </c>
       <c r="J31" s="2" t="n">
-        <v>28125.52905279903</v>
+        <v>306.5485944726447</v>
       </c>
       <c r="K31" s="2" t="n">
-        <v>29654.33031092169</v>
+        <v>306.5485944726447</v>
       </c>
       <c r="L31" s="2" t="n">
-        <v>31044.54895603916</v>
+        <v>306.5485944726447</v>
       </c>
       <c r="M31" s="2" t="n">
-        <v>32256.73667984891</v>
+        <v>306.5485944726447</v>
       </c>
       <c r="N31" s="2" t="n">
-        <v>33239.72047130691</v>
+        <v>306.5485944726447</v>
       </c>
       <c r="O31" s="2" t="n">
-        <v>33933.38931404932</v>
+        <v>306.5485944726447</v>
       </c>
       <c r="P31" s="1" t="inlineStr"/>
     </row>
     <row r="32" ht="15" customHeight="1">
       <c r="A32" s="1" t="inlineStr">
         <is>
-          <t>L_z_i</t>
+          <t>Hт_i</t>
         </is>
       </c>
       <c r="B32" s="1" t="inlineStr">
         <is>
-          <t>Действительная работа сжатия i-й ступени</t>
+          <t>Теоретический напор i-й ступени</t>
         </is>
       </c>
       <c r="C32" s="1" t="inlineStr"/>
       <c r="D32" s="2" t="n">
-        <v>16797.45478263309</v>
+        <v>16967.12604306373</v>
       </c>
       <c r="E32" s="2" t="n">
-        <v>18689.4645905753</v>
+        <v>19070.88223528092</v>
       </c>
       <c r="F32" s="2" t="n">
-        <v>20425.79679468683</v>
+        <v>21057.52246874931</v>
       </c>
       <c r="G32" s="2" t="n">
-        <v>22032.09034105915</v>
+        <v>22950.09410526995</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>23521.18460449959</v>
+        <v>24759.14168894694</v>
       </c>
       <c r="I32" s="2" t="n">
-        <v>24897.7859435645</v>
+        <v>26487.00632294096</v>
       </c>
       <c r="J32" s="2" t="n">
-        <v>26437.99730963109</v>
+        <v>28125.52905279903</v>
       </c>
       <c r="K32" s="2" t="n">
-        <v>27875.07049226639</v>
+        <v>29654.33031092169</v>
       </c>
       <c r="L32" s="2" t="n">
-        <v>29181.87601867681</v>
+        <v>31044.54895603916</v>
       </c>
       <c r="M32" s="2" t="n">
-        <v>30321.33247905798</v>
+        <v>32256.73667984891</v>
       </c>
       <c r="N32" s="2" t="n">
-        <v>31245.33724302849</v>
+        <v>33239.72047130691</v>
       </c>
       <c r="O32" s="2" t="n">
-        <v>31897.38595520635</v>
+        <v>33933.38931404932</v>
       </c>
       <c r="P32" s="1" t="inlineStr"/>
     </row>
     <row r="33" ht="15" customHeight="1">
       <c r="A33" s="1" t="inlineStr">
         <is>
-          <t>H_ад_i</t>
+          <t>L_z_i</t>
         </is>
       </c>
       <c r="B33" s="1" t="inlineStr">
         <is>
-          <t>Адиабатическая работа сжатия i-й ступени</t>
+          <t>Действительная работа сжатия i-й ступени</t>
         </is>
       </c>
       <c r="C33" s="1" t="inlineStr"/>
       <c r="D33" s="2" t="n">
-        <v>13701.87693398603</v>
+        <v>16797.45478263309</v>
       </c>
       <c r="E33" s="2" t="n">
-        <v>15617.01385068403</v>
+        <v>18689.4645905753</v>
       </c>
       <c r="F33" s="2" t="n">
-        <v>17413.88007155858</v>
+        <v>20425.79679468683</v>
       </c>
       <c r="G33" s="2" t="n">
-        <v>19087.25918979651</v>
+        <v>22032.09034105915</v>
       </c>
       <c r="H33" s="2" t="n">
-        <v>20623.27203085376</v>
+        <v>23521.18460449959</v>
       </c>
       <c r="I33" s="2" t="n">
-        <v>22003.16976086839</v>
+        <v>24897.7859435645</v>
       </c>
       <c r="J33" s="2" t="n">
-        <v>23450.49881419504</v>
+        <v>26437.99730963109</v>
       </c>
       <c r="K33" s="2" t="n">
-        <v>24708.63115599736</v>
+        <v>27875.07049226639</v>
       </c>
       <c r="L33" s="2" t="n">
-        <v>25732.59482627098</v>
+        <v>29181.87601867681</v>
       </c>
       <c r="M33" s="2" t="n">
-        <v>26471.29676564151</v>
+        <v>30321.33247905798</v>
       </c>
       <c r="N33" s="2" t="n">
-        <v>26869.11978064452</v>
+        <v>31245.33724302849</v>
       </c>
       <c r="O33" s="2" t="n">
-        <v>26870.38869889748</v>
+        <v>31897.38595520635</v>
       </c>
       <c r="P33" s="1" t="inlineStr"/>
     </row>
     <row r="34" ht="15" customHeight="1">
       <c r="A34" s="1" t="inlineStr">
         <is>
-          <t>ΔT_полн_i</t>
+          <t>H_ад_i</t>
         </is>
       </c>
       <c r="B34" s="1" t="inlineStr">
         <is>
-          <t>Повышение полной температуры в ступени</t>
+          <t>Адиабатическая работа сжатия i-й ступени</t>
         </is>
       </c>
       <c r="C34" s="1" t="inlineStr"/>
       <c r="D34" s="2" t="n">
-        <v>16.6972711556989</v>
+        <v>13701.87693398603</v>
       </c>
       <c r="E34" s="2" t="n">
-        <v>18.50442038670822</v>
+        <v>15617.01385068403</v>
       </c>
       <c r="F34" s="2" t="n">
-        <v>20.11894020580701</v>
+        <v>17413.88007155858</v>
       </c>
       <c r="G34" s="2" t="n">
-        <v>21.64822137575578</v>
+        <v>19087.25918979651</v>
       </c>
       <c r="H34" s="2" t="n">
-        <v>22.99361339494931</v>
+        <v>20623.27203085376</v>
       </c>
       <c r="I34" s="2" t="n">
-        <v>24.21836985820667</v>
+        <v>22003.16976086839</v>
       </c>
       <c r="J34" s="2" t="n">
-        <v>25.542462618911</v>
+        <v>23450.49881419504</v>
       </c>
       <c r="K34" s="2" t="n">
-        <v>26.74370321551575</v>
+        <v>24708.63115599736</v>
       </c>
       <c r="L34" s="2" t="n">
-        <v>27.75136266990286</v>
+        <v>25732.59482627098</v>
       </c>
       <c r="M34" s="2" t="n">
-        <v>28.63014872286476</v>
+        <v>26471.29676564151</v>
       </c>
       <c r="N34" s="2" t="n">
-        <v>29.28231493183464</v>
+        <v>26869.11978064452</v>
       </c>
       <c r="O34" s="2" t="n">
-        <v>29.65175826002295</v>
+        <v>26870.38869889748</v>
       </c>
       <c r="P34" s="1" t="inlineStr"/>
     </row>
     <row r="35" ht="15" customHeight="1">
       <c r="A35" s="1" t="inlineStr">
         <is>
-          <t>T3_полн_i</t>
+          <t>ΔT_полн_i</t>
         </is>
       </c>
       <c r="B35" s="1" t="inlineStr">
         <is>
-          <t>Полная температура на выходе из ступени</t>
+          <t>Повышение полной температуры в ступени</t>
         </is>
       </c>
       <c r="C35" s="1" t="inlineStr"/>
       <c r="D35" s="2" t="n">
-        <v>304.6972711556989</v>
+        <v>16.6972711556989</v>
       </c>
       <c r="E35" s="2" t="n">
-        <v>342.7216074711233</v>
+        <v>18.50442038670822</v>
       </c>
       <c r="F35" s="2" t="n">
-        <v>380.5533143746371</v>
+        <v>20.11894020580701</v>
       </c>
       <c r="G35" s="2" t="n">
-        <v>418.299782629001</v>
+        <v>21.64822137575578</v>
       </c>
       <c r="H35" s="2" t="n">
-        <v>455.8623617326095</v>
+        <v>22.99361339494931</v>
       </c>
       <c r="I35" s="2" t="n">
-        <v>493.3043052802819</v>
+        <v>24.21836985820667</v>
       </c>
       <c r="J35" s="2" t="n">
-        <v>530.8455851254013</v>
+        <v>25.542462618911</v>
       </c>
       <c r="K35" s="2" t="n">
-        <v>568.2640128064211</v>
+        <v>26.74370321551575</v>
       </c>
       <c r="L35" s="2" t="n">
-        <v>605.4888593452233</v>
+        <v>27.75136266990286</v>
       </c>
       <c r="M35" s="2" t="n">
-        <v>642.5848324826002</v>
+        <v>28.63014872286476</v>
       </c>
       <c r="N35" s="2" t="n">
-        <v>679.4541857759853</v>
+        <v>29.28231493183464</v>
       </c>
       <c r="O35" s="2" t="n">
-        <v>716.0408161885885</v>
+        <v>29.65175826002295</v>
       </c>
       <c r="P35" s="1" t="inlineStr"/>
     </row>
-    <row r="36" ht="30" customHeight="1">
+    <row r="36" ht="15" customHeight="1">
       <c r="A36" s="1" t="inlineStr">
         <is>
-          <t>T1_полн_i_plus_1</t>
+          <t>T3_полн_i</t>
         </is>
       </c>
       <c r="B36" s="1" t="inlineStr">
         <is>
-          <t>Полная температура на входе в следующую ступень</t>
+          <t>Полная температура на выходе из ступени</t>
         </is>
       </c>
       <c r="C36" s="1" t="inlineStr"/>
@@ -1790,115 +1768,115 @@
       </c>
       <c r="P36" s="1" t="inlineStr"/>
     </row>
-    <row r="37" ht="15" customHeight="1">
+    <row r="37" ht="30" customHeight="1">
       <c r="A37" s="1" t="inlineStr">
         <is>
-          <t>π_полн_i</t>
+          <t>T1_полн_i_plus_1</t>
         </is>
       </c>
       <c r="B37" s="1" t="inlineStr">
         <is>
-          <t>Степень повышения полного давления в ступени</t>
+          <t>Полная температура на входе в следующую ступень</t>
         </is>
       </c>
       <c r="C37" s="1" t="inlineStr"/>
       <c r="D37" s="2" t="n">
-        <v>1.175559285399187</v>
+        <v>304.6972711556989</v>
       </c>
       <c r="E37" s="2" t="n">
-        <v>1.177892225128341</v>
+        <v>342.7216074711233</v>
       </c>
       <c r="F37" s="2" t="n">
-        <v>1.178483449737299</v>
+        <v>380.5533143746371</v>
       </c>
       <c r="G37" s="2" t="n">
-        <v>1.177740365938578</v>
+        <v>418.299782629001</v>
       </c>
       <c r="H37" s="2" t="n">
-        <v>1.175894000936239</v>
+        <v>455.8623617326095</v>
       </c>
       <c r="I37" s="2" t="n">
-        <v>1.173036766366976</v>
+        <v>493.3043052802819</v>
       </c>
       <c r="J37" s="2" t="n">
-        <v>1.171122407075676</v>
+        <v>530.8455851254013</v>
       </c>
       <c r="K37" s="2" t="n">
-        <v>1.168108071555353</v>
+        <v>568.2640128064211</v>
       </c>
       <c r="L37" s="2" t="n">
-        <v>1.163909173397865</v>
+        <v>605.4888593452233</v>
       </c>
       <c r="M37" s="2" t="n">
-        <v>1.158409204291314</v>
+        <v>642.5848324826002</v>
       </c>
       <c r="N37" s="2" t="n">
-        <v>1.151515127689758</v>
+        <v>679.4541857759853</v>
       </c>
       <c r="O37" s="2" t="n">
-        <v>1.143155604508661</v>
+        <v>716.0408161885885</v>
       </c>
       <c r="P37" s="1" t="inlineStr"/>
     </row>
     <row r="38" ht="15" customHeight="1">
       <c r="A38" s="1" t="inlineStr">
         <is>
-          <t>P3_полн_i</t>
+          <t>π_полн_i</t>
         </is>
       </c>
       <c r="B38" s="1" t="inlineStr">
         <is>
-          <t>Полное давление на выходе из ступени</t>
+          <t>Степень повышения полного давления в ступени</t>
         </is>
       </c>
       <c r="C38" s="1" t="inlineStr"/>
       <c r="D38" s="2" t="n">
-        <v>117900.225235523</v>
+        <v>1.175559285399187</v>
       </c>
       <c r="E38" s="2" t="n">
-        <v>305713.5403829411</v>
+        <v>1.177892225128341</v>
       </c>
       <c r="F38" s="2" t="n">
-        <v>493540.4789454677</v>
+        <v>1.178483449737299</v>
       </c>
       <c r="G38" s="2" t="n">
-        <v>680784.4350698986</v>
+        <v>1.177740365938578</v>
       </c>
       <c r="H38" s="2" t="n">
-        <v>866978.2776241348</v>
+        <v>1.175894000936239</v>
       </c>
       <c r="I38" s="2" t="n">
-        <v>1051677.76500542</v>
+        <v>1.173036766366976</v>
       </c>
       <c r="J38" s="2" t="n">
-        <v>1236462.704180656</v>
+        <v>1.171122407075676</v>
       </c>
       <c r="K38" s="2" t="n">
-        <v>1419301.401627094</v>
+        <v>1.168108071555353</v>
       </c>
       <c r="L38" s="2" t="n">
-        <v>1599552.097199386</v>
+        <v>1.163909173397865</v>
       </c>
       <c r="M38" s="2" t="n">
-        <v>1776470.195601449</v>
+        <v>1.158409204291314</v>
       </c>
       <c r="N38" s="2" t="n">
-        <v>1949276.618580578</v>
+        <v>1.151515127689758</v>
       </c>
       <c r="O38" s="2" t="n">
-        <v>2117173.208233083</v>
+        <v>1.143155604508661</v>
       </c>
       <c r="P38" s="1" t="inlineStr"/>
     </row>
     <row r="39" ht="15" customHeight="1">
       <c r="A39" s="1" t="inlineStr">
         <is>
-          <t>P1_полн_i_plus_1</t>
+          <t>P3_полн_i</t>
         </is>
       </c>
       <c r="B39" s="1" t="inlineStr">
         <is>
-          <t>Полное давление перед следующей ступенью</t>
+          <t>Полное давление на выходе из ступени</t>
         </is>
       </c>
       <c r="C39" s="1" t="inlineStr"/>
@@ -1940,2155 +1918,2205 @@
       </c>
       <c r="P39" s="1" t="inlineStr"/>
     </row>
-    <row r="40" ht="30" customHeight="1">
+    <row r="40" ht="15" customHeight="1">
       <c r="A40" s="1" t="inlineStr">
         <is>
-          <t>a_кр_1_i</t>
+          <t>P1_полн_i_plus_1</t>
         </is>
       </c>
       <c r="B40" s="1" t="inlineStr">
         <is>
-          <t>Критическая скорость потока на входе в ступень</t>
+          <t>Полное давление перед следующей ступенью</t>
         </is>
       </c>
       <c r="C40" s="1" t="inlineStr"/>
       <c r="D40" s="2" t="n">
-        <v>310.7487734256569</v>
+        <v>117900.225235523</v>
       </c>
       <c r="E40" s="2" t="n">
-        <v>329.6005504723648</v>
+        <v>305713.5403829411</v>
       </c>
       <c r="F40" s="2" t="n">
-        <v>347.3735553312965</v>
+        <v>493540.4789454677</v>
       </c>
       <c r="G40" s="2" t="n">
-        <v>364.3350972913221</v>
+        <v>680784.4350698986</v>
       </c>
       <c r="H40" s="2" t="n">
-        <v>380.445728537063</v>
+        <v>866978.2776241348</v>
       </c>
       <c r="I40" s="2" t="n">
-        <v>395.8808441843627</v>
+        <v>1051677.76500542</v>
       </c>
       <c r="J40" s="2" t="n">
-        <v>410.6535144715717</v>
+        <v>1236462.704180656</v>
       </c>
       <c r="K40" s="2" t="n">
-        <v>424.8775489240568</v>
+        <v>1419301.401627094</v>
       </c>
       <c r="L40" s="2" t="n">
-        <v>438.5475167594254</v>
+        <v>1599552.097199386</v>
       </c>
       <c r="M40" s="2" t="n">
-        <v>451.8304907351089</v>
+        <v>1776470.195601449</v>
       </c>
       <c r="N40" s="2" t="n">
-        <v>464.6939992401076</v>
+        <v>1949276.618580578</v>
       </c>
       <c r="O40" s="2" t="n">
-        <v>477.1612274741949</v>
+        <v>2117173.208233083</v>
       </c>
       <c r="P40" s="1" t="inlineStr"/>
     </row>
     <row r="41" ht="30" customHeight="1">
       <c r="A41" s="1" t="inlineStr">
         <is>
-          <t>a_кр_3_i</t>
+          <t>a_кр_1_i</t>
         </is>
       </c>
       <c r="B41" s="1" t="inlineStr">
         <is>
-          <t>Критическая скорость потока на выходе из ступени</t>
+          <t>Критическая скорость потока на входе в ступень</t>
         </is>
       </c>
       <c r="C41" s="1" t="inlineStr"/>
       <c r="D41" s="2" t="n">
-        <v>319.5245220964998</v>
+        <v>310.7487734256569</v>
       </c>
       <c r="E41" s="2" t="n">
-        <v>338.7305720009615</v>
+        <v>329.6005504723648</v>
       </c>
       <c r="F41" s="2" t="n">
-        <v>356.8651842260853</v>
+        <v>347.3735553312965</v>
       </c>
       <c r="G41" s="2" t="n">
-        <v>373.9886443846121</v>
+        <v>364.3350972913221</v>
       </c>
       <c r="H41" s="2" t="n">
-        <v>390.2609971889856</v>
+        <v>380.445728537063</v>
       </c>
       <c r="I41" s="2" t="n">
-        <v>405.7485774550155</v>
+        <v>395.8808441843627</v>
       </c>
       <c r="J41" s="2" t="n">
-        <v>420.6690040022493</v>
+        <v>410.6535144715717</v>
       </c>
       <c r="K41" s="2" t="n">
-        <v>434.9371010045424</v>
+        <v>424.8775489240568</v>
       </c>
       <c r="L41" s="2" t="n">
-        <v>448.7045308344883</v>
+        <v>438.5475167594254</v>
       </c>
       <c r="M41" s="2" t="n">
-        <v>461.97472048923</v>
+        <v>451.8304907351089</v>
       </c>
       <c r="N41" s="2" t="n">
-        <v>474.7446295243685</v>
+        <v>464.6939992401076</v>
       </c>
       <c r="O41" s="2" t="n">
-        <v>487.0511463806778</v>
+        <v>477.1612274741949</v>
       </c>
       <c r="P41" s="1" t="inlineStr"/>
     </row>
     <row r="42" ht="30" customHeight="1">
       <c r="A42" s="1" t="inlineStr">
         <is>
-          <t>r_ср1_отн_i</t>
+          <t>a_кр_3_i</t>
         </is>
       </c>
       <c r="B42" s="1" t="inlineStr">
         <is>
-          <t>Относительный средний радиус на входе в ступень</t>
+          <t>Критическая скорость потока на выходе из ступени</t>
         </is>
       </c>
       <c r="C42" s="1" t="inlineStr"/>
       <c r="D42" s="2" t="n">
-        <v>0.7697077367416805</v>
+        <v>319.5245220964998</v>
       </c>
       <c r="E42" s="2" t="n">
-        <v>0.7826118504833496</v>
+        <v>338.7305720009615</v>
       </c>
       <c r="F42" s="2" t="n">
-        <v>0.7965395820078109</v>
+        <v>356.8651842260853</v>
       </c>
       <c r="G42" s="2" t="n">
-        <v>0.8114382241209841</v>
+        <v>373.9886443846121</v>
       </c>
       <c r="H42" s="2" t="n">
-        <v>0.8272553209833634</v>
+        <v>390.2609971889856</v>
       </c>
       <c r="I42" s="2" t="n">
-        <v>0.8439392331780717</v>
+        <v>405.7485774550155</v>
       </c>
       <c r="J42" s="2" t="n">
-        <v>0.8614395980974688</v>
+        <v>420.6690040022493</v>
       </c>
       <c r="K42" s="2" t="n">
-        <v>0.8797076910626043</v>
+        <v>434.9371010045424</v>
       </c>
       <c r="L42" s="2" t="n">
-        <v>0.8986966957379452</v>
+        <v>448.7045308344883</v>
       </c>
       <c r="M42" s="2" t="n">
-        <v>0.9183618942536413</v>
+        <v>461.97472048923</v>
       </c>
       <c r="N42" s="2" t="n">
-        <v>0.9386607882377982</v>
+        <v>474.7446295243685</v>
       </c>
       <c r="O42" s="2" t="n">
-        <v>0.9595531619480527</v>
+        <v>487.0511463806778</v>
       </c>
       <c r="P42" s="1" t="inlineStr"/>
     </row>
     <row r="43" ht="30" customHeight="1">
       <c r="A43" s="1" t="inlineStr">
         <is>
-          <t>c_u1_отн_i</t>
+          <t>r_ср1_отн_i</t>
         </is>
       </c>
       <c r="B43" s="1" t="inlineStr">
         <is>
-          <t>Безразмерная окружная составляющая скорости на входе</t>
+          <t>Относительный средний радиус на входе в ступень</t>
         </is>
       </c>
       <c r="C43" s="1" t="inlineStr"/>
       <c r="D43" s="2" t="n">
-        <v>0.2675658145409672</v>
+        <v>0.7697077367416805</v>
       </c>
       <c r="E43" s="2" t="n">
-        <v>0.2616490023434986</v>
+        <v>0.7826118504833496</v>
       </c>
       <c r="F43" s="2" t="n">
-        <v>0.2576095825081036</v>
+        <v>0.7965395820078109</v>
       </c>
       <c r="G43" s="2" t="n">
-        <v>0.2552316373223689</v>
+        <v>0.8114382241209841</v>
       </c>
       <c r="H43" s="2" t="n">
-        <v>0.2543820897171053</v>
+        <v>0.8272553209833634</v>
       </c>
       <c r="I43" s="2" t="n">
-        <v>0.2549786247517394</v>
+        <v>0.8439392331780717</v>
       </c>
       <c r="J43" s="2" t="n">
-        <v>0.2570008412996226</v>
+        <v>0.8614395980974688</v>
       </c>
       <c r="K43" s="2" t="n">
-        <v>0.2604957112317619</v>
+        <v>0.8797076910626043</v>
       </c>
       <c r="L43" s="2" t="n">
-        <v>0.2655491738474892</v>
+        <v>0.8986966957379452</v>
       </c>
       <c r="M43" s="2" t="n">
-        <v>0.2722944518517804</v>
+        <v>0.9183618942536413</v>
       </c>
       <c r="N43" s="2" t="n">
-        <v>0.2809134165726251</v>
+        <v>0.9386607882377982</v>
       </c>
       <c r="O43" s="2" t="n">
-        <v>0.2916156103246133</v>
+        <v>0.9595531619480527</v>
       </c>
       <c r="P43" s="1" t="inlineStr"/>
     </row>
-    <row r="44" ht="15" customHeight="1">
+    <row r="44" ht="30" customHeight="1">
       <c r="A44" s="1" t="inlineStr">
         <is>
-          <t>α_1_i</t>
+          <t>c_u1_отн_i</t>
         </is>
       </c>
       <c r="B44" s="1" t="inlineStr">
         <is>
-          <t>Угол абсолютной скорости на входе в РК</t>
+          <t>Безразмерная окружная составляющая скорости на входе</t>
         </is>
       </c>
       <c r="C44" s="1" t="inlineStr"/>
       <c r="D44" s="2" t="n">
-        <v>1.180296158977294</v>
+        <v>0.2675658145409672</v>
       </c>
       <c r="E44" s="2" t="n">
-        <v>1.17354769367773</v>
+        <v>0.2616490023434986</v>
       </c>
       <c r="F44" s="2" t="n">
-        <v>1.163593381597623</v>
+        <v>0.2576095825081036</v>
       </c>
       <c r="G44" s="2" t="n">
-        <v>1.15038850731903</v>
+        <v>0.2552316373223689</v>
       </c>
       <c r="H44" s="2" t="n">
-        <v>1.133775838988559</v>
+        <v>0.2543820897171053</v>
       </c>
       <c r="I44" s="2" t="n">
-        <v>1.113517639280561</v>
+        <v>0.2549786247517394</v>
       </c>
       <c r="J44" s="2" t="n">
-        <v>1.089269891516375</v>
+        <v>0.2570008412996226</v>
       </c>
       <c r="K44" s="2" t="n">
-        <v>1.060567821445653</v>
+        <v>0.2604957112317619</v>
       </c>
       <c r="L44" s="2" t="n">
-        <v>1.026876578551888</v>
+        <v>0.2655491738474892</v>
       </c>
       <c r="M44" s="2" t="n">
-        <v>0.9876014776906153</v>
+        <v>0.2722944518517804</v>
       </c>
       <c r="N44" s="2" t="n">
-        <v>0.9421326350930992</v>
+        <v>0.2809134165726251</v>
       </c>
       <c r="O44" s="2" t="n">
-        <v>0.8899613152251319</v>
+        <v>0.2916156103246133</v>
       </c>
       <c r="P44" s="1" t="inlineStr"/>
     </row>
     <row r="45" ht="15" customHeight="1">
       <c r="A45" s="1" t="inlineStr">
         <is>
-          <t>c_a1_i</t>
+          <t>α_1_i</t>
         </is>
       </c>
       <c r="B45" s="1" t="inlineStr">
         <is>
-          <t>Осевая скорость на входе в ступень</t>
+          <t>Угол абсолютной скорости на входе в РК</t>
         </is>
       </c>
       <c r="C45" s="1" t="inlineStr"/>
       <c r="D45" s="2" t="n">
-        <v>199.2565864072191</v>
+        <v>1.180296158977294</v>
       </c>
       <c r="E45" s="2" t="n">
-        <v>191.1748507347584</v>
+        <v>1.17354769367773</v>
       </c>
       <c r="F45" s="2" t="n">
-        <v>183.0931150622978</v>
+        <v>1.163593381597623</v>
       </c>
       <c r="G45" s="2" t="n">
-        <v>175.0113793898372</v>
+        <v>1.15038850731903</v>
       </c>
       <c r="H45" s="2" t="n">
-        <v>166.9296437173765</v>
+        <v>1.133775838988559</v>
       </c>
       <c r="I45" s="2" t="n">
-        <v>158.8479080449159</v>
+        <v>1.113517639280561</v>
       </c>
       <c r="J45" s="2" t="n">
-        <v>150.7661723724553</v>
+        <v>1.089269891516375</v>
       </c>
       <c r="K45" s="2" t="n">
-        <v>142.6844366999946</v>
+        <v>1.060567821445653</v>
       </c>
       <c r="L45" s="2" t="n">
-        <v>134.602701027534</v>
+        <v>1.026876578551888</v>
       </c>
       <c r="M45" s="2" t="n">
-        <v>126.5209653550734</v>
+        <v>0.9876014776906153</v>
       </c>
       <c r="N45" s="2" t="n">
-        <v>118.4392296826127</v>
+        <v>0.9421326350930992</v>
       </c>
       <c r="O45" s="2" t="n">
-        <v>110.3574940101521</v>
+        <v>0.8899613152251319</v>
       </c>
       <c r="P45" s="1" t="inlineStr"/>
     </row>
     <row r="46" ht="15" customHeight="1">
       <c r="A46" s="1" t="inlineStr">
         <is>
-          <t>λ_1_i</t>
+          <t>c_a1_i</t>
         </is>
       </c>
       <c r="B46" s="1" t="inlineStr">
         <is>
-          <t>Приведенная скорость на входе в ступень</t>
+          <t>Осевая скорость на входе в ступень</t>
         </is>
       </c>
       <c r="C46" s="1" t="inlineStr"/>
       <c r="D46" s="2" t="n">
-        <v>0.6934155588636786</v>
+        <v>199.2565864072191</v>
       </c>
       <c r="E46" s="2" t="n">
-        <v>0.6290007738192603</v>
+        <v>191.1748507347584</v>
       </c>
       <c r="F46" s="2" t="n">
-        <v>0.574014360850995</v>
+        <v>183.0931150622978</v>
       </c>
       <c r="G46" s="2" t="n">
-        <v>0.5261763607748462</v>
+        <v>175.0113793898372</v>
       </c>
       <c r="H46" s="2" t="n">
-        <v>0.4842889204649947</v>
+        <v>166.9296437173765</v>
       </c>
       <c r="I46" s="2" t="n">
-        <v>0.4471981639398266</v>
+        <v>158.8479080449159</v>
       </c>
       <c r="J46" s="2" t="n">
-        <v>0.4142409216095714</v>
+        <v>150.7661723724553</v>
       </c>
       <c r="K46" s="2" t="n">
-        <v>0.3848409007715879</v>
+        <v>142.6844366999946</v>
       </c>
       <c r="L46" s="2" t="n">
-        <v>0.358692486055376</v>
+        <v>134.602701027534</v>
       </c>
       <c r="M46" s="2" t="n">
-        <v>0.335469182640696</v>
+        <v>126.5209653550734</v>
       </c>
       <c r="N46" s="2" t="n">
-        <v>0.3151227911923925</v>
+        <v>118.4392296826127</v>
       </c>
       <c r="O46" s="2" t="n">
-        <v>0.2976385445704193</v>
+        <v>110.3574940101521</v>
       </c>
       <c r="P46" s="1" t="inlineStr"/>
     </row>
     <row r="47" ht="15" customHeight="1">
       <c r="A47" s="1" t="inlineStr">
         <is>
-          <t>q_1_i</t>
+          <t>λ_1_i</t>
         </is>
       </c>
       <c r="B47" s="1" t="inlineStr">
         <is>
-          <t>Газодинамическая функция расхода на входе</t>
+          <t>Приведенная скорость на входе в ступень</t>
         </is>
       </c>
       <c r="C47" s="1" t="inlineStr"/>
       <c r="D47" s="2" t="n">
-        <v>0.8876763917513479</v>
+        <v>0.6934155588636786</v>
       </c>
       <c r="E47" s="2" t="n">
-        <v>0.8367187220902095</v>
+        <v>0.6290007738192603</v>
       </c>
       <c r="F47" s="2" t="n">
-        <v>0.7864274238623349</v>
+        <v>0.574014360850995</v>
       </c>
       <c r="G47" s="2" t="n">
-        <v>0.7378118937190112</v>
+        <v>0.5261763607748462</v>
       </c>
       <c r="H47" s="2" t="n">
-        <v>0.6918457719220593</v>
+        <v>0.4842889204649947</v>
       </c>
       <c r="I47" s="2" t="n">
-        <v>0.6486182523825925</v>
+        <v>0.4471981639398266</v>
       </c>
       <c r="J47" s="2" t="n">
-        <v>0.608383057920596</v>
+        <v>0.4142409216095714</v>
       </c>
       <c r="K47" s="2" t="n">
-        <v>0.571105333397828</v>
+        <v>0.3848409007715879</v>
       </c>
       <c r="L47" s="2" t="n">
-        <v>0.5369562412061231</v>
+        <v>0.358692486055376</v>
       </c>
       <c r="M47" s="2" t="n">
-        <v>0.5058253851811065</v>
+        <v>0.335469182640696</v>
       </c>
       <c r="N47" s="2" t="n">
-        <v>0.4780003690667221</v>
+        <v>0.3151227911923925</v>
       </c>
       <c r="O47" s="2" t="n">
-        <v>0.4537118711400231</v>
+        <v>0.2976385445704193</v>
       </c>
       <c r="P47" s="1" t="inlineStr"/>
     </row>
     <row r="48" ht="15" customHeight="1">
       <c r="A48" s="1" t="inlineStr">
         <is>
-          <t>F_1_i</t>
+          <t>q_1_i</t>
         </is>
       </c>
       <c r="B48" s="1" t="inlineStr">
         <is>
-          <t>Кольцевая площадь на входе в ступень</t>
+          <t>Газодинамическая функция расхода на входе</t>
         </is>
       </c>
       <c r="C48" s="1" t="inlineStr"/>
       <c r="D48" s="2" t="n">
-        <v>0.3009117955899137</v>
+        <v>0.8876763917513479</v>
       </c>
       <c r="E48" s="2" t="n">
-        <v>0.1312547944711213</v>
+        <v>0.8367187220902095</v>
       </c>
       <c r="F48" s="2" t="n">
-        <v>0.09163894407812001</v>
+        <v>0.7864274238623349</v>
       </c>
       <c r="G48" s="2" t="n">
-        <v>0.07466934589439193</v>
+        <v>0.7378118937190112</v>
       </c>
       <c r="H48" s="2" t="n">
-        <v>0.06571582737082768</v>
+        <v>0.6918457719220593</v>
       </c>
       <c r="I48" s="2" t="n">
-        <v>0.06059354891620095</v>
+        <v>0.6486182523825925</v>
       </c>
       <c r="J48" s="2" t="n">
-        <v>0.05763976482606604</v>
+        <v>0.608383057920596</v>
       </c>
       <c r="K48" s="2" t="n">
-        <v>0.05609774057576191</v>
+        <v>0.571105333397828</v>
       </c>
       <c r="L48" s="2" t="n">
-        <v>0.05556606751348679</v>
+        <v>0.5369562412061231</v>
       </c>
       <c r="M48" s="2" t="n">
-        <v>0.05586177064312022</v>
+        <v>0.5058253851811065</v>
       </c>
       <c r="N48" s="2" t="n">
-        <v>0.05687360435199427</v>
+        <v>0.4780003690667221</v>
       </c>
       <c r="O48" s="2" t="n">
-        <v>0.05857117009930012</v>
+        <v>0.4537118711400231</v>
       </c>
       <c r="P48" s="1" t="inlineStr"/>
     </row>
     <row r="49" ht="15" customHeight="1">
       <c r="A49" s="1" t="inlineStr">
         <is>
-          <t>c_a3_отн_i</t>
+          <t>F_1_i</t>
         </is>
       </c>
       <c r="B49" s="1" t="inlineStr">
         <is>
-          <t>Коэффициент расхода на выходе из ступени</t>
+          <t>Кольцевая площадь на входе в ступень</t>
         </is>
       </c>
       <c r="C49" s="1" t="inlineStr"/>
       <c r="D49" s="2" t="n">
-        <v>0.6236363636363637</v>
+        <v>0.3009117955899137</v>
       </c>
       <c r="E49" s="2" t="n">
-        <v>0.5972727272727273</v>
+        <v>0.1312547944711213</v>
       </c>
       <c r="F49" s="2" t="n">
-        <v>0.5709090909090909</v>
+        <v>0.09163894407812001</v>
       </c>
       <c r="G49" s="2" t="n">
-        <v>0.5445454545454546</v>
+        <v>0.07466934589439193</v>
       </c>
       <c r="H49" s="2" t="n">
-        <v>0.5181818181818182</v>
+        <v>0.06571582737082768</v>
       </c>
       <c r="I49" s="2" t="n">
-        <v>0.4918181818181818</v>
+        <v>0.06059354891620095</v>
       </c>
       <c r="J49" s="2" t="n">
-        <v>0.4654545454545455</v>
+        <v>0.05763976482606604</v>
       </c>
       <c r="K49" s="2" t="n">
-        <v>0.4390909090909091</v>
+        <v>0.05609774057576191</v>
       </c>
       <c r="L49" s="2" t="n">
-        <v>0.4127272727272727</v>
+        <v>0.05556606751348679</v>
       </c>
       <c r="M49" s="2" t="n">
-        <v>0.3863636363636364</v>
+        <v>0.05586177064312022</v>
       </c>
       <c r="N49" s="2" t="n">
-        <v>0.36</v>
+        <v>0.05687360435199427</v>
       </c>
       <c r="O49" s="2" t="n">
-        <v>0.3336363636363636</v>
+        <v>0.05857117009930012</v>
       </c>
       <c r="P49" s="1" t="inlineStr"/>
     </row>
     <row r="50" ht="15" customHeight="1">
       <c r="A50" s="1" t="inlineStr">
         <is>
-          <t>c_a3_i</t>
+          <t>c_a3_отн_i</t>
         </is>
       </c>
       <c r="B50" s="1" t="inlineStr">
         <is>
-          <t>Осевая скорость на выходе из ступени</t>
+          <t>Коэффициент расхода на выходе из ступени</t>
         </is>
       </c>
       <c r="C50" s="1" t="inlineStr"/>
       <c r="D50" s="2" t="n">
-        <v>191.1748507347584</v>
+        <v>0.6236363636363637</v>
       </c>
       <c r="E50" s="2" t="n">
-        <v>183.0931150622978</v>
+        <v>0.5972727272727273</v>
       </c>
       <c r="F50" s="2" t="n">
-        <v>175.0113793898372</v>
+        <v>0.5709090909090909</v>
       </c>
       <c r="G50" s="2" t="n">
-        <v>166.9296437173765</v>
+        <v>0.5445454545454546</v>
       </c>
       <c r="H50" s="2" t="n">
-        <v>158.8479080449159</v>
+        <v>0.5181818181818182</v>
       </c>
       <c r="I50" s="2" t="n">
-        <v>150.7661723724553</v>
+        <v>0.4918181818181818</v>
       </c>
       <c r="J50" s="2" t="n">
-        <v>142.6844366999946</v>
+        <v>0.4654545454545455</v>
       </c>
       <c r="K50" s="2" t="n">
-        <v>134.602701027534</v>
+        <v>0.4390909090909091</v>
       </c>
       <c r="L50" s="2" t="n">
-        <v>126.5209653550734</v>
+        <v>0.4127272727272727</v>
       </c>
       <c r="M50" s="2" t="n">
-        <v>118.4392296826127</v>
+        <v>0.3863636363636364</v>
       </c>
       <c r="N50" s="2" t="n">
-        <v>110.3574940101521</v>
+        <v>0.36</v>
       </c>
       <c r="O50" s="2" t="n">
-        <v>102.2757583376915</v>
+        <v>0.3336363636363636</v>
       </c>
       <c r="P50" s="1" t="inlineStr"/>
     </row>
-    <row r="51" ht="30" customHeight="1">
+    <row r="51" ht="15" customHeight="1">
       <c r="A51" s="1" t="inlineStr">
         <is>
-          <t>λ_3_i_0</t>
+          <t>c_a3_i</t>
         </is>
       </c>
       <c r="B51" s="1" t="inlineStr">
         <is>
-          <t>Приведенная скорость на выходе (1-е приближение)</t>
+          <t>Осевая скорость на выходе из ступени</t>
         </is>
       </c>
       <c r="C51" s="1" t="inlineStr"/>
       <c r="D51" s="2" t="n">
-        <v>0.6470187781110718</v>
+        <v>191.1748507347584</v>
       </c>
       <c r="E51" s="2" t="n">
-        <v>0.586173210716883</v>
+        <v>183.0931150622978</v>
       </c>
       <c r="F51" s="2" t="n">
-        <v>0.5340840464310409</v>
+        <v>175.0113793898372</v>
       </c>
       <c r="G51" s="2" t="n">
-        <v>0.4889237180942501</v>
+        <v>166.9296437173765</v>
       </c>
       <c r="H51" s="2" t="n">
-        <v>0.4492521137640234</v>
+        <v>158.8479080449159</v>
       </c>
       <c r="I51" s="2" t="n">
-        <v>0.4141235259565256</v>
+        <v>150.7661723724553</v>
       </c>
       <c r="J51" s="2" t="n">
-        <v>0.3827019947765132</v>
+        <v>142.6844366999946</v>
       </c>
       <c r="K51" s="2" t="n">
-        <v>0.3546465340521764</v>
+        <v>134.602701027534</v>
       </c>
       <c r="L51" s="2" t="n">
-        <v>0.3295241151493359</v>
+        <v>126.5209653550734</v>
       </c>
       <c r="M51" s="2" t="n">
-        <v>0.3071447039852674</v>
+        <v>118.4392296826127</v>
       </c>
       <c r="N51" s="2" t="n">
-        <v>0.2874041760296047</v>
+        <v>110.3574940101521</v>
       </c>
       <c r="O51" s="2" t="n">
-        <v>0.2702406194692441</v>
+        <v>102.2757583376915</v>
       </c>
       <c r="P51" s="1" t="inlineStr"/>
     </row>
-    <row r="52" ht="15" customHeight="1">
+    <row r="52" ht="30" customHeight="1">
       <c r="A52" s="1" t="inlineStr">
         <is>
-          <t>q_3_i</t>
+          <t>λ_3_i_0</t>
         </is>
       </c>
       <c r="B52" s="1" t="inlineStr">
         <is>
-          <t>Газодинамическая функция расхода на выходе</t>
+          <t>Приведенная скорость на выходе (1-е приближение)</t>
         </is>
       </c>
       <c r="C52" s="1" t="inlineStr"/>
       <c r="D52" s="2" t="n">
-        <v>0.8518815630867524</v>
+        <v>0.6470187781110718</v>
       </c>
       <c r="E52" s="2" t="n">
-        <v>0.7980928600064215</v>
+        <v>0.586173210716883</v>
       </c>
       <c r="F52" s="2" t="n">
-        <v>0.7461548093475975</v>
+        <v>0.5340840464310409</v>
       </c>
       <c r="G52" s="2" t="n">
-        <v>0.697097433111779</v>
+        <v>0.4889237180942501</v>
       </c>
       <c r="H52" s="2" t="n">
-        <v>0.6510781569448195</v>
+        <v>0.4492521137640234</v>
       </c>
       <c r="I52" s="2" t="n">
-        <v>0.6082361540873048</v>
+        <v>0.4141235259565256</v>
       </c>
       <c r="J52" s="2" t="n">
-        <v>0.5683324138660786</v>
+        <v>0.3827019947765132</v>
       </c>
       <c r="K52" s="2" t="n">
-        <v>0.5315580405223252</v>
+        <v>0.3546465340521764</v>
       </c>
       <c r="L52" s="2" t="n">
-        <v>0.4977046335060994</v>
+        <v>0.3295241151493359</v>
       </c>
       <c r="M52" s="2" t="n">
-        <v>0.4668911352930197</v>
+        <v>0.3071447039852674</v>
       </c>
       <c r="N52" s="2" t="n">
-        <v>0.439236548039308</v>
+        <v>0.2874041760296047</v>
       </c>
       <c r="O52" s="2" t="n">
-        <v>0.4148482593599832</v>
+        <v>0.2702406194692441</v>
       </c>
       <c r="P52" s="1" t="inlineStr"/>
     </row>
-    <row r="53" ht="30" customHeight="1">
+    <row r="53" ht="15" customHeight="1">
       <c r="A53" s="1" t="inlineStr">
         <is>
-          <t>F_3_i_0</t>
+          <t>q_3_i</t>
         </is>
       </c>
       <c r="B53" s="1" t="inlineStr">
         <is>
-          <t>Кольцевая площадь на выходе (1-е приближение)</t>
+          <t>Газодинамическая функция расхода на выходе</t>
         </is>
       </c>
       <c r="C53" s="1" t="inlineStr"/>
       <c r="D53" s="2" t="n">
-        <v>0.2743520218633287</v>
+        <v>0.8518815630867524</v>
       </c>
       <c r="E53" s="2" t="n">
-        <v>0.1201125559303119</v>
+        <v>0.7980928600064215</v>
       </c>
       <c r="F53" s="2" t="n">
-        <v>0.08421335092644007</v>
+        <v>0.7461548093475975</v>
       </c>
       <c r="G53" s="2" t="n">
-        <v>0.06891030788799436</v>
+        <v>0.697097433111779</v>
       </c>
       <c r="H53" s="2" t="n">
-        <v>0.06094200283320824</v>
+        <v>0.6510781569448195</v>
       </c>
       <c r="I53" s="2" t="n">
-        <v>0.05648887770844104</v>
+        <v>0.6082361540873048</v>
       </c>
       <c r="J53" s="2" t="n">
-        <v>0.05400111276892245</v>
+        <v>0.5683324138660786</v>
       </c>
       <c r="K53" s="2" t="n">
-        <v>0.05285615546139544</v>
+        <v>0.5315580405223252</v>
       </c>
       <c r="L53" s="2" t="n">
-        <v>0.05272852012561755</v>
+        <v>0.4977046335060994</v>
       </c>
       <c r="M53" s="2" t="n">
-        <v>0.05344840716338015</v>
+        <v>0.4668911352930197</v>
       </c>
       <c r="N53" s="2" t="n">
-        <v>0.05494609946622748</v>
+        <v>0.439236548039308</v>
       </c>
       <c r="O53" s="2" t="n">
-        <v>0.05723387284064647</v>
+        <v>0.4148482593599832</v>
       </c>
       <c r="P53" s="1" t="inlineStr"/>
     </row>
     <row r="54" ht="30" customHeight="1">
       <c r="A54" s="1" t="inlineStr">
         <is>
-          <t>d3_отн_i_0</t>
+          <t>F_3_i_0</t>
         </is>
       </c>
       <c r="B54" s="1" t="inlineStr">
         <is>
-          <t>Относительный диаметр втулки на выходе (1-е приближение)</t>
+          <t>Кольцевая площадь на выходе (1-е приближение)</t>
         </is>
       </c>
       <c r="C54" s="1" t="inlineStr"/>
       <c r="D54" s="2" t="n">
-        <v>0.496259530291237</v>
+        <v>0.2743520218633287</v>
       </c>
       <c r="E54" s="2" t="n">
-        <v>0.8185445247137505</v>
+        <v>0.1201125559303119</v>
       </c>
       <c r="F54" s="2" t="n">
-        <v>0.8767216867967569</v>
+        <v>0.08421335092644007</v>
       </c>
       <c r="G54" s="2" t="n">
-        <v>0.9003793199997074</v>
+        <v>0.06891030788799436</v>
       </c>
       <c r="H54" s="2" t="n">
-        <v>0.9124550510696275</v>
+        <v>0.06094200283320824</v>
       </c>
       <c r="I54" s="2" t="n">
-        <v>0.9191345262736552</v>
+        <v>0.05648887770844104</v>
       </c>
       <c r="J54" s="2" t="n">
-        <v>0.9228450067431002</v>
+        <v>0.05400111276892245</v>
       </c>
       <c r="K54" s="2" t="n">
-        <v>0.9245476971002226</v>
+        <v>0.05285615546139544</v>
       </c>
       <c r="L54" s="2" t="n">
-        <v>0.9247373120971561</v>
+        <v>0.05272852012561755</v>
       </c>
       <c r="M54" s="2" t="n">
-        <v>0.9236673388761331</v>
+        <v>0.05344840716338015</v>
       </c>
       <c r="N54" s="2" t="n">
-        <v>0.9214373268864954</v>
+        <v>0.05494609946622748</v>
       </c>
       <c r="O54" s="2" t="n">
-        <v>0.9180204543028089</v>
+        <v>0.05723387284064647</v>
       </c>
       <c r="P54" s="1" t="inlineStr"/>
     </row>
     <row r="55" ht="30" customHeight="1">
       <c r="A55" s="1" t="inlineStr">
         <is>
-          <t>r_ср3_отн_i</t>
+          <t>d3_отн_i_0</t>
         </is>
       </c>
       <c r="B55" s="1" t="inlineStr">
         <is>
-          <t>Относительный средний радиус на выходе из ступени</t>
+          <t>Относительный диаметр втулки на выходе (1-е приближение)</t>
         </is>
       </c>
       <c r="C55" s="1" t="inlineStr"/>
       <c r="D55" s="2" t="n">
-        <v>0.7914114817012881</v>
+        <v>0.496259530291237</v>
       </c>
       <c r="E55" s="2" t="n">
-        <v>0.9175642260339907</v>
+        <v>0.8185445247137505</v>
       </c>
       <c r="F55" s="2" t="n">
-        <v>0.9436523966497012</v>
+        <v>0.8767216867967569</v>
       </c>
       <c r="G55" s="2" t="n">
-        <v>0.9544615921341284</v>
+        <v>0.9003793199997074</v>
       </c>
       <c r="H55" s="2" t="n">
-        <v>0.9600071988288605</v>
+        <v>0.9124550510696275</v>
       </c>
       <c r="I55" s="2" t="n">
-        <v>0.9630603322341956</v>
+        <v>0.9191345262736552</v>
       </c>
       <c r="J55" s="2" t="n">
-        <v>0.9647162909970507</v>
+        <v>0.9228450067431002</v>
       </c>
       <c r="K55" s="2" t="n">
-        <v>0.9654026903433606</v>
+        <v>0.9245476971002226</v>
       </c>
       <c r="L55" s="2" t="n">
-        <v>0.9653300977116198</v>
+        <v>0.9247373120971561</v>
       </c>
       <c r="M55" s="2" t="n">
-        <v>0.9645907141301797</v>
+        <v>0.9236673388761331</v>
       </c>
       <c r="N55" s="2" t="n">
-        <v>0.9631964275673923</v>
+        <v>0.9214373268864954</v>
       </c>
       <c r="O55" s="2" t="n">
-        <v>0.961087937215221</v>
+        <v>0.9180204543028089</v>
       </c>
       <c r="P55" s="1" t="inlineStr"/>
     </row>
     <row r="56" ht="30" customHeight="1">
       <c r="A56" s="1" t="inlineStr">
         <is>
-          <t>c_3u_отн_i</t>
+          <t>r_ср3_отн_i</t>
         </is>
       </c>
       <c r="B56" s="1" t="inlineStr">
         <is>
-          <t>Безразмерная окружная составляющая скорости на выходе</t>
+          <t>Относительный средний радиус на выходе из ступени</t>
         </is>
       </c>
       <c r="C56" s="1" t="inlineStr"/>
       <c r="D56" s="2" t="n">
-        <v>0.2803314260408126</v>
+        <v>0.7914114817012881</v>
       </c>
       <c r="E56" s="2" t="n">
-        <v>0.3458492759403646</v>
+        <v>0.9175642260339907</v>
       </c>
       <c r="F56" s="2" t="n">
-        <v>0.351047131535497</v>
+        <v>0.9436523966497012</v>
       </c>
       <c r="G56" s="2" t="n">
-        <v>0.3474108361019247</v>
+        <v>0.9544615921341284</v>
       </c>
       <c r="H56" s="2" t="n">
-        <v>0.3409913965417674</v>
+        <v>0.9600071988288605</v>
       </c>
       <c r="I56" s="2" t="n">
-        <v>0.333471026166709</v>
+        <v>0.9630603322341956</v>
       </c>
       <c r="J56" s="2" t="n">
-        <v>0.325570138399774</v>
+        <v>0.9647162909970507</v>
       </c>
       <c r="K56" s="2" t="n">
-        <v>0.3176637807777642</v>
+        <v>0.9654026903433606</v>
       </c>
       <c r="L56" s="2" t="n">
-        <v>0.3100444252741181</v>
+        <v>0.9653300977116198</v>
       </c>
       <c r="M56" s="2" t="n">
-        <v>0.3029957910776013</v>
+        <v>0.9645907141301797</v>
       </c>
       <c r="N56" s="2" t="n">
-        <v>0.2968234119960466</v>
+        <v>0.9631964275673923</v>
       </c>
       <c r="O56" s="2" t="n">
-        <v>0.2918471447312225</v>
+        <v>0.961087937215221</v>
       </c>
       <c r="P56" s="1" t="inlineStr"/>
     </row>
     <row r="57" ht="30" customHeight="1">
       <c r="A57" s="1" t="inlineStr">
         <is>
-          <t>α_3_i</t>
+          <t>c_3u_отн_i</t>
         </is>
       </c>
       <c r="B57" s="1" t="inlineStr">
         <is>
-          <t>Угол абсолютной скорости на выходе из ступени</t>
+          <t>Безразмерная окружная составляющая скорости на выходе</t>
         </is>
       </c>
       <c r="C57" s="1" t="inlineStr"/>
       <c r="D57" s="2" t="n">
-        <v>1.148349100413499</v>
+        <v>0.2803314260408126</v>
       </c>
       <c r="E57" s="2" t="n">
-        <v>1.045925568107925</v>
+        <v>0.3458492759403646</v>
       </c>
       <c r="F57" s="2" t="n">
-        <v>1.019499110376512</v>
+        <v>0.351047131535497</v>
       </c>
       <c r="G57" s="2" t="n">
-        <v>1.002915226818822</v>
+        <v>0.3474108361019247</v>
       </c>
       <c r="H57" s="2" t="n">
-        <v>0.9887803620450216</v>
+        <v>0.3409913965417674</v>
       </c>
       <c r="I57" s="2" t="n">
-        <v>0.9749630666974607</v>
+        <v>0.333471026166709</v>
       </c>
       <c r="J57" s="2" t="n">
-        <v>0.9604281068418332</v>
+        <v>0.325570138399774</v>
       </c>
       <c r="K57" s="2" t="n">
-        <v>0.9444996836152652</v>
+        <v>0.3176637807777642</v>
       </c>
       <c r="L57" s="2" t="n">
-        <v>0.9265219325482024</v>
+        <v>0.3100444252741181</v>
       </c>
       <c r="M57" s="2" t="n">
-        <v>0.9057489472864968</v>
+        <v>0.3029957910776013</v>
       </c>
       <c r="N57" s="2" t="n">
-        <v>0.8812882212871602</v>
+        <v>0.2968234119960466</v>
       </c>
       <c r="O57" s="2" t="n">
-        <v>0.8521100845146086</v>
+        <v>0.2918471447312225</v>
       </c>
       <c r="P57" s="1" t="inlineStr"/>
     </row>
-    <row r="58" ht="15" customHeight="1">
+    <row r="58" ht="30" customHeight="1">
       <c r="A58" s="1" t="inlineStr">
         <is>
-          <t>λ_3_i</t>
+          <t>α_3_i</t>
         </is>
       </c>
       <c r="B58" s="1" t="inlineStr">
         <is>
-          <t>Приведенная скорость на выходе из ступени</t>
+          <t>Угол абсолютной скорости на выходе из ступени</t>
         </is>
       </c>
       <c r="C58" s="1" t="inlineStr"/>
       <c r="D58" s="2" t="n">
-        <v>0.6559785963090488</v>
+        <v>1.148349100413499</v>
       </c>
       <c r="E58" s="2" t="n">
-        <v>0.6246063457694964</v>
+        <v>1.045925568107925</v>
       </c>
       <c r="F58" s="2" t="n">
-        <v>0.5757065070246412</v>
+        <v>1.019499110376512</v>
       </c>
       <c r="G58" s="2" t="n">
-        <v>0.5294507601125176</v>
+        <v>1.002915226818822</v>
       </c>
       <c r="H58" s="2" t="n">
-        <v>0.4872531702268296</v>
+        <v>0.9887803620450216</v>
       </c>
       <c r="I58" s="2" t="n">
-        <v>0.4489353796842664</v>
+        <v>0.9749630666974607</v>
       </c>
       <c r="J58" s="2" t="n">
-        <v>0.4139239072289042</v>
+        <v>0.9604281068418332</v>
       </c>
       <c r="K58" s="2" t="n">
-        <v>0.3819733439588067</v>
+        <v>0.9444996836152652</v>
       </c>
       <c r="L58" s="2" t="n">
-        <v>0.3526664394879173</v>
+        <v>0.9265219325482024</v>
       </c>
       <c r="M58" s="2" t="n">
-        <v>0.3258102099036672</v>
+        <v>0.9057489472864968</v>
       </c>
       <c r="N58" s="2" t="n">
-        <v>0.3012816010392996</v>
+        <v>0.8812882212871602</v>
       </c>
       <c r="O58" s="2" t="n">
-        <v>0.278992643690011</v>
+        <v>0.8521100845146086</v>
       </c>
       <c r="P58" s="1" t="inlineStr"/>
     </row>
-    <row r="59" ht="30" customHeight="1">
+    <row r="59" ht="15" customHeight="1">
       <c r="A59" s="1" t="inlineStr">
         <is>
-          <t>F_3_i</t>
+          <t>λ_3_i</t>
         </is>
       </c>
       <c r="B59" s="1" t="inlineStr">
         <is>
-          <t>Действительная кольцевая площадь на выходе из ступени</t>
+          <t>Приведенная скорость на выходе из ступени</t>
         </is>
       </c>
       <c r="C59" s="1" t="inlineStr"/>
       <c r="D59" s="2" t="n">
-        <v>0.2720258280079406</v>
+        <v>0.6559785963090488</v>
       </c>
       <c r="E59" s="2" t="n">
-        <v>0.1150773962795963</v>
+        <v>0.6246063457694964</v>
       </c>
       <c r="F59" s="2" t="n">
-        <v>0.07972938889514986</v>
+        <v>0.5757065070246412</v>
       </c>
       <c r="G59" s="2" t="n">
-        <v>0.06479319133468478</v>
+        <v>0.5294507601125176</v>
       </c>
       <c r="H59" s="2" t="n">
-        <v>0.0570642191435431</v>
+        <v>0.4872531702268296</v>
       </c>
       <c r="I59" s="2" t="n">
-        <v>0.05278992205645663</v>
+        <v>0.4489353796842664</v>
       </c>
       <c r="J59" s="2" t="n">
-        <v>0.05046595153123931</v>
+        <v>0.4139239072289042</v>
       </c>
       <c r="K59" s="2" t="n">
-        <v>0.04950148906418269</v>
+        <v>0.3819733439588067</v>
       </c>
       <c r="L59" s="2" t="n">
-        <v>0.04960352169899662</v>
+        <v>0.3526664394879173</v>
       </c>
       <c r="M59" s="2" t="n">
-        <v>0.05064232585954236</v>
+        <v>0.3258102099036672</v>
       </c>
       <c r="N59" s="2" t="n">
-        <v>0.05259907661212716</v>
+        <v>0.3012816010392996</v>
       </c>
       <c r="O59" s="2" t="n">
-        <v>0.05555276895854432</v>
+        <v>0.278992643690011</v>
       </c>
       <c r="P59" s="1" t="inlineStr"/>
     </row>
     <row r="60" ht="30" customHeight="1">
       <c r="A60" s="1" t="inlineStr">
         <is>
-          <t>F_1_i_plus_1</t>
+          <t>F_3_i</t>
         </is>
       </c>
       <c r="B60" s="1" t="inlineStr">
         <is>
-          <t>Кольцевая площадь на входе в следующую ступень</t>
+          <t>Действительная кольцевая площадь на выходе из ступени</t>
         </is>
       </c>
       <c r="C60" s="1" t="inlineStr"/>
       <c r="D60" s="2" t="n">
+        <v>0.2720258280079406</v>
+      </c>
+      <c r="E60" s="2" t="n">
         <v>0.1150773962795963</v>
       </c>
-      <c r="E60" s="2" t="n">
+      <c r="F60" s="2" t="n">
         <v>0.07972938889514986</v>
       </c>
-      <c r="F60" s="2" t="n">
+      <c r="G60" s="2" t="n">
         <v>0.06479319133468478</v>
       </c>
-      <c r="G60" s="2" t="n">
+      <c r="H60" s="2" t="n">
         <v>0.0570642191435431</v>
       </c>
-      <c r="H60" s="2" t="n">
+      <c r="I60" s="2" t="n">
         <v>0.05278992205645663</v>
       </c>
-      <c r="I60" s="2" t="n">
+      <c r="J60" s="2" t="n">
         <v>0.05046595153123931</v>
       </c>
-      <c r="J60" s="2" t="n">
+      <c r="K60" s="2" t="n">
         <v>0.04950148906418269</v>
       </c>
-      <c r="K60" s="2" t="n">
+      <c r="L60" s="2" t="n">
         <v>0.04960352169899662</v>
       </c>
-      <c r="L60" s="2" t="n">
+      <c r="M60" s="2" t="n">
         <v>0.05064232585954236</v>
       </c>
-      <c r="M60" s="2" t="n">
+      <c r="N60" s="2" t="n">
         <v>0.05259907661212716</v>
       </c>
-      <c r="N60" s="2" t="n">
+      <c r="O60" s="2" t="n">
         <v>0.05555276895854432</v>
-      </c>
-      <c r="O60" s="2" t="n">
-        <v>0.05850646130496148</v>
       </c>
       <c r="P60" s="1" t="inlineStr"/>
     </row>
     <row r="61" ht="30" customHeight="1">
       <c r="A61" s="1" t="inlineStr">
         <is>
-          <t>d3_отн_i</t>
+          <t>F_1_i_plus_1</t>
         </is>
       </c>
       <c r="B61" s="1" t="inlineStr">
         <is>
-          <t>Относительный диаметр втулки на выходе из ступени</t>
+          <t>Кольцевая площадь на входе в следующую ступень</t>
         </is>
       </c>
       <c r="C61" s="1" t="inlineStr"/>
       <c r="D61" s="2" t="n">
-        <v>0.5026572059935642</v>
+        <v>0.1150773962795963</v>
       </c>
       <c r="E61" s="2" t="n">
-        <v>0.8269511580466603</v>
+        <v>0.07972938889514986</v>
       </c>
       <c r="F61" s="2" t="n">
-        <v>0.8837192378835317</v>
+        <v>0.06479319133468478</v>
       </c>
       <c r="G61" s="2" t="n">
-        <v>0.9066387713518712</v>
+        <v>0.0570642191435431</v>
       </c>
       <c r="H61" s="2" t="n">
-        <v>0.9182742747166943</v>
+        <v>0.05278992205645663</v>
       </c>
       <c r="I61" s="2" t="n">
-        <v>0.9246460982700778</v>
+        <v>0.05046595153123931</v>
       </c>
       <c r="J61" s="2" t="n">
-        <v>0.9280921528761098</v>
+        <v>0.04950148906418269</v>
       </c>
       <c r="K61" s="2" t="n">
-        <v>0.9295185361489017</v>
+        <v>0.04960352169899662</v>
       </c>
       <c r="L61" s="2" t="n">
-        <v>0.929367739431411</v>
+        <v>0.05064232585954236</v>
       </c>
       <c r="M61" s="2" t="n">
-        <v>0.9278310684452963</v>
+        <v>0.05259907661212716</v>
       </c>
       <c r="N61" s="2" t="n">
-        <v>0.9249295736201615</v>
+        <v>0.05555276895854432</v>
       </c>
       <c r="O61" s="2" t="n">
-        <v>0.9205324796666424</v>
+        <v>0.05850646130496148</v>
       </c>
       <c r="P61" s="1" t="inlineStr"/>
     </row>
-    <row r="62" ht="15" customHeight="1">
+    <row r="62" ht="30" customHeight="1">
       <c r="A62" s="1" t="inlineStr">
         <is>
-          <t>r_ср2_отн_i</t>
+          <t>d3_отн_i</t>
         </is>
       </c>
       <c r="B62" s="1" t="inlineStr">
         <is>
-          <t>Относительный средний радиус на выходе из РК</t>
+          <t>Относительный диаметр втулки на выходе из ступени</t>
         </is>
       </c>
       <c r="C62" s="1" t="inlineStr"/>
       <c r="D62" s="2" t="n">
-        <v>0.7805596092214843</v>
+        <v>0.5026572059935642</v>
       </c>
       <c r="E62" s="2" t="n">
-        <v>0.8500880382586702</v>
+        <v>0.8269511580466603</v>
       </c>
       <c r="F62" s="2" t="n">
-        <v>0.8700959893287561</v>
+        <v>0.8837192378835317</v>
       </c>
       <c r="G62" s="2" t="n">
-        <v>0.8829499081275562</v>
+        <v>0.9066387713518712</v>
       </c>
       <c r="H62" s="2" t="n">
-        <v>0.893631259906112</v>
+        <v>0.9182742747166943</v>
       </c>
       <c r="I62" s="2" t="n">
-        <v>0.9034997827061337</v>
+        <v>0.9246460982700778</v>
       </c>
       <c r="J62" s="2" t="n">
-        <v>0.9130779445472598</v>
+        <v>0.9280921528761098</v>
       </c>
       <c r="K62" s="2" t="n">
-        <v>0.9225551907029824</v>
+        <v>0.9295185361489017</v>
       </c>
       <c r="L62" s="2" t="n">
-        <v>0.9320133967247826</v>
+        <v>0.929367739431411</v>
       </c>
       <c r="M62" s="2" t="n">
-        <v>0.9414763041919105</v>
+        <v>0.9278310684452963</v>
       </c>
       <c r="N62" s="2" t="n">
-        <v>0.9509286079025953</v>
+        <v>0.9249295736201615</v>
       </c>
       <c r="O62" s="2" t="n">
-        <v>0.9603205495816369</v>
+        <v>0.9205324796666424</v>
       </c>
       <c r="P62" s="1" t="inlineStr"/>
     </row>
-    <row r="63" ht="30" customHeight="1">
+    <row r="63" ht="15" customHeight="1">
       <c r="A63" s="1" t="inlineStr">
         <is>
-          <t>c_u2_отн_i</t>
+          <t>r_ср2_отн_i</t>
         </is>
       </c>
       <c r="B63" s="1" t="inlineStr">
         <is>
-          <t>Безразмерная окружная составляющая скорости на выходе из РК</t>
+          <t>Относительный средний радиус на выходе из РК</t>
         </is>
       </c>
       <c r="C63" s="1" t="inlineStr"/>
       <c r="D63" s="2" t="n">
-        <v>0.4951608024475138</v>
+        <v>0.7805596092214843</v>
       </c>
       <c r="E63" s="2" t="n">
-        <v>0.4796111464536851</v>
+        <v>0.8500880382586702</v>
       </c>
       <c r="F63" s="2" t="n">
-        <v>0.4933697911469953</v>
+        <v>0.8700959893287561</v>
       </c>
       <c r="G63" s="2" t="n">
-        <v>0.511158425729244</v>
+        <v>0.8829499081275562</v>
       </c>
       <c r="H63" s="2" t="n">
-        <v>0.5303221251053101</v>
+        <v>0.893631259906112</v>
       </c>
       <c r="I63" s="2" t="n">
-        <v>0.5501351231747619</v>
+        <v>0.9034997827061337</v>
       </c>
       <c r="J63" s="2" t="n">
-        <v>0.5702552370692163</v>
+        <v>0.9130779445472598</v>
       </c>
       <c r="K63" s="2" t="n">
-        <v>0.5904530661631379</v>
+        <v>0.9225551907029824</v>
       </c>
       <c r="L63" s="2" t="n">
-        <v>0.6105143851335061</v>
+        <v>0.9320133967247826</v>
       </c>
       <c r="M63" s="2" t="n">
-        <v>0.630205686088978</v>
+        <v>0.9414763041919105</v>
       </c>
       <c r="N63" s="2" t="n">
-        <v>0.6492618491206571</v>
+        <v>0.9509286079025953</v>
       </c>
       <c r="O63" s="2" t="n">
-        <v>0.6674038058680815</v>
+        <v>0.9603205495816369</v>
       </c>
       <c r="P63" s="1" t="inlineStr"/>
     </row>
-    <row r="64" ht="15" customHeight="1">
+    <row r="64" ht="30" customHeight="1">
       <c r="A64" s="1" t="inlineStr">
         <is>
-          <t>β_1_i</t>
+          <t>c_u2_отн_i</t>
         </is>
       </c>
       <c r="B64" s="1" t="inlineStr">
         <is>
-          <t>Угол относительной скорости на входе в РК</t>
+          <t>Безразмерная окружная составляющая скорости на выходе из РК</t>
         </is>
       </c>
       <c r="C64" s="1" t="inlineStr"/>
       <c r="D64" s="2" t="n">
-        <v>0.9130337357818</v>
+        <v>0.4951608024475138</v>
       </c>
       <c r="E64" s="2" t="n">
-        <v>0.8748613108903142</v>
+        <v>0.4796111464536851</v>
       </c>
       <c r="F64" s="2" t="n">
-        <v>0.8367019754879613</v>
+        <v>0.4933697911469953</v>
       </c>
       <c r="G64" s="2" t="n">
-        <v>0.7984417849023867</v>
+        <v>0.511158425729244</v>
       </c>
       <c r="H64" s="2" t="n">
-        <v>0.760052506592651</v>
+        <v>0.5303221251053101</v>
       </c>
       <c r="I64" s="2" t="n">
-        <v>0.7215557875774173</v>
+        <v>0.5501351231747619</v>
       </c>
       <c r="J64" s="2" t="n">
-        <v>0.6830253822830016</v>
+        <v>0.5702552370692163</v>
       </c>
       <c r="K64" s="2" t="n">
-        <v>0.6445808950740264</v>
+        <v>0.5904530661631379</v>
       </c>
       <c r="L64" s="2" t="n">
-        <v>0.6063535228830391</v>
+        <v>0.6105143851335061</v>
       </c>
       <c r="M64" s="2" t="n">
-        <v>0.5684827367765299</v>
+        <v>0.630205686088978</v>
       </c>
       <c r="N64" s="2" t="n">
-        <v>0.5311064742865111</v>
+        <v>0.6492618491206571</v>
       </c>
       <c r="O64" s="2" t="n">
-        <v>0.4943374292495647</v>
+        <v>0.6674038058680815</v>
       </c>
       <c r="P64" s="1" t="inlineStr"/>
     </row>
-    <row r="65" ht="30" customHeight="1">
+    <row r="65" ht="15" customHeight="1">
       <c r="A65" s="1" t="inlineStr">
         <is>
-          <t>c_a2_отн_i</t>
+          <t>β_1_i</t>
         </is>
       </c>
       <c r="B65" s="1" t="inlineStr">
         <is>
-          <t>Относительная осевая скорость на выходе из РК</t>
+          <t>Угол относительной скорости на входе в РК</t>
         </is>
       </c>
       <c r="C65" s="1" t="inlineStr"/>
       <c r="D65" s="2" t="n">
-        <v>0.6368181818181818</v>
+        <v>0.9130337357818</v>
       </c>
       <c r="E65" s="2" t="n">
-        <v>0.6104545454545455</v>
+        <v>0.8748613108903142</v>
       </c>
       <c r="F65" s="2" t="n">
-        <v>0.5840909090909091</v>
+        <v>0.8367019754879613</v>
       </c>
       <c r="G65" s="2" t="n">
-        <v>0.5577272727272727</v>
+        <v>0.7984417849023867</v>
       </c>
       <c r="H65" s="2" t="n">
-        <v>0.5313636363636364</v>
+        <v>0.760052506592651</v>
       </c>
       <c r="I65" s="2" t="n">
-        <v>0.505</v>
+        <v>0.7215557875774173</v>
       </c>
       <c r="J65" s="2" t="n">
-        <v>0.4786363636363636</v>
+        <v>0.6830253822830016</v>
       </c>
       <c r="K65" s="2" t="n">
-        <v>0.4522727272727273</v>
+        <v>0.6445808950740264</v>
       </c>
       <c r="L65" s="2" t="n">
-        <v>0.4259090909090909</v>
+        <v>0.6063535228830391</v>
       </c>
       <c r="M65" s="2" t="n">
-        <v>0.3995454545454545</v>
+        <v>0.5684827367765299</v>
       </c>
       <c r="N65" s="2" t="n">
-        <v>0.3731818181818182</v>
+        <v>0.5311064742865111</v>
       </c>
       <c r="O65" s="2" t="n">
-        <v>0.3468181818181818</v>
+        <v>0.4943374292495647</v>
       </c>
       <c r="P65" s="1" t="inlineStr"/>
     </row>
-    <row r="66" ht="15" customHeight="1">
+    <row r="66" ht="30" customHeight="1">
       <c r="A66" s="1" t="inlineStr">
         <is>
-          <t>β_2_i</t>
+          <t>c_a2_отн_i</t>
         </is>
       </c>
       <c r="B66" s="1" t="inlineStr">
         <is>
-          <t>Угол относительной скорости на выходе из РК</t>
+          <t>Относительная осевая скорость на выходе из РК</t>
         </is>
       </c>
       <c r="C66" s="1" t="inlineStr"/>
       <c r="D66" s="2" t="n">
-        <v>1.149470499626858</v>
+        <v>0.6368181818181818</v>
       </c>
       <c r="E66" s="2" t="n">
-        <v>1.025328281506466</v>
+        <v>0.6104545454545455</v>
       </c>
       <c r="F66" s="2" t="n">
-        <v>0.9979591178031184</v>
+        <v>0.5840909090909091</v>
       </c>
       <c r="G66" s="2" t="n">
-        <v>0.9828268660091499</v>
+        <v>0.5577272727272727</v>
       </c>
       <c r="H66" s="2" t="n">
-        <v>0.9710736479752523</v>
+        <v>0.5313636363636364</v>
       </c>
       <c r="I66" s="2" t="n">
-        <v>0.9602502514475583</v>
+        <v>0.505</v>
       </c>
       <c r="J66" s="2" t="n">
-        <v>0.9492481850610934</v>
+        <v>0.4786363636363636</v>
       </c>
       <c r="K66" s="2" t="n">
-        <v>0.9374216670208639</v>
+        <v>0.4522727272727273</v>
       </c>
       <c r="L66" s="2" t="n">
-        <v>0.924196142381593</v>
+        <v>0.4259090909090909</v>
       </c>
       <c r="M66" s="2" t="n">
-        <v>0.9089535843846798</v>
+        <v>0.3995454545454545</v>
       </c>
       <c r="N66" s="2" t="n">
-        <v>0.8909761330468265</v>
+        <v>0.3731818181818182</v>
       </c>
       <c r="O66" s="2" t="n">
-        <v>0.8694555233106508</v>
+        <v>0.3468181818181818</v>
       </c>
       <c r="P66" s="1" t="inlineStr"/>
     </row>
     <row r="67" ht="15" customHeight="1">
       <c r="A67" s="1" t="inlineStr">
         <is>
-          <t>α_2_i</t>
+          <t>β_2_i</t>
         </is>
       </c>
       <c r="B67" s="1" t="inlineStr">
         <is>
-          <t>Угол абсолютной скорости на выходе из РК</t>
+          <t>Угол относительной скорости на выходе из РК</t>
         </is>
       </c>
       <c r="C67" s="1" t="inlineStr"/>
       <c r="D67" s="2" t="n">
-        <v>0.9098923318704959</v>
+        <v>1.149470499626858</v>
       </c>
       <c r="E67" s="2" t="n">
-        <v>0.9048592082754372</v>
+        <v>1.025328281506466</v>
       </c>
       <c r="F67" s="2" t="n">
-        <v>0.8693990341364447</v>
+        <v>0.9979591178031184</v>
       </c>
       <c r="G67" s="2" t="n">
-        <v>0.8289382873161977</v>
+        <v>0.9828268660091499</v>
       </c>
       <c r="H67" s="2" t="n">
-        <v>0.7863791607528087</v>
+        <v>0.9710736479752523</v>
       </c>
       <c r="I67" s="2" t="n">
-        <v>0.7426475977563408</v>
+        <v>0.9602502514475583</v>
       </c>
       <c r="J67" s="2" t="n">
-        <v>0.6982710232411901</v>
+        <v>0.9492481850610934</v>
       </c>
       <c r="K67" s="2" t="n">
-        <v>0.6536474291487642</v>
+        <v>0.9374216670208639</v>
       </c>
       <c r="L67" s="2" t="n">
-        <v>0.6091291160368223</v>
+        <v>0.924196142381593</v>
       </c>
       <c r="M67" s="2" t="n">
-        <v>0.5650394600392833</v>
+        <v>0.9089535843846798</v>
       </c>
       <c r="N67" s="2" t="n">
-        <v>0.5216678776691375</v>
+        <v>0.8909761330468265</v>
       </c>
       <c r="O67" s="2" t="n">
-        <v>0.4792458653577785</v>
+        <v>0.8694555233106508</v>
       </c>
       <c r="P67" s="1" t="inlineStr"/>
     </row>
     <row r="68" ht="15" customHeight="1">
       <c r="A68" s="1" t="inlineStr">
         <is>
-          <t>ε_рк_i</t>
+          <t>α_2_i</t>
         </is>
       </c>
       <c r="B68" s="1" t="inlineStr">
         <is>
-          <t>Диффузность решетки РК</t>
+          <t>Угол абсолютной скорости на выходе из РК</t>
         </is>
       </c>
       <c r="C68" s="1" t="inlineStr"/>
       <c r="D68" s="2" t="n">
-        <v>0.2364367638450576</v>
+        <v>0.9098923318704959</v>
       </c>
       <c r="E68" s="2" t="n">
-        <v>0.1504669706161518</v>
+        <v>0.9048592082754372</v>
       </c>
       <c r="F68" s="2" t="n">
-        <v>0.1612571423151571</v>
+        <v>0.8693990341364447</v>
       </c>
       <c r="G68" s="2" t="n">
-        <v>0.1843850811067632</v>
+        <v>0.8289382873161977</v>
       </c>
       <c r="H68" s="2" t="n">
-        <v>0.2110211413826013</v>
+        <v>0.7863791607528087</v>
       </c>
       <c r="I68" s="2" t="n">
-        <v>0.2386944638701409</v>
+        <v>0.7426475977563408</v>
       </c>
       <c r="J68" s="2" t="n">
-        <v>0.2662228027780918</v>
+        <v>0.6982710232411901</v>
       </c>
       <c r="K68" s="2" t="n">
-        <v>0.2928407719468376</v>
+        <v>0.6536474291487642</v>
       </c>
       <c r="L68" s="2" t="n">
-        <v>0.3178426194985539</v>
+        <v>0.6091291160368223</v>
       </c>
       <c r="M68" s="2" t="n">
-        <v>0.3404708476081498</v>
+        <v>0.5650394600392833</v>
       </c>
       <c r="N68" s="2" t="n">
-        <v>0.3598696587603154</v>
+        <v>0.5216678776691375</v>
       </c>
       <c r="O68" s="2" t="n">
-        <v>0.3751180940610861</v>
+        <v>0.4792458653577785</v>
       </c>
       <c r="P68" s="1" t="inlineStr"/>
     </row>
     <row r="69" ht="15" customHeight="1">
       <c r="A69" s="1" t="inlineStr">
         <is>
-          <t>ε_на_i</t>
+          <t>ε_рк_i</t>
         </is>
       </c>
       <c r="B69" s="1" t="inlineStr">
         <is>
-          <t>Диффузность решетки НА</t>
+          <t>Диффузность решетки РК</t>
         </is>
       </c>
       <c r="C69" s="1" t="inlineStr"/>
       <c r="D69" s="2" t="n">
-        <v>0.238456768543003</v>
+        <v>0.2364367638450576</v>
       </c>
       <c r="E69" s="2" t="n">
-        <v>0.1410663598324875</v>
+        <v>0.1504669706161518</v>
       </c>
       <c r="F69" s="2" t="n">
-        <v>0.1501000762400676</v>
+        <v>0.1612571423151571</v>
       </c>
       <c r="G69" s="2" t="n">
-        <v>0.1739769395026247</v>
+        <v>0.1843850811067632</v>
       </c>
       <c r="H69" s="2" t="n">
-        <v>0.202401201292213</v>
+        <v>0.2110211413826013</v>
       </c>
       <c r="I69" s="2" t="n">
-        <v>0.2323154689411199</v>
+        <v>0.2386944638701409</v>
       </c>
       <c r="J69" s="2" t="n">
-        <v>0.2621570836006432</v>
+        <v>0.2662228027780918</v>
       </c>
       <c r="K69" s="2" t="n">
-        <v>0.290852254466501</v>
+        <v>0.2928407719468376</v>
       </c>
       <c r="L69" s="2" t="n">
-        <v>0.3173928165113801</v>
+        <v>0.3178426194985539</v>
       </c>
       <c r="M69" s="2" t="n">
-        <v>0.3407094872472135</v>
+        <v>0.3404708476081498</v>
       </c>
       <c r="N69" s="2" t="n">
-        <v>0.3596203436180228</v>
+        <v>0.3598696587603154</v>
       </c>
       <c r="O69" s="2" t="n">
-        <v>0.37286421915683</v>
+        <v>0.3751180940610861</v>
       </c>
       <c r="P69" s="1" t="inlineStr"/>
     </row>
     <row r="70" ht="15" customHeight="1">
       <c r="A70" s="1" t="inlineStr">
         <is>
-          <t>W_1_i</t>
+          <t>ε_на_i</t>
         </is>
       </c>
       <c r="B70" s="1" t="inlineStr">
         <is>
-          <t>Относительная скорость на входе в РК</t>
+          <t>Диффузность решетки НА</t>
         </is>
       </c>
       <c r="C70" s="1" t="inlineStr"/>
       <c r="D70" s="2" t="n">
-        <v>251.7894146864385</v>
+        <v>0.238456768543003</v>
       </c>
       <c r="E70" s="2" t="n">
-        <v>249.1024900209453</v>
+        <v>0.1410663598324875</v>
       </c>
       <c r="F70" s="2" t="n">
-        <v>246.6107242604538</v>
+        <v>0.1501000762400676</v>
       </c>
       <c r="G70" s="2" t="n">
-        <v>244.3372984316917</v>
+        <v>0.1739769395026247</v>
       </c>
       <c r="H70" s="2" t="n">
-        <v>242.2923887858165</v>
+        <v>0.202401201292213</v>
       </c>
       <c r="I70" s="2" t="n">
-        <v>240.4769672604629</v>
+        <v>0.2323154689411199</v>
       </c>
       <c r="J70" s="2" t="n">
-        <v>238.8781441276591</v>
+        <v>0.2621570836006432</v>
       </c>
       <c r="K70" s="2" t="n">
-        <v>237.4656501333595</v>
+        <v>0.290852254466501</v>
       </c>
       <c r="L70" s="2" t="n">
-        <v>236.1969574055916</v>
+        <v>0.3173928165113801</v>
       </c>
       <c r="M70" s="2" t="n">
-        <v>235.0144241906794</v>
+        <v>0.3407094872472135</v>
       </c>
       <c r="N70" s="2" t="n">
-        <v>233.8442343661209</v>
+        <v>0.3596203436180228</v>
       </c>
       <c r="O70" s="2" t="n">
-        <v>232.6016263665796</v>
+        <v>0.37286421915683</v>
       </c>
       <c r="P70" s="1" t="inlineStr"/>
     </row>
     <row r="71" ht="15" customHeight="1">
       <c r="A71" s="1" t="inlineStr">
         <is>
-          <t>c_a2_i</t>
+          <t>W_1_i</t>
         </is>
       </c>
       <c r="B71" s="1" t="inlineStr">
         <is>
-          <t>Осевая скорость на выходе из РК</t>
+          <t>Относительная скорость на входе в РК</t>
         </is>
       </c>
       <c r="C71" s="1" t="inlineStr"/>
       <c r="D71" s="2" t="n">
-        <v>195.2157185709887</v>
+        <v>251.7894146864385</v>
       </c>
       <c r="E71" s="2" t="n">
-        <v>187.1339828985281</v>
+        <v>249.1024900209453</v>
       </c>
       <c r="F71" s="2" t="n">
-        <v>179.0522472260675</v>
+        <v>246.6107242604538</v>
       </c>
       <c r="G71" s="2" t="n">
-        <v>170.9705115536069</v>
+        <v>244.3372984316917</v>
       </c>
       <c r="H71" s="2" t="n">
-        <v>162.8887758811462</v>
+        <v>242.2923887858165</v>
       </c>
       <c r="I71" s="2" t="n">
-        <v>154.8070402086856</v>
+        <v>240.4769672604629</v>
       </c>
       <c r="J71" s="2" t="n">
-        <v>146.7253045362249</v>
+        <v>238.8781441276591</v>
       </c>
       <c r="K71" s="2" t="n">
-        <v>138.6435688637643</v>
+        <v>237.4656501333595</v>
       </c>
       <c r="L71" s="2" t="n">
-        <v>130.5618331913037</v>
+        <v>236.1969574055916</v>
       </c>
       <c r="M71" s="2" t="n">
-        <v>122.480097518843</v>
+        <v>235.0144241906794</v>
       </c>
       <c r="N71" s="2" t="n">
-        <v>114.3983618463824</v>
+        <v>233.8442343661209</v>
       </c>
       <c r="O71" s="2" t="n">
-        <v>106.3166261739218</v>
+        <v>232.6016263665796</v>
       </c>
       <c r="P71" s="1" t="inlineStr"/>
     </row>
     <row r="72" ht="15" customHeight="1">
       <c r="A72" s="1" t="inlineStr">
         <is>
-          <t>c_2_i</t>
+          <t>c_a2_i</t>
         </is>
       </c>
       <c r="B72" s="1" t="inlineStr">
         <is>
-          <t>Абсолютная скорость на выходе из РК</t>
+          <t>Осевая скорость на выходе из РК</t>
         </is>
       </c>
       <c r="C72" s="1" t="inlineStr"/>
       <c r="D72" s="2" t="n">
-        <v>247.28452908</v>
+        <v>195.2157185709887</v>
       </c>
       <c r="E72" s="2" t="n">
-        <v>237.9815544364363</v>
+        <v>187.1339828985281</v>
       </c>
       <c r="F72" s="2" t="n">
-        <v>234.3795941484085</v>
+        <v>179.0522472260675</v>
       </c>
       <c r="G72" s="2" t="n">
-        <v>231.9142224061601</v>
+        <v>170.9705115536069</v>
       </c>
       <c r="H72" s="2" t="n">
-        <v>230.133866067011</v>
+        <v>162.8887758811462</v>
       </c>
       <c r="I72" s="2" t="n">
-        <v>228.9229812149858</v>
+        <v>154.8070402086856</v>
       </c>
       <c r="J72" s="2" t="n">
-        <v>228.2261602651597</v>
+        <v>146.7253045362249</v>
       </c>
       <c r="K72" s="2" t="n">
-        <v>227.999923292236</v>
+        <v>138.6435688637643</v>
       </c>
       <c r="L72" s="2" t="n">
-        <v>228.1937458904654</v>
+        <v>130.5618331913037</v>
       </c>
       <c r="M72" s="2" t="n">
-        <v>228.7427276681898</v>
+        <v>122.480097518843</v>
       </c>
       <c r="N72" s="2" t="n">
-        <v>229.5649111126124</v>
+        <v>114.3983618463824</v>
       </c>
       <c r="O72" s="2" t="n">
-        <v>230.5666674764105</v>
+        <v>106.3166261739218</v>
       </c>
       <c r="P72" s="1" t="inlineStr"/>
     </row>
     <row r="73" ht="15" customHeight="1">
       <c r="A73" s="1" t="inlineStr">
         <is>
-          <t>τ_1_i</t>
+          <t>c_2_i</t>
         </is>
       </c>
       <c r="B73" s="1" t="inlineStr">
         <is>
-          <t>Температурная функция на входе в РК</t>
+          <t>Абсолютная скорость на выходе из РК</t>
         </is>
       </c>
       <c r="C73" s="1" t="inlineStr"/>
       <c r="D73" s="2" t="n">
-        <v>0.9198717705829682</v>
+        <v>247.28452908</v>
       </c>
       <c r="E73" s="2" t="n">
-        <v>0.9343717516022703</v>
+        <v>237.9815544364363</v>
       </c>
       <c r="F73" s="2" t="n">
-        <v>0.9456738513371452</v>
+        <v>234.3795941484085</v>
       </c>
       <c r="G73" s="2" t="n">
-        <v>0.9544810706406721</v>
+        <v>231.9142224061601</v>
       </c>
       <c r="H73" s="2" t="n">
-        <v>0.9616684573121036</v>
+        <v>230.133866067011</v>
       </c>
       <c r="I73" s="2" t="n">
-        <v>0.9675039353435879</v>
+        <v>228.9229812149858</v>
       </c>
       <c r="J73" s="2" t="n">
-        <v>0.9723363601852713</v>
+        <v>228.2261602651597</v>
       </c>
       <c r="K73" s="2" t="n">
-        <v>0.9763162299517529</v>
+        <v>227.999923292236</v>
       </c>
       <c r="L73" s="2" t="n">
-        <v>0.9796348119488701</v>
+        <v>228.1937458904654</v>
       </c>
       <c r="M73" s="2" t="n">
-        <v>0.9823328970460875</v>
+        <v>228.7427276681898</v>
       </c>
       <c r="N73" s="2" t="n">
-        <v>0.9845454709023621</v>
+        <v>229.5649111126124</v>
       </c>
       <c r="O73" s="2" t="n">
-        <v>0.9863414798135992</v>
+        <v>230.5666674764105</v>
       </c>
       <c r="P73" s="1" t="inlineStr"/>
     </row>
     <row r="74" ht="15" customHeight="1">
       <c r="A74" s="1" t="inlineStr">
         <is>
-          <t>T_1_i</t>
+          <t>τ_1_i</t>
         </is>
       </c>
       <c r="B74" s="1" t="inlineStr">
         <is>
-          <t>Статическая температура на входе в РК</t>
+          <t>Температурная функция на входе в РК</t>
         </is>
       </c>
       <c r="C74" s="1" t="inlineStr"/>
       <c r="D74" s="2" t="n">
-        <v>264.9230699278949</v>
+        <v>0.9198717705829682</v>
       </c>
       <c r="E74" s="2" t="n">
-        <v>302.9393809956259</v>
+        <v>0.9343717516022703</v>
       </c>
       <c r="F74" s="2" t="n">
-        <v>340.8533627745312</v>
+        <v>0.9456738513371452</v>
       </c>
       <c r="G74" s="2" t="n">
-        <v>378.5964068562916</v>
+        <v>0.9544810706406721</v>
       </c>
       <c r="H74" s="2" t="n">
-        <v>416.2762214324989</v>
+        <v>0.9616684573121036</v>
       </c>
       <c r="I74" s="2" t="n">
-        <v>453.842488535186</v>
+        <v>0.9675039353435879</v>
       </c>
       <c r="J74" s="2" t="n">
-        <v>491.324598928213</v>
+        <v>0.9723363601852713</v>
       </c>
       <c r="K74" s="2" t="n">
-        <v>528.6950671020987</v>
+        <v>0.9763162299517529</v>
       </c>
       <c r="L74" s="2" t="n">
-        <v>565.9717639113386</v>
+        <v>0.9796348119488701</v>
       </c>
       <c r="M74" s="2" t="n">
-        <v>603.1078831527154</v>
+        <v>0.9823328970460875</v>
       </c>
       <c r="N74" s="2" t="n">
-        <v>640.1237707477241</v>
+        <v>0.9845454709023621</v>
       </c>
       <c r="O74" s="2" t="n">
-        <v>677.0139991251236</v>
+        <v>0.9863414798135992</v>
       </c>
       <c r="P74" s="1" t="inlineStr"/>
     </row>
     <row r="75" ht="15" customHeight="1">
       <c r="A75" s="1" t="inlineStr">
         <is>
-          <t>a_1_i</t>
+          <t>T_1_i</t>
         </is>
       </c>
       <c r="B75" s="1" t="inlineStr">
         <is>
-          <t>Скорость звука на входе в РК</t>
+          <t>Статическая температура на входе в РК</t>
         </is>
       </c>
       <c r="C75" s="1" t="inlineStr"/>
       <c r="D75" s="2" t="n">
-        <v>298.0389802067385</v>
+        <v>264.9230699278949</v>
       </c>
       <c r="E75" s="2" t="n">
-        <v>318.6014723186276</v>
+        <v>302.9393809956259</v>
       </c>
       <c r="F75" s="2" t="n">
-        <v>337.8060659838801</v>
+        <v>340.8533627745312</v>
       </c>
       <c r="G75" s="2" t="n">
-        <v>355.9464532230144</v>
+        <v>378.5964068562916</v>
       </c>
       <c r="H75" s="2" t="n">
-        <v>373.082946582965</v>
+        <v>416.2762214324989</v>
       </c>
       <c r="I75" s="2" t="n">
-        <v>389.395436741228</v>
+        <v>453.842488535186</v>
       </c>
       <c r="J75" s="2" t="n">
-        <v>404.9335931204457</v>
+        <v>491.324598928213</v>
       </c>
       <c r="K75" s="2" t="n">
-        <v>419.8160494160329</v>
+        <v>528.6950671020987</v>
       </c>
       <c r="L75" s="2" t="n">
-        <v>434.0589954920686</v>
+        <v>565.9717639113386</v>
       </c>
       <c r="M75" s="2" t="n">
-        <v>447.8214368375179</v>
+        <v>603.1078831527154</v>
       </c>
       <c r="N75" s="2" t="n">
-        <v>461.0892039392522</v>
+        <v>640.1237707477241</v>
       </c>
       <c r="O75" s="2" t="n">
-        <v>473.8913655885228</v>
+        <v>677.0139991251236</v>
       </c>
       <c r="P75" s="1" t="inlineStr"/>
     </row>
-    <row r="76" ht="30" customHeight="1">
+    <row r="76" ht="15" customHeight="1">
       <c r="A76" s="1" t="inlineStr">
         <is>
-          <t>M_w1_i</t>
+          <t>a_1_i</t>
         </is>
       </c>
       <c r="B76" s="1" t="inlineStr">
         <is>
-          <t>Число Маха относительной скорости на входе в РК</t>
+          <t>Скорость звука на входе в РК</t>
         </is>
       </c>
       <c r="C76" s="1" t="inlineStr"/>
       <c r="D76" s="2" t="n">
-        <v>0.8448204141343578</v>
+        <v>298.0389802067385</v>
       </c>
       <c r="E76" s="2" t="n">
-        <v>0.7818623316712811</v>
+        <v>318.6014723186276</v>
       </c>
       <c r="F76" s="2" t="n">
-        <v>0.7300363998561882</v>
+        <v>337.8060659838801</v>
       </c>
       <c r="G76" s="2" t="n">
-        <v>0.6864439755454026</v>
+        <v>355.9464532230144</v>
       </c>
       <c r="H76" s="2" t="n">
-        <v>0.6494330309250312</v>
+        <v>373.082946582965</v>
       </c>
       <c r="I76" s="2" t="n">
-        <v>0.6175649341783925</v>
+        <v>389.395436741228</v>
       </c>
       <c r="J76" s="2" t="n">
-        <v>0.5899193057480068</v>
+        <v>404.9335931204457</v>
       </c>
       <c r="K76" s="2" t="n">
-        <v>0.5656421436571468</v>
+        <v>419.8160494160329</v>
       </c>
       <c r="L76" s="2" t="n">
-        <v>0.5441586509175513</v>
+        <v>434.0589954920686</v>
       </c>
       <c r="M76" s="2" t="n">
-        <v>0.5247949402563977</v>
+        <v>447.8214368375179</v>
       </c>
       <c r="N76" s="2" t="n">
-        <v>0.5071561692798375</v>
+        <v>461.0892039392522</v>
       </c>
       <c r="O76" s="2" t="n">
-        <v>0.4908332230905137</v>
+        <v>473.8913655885228</v>
       </c>
       <c r="P76" s="1" t="inlineStr"/>
     </row>
     <row r="77" ht="30" customHeight="1">
       <c r="A77" s="1" t="inlineStr">
         <is>
-          <t>λ_c2_i</t>
+          <t>M_w1_i</t>
         </is>
       </c>
       <c r="B77" s="1" t="inlineStr">
         <is>
-          <t>Приведенная абсолютная скорость на выходе из РК</t>
+          <t>Число Маха относительной скорости на входе в РК</t>
         </is>
       </c>
       <c r="C77" s="1" t="inlineStr"/>
       <c r="D77" s="2" t="n">
-        <v>0.7739140879000126</v>
+        <v>0.8448204141343578</v>
       </c>
       <c r="E77" s="2" t="n">
-        <v>0.7025688677305478</v>
+        <v>0.7818623316712811</v>
       </c>
       <c r="F77" s="2" t="n">
-        <v>0.6567734946088818</v>
+        <v>0.7300363998561882</v>
       </c>
       <c r="G77" s="2" t="n">
-        <v>0.6201103319267046</v>
+        <v>0.6864439755454026</v>
       </c>
       <c r="H77" s="2" t="n">
-        <v>0.5896922001548817</v>
+        <v>0.6494330309250312</v>
       </c>
       <c r="I77" s="2" t="n">
-        <v>0.5641990975072881</v>
+        <v>0.6175649341783925</v>
       </c>
       <c r="J77" s="2" t="n">
-        <v>0.5425314394305585</v>
+        <v>0.5899193057480068</v>
       </c>
       <c r="K77" s="2" t="n">
-        <v>0.5242135535589888</v>
+        <v>0.5656421436571468</v>
       </c>
       <c r="L77" s="2" t="n">
-        <v>0.5085612696312135</v>
+        <v>0.5441586509175513</v>
       </c>
       <c r="M77" s="2" t="n">
-        <v>0.4951412220693632</v>
+        <v>0.5247949402563977</v>
       </c>
       <c r="N77" s="2" t="n">
-        <v>0.4835545192846229</v>
+        <v>0.5071561692798375</v>
       </c>
       <c r="O77" s="2" t="n">
-        <v>0.4733931316860104</v>
+        <v>0.4908332230905137</v>
       </c>
       <c r="P77" s="1" t="inlineStr"/>
     </row>
-    <row r="78" ht="15" customHeight="1">
+    <row r="78" ht="30" customHeight="1">
       <c r="A78" s="1" t="inlineStr">
         <is>
-          <t>T2_полн_i</t>
+          <t>λ_c2_i</t>
         </is>
       </c>
       <c r="B78" s="1" t="inlineStr">
         <is>
-          <t>Полная температура на выходе из РК</t>
+          <t>Приведенная абсолютная скорость на выходе из РК</t>
         </is>
       </c>
       <c r="C78" s="1" t="inlineStr"/>
       <c r="D78" s="2" t="n">
-        <v>304.6972711556989</v>
+        <v>0.7739140879000126</v>
       </c>
       <c r="E78" s="2" t="n">
-        <v>342.7216074711233</v>
+        <v>0.7025688677305478</v>
       </c>
       <c r="F78" s="2" t="n">
-        <v>380.5533143746371</v>
+        <v>0.6567734946088818</v>
       </c>
       <c r="G78" s="2" t="n">
-        <v>418.299782629001</v>
+        <v>0.6201103319267046</v>
       </c>
       <c r="H78" s="2" t="n">
-        <v>455.8623617326095</v>
+        <v>0.5896922001548817</v>
       </c>
       <c r="I78" s="2" t="n">
-        <v>493.3043052802819</v>
+        <v>0.5641990975072881</v>
       </c>
       <c r="J78" s="2" t="n">
-        <v>530.8455851254013</v>
+        <v>0.5425314394305585</v>
       </c>
       <c r="K78" s="2" t="n">
-        <v>568.2640128064211</v>
+        <v>0.5242135535589888</v>
       </c>
       <c r="L78" s="2" t="n">
-        <v>605.4888593452233</v>
+        <v>0.5085612696312135</v>
       </c>
       <c r="M78" s="2" t="n">
-        <v>642.5848324826002</v>
+        <v>0.4951412220693632</v>
       </c>
       <c r="N78" s="2" t="n">
-        <v>679.4541857759853</v>
+        <v>0.4835545192846229</v>
       </c>
       <c r="O78" s="2" t="n">
-        <v>716.0408161885885</v>
+        <v>0.4733931316860104</v>
       </c>
       <c r="P78" s="1" t="inlineStr"/>
     </row>
     <row r="79" ht="15" customHeight="1">
       <c r="A79" s="1" t="inlineStr">
         <is>
-          <t>τ_2_i</t>
+          <t>T2_полн_i</t>
         </is>
       </c>
       <c r="B79" s="1" t="inlineStr">
         <is>
-          <t>Температурная функция на выходе из РК</t>
+          <t>Полная температура на выходе из РК</t>
         </is>
       </c>
       <c r="C79" s="1" t="inlineStr"/>
       <c r="D79" s="2" t="n">
-        <v>0.9006486075029659</v>
+        <v>304.6972711556989</v>
       </c>
       <c r="E79" s="2" t="n">
-        <v>0.9186155927206895</v>
+        <v>342.7216074711233</v>
       </c>
       <c r="F79" s="2" t="n">
-        <v>0.9290813257877711</v>
+        <v>380.5533143746371</v>
       </c>
       <c r="G79" s="2" t="n">
-        <v>0.9371529110515402</v>
+        <v>418.299782629001</v>
       </c>
       <c r="H79" s="2" t="n">
-        <v>0.9434956981360756</v>
+        <v>455.8623617326095</v>
       </c>
       <c r="I79" s="2" t="n">
-        <v>0.9486821920661557</v>
+        <v>493.3043052802819</v>
       </c>
       <c r="J79" s="2" t="n">
-        <v>0.9529306488556853</v>
+        <v>530.8455851254013</v>
       </c>
       <c r="K79" s="2" t="n">
-        <v>0.9565028945546096</v>
+        <v>568.2640128064211</v>
       </c>
       <c r="L79" s="2" t="n">
-        <v>0.959398073182831</v>
+        <v>605.4888593452233</v>
       </c>
       <c r="M79" s="2" t="n">
-        <v>0.9618447489108495</v>
+        <v>642.5848324826002</v>
       </c>
       <c r="N79" s="2" t="n">
-        <v>0.9639490928348131</v>
+        <v>679.4541857759853</v>
       </c>
       <c r="O79" s="2" t="n">
-        <v>0.9657748293183122</v>
+        <v>716.0408161885885</v>
       </c>
       <c r="P79" s="1" t="inlineStr"/>
     </row>
     <row r="80" ht="15" customHeight="1">
       <c r="A80" s="1" t="inlineStr">
         <is>
-          <t>T_2_i</t>
+          <t>τ_2_i</t>
         </is>
       </c>
       <c r="B80" s="1" t="inlineStr">
         <is>
-          <t>Статическая температура на выходе из РК</t>
+          <t>Температурная функция на выходе из РК</t>
         </is>
       </c>
       <c r="C80" s="1" t="inlineStr"/>
       <c r="D80" s="2" t="n">
-        <v>618.1953492286352</v>
+        <v>0.9006486075029659</v>
       </c>
       <c r="E80" s="2" t="n">
-        <v>630.527691286045</v>
+        <v>0.9186155927206895</v>
       </c>
       <c r="F80" s="2" t="n">
-        <v>637.711255946491</v>
+        <v>0.9290813257877711</v>
       </c>
       <c r="G80" s="2" t="n">
-        <v>643.2515037516795</v>
+        <v>0.9371529110515402</v>
       </c>
       <c r="H80" s="2" t="n">
-        <v>647.6051234032751</v>
+        <v>0.9434956981360756</v>
       </c>
       <c r="I80" s="2" t="n">
-        <v>651.1650760858951</v>
+        <v>0.9486821920661557</v>
       </c>
       <c r="J80" s="2" t="n">
-        <v>654.0811703393106</v>
+        <v>0.9529306488556853</v>
       </c>
       <c r="K80" s="2" t="n">
-        <v>656.5331206992845</v>
+        <v>0.9565028945546096</v>
       </c>
       <c r="L80" s="2" t="n">
-        <v>658.5203396304444</v>
+        <v>0.959398073182831</v>
       </c>
       <c r="M80" s="2" t="n">
-        <v>660.1997110784556</v>
+        <v>0.9618447489108495</v>
       </c>
       <c r="N80" s="2" t="n">
-        <v>661.6441097219828</v>
+        <v>0.9639490928348131</v>
       </c>
       <c r="O80" s="2" t="n">
-        <v>662.8972752669174</v>
+        <v>0.9657748293183122</v>
       </c>
       <c r="P80" s="1" t="inlineStr"/>
     </row>
     <row r="81" ht="15" customHeight="1">
       <c r="A81" s="1" t="inlineStr">
         <is>
-          <t>a_2_i</t>
+          <t>T_2_i</t>
         </is>
       </c>
       <c r="B81" s="1" t="inlineStr">
         <is>
-          <t>Скорость звука на выходе из РК</t>
+          <t>Статическая температура на выходе из РК</t>
         </is>
       </c>
       <c r="C81" s="1" t="inlineStr"/>
       <c r="D81" s="2" t="n">
-        <v>455.2023097056071</v>
+        <v>618.1953492286352</v>
       </c>
       <c r="E81" s="2" t="n">
-        <v>459.5459468369926</v>
+        <v>630.527691286045</v>
       </c>
       <c r="F81" s="2" t="n">
-        <v>462.0107673069759</v>
+        <v>637.711255946491</v>
       </c>
       <c r="G81" s="2" t="n">
-        <v>463.8696816901759</v>
+        <v>643.2515037516795</v>
       </c>
       <c r="H81" s="2" t="n">
-        <v>465.2449251931451</v>
+        <v>647.6051234032751</v>
       </c>
       <c r="I81" s="2" t="n">
-        <v>466.2991149814897</v>
+        <v>651.1650760858951</v>
       </c>
       <c r="J81" s="2" t="n">
-        <v>467.0828615584704</v>
+        <v>654.0811703393106</v>
       </c>
       <c r="K81" s="2" t="n">
-        <v>467.662357643633</v>
+        <v>656.5331206992845</v>
       </c>
       <c r="L81" s="2" t="n">
-        <v>468.0735522884636</v>
+        <v>658.5203396304444</v>
       </c>
       <c r="M81" s="2" t="n">
-        <v>468.4011802428435</v>
+        <v>660.1997110784556</v>
       </c>
       <c r="N81" s="2" t="n">
-        <v>468.6286750273001</v>
+        <v>661.6441097219828</v>
       </c>
       <c r="O81" s="2" t="n">
-        <v>468.7767936030652</v>
+        <v>662.8972752669174</v>
       </c>
       <c r="P81" s="1" t="inlineStr"/>
     </row>
     <row r="82" ht="15" customHeight="1">
       <c r="A82" s="1" t="inlineStr">
         <is>
-          <t>M_c2_ср_i</t>
+          <t>a_2_i</t>
         </is>
       </c>
       <c r="B82" s="1" t="inlineStr">
         <is>
-          <t>Среднее число Маха на выходе из РК</t>
+          <t>Скорость звука на выходе из РК</t>
         </is>
       </c>
       <c r="C82" s="1" t="inlineStr"/>
       <c r="D82" s="2" t="n">
+        <v>455.2023097056071</v>
+      </c>
+      <c r="E82" s="2" t="n">
+        <v>459.5459468369926</v>
+      </c>
+      <c r="F82" s="2" t="n">
+        <v>462.0107673069759</v>
+      </c>
+      <c r="G82" s="2" t="n">
+        <v>463.8696816901759</v>
+      </c>
+      <c r="H82" s="2" t="n">
+        <v>465.2449251931451</v>
+      </c>
+      <c r="I82" s="2" t="n">
+        <v>466.2991149814897</v>
+      </c>
+      <c r="J82" s="2" t="n">
+        <v>467.0828615584704</v>
+      </c>
+      <c r="K82" s="2" t="n">
+        <v>467.662357643633</v>
+      </c>
+      <c r="L82" s="2" t="n">
+        <v>468.0735522884636</v>
+      </c>
+      <c r="M82" s="2" t="n">
+        <v>468.4011802428435</v>
+      </c>
+      <c r="N82" s="2" t="n">
+        <v>468.6286750273001</v>
+      </c>
+      <c r="O82" s="2" t="n">
+        <v>468.7767936030652</v>
+      </c>
+      <c r="P82" s="1" t="inlineStr"/>
+    </row>
+    <row r="83" ht="15" customHeight="1">
+      <c r="A83" s="1" t="inlineStr">
+        <is>
+          <t>M_c2_ср_i</t>
+        </is>
+      </c>
+      <c r="B83" s="1" t="inlineStr">
+        <is>
+          <t>Среднее число Маха на выходе из РК</t>
+        </is>
+      </c>
+      <c r="C83" s="1" t="inlineStr"/>
+      <c r="D83" s="2" t="n">
         <v>0.5432409366286526</v>
       </c>
-      <c r="E82" s="2" t="n">
+      <c r="E83" s="2" t="n">
         <v>0.5178623727930555</v>
       </c>
-      <c r="F82" s="2" t="n">
+      <c r="F83" s="2" t="n">
         <v>0.5073033157096933</v>
       </c>
-      <c r="G82" s="2" t="n">
+      <c r="G83" s="2" t="n">
         <v>0.4999555512253943</v>
       </c>
-      <c r="H82" s="2" t="n">
+      <c r="H83" s="2" t="n">
         <v>0.4946509969377347</v>
       </c>
-      <c r="I82" s="2" t="n">
+      <c r="I83" s="2" t="n">
         <v>0.4909359118643687</v>
       </c>
-      <c r="J82" s="2" t="n">
+      <c r="J83" s="2" t="n">
         <v>0.4886202835695136</v>
       </c>
-      <c r="K82" s="2" t="n">
+      <c r="K83" s="2" t="n">
         <v>0.4875310564678288</v>
       </c>
-      <c r="L82" s="2" t="n">
+      <c r="L83" s="2" t="n">
         <v>0.4875168545088711</v>
       </c>
-      <c r="M82" s="2" t="n">
+      <c r="M83" s="2" t="n">
         <v>0.4883478891953212</v>
       </c>
-      <c r="N82" s="2" t="n">
+      <c r="N83" s="2" t="n">
         <v>0.4898652672059366</v>
       </c>
-      <c r="O82" s="2" t="n">
+      <c r="O83" s="2" t="n">
         <v>0.4918474434373172</v>
       </c>
-      <c r="P82" s="1" t="inlineStr"/>
+      <c r="P83" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Changes in limits of Ht_average
</commit_message>
<xml_diff>
--- a/results/Поступенчатый_расчет_ступеней.xlsx
+++ b/results/Поступенчатый_расчет_ступеней.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T83"/>
+  <dimension ref="A1:S83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -433,17 +433,16 @@
     <col width="21" customWidth="1" min="7" max="7"/>
     <col width="22" customWidth="1" min="8" max="8"/>
     <col width="22" customWidth="1" min="9" max="9"/>
-    <col width="22" customWidth="1" min="10" max="10"/>
+    <col width="21" customWidth="1" min="10" max="10"/>
     <col width="22" customWidth="1" min="11" max="11"/>
     <col width="22" customWidth="1" min="12" max="12"/>
     <col width="22" customWidth="1" min="13" max="13"/>
-    <col width="21" customWidth="1" min="14" max="14"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
     <col width="22" customWidth="1" min="15" max="15"/>
     <col width="22" customWidth="1" min="16" max="16"/>
-    <col width="21" customWidth="1" min="17" max="17"/>
-    <col width="21" customWidth="1" min="18" max="18"/>
-    <col width="22" customWidth="1" min="19" max="19"/>
-    <col width="22" customWidth="1" min="20" max="20"/>
+    <col width="22" customWidth="1" min="17" max="17"/>
+    <col width="22" customWidth="1" min="18" max="18"/>
+    <col width="21" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1">
@@ -538,11 +537,6 @@
         </is>
       </c>
       <c r="S1" s="1" t="inlineStr">
-        <is>
-          <t>Ступень 16</t>
-        </is>
-      </c>
-      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>СА</t>
         </is>
@@ -578,7 +572,6 @@
       <c r="Q2" s="1" t="inlineStr"/>
       <c r="R2" s="1" t="inlineStr"/>
       <c r="S2" s="1" t="inlineStr"/>
-      <c r="T2" s="1" t="inlineStr"/>
     </row>
     <row r="3" ht="15" customHeight="1">
       <c r="A3" s="1" t="inlineStr">
@@ -610,7 +603,6 @@
       <c r="Q3" s="1" t="inlineStr"/>
       <c r="R3" s="1" t="inlineStr"/>
       <c r="S3" s="1" t="inlineStr"/>
-      <c r="T3" s="1" t="inlineStr"/>
     </row>
     <row r="4" ht="15" customHeight="1">
       <c r="A4" s="1" t="inlineStr">
@@ -642,7 +634,6 @@
       <c r="Q4" s="1" t="inlineStr"/>
       <c r="R4" s="1" t="inlineStr"/>
       <c r="S4" s="1" t="inlineStr"/>
-      <c r="T4" s="1" t="inlineStr"/>
     </row>
     <row r="5" ht="15" customHeight="1">
       <c r="A5" s="1" t="inlineStr">
@@ -674,7 +665,6 @@
       <c r="Q5" s="1" t="inlineStr"/>
       <c r="R5" s="1" t="inlineStr"/>
       <c r="S5" s="1" t="inlineStr"/>
-      <c r="T5" s="1" t="inlineStr"/>
     </row>
     <row r="6" ht="15" customHeight="1">
       <c r="A6" s="1" t="inlineStr">
@@ -706,7 +696,6 @@
       <c r="Q6" s="1" t="inlineStr"/>
       <c r="R6" s="1" t="inlineStr"/>
       <c r="S6" s="1" t="inlineStr"/>
-      <c r="T6" s="1" t="inlineStr"/>
     </row>
     <row r="7" ht="15" customHeight="1">
       <c r="A7" s="1" t="inlineStr">
@@ -738,7 +727,6 @@
       <c r="Q7" s="1" t="inlineStr"/>
       <c r="R7" s="1" t="inlineStr"/>
       <c r="S7" s="1" t="inlineStr"/>
-      <c r="T7" s="1" t="inlineStr"/>
     </row>
     <row r="8" ht="15" customHeight="1">
       <c r="A8" s="1" t="inlineStr">
@@ -767,8 +755,7 @@
       <c r="P8" s="1" t="inlineStr"/>
       <c r="Q8" s="1" t="inlineStr"/>
       <c r="R8" s="1" t="inlineStr"/>
-      <c r="S8" s="1" t="inlineStr"/>
-      <c r="T8" s="2" t="n">
+      <c r="S8" s="2" t="n">
         <v>477.1612274741949</v>
       </c>
     </row>
@@ -799,8 +786,7 @@
       <c r="P9" s="1" t="inlineStr"/>
       <c r="Q9" s="1" t="inlineStr"/>
       <c r="R9" s="1" t="inlineStr"/>
-      <c r="S9" s="1" t="inlineStr"/>
-      <c r="T9" s="2" t="n">
+      <c r="S9" s="2" t="n">
         <v>0.9595531619480527</v>
       </c>
     </row>
@@ -831,9 +817,8 @@
       <c r="P10" s="1" t="inlineStr"/>
       <c r="Q10" s="1" t="inlineStr"/>
       <c r="R10" s="1" t="inlineStr"/>
-      <c r="S10" s="1" t="inlineStr"/>
-      <c r="T10" s="2" t="n">
-        <v>107.3941909302498</v>
+      <c r="S10" s="2" t="n">
+        <v>107.1825264245426</v>
       </c>
     </row>
     <row r="11" ht="15" customHeight="1">
@@ -863,8 +848,7 @@
       <c r="P11" s="1" t="inlineStr"/>
       <c r="Q11" s="1" t="inlineStr"/>
       <c r="R11" s="1" t="inlineStr"/>
-      <c r="S11" s="1" t="inlineStr"/>
-      <c r="T11" s="2" t="n">
+      <c r="S11" s="2" t="n">
         <v>0.4537118711400231</v>
       </c>
     </row>
@@ -895,9 +879,8 @@
       <c r="P12" s="1" t="inlineStr"/>
       <c r="Q12" s="1" t="inlineStr"/>
       <c r="R12" s="1" t="inlineStr"/>
-      <c r="S12" s="1" t="inlineStr"/>
-      <c r="T12" s="2" t="n">
-        <v>0.05491106614839087</v>
+      <c r="S12" s="2" t="n">
+        <v>0.05503600366715333</v>
       </c>
     </row>
     <row r="13" ht="15" customHeight="1">
@@ -927,8 +910,7 @@
       <c r="P13" s="1" t="inlineStr"/>
       <c r="Q13" s="1" t="inlineStr"/>
       <c r="R13" s="1" t="inlineStr"/>
-      <c r="S13" s="1" t="inlineStr"/>
-      <c r="T13" s="2" t="n">
+      <c r="S13" s="2" t="n">
         <v>1.570796326794897</v>
       </c>
     </row>
@@ -959,9 +941,8 @@
       <c r="P14" s="1" t="inlineStr"/>
       <c r="Q14" s="1" t="inlineStr"/>
       <c r="R14" s="1" t="inlineStr"/>
-      <c r="S14" s="1" t="inlineStr"/>
-      <c r="T14" s="2" t="n">
-        <v>0.05491106614839087</v>
+      <c r="S14" s="2" t="n">
+        <v>0.05503600366715333</v>
       </c>
     </row>
     <row r="15" ht="15" customHeight="1">
@@ -991,9 +972,8 @@
       <c r="P15" s="1" t="inlineStr"/>
       <c r="Q15" s="1" t="inlineStr"/>
       <c r="R15" s="1" t="inlineStr"/>
-      <c r="S15" s="1" t="inlineStr"/>
-      <c r="T15" s="2" t="n">
-        <v>0.3452273254016311</v>
+      <c r="S15" s="2" t="n">
+        <v>0.3446443080405253</v>
       </c>
     </row>
     <row r="16" ht="15" customHeight="1">
@@ -1023,9 +1003,8 @@
       <c r="P16" s="1" t="inlineStr"/>
       <c r="Q16" s="1" t="inlineStr"/>
       <c r="R16" s="1" t="inlineStr"/>
-      <c r="S16" s="1" t="inlineStr"/>
-      <c r="T16" s="2" t="n">
-        <v>0.5071108561666231</v>
+      <c r="S16" s="2" t="n">
+        <v>0.5062544510926434</v>
       </c>
     </row>
     <row r="17" ht="15" customHeight="1">
@@ -1055,9 +1034,8 @@
       <c r="P17" s="1" t="inlineStr"/>
       <c r="Q17" s="1" t="inlineStr"/>
       <c r="R17" s="1" t="inlineStr"/>
-      <c r="S17" s="1" t="inlineStr"/>
-      <c r="T17" s="2" t="n">
-        <v>0.7928308206805679</v>
+      <c r="S17" s="2" t="n">
+        <v>0.7925571175792675</v>
       </c>
     </row>
     <row r="18" ht="15" customHeight="1">
@@ -1087,9 +1065,8 @@
       <c r="P18" s="1" t="inlineStr"/>
       <c r="Q18" s="1" t="inlineStr"/>
       <c r="R18" s="1" t="inlineStr"/>
-      <c r="S18" s="1" t="inlineStr"/>
-      <c r="T18" s="2" t="n">
-        <v>0.861508375559446</v>
+      <c r="S18" s="2" t="n">
+        <v>0.8596778720441994</v>
       </c>
     </row>
     <row r="19" ht="15" customHeight="1">
@@ -1119,9 +1096,8 @@
       <c r="P19" s="1" t="inlineStr"/>
       <c r="Q19" s="1" t="inlineStr"/>
       <c r="R19" s="1" t="inlineStr"/>
-      <c r="S19" s="1" t="inlineStr"/>
-      <c r="T19" s="2" t="n">
-        <v>0.7092879512354505</v>
+      <c r="S19" s="2" t="n">
+        <v>0.7111184547506971</v>
       </c>
     </row>
     <row r="20" ht="15" customHeight="1">
@@ -1151,9 +1127,8 @@
       <c r="P20" s="1" t="inlineStr"/>
       <c r="Q20" s="1" t="inlineStr"/>
       <c r="R20" s="1" t="inlineStr"/>
-      <c r="S20" s="1" t="inlineStr"/>
-      <c r="T20" s="2" t="n">
-        <v>141.5268009329557</v>
+      <c r="S20" s="2" t="n">
+        <v>141.4703657841591</v>
       </c>
     </row>
     <row r="21" ht="30" customHeight="1">
@@ -1183,9 +1158,8 @@
       <c r="P21" s="1" t="inlineStr"/>
       <c r="Q21" s="1" t="inlineStr"/>
       <c r="R21" s="1" t="inlineStr"/>
-      <c r="S21" s="1" t="inlineStr"/>
-      <c r="T21" s="2" t="n">
-        <v>0.919408386540464</v>
+      <c r="S21" s="2" t="n">
+        <v>0.9193151445039431</v>
       </c>
     </row>
     <row r="22" ht="15" customHeight="1">
@@ -1215,9 +1189,8 @@
       <c r="P22" s="1" t="inlineStr"/>
       <c r="Q22" s="1" t="inlineStr"/>
       <c r="R22" s="1" t="inlineStr"/>
-      <c r="S22" s="1" t="inlineStr"/>
-      <c r="T22" s="2" t="n">
-        <v>0.6259083085630148</v>
+      <c r="S22" s="2" t="n">
+        <v>0.6258448319119204</v>
       </c>
     </row>
     <row r="23" ht="15" customHeight="1">
@@ -1247,9 +1220,8 @@
       <c r="P23" s="1" t="inlineStr"/>
       <c r="Q23" s="1" t="inlineStr"/>
       <c r="R23" s="1" t="inlineStr"/>
-      <c r="S23" s="1" t="inlineStr"/>
-      <c r="T23" s="2" t="n">
-        <v>0.02743229298496425</v>
+      <c r="S23" s="2" t="n">
+        <v>0.02746403131051145</v>
       </c>
     </row>
     <row r="24" ht="15" customHeight="1">
@@ -1279,9 +1251,8 @@
       <c r="P24" s="1" t="inlineStr"/>
       <c r="Q24" s="1" t="inlineStr"/>
       <c r="R24" s="1" t="inlineStr"/>
-      <c r="S24" s="1" t="inlineStr"/>
-      <c r="T24" s="2" t="n">
-        <v>0.1677727845656561</v>
+      <c r="S24" s="2" t="n">
+        <v>0.168064293246209</v>
       </c>
     </row>
     <row r="25" ht="30" customHeight="1">
@@ -1300,51 +1271,48 @@
         <v>1.399944336209296</v>
       </c>
       <c r="E25" s="2" t="n">
-        <v>1.398030109901669</v>
+        <v>1.397925561088529</v>
       </c>
       <c r="F25" s="2" t="n">
-        <v>1.397119376129521</v>
+        <v>1.395818006608158</v>
       </c>
       <c r="G25" s="2" t="n">
-        <v>1.395156317152682</v>
+        <v>1.39503266988259</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>1.393623697897493</v>
+        <v>1.393257398883002</v>
       </c>
       <c r="I25" s="2" t="n">
-        <v>1.392036202062929</v>
+        <v>1.390896057070977</v>
       </c>
       <c r="J25" s="2" t="n">
-        <v>1.389809783724452</v>
+        <v>1.388904920518764</v>
       </c>
       <c r="K25" s="2" t="n">
-        <v>1.387086457843369</v>
+        <v>1.386004386389407</v>
       </c>
       <c r="L25" s="2" t="n">
-        <v>1.384896195015433</v>
+        <v>1.383337910643934</v>
       </c>
       <c r="M25" s="2" t="n">
-        <v>1.382177452656831</v>
+        <v>1.380449879843793</v>
       </c>
       <c r="N25" s="2" t="n">
-        <v>1.378497276781724</v>
+        <v>1.376615395737872</v>
       </c>
       <c r="O25" s="2" t="n">
-        <v>1.375867872658643</v>
+        <v>1.373817483070391</v>
       </c>
       <c r="P25" s="2" t="n">
-        <v>1.373209687129157</v>
+        <v>1.370798140159712</v>
       </c>
       <c r="Q25" s="2" t="n">
-        <v>1.370399242345619</v>
+        <v>1.367827181223123</v>
       </c>
       <c r="R25" s="2" t="n">
-        <v>1.36763080914184</v>
-      </c>
-      <c r="S25" s="2" t="n">
         <v>1.364566577433034</v>
       </c>
-      <c r="T25" s="1" t="inlineStr"/>
+      <c r="S25" s="1" t="inlineStr"/>
     </row>
     <row r="26" ht="15" customHeight="1">
       <c r="A26" s="1" t="inlineStr">
@@ -1362,51 +1330,48 @@
         <v>0.65</v>
       </c>
       <c r="E26" s="2" t="n">
-        <v>0.6306666666666667</v>
+        <v>0.6292857142857143</v>
       </c>
       <c r="F26" s="2" t="n">
-        <v>0.6113333333333334</v>
+        <v>0.6085714285714285</v>
       </c>
       <c r="G26" s="2" t="n">
-        <v>0.592</v>
+        <v>0.5878571428571429</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>0.5726666666666667</v>
+        <v>0.5671428571428572</v>
       </c>
       <c r="I26" s="2" t="n">
-        <v>0.5533333333333333</v>
+        <v>0.5464285714285715</v>
       </c>
       <c r="J26" s="2" t="n">
-        <v>0.534</v>
+        <v>0.5257142857142857</v>
       </c>
       <c r="K26" s="2" t="n">
-        <v>0.5146666666666667</v>
+        <v>0.505</v>
       </c>
       <c r="L26" s="2" t="n">
-        <v>0.4953333333333333</v>
+        <v>0.4842857142857143</v>
       </c>
       <c r="M26" s="2" t="n">
-        <v>0.476</v>
+        <v>0.4635714285714286</v>
       </c>
       <c r="N26" s="2" t="n">
-        <v>0.4566666666666667</v>
+        <v>0.4428571428571428</v>
       </c>
       <c r="O26" s="2" t="n">
-        <v>0.4373333333333334</v>
+        <v>0.4221428571428572</v>
       </c>
       <c r="P26" s="2" t="n">
-        <v>0.418</v>
+        <v>0.4014285714285714</v>
       </c>
       <c r="Q26" s="2" t="n">
-        <v>0.3986666666666667</v>
+        <v>0.3807142857142857</v>
       </c>
       <c r="R26" s="2" t="n">
-        <v>0.3793333333333334</v>
-      </c>
-      <c r="S26" s="2" t="n">
         <v>0.36</v>
       </c>
-      <c r="T26" s="1" t="inlineStr"/>
+      <c r="S26" s="1" t="inlineStr"/>
     </row>
     <row r="27" ht="15" customHeight="1">
       <c r="A27" s="1" t="inlineStr">
@@ -1421,54 +1386,51 @@
       </c>
       <c r="C27" s="1" t="inlineStr"/>
       <c r="D27" s="2" t="n">
-        <v>0.6306666666666667</v>
+        <v>0.6292857142857143</v>
       </c>
       <c r="E27" s="2" t="n">
-        <v>0.6113333333333334</v>
+        <v>0.6085714285714285</v>
       </c>
       <c r="F27" s="2" t="n">
-        <v>0.592</v>
+        <v>0.5878571428571429</v>
       </c>
       <c r="G27" s="2" t="n">
-        <v>0.5726666666666667</v>
+        <v>0.5671428571428572</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>0.5533333333333333</v>
+        <v>0.5464285714285715</v>
       </c>
       <c r="I27" s="2" t="n">
-        <v>0.534</v>
+        <v>0.5257142857142857</v>
       </c>
       <c r="J27" s="2" t="n">
-        <v>0.5146666666666667</v>
+        <v>0.505</v>
       </c>
       <c r="K27" s="2" t="n">
-        <v>0.4953333333333333</v>
+        <v>0.4842857142857143</v>
       </c>
       <c r="L27" s="2" t="n">
-        <v>0.476</v>
+        <v>0.4635714285714286</v>
       </c>
       <c r="M27" s="2" t="n">
-        <v>0.4566666666666667</v>
+        <v>0.4428571428571428</v>
       </c>
       <c r="N27" s="2" t="n">
-        <v>0.4373333333333334</v>
+        <v>0.4221428571428572</v>
       </c>
       <c r="O27" s="2" t="n">
-        <v>0.418</v>
+        <v>0.4014285714285714</v>
       </c>
       <c r="P27" s="2" t="n">
-        <v>0.3986666666666667</v>
+        <v>0.3807142857142857</v>
       </c>
       <c r="Q27" s="2" t="n">
-        <v>0.3793333333333334</v>
+        <v>0.36</v>
       </c>
       <c r="R27" s="2" t="n">
-        <v>0.36</v>
-      </c>
-      <c r="S27" s="2" t="n">
-        <v>0.3406666666666666</v>
-      </c>
-      <c r="T27" s="1" t="inlineStr"/>
+        <v>0.3392857142857142</v>
+      </c>
+      <c r="S27" s="1" t="inlineStr"/>
     </row>
     <row r="28" ht="15" customHeight="1">
       <c r="A28" s="1" t="inlineStr">
@@ -1486,51 +1448,48 @@
         <v>100292.8790575521</v>
       </c>
       <c r="E28" s="2" t="n">
-        <v>217076.2130468525</v>
+        <v>225417.879760374</v>
       </c>
       <c r="F28" s="2" t="n">
-        <v>333859.5470361529</v>
+        <v>350542.8804631958</v>
       </c>
       <c r="G28" s="2" t="n">
-        <v>450642.8810254533</v>
+        <v>475667.8811660177</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>567426.2150147536</v>
+        <v>600792.8818688395</v>
       </c>
       <c r="I28" s="2" t="n">
-        <v>684209.5490040539</v>
+        <v>725917.8825716614</v>
       </c>
       <c r="J28" s="2" t="n">
-        <v>800992.8829933545</v>
+        <v>851042.8832744833</v>
       </c>
       <c r="K28" s="2" t="n">
-        <v>917776.2169826548</v>
+        <v>976167.8839773049</v>
       </c>
       <c r="L28" s="2" t="n">
-        <v>1034559.550971955</v>
+        <v>1101292.884680127</v>
       </c>
       <c r="M28" s="2" t="n">
-        <v>1151342.884961256</v>
+        <v>1226417.885382949</v>
       </c>
       <c r="N28" s="2" t="n">
-        <v>1268126.218950556</v>
+        <v>1351542.886085771</v>
       </c>
       <c r="O28" s="2" t="n">
-        <v>1384909.552939856</v>
+        <v>1476667.886788592</v>
       </c>
       <c r="P28" s="2" t="n">
-        <v>1501692.886929157</v>
+        <v>1601792.887491414</v>
       </c>
       <c r="Q28" s="2" t="n">
-        <v>1618476.220918457</v>
+        <v>1726917.888194236</v>
       </c>
       <c r="R28" s="2" t="n">
-        <v>1735259.554907757</v>
-      </c>
-      <c r="S28" s="2" t="n">
         <v>1852042.888897058</v>
       </c>
-      <c r="T28" s="1" t="inlineStr"/>
+      <c r="S28" s="1" t="inlineStr"/>
     </row>
     <row r="29" ht="15" customHeight="1">
       <c r="A29" s="1" t="inlineStr">
@@ -1548,51 +1507,48 @@
         <v>288</v>
       </c>
       <c r="E29" s="2" t="n">
-        <v>314.5592705285711</v>
+        <v>316.4563612806118</v>
       </c>
       <c r="F29" s="2" t="n">
-        <v>341.1185410571421</v>
+        <v>344.9127225612236</v>
       </c>
       <c r="G29" s="2" t="n">
-        <v>367.6778115857131</v>
+        <v>373.3690838418355</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>394.2370821142841</v>
+        <v>401.8254451224473</v>
       </c>
       <c r="I29" s="2" t="n">
-        <v>420.7963526428552</v>
+        <v>430.2818064030591</v>
       </c>
       <c r="J29" s="2" t="n">
-        <v>447.3556231714263</v>
+        <v>458.738167683671</v>
       </c>
       <c r="K29" s="2" t="n">
-        <v>473.9148936999973</v>
+        <v>487.1945289642828</v>
       </c>
       <c r="L29" s="2" t="n">
-        <v>500.4741642285683</v>
+        <v>515.6508902448945</v>
       </c>
       <c r="M29" s="2" t="n">
-        <v>527.0334347571393</v>
+        <v>544.1072515255064</v>
       </c>
       <c r="N29" s="2" t="n">
-        <v>553.5927052857104</v>
+        <v>572.5636128061183</v>
       </c>
       <c r="O29" s="2" t="n">
-        <v>580.1519758142814</v>
+        <v>601.01997408673</v>
       </c>
       <c r="P29" s="2" t="n">
-        <v>606.7112463428525</v>
+        <v>629.4763353673419</v>
       </c>
       <c r="Q29" s="2" t="n">
-        <v>633.2705168714235</v>
+        <v>657.9326966479537</v>
       </c>
       <c r="R29" s="2" t="n">
-        <v>659.8297873999945</v>
-      </c>
-      <c r="S29" s="2" t="n">
         <v>686.3890579285655</v>
       </c>
-      <c r="T29" s="1" t="inlineStr"/>
+      <c r="S29" s="1" t="inlineStr"/>
     </row>
     <row r="30" ht="30" customHeight="1">
       <c r="A30" s="1" t="inlineStr">
@@ -1610,51 +1566,48 @@
         <v>0.43</v>
       </c>
       <c r="E30" s="2" t="n">
-        <v>0.4624883110069641</v>
+        <v>0.4648089046503187</v>
       </c>
       <c r="F30" s="2" t="n">
-        <v>0.4949766220139281</v>
+        <v>0.4996178093006373</v>
       </c>
       <c r="G30" s="2" t="n">
-        <v>0.5274649330208923</v>
+        <v>0.534426713950956</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>0.5599532440278563</v>
+        <v>0.5692356186012746</v>
       </c>
       <c r="I30" s="2" t="n">
-        <v>0.5924415550348203</v>
+        <v>0.6040445232515932</v>
       </c>
       <c r="J30" s="2" t="n">
-        <v>0.6249298660417845</v>
+        <v>0.6388534279019119</v>
       </c>
       <c r="K30" s="2" t="n">
-        <v>0.6574181770487485</v>
+        <v>0.6736623325522305</v>
       </c>
       <c r="L30" s="2" t="n">
-        <v>0.6899064880557126</v>
+        <v>0.7084712372025492</v>
       </c>
       <c r="M30" s="2" t="n">
-        <v>0.7223947990626767</v>
+        <v>0.7432801418528678</v>
       </c>
       <c r="N30" s="2" t="n">
-        <v>0.7548831100696407</v>
+        <v>0.7780890465031864</v>
       </c>
       <c r="O30" s="2" t="n">
-        <v>0.7873714210766047</v>
+        <v>0.812897951153505</v>
       </c>
       <c r="P30" s="2" t="n">
-        <v>0.8198597320835689</v>
+        <v>0.8477068558038238</v>
       </c>
       <c r="Q30" s="2" t="n">
-        <v>0.852348043090533</v>
+        <v>0.8825157604541425</v>
       </c>
       <c r="R30" s="2" t="n">
-        <v>0.8848363540974971</v>
-      </c>
-      <c r="S30" s="2" t="n">
         <v>0.9173246651044611</v>
       </c>
-      <c r="T30" s="1" t="inlineStr"/>
+      <c r="S30" s="1" t="inlineStr"/>
     </row>
     <row r="31" ht="30" customHeight="1">
       <c r="A31" s="1" t="inlineStr">
@@ -1713,10 +1666,7 @@
       <c r="R31" s="2" t="n">
         <v>306.5485944726447</v>
       </c>
-      <c r="S31" s="2" t="n">
-        <v>306.5485944726447</v>
-      </c>
-      <c r="T31" s="1" t="inlineStr"/>
+      <c r="S31" s="1" t="inlineStr"/>
     </row>
     <row r="32" ht="15" customHeight="1">
       <c r="A32" s="1" t="inlineStr">
@@ -1734,51 +1684,48 @@
         <v>16967.12604306373</v>
       </c>
       <c r="E32" s="2" t="n">
-        <v>18522.44457042484</v>
+        <v>18630.78159248007</v>
       </c>
       <c r="F32" s="2" t="n">
-        <v>20010.85352487777</v>
+        <v>20218.5607708968</v>
       </c>
       <c r="G32" s="2" t="n">
-        <v>21443.52757416789</v>
+        <v>21743.63912220311</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>22826.43669504646</v>
+        <v>23213.0501078087</v>
       </c>
       <c r="I32" s="2" t="n">
-        <v>24164.78508955374</v>
+        <v>24632.76848581418</v>
       </c>
       <c r="J32" s="2" t="n">
-        <v>25460.68314778449</v>
+        <v>26002.0239099061</v>
       </c>
       <c r="K32" s="2" t="n">
-        <v>26711.24295341488</v>
+        <v>27318.78381964874</v>
       </c>
       <c r="L32" s="2" t="n">
-        <v>27912.59985073472</v>
+        <v>28574.47174295057</v>
       </c>
       <c r="M32" s="2" t="n">
-        <v>29057.20999885778</v>
+        <v>29758.48274205851</v>
       </c>
       <c r="N32" s="2" t="n">
-        <v>30135.06929757995</v>
+        <v>30856.11876136259</v>
       </c>
       <c r="O32" s="2" t="n">
-        <v>31131.51671175844</v>
+        <v>31847.15753258983</v>
       </c>
       <c r="P32" s="2" t="n">
-        <v>32030.58870804145</v>
+        <v>32709.42570822144</v>
       </c>
       <c r="Q32" s="2" t="n">
-        <v>32813.11863637829</v>
+        <v>33415.02270248366</v>
       </c>
       <c r="R32" s="2" t="n">
-        <v>33455.75153274887</v>
-      </c>
-      <c r="S32" s="2" t="n">
         <v>33933.38931404932</v>
       </c>
-      <c r="T32" s="1" t="inlineStr"/>
+      <c r="S32" s="1" t="inlineStr"/>
     </row>
     <row r="33" ht="15" customHeight="1">
       <c r="A33" s="1" t="inlineStr">
@@ -1796,51 +1743,48 @@
         <v>16797.45478263309</v>
       </c>
       <c r="E33" s="2" t="n">
-        <v>18151.99567901635</v>
+        <v>18258.16596063047</v>
       </c>
       <c r="F33" s="2" t="n">
-        <v>19410.52791913144</v>
+        <v>19612.0039477699</v>
       </c>
       <c r="G33" s="2" t="n">
-        <v>20585.78647120117</v>
+        <v>20873.89355731498</v>
       </c>
       <c r="H33" s="2" t="n">
-        <v>21685.11486029413</v>
+        <v>22052.39760241826</v>
       </c>
       <c r="I33" s="2" t="n">
-        <v>22714.89798418052</v>
+        <v>23154.80237666533</v>
       </c>
       <c r="J33" s="2" t="n">
-        <v>23933.04215891742</v>
+        <v>24441.90247531174</v>
       </c>
       <c r="K33" s="2" t="n">
-        <v>25108.56837620999</v>
+        <v>25679.65679046981</v>
       </c>
       <c r="L33" s="2" t="n">
-        <v>26237.84385969064</v>
+        <v>26860.00343837353</v>
       </c>
       <c r="M33" s="2" t="n">
-        <v>27313.77739892632</v>
+        <v>27972.97377753499</v>
       </c>
       <c r="N33" s="2" t="n">
-        <v>28326.96513972515</v>
+        <v>29004.75163568083</v>
       </c>
       <c r="O33" s="2" t="n">
-        <v>29263.62570905293</v>
+        <v>29936.32808063443</v>
       </c>
       <c r="P33" s="2" t="n">
-        <v>30108.75338555896</v>
+        <v>30746.86016572815</v>
       </c>
       <c r="Q33" s="2" t="n">
-        <v>30844.33151819559</v>
+        <v>31410.12134033464</v>
       </c>
       <c r="R33" s="2" t="n">
-        <v>31448.40644078394</v>
-      </c>
-      <c r="S33" s="2" t="n">
         <v>31897.38595520635</v>
       </c>
-      <c r="T33" s="1" t="inlineStr"/>
+      <c r="S33" s="1" t="inlineStr"/>
     </row>
     <row r="34" ht="15" customHeight="1">
       <c r="A34" s="1" t="inlineStr">
@@ -1858,51 +1802,48 @@
         <v>13701.87693398603</v>
       </c>
       <c r="E34" s="2" t="n">
-        <v>15076.69597297022</v>
+        <v>15183.18715242576</v>
       </c>
       <c r="F34" s="2" t="n">
-        <v>16380.32104836129</v>
+        <v>16585.02366398544</v>
       </c>
       <c r="G34" s="2" t="n">
-        <v>17612.45722779648</v>
+        <v>17906.52312846286</v>
       </c>
       <c r="H34" s="2" t="n">
-        <v>18768.90312231542</v>
+        <v>19142.33211474175</v>
       </c>
       <c r="I34" s="2" t="n">
-        <v>19845.7876917099</v>
+        <v>20287.40656738138</v>
       </c>
       <c r="J34" s="2" t="n">
-        <v>21061.22894992113</v>
+        <v>21560.80915145568</v>
       </c>
       <c r="K34" s="2" t="n">
-        <v>22205.82054603481</v>
+        <v>22748.12080720581</v>
       </c>
       <c r="L34" s="2" t="n">
-        <v>23267.30088055942</v>
+        <v>23831.00891765521</v>
       </c>
       <c r="M34" s="2" t="n">
-        <v>24230.49891283819</v>
+        <v>24789.99333265435</v>
       </c>
       <c r="N34" s="2" t="n">
-        <v>25078.5381918534</v>
+        <v>25602.7462639698</v>
       </c>
       <c r="O34" s="2" t="n">
-        <v>25791.39094590568</v>
+        <v>26243.62718943152</v>
       </c>
       <c r="P34" s="2" t="n">
-        <v>26348.87669288917</v>
+        <v>26686.81663025726</v>
       </c>
       <c r="Q34" s="2" t="n">
-        <v>26729.44485873016</v>
+        <v>26904.66888708492</v>
       </c>
       <c r="R34" s="2" t="n">
-        <v>26910.5198447063</v>
-      </c>
-      <c r="S34" s="2" t="n">
         <v>26870.38869889748</v>
       </c>
-      <c r="T34" s="1" t="inlineStr"/>
+      <c r="S34" s="1" t="inlineStr"/>
     </row>
     <row r="35" ht="15" customHeight="1">
       <c r="A35" s="1" t="inlineStr">
@@ -1920,51 +1861,48 @@
         <v>16.6972711556989</v>
       </c>
       <c r="E35" s="2" t="n">
-        <v>17.98195958095144</v>
+        <v>18.08373681547279</v>
       </c>
       <c r="F35" s="2" t="n">
-        <v>19.19721130784214</v>
+        <v>19.35093521240871</v>
       </c>
       <c r="G35" s="2" t="n">
-        <v>20.28741714564764</v>
+        <v>20.56673424835787</v>
       </c>
       <c r="H35" s="2" t="n">
-        <v>21.31133604977339</v>
+        <v>21.65781275498967</v>
       </c>
       <c r="I35" s="2" t="n">
-        <v>22.2586935435603</v>
+        <v>22.64232024894013</v>
       </c>
       <c r="J35" s="2" t="n">
-        <v>23.35654027139916</v>
+        <v>23.81327704394781</v>
       </c>
       <c r="K35" s="2" t="n">
-        <v>24.38033301608176</v>
+        <v>24.88456689222609</v>
       </c>
       <c r="L35" s="2" t="n">
-        <v>25.37276372176333</v>
+        <v>25.89839154897781</v>
       </c>
       <c r="M35" s="2" t="n">
-        <v>26.27823905870514</v>
+        <v>26.82431759468589</v>
       </c>
       <c r="N35" s="2" t="n">
-        <v>27.06263816738749</v>
+        <v>27.61009078020989</v>
       </c>
       <c r="O35" s="2" t="n">
-        <v>27.81633101439324</v>
+        <v>28.34277284468556</v>
       </c>
       <c r="P35" s="2" t="n">
-        <v>28.47226781897626</v>
+        <v>28.93863549455284</v>
       </c>
       <c r="Q35" s="2" t="n">
-        <v>29.00758532167604</v>
+        <v>29.38971940023348</v>
       </c>
       <c r="R35" s="2" t="n">
-        <v>29.41405527703473</v>
-      </c>
-      <c r="S35" s="2" t="n">
         <v>29.65175826002295</v>
       </c>
-      <c r="T35" s="1" t="inlineStr"/>
+      <c r="S35" s="1" t="inlineStr"/>
     </row>
     <row r="36" ht="15" customHeight="1">
       <c r="A36" s="1" t="inlineStr">
@@ -1982,51 +1920,48 @@
         <v>304.6972711556989</v>
       </c>
       <c r="E36" s="2" t="n">
-        <v>332.5412301095225</v>
+        <v>334.5400980960846</v>
       </c>
       <c r="F36" s="2" t="n">
-        <v>360.3157523649842</v>
+        <v>364.2636577736324</v>
       </c>
       <c r="G36" s="2" t="n">
-        <v>387.9652287313608</v>
+        <v>393.9358180901934</v>
       </c>
       <c r="H36" s="2" t="n">
-        <v>415.5484181640575</v>
+        <v>423.4832578774369</v>
       </c>
       <c r="I36" s="2" t="n">
-        <v>443.0550461864155</v>
+        <v>452.9241266519992</v>
       </c>
       <c r="J36" s="2" t="n">
-        <v>470.7121634428254</v>
+        <v>482.5514447276188</v>
       </c>
       <c r="K36" s="2" t="n">
-        <v>498.295226716079</v>
+        <v>512.0790958565088</v>
       </c>
       <c r="L36" s="2" t="n">
-        <v>525.8469279503316</v>
+        <v>541.5492817938723</v>
       </c>
       <c r="M36" s="2" t="n">
-        <v>553.3116738158444</v>
+        <v>570.9315691201923</v>
       </c>
       <c r="N36" s="2" t="n">
-        <v>580.6553434530979</v>
+        <v>600.1737035863282</v>
       </c>
       <c r="O36" s="2" t="n">
-        <v>607.9683068286746</v>
+        <v>629.3627469314156</v>
       </c>
       <c r="P36" s="2" t="n">
-        <v>635.1835141618287</v>
+        <v>658.4149708618947</v>
       </c>
       <c r="Q36" s="2" t="n">
-        <v>662.2781021930996</v>
+        <v>687.3224160481872</v>
       </c>
       <c r="R36" s="2" t="n">
-        <v>689.2438426770293</v>
-      </c>
-      <c r="S36" s="2" t="n">
         <v>716.0408161885885</v>
       </c>
-      <c r="T36" s="1" t="inlineStr"/>
+      <c r="S36" s="1" t="inlineStr"/>
     </row>
     <row r="37" ht="30" customHeight="1">
       <c r="A37" s="1" t="inlineStr">
@@ -2044,51 +1979,48 @@
         <v>304.6972711556989</v>
       </c>
       <c r="E37" s="2" t="n">
-        <v>332.5412301095225</v>
+        <v>334.5400980960846</v>
       </c>
       <c r="F37" s="2" t="n">
-        <v>360.3157523649842</v>
+        <v>364.2636577736324</v>
       </c>
       <c r="G37" s="2" t="n">
-        <v>387.9652287313608</v>
+        <v>393.9358180901934</v>
       </c>
       <c r="H37" s="2" t="n">
-        <v>415.5484181640575</v>
+        <v>423.4832578774369</v>
       </c>
       <c r="I37" s="2" t="n">
-        <v>443.0550461864155</v>
+        <v>452.9241266519992</v>
       </c>
       <c r="J37" s="2" t="n">
-        <v>470.7121634428254</v>
+        <v>482.5514447276188</v>
       </c>
       <c r="K37" s="2" t="n">
-        <v>498.295226716079</v>
+        <v>512.0790958565088</v>
       </c>
       <c r="L37" s="2" t="n">
-        <v>525.8469279503316</v>
+        <v>541.5492817938723</v>
       </c>
       <c r="M37" s="2" t="n">
-        <v>553.3116738158444</v>
+        <v>570.9315691201923</v>
       </c>
       <c r="N37" s="2" t="n">
-        <v>580.6553434530979</v>
+        <v>600.1737035863282</v>
       </c>
       <c r="O37" s="2" t="n">
-        <v>607.9683068286746</v>
+        <v>629.3627469314156</v>
       </c>
       <c r="P37" s="2" t="n">
-        <v>635.1835141618287</v>
+        <v>658.4149708618947</v>
       </c>
       <c r="Q37" s="2" t="n">
-        <v>662.2781021930996</v>
+        <v>687.3224160481872</v>
       </c>
       <c r="R37" s="2" t="n">
-        <v>689.2438426770293</v>
-      </c>
-      <c r="S37" s="2" t="n">
         <v>716.0408161885885</v>
       </c>
-      <c r="T37" s="1" t="inlineStr"/>
+      <c r="S37" s="1" t="inlineStr"/>
     </row>
     <row r="38" ht="15" customHeight="1">
       <c r="A38" s="1" t="inlineStr">
@@ -2106,51 +2038,48 @@
         <v>1.175559285399187</v>
       </c>
       <c r="E38" s="2" t="n">
-        <v>1.176956036090575</v>
+        <v>1.177149157361195</v>
       </c>
       <c r="F38" s="2" t="n">
-        <v>1.177314556774188</v>
+        <v>1.177580116958397</v>
       </c>
       <c r="G38" s="2" t="n">
-        <v>1.176870346260679</v>
+        <v>1.177095915781244</v>
       </c>
       <c r="H38" s="2" t="n">
-        <v>1.175734201092261</v>
+        <v>1.175855347567406</v>
       </c>
       <c r="I38" s="2" t="n">
-        <v>1.17400542811149</v>
+        <v>1.173962116210552</v>
       </c>
       <c r="J38" s="2" t="n">
-        <v>1.173698204745806</v>
+        <v>1.173396175963183</v>
       </c>
       <c r="K38" s="2" t="n">
-        <v>1.172847504293333</v>
+        <v>1.172215437821457</v>
       </c>
       <c r="L38" s="2" t="n">
-        <v>1.171437473220811</v>
+        <v>1.170376301404517</v>
       </c>
       <c r="M38" s="2" t="n">
-        <v>1.169448963439853</v>
+        <v>1.167847518639031</v>
       </c>
       <c r="N38" s="2" t="n">
-        <v>1.166851812849547</v>
+        <v>1.164588351389238</v>
       </c>
       <c r="O38" s="2" t="n">
-        <v>1.163584415306085</v>
+        <v>1.160528026232</v>
       </c>
       <c r="P38" s="2" t="n">
-        <v>1.159616698752758</v>
+        <v>1.155630506097777</v>
       </c>
       <c r="Q38" s="2" t="n">
-        <v>1.154911296973687</v>
+        <v>1.149848870725617</v>
       </c>
       <c r="R38" s="2" t="n">
-        <v>1.149431198653191</v>
-      </c>
-      <c r="S38" s="2" t="n">
         <v>1.143155604508661</v>
       </c>
-      <c r="T38" s="1" t="inlineStr"/>
+      <c r="S38" s="1" t="inlineStr"/>
     </row>
     <row r="39" ht="15" customHeight="1">
       <c r="A39" s="1" t="inlineStr">
@@ -2168,51 +2097,48 @@
         <v>117900.225235523</v>
       </c>
       <c r="E39" s="2" t="n">
-        <v>255489.1592371767</v>
+        <v>265350.4672140714</v>
       </c>
       <c r="F39" s="2" t="n">
-        <v>393057.7046436996</v>
+        <v>412792.3261747835</v>
       </c>
       <c r="G39" s="2" t="n">
-        <v>530348.2434323351</v>
+        <v>559906.7201888376</v>
       </c>
       <c r="H39" s="2" t="n">
-        <v>667142.4075891768</v>
+        <v>706445.5229259076</v>
       </c>
       <c r="I39" s="2" t="n">
-        <v>803265.7244964738</v>
+        <v>852200.0936189106</v>
       </c>
       <c r="J39" s="2" t="n">
-        <v>940123.9087834673</v>
+        <v>998610.46481496</v>
       </c>
       <c r="K39" s="2" t="n">
-        <v>1076411.545587883</v>
+        <v>1144279.063503702</v>
       </c>
       <c r="L39" s="2" t="n">
-        <v>1211921.826287044</v>
+        <v>1288927.093135038</v>
       </c>
       <c r="M39" s="2" t="n">
-        <v>1346436.74338179</v>
+        <v>1432269.084259004</v>
       </c>
       <c r="N39" s="2" t="n">
-        <v>1479715.377504498</v>
+        <v>1573991.10153848</v>
       </c>
       <c r="O39" s="2" t="n">
-        <v>1611459.172409335</v>
+        <v>1713714.468054943</v>
       </c>
       <c r="P39" s="2" t="n">
-        <v>1741388.148081287</v>
+        <v>1851080.725235523</v>
       </c>
       <c r="Q39" s="2" t="n">
-        <v>1869196.471422007</v>
+        <v>1985694.583576011</v>
       </c>
       <c r="R39" s="2" t="n">
-        <v>1994561.470172026</v>
-      </c>
-      <c r="S39" s="2" t="n">
         <v>2117173.208233083</v>
       </c>
-      <c r="T39" s="1" t="inlineStr"/>
+      <c r="S39" s="1" t="inlineStr"/>
     </row>
     <row r="40" ht="15" customHeight="1">
       <c r="A40" s="1" t="inlineStr">
@@ -2230,51 +2156,48 @@
         <v>117900.225235523</v>
       </c>
       <c r="E40" s="2" t="n">
-        <v>255489.1592371767</v>
+        <v>265350.4672140714</v>
       </c>
       <c r="F40" s="2" t="n">
-        <v>393057.7046436996</v>
+        <v>412792.3261747835</v>
       </c>
       <c r="G40" s="2" t="n">
-        <v>530348.2434323351</v>
+        <v>559906.7201888376</v>
       </c>
       <c r="H40" s="2" t="n">
-        <v>667142.4075891768</v>
+        <v>706445.5229259076</v>
       </c>
       <c r="I40" s="2" t="n">
-        <v>803265.7244964738</v>
+        <v>852200.0936189106</v>
       </c>
       <c r="J40" s="2" t="n">
-        <v>940123.9087834673</v>
+        <v>998610.46481496</v>
       </c>
       <c r="K40" s="2" t="n">
-        <v>1076411.545587883</v>
+        <v>1144279.063503702</v>
       </c>
       <c r="L40" s="2" t="n">
-        <v>1211921.826287044</v>
+        <v>1288927.093135038</v>
       </c>
       <c r="M40" s="2" t="n">
-        <v>1346436.74338179</v>
+        <v>1432269.084259004</v>
       </c>
       <c r="N40" s="2" t="n">
-        <v>1479715.377504498</v>
+        <v>1573991.10153848</v>
       </c>
       <c r="O40" s="2" t="n">
-        <v>1611459.172409335</v>
+        <v>1713714.468054943</v>
       </c>
       <c r="P40" s="2" t="n">
-        <v>1741388.148081287</v>
+        <v>1851080.725235523</v>
       </c>
       <c r="Q40" s="2" t="n">
-        <v>1869196.471422007</v>
+        <v>1985694.583576011</v>
       </c>
       <c r="R40" s="2" t="n">
-        <v>1994561.470172026</v>
-      </c>
-      <c r="S40" s="2" t="n">
         <v>2117173.208233083</v>
       </c>
-      <c r="T40" s="1" t="inlineStr"/>
+      <c r="S40" s="1" t="inlineStr"/>
     </row>
     <row r="41" ht="30" customHeight="1">
       <c r="A41" s="1" t="inlineStr">
@@ -2292,51 +2215,48 @@
         <v>310.7487734256569</v>
       </c>
       <c r="E41" s="2" t="n">
-        <v>324.6688112316239</v>
+        <v>325.6412920534009</v>
       </c>
       <c r="F41" s="2" t="n">
-        <v>338.0515793090531</v>
+        <v>339.860328445252</v>
       </c>
       <c r="G41" s="2" t="n">
-        <v>350.862209958119</v>
+        <v>353.5607325376019</v>
       </c>
       <c r="H41" s="2" t="n">
-        <v>363.2301909542014</v>
+        <v>366.6891593767065</v>
       </c>
       <c r="I41" s="2" t="n">
-        <v>375.1766092304147</v>
+        <v>379.3166107530025</v>
       </c>
       <c r="J41" s="2" t="n">
-        <v>386.7059416936959</v>
+        <v>391.5413584539659</v>
       </c>
       <c r="K41" s="2" t="n">
-        <v>397.8563095118959</v>
+        <v>403.32604206627</v>
       </c>
       <c r="L41" s="2" t="n">
-        <v>408.7173575831252</v>
+        <v>414.7702463409155</v>
       </c>
       <c r="M41" s="2" t="n">
-        <v>419.249265744434</v>
+        <v>425.8743045830093</v>
       </c>
       <c r="N41" s="2" t="n">
-        <v>429.4426618693322</v>
+        <v>436.6134499325574</v>
       </c>
       <c r="O41" s="2" t="n">
-        <v>439.4469858198541</v>
+        <v>447.1401723128121</v>
       </c>
       <c r="P41" s="2" t="n">
-        <v>449.2103721206494</v>
+        <v>457.3909295893897</v>
       </c>
       <c r="Q41" s="2" t="n">
-        <v>458.739164603982</v>
+        <v>467.4010982997746</v>
       </c>
       <c r="R41" s="2" t="n">
-        <v>468.0602766896044</v>
-      </c>
-      <c r="S41" s="2" t="n">
         <v>477.1612274741949</v>
       </c>
-      <c r="T41" s="1" t="inlineStr"/>
+      <c r="S41" s="1" t="inlineStr"/>
     </row>
     <row r="42" ht="30" customHeight="1">
       <c r="A42" s="1" t="inlineStr">
@@ -2351,54 +2271,51 @@
       </c>
       <c r="C42" s="1" t="inlineStr"/>
       <c r="D42" s="2" t="n">
-        <v>319.538806481394</v>
+        <v>319.5338237912142</v>
       </c>
       <c r="E42" s="2" t="n">
-        <v>333.774424617516</v>
+        <v>334.7109771300942</v>
       </c>
       <c r="F42" s="2" t="n">
-        <v>347.3317688252171</v>
+        <v>349.222944744292</v>
       </c>
       <c r="G42" s="2" t="n">
-        <v>360.3293224315304</v>
+        <v>363.0714408965355</v>
       </c>
       <c r="H42" s="2" t="n">
-        <v>372.8297737710806</v>
+        <v>376.3080358645553</v>
       </c>
       <c r="I42" s="2" t="n">
-        <v>384.842687051213</v>
+        <v>389.0522517673508</v>
       </c>
       <c r="J42" s="2" t="n">
-        <v>396.509668398383</v>
+        <v>401.3995426568525</v>
       </c>
       <c r="K42" s="2" t="n">
-        <v>407.8266612290232</v>
+        <v>413.3312413404398</v>
       </c>
       <c r="L42" s="2" t="n">
-        <v>418.7770733157024</v>
+        <v>424.8720601328997</v>
       </c>
       <c r="M42" s="2" t="n">
-        <v>429.3336446966811</v>
+        <v>435.9907411935118</v>
       </c>
       <c r="N42" s="2" t="n">
-        <v>439.6375871105478</v>
+        <v>446.8252619518367</v>
       </c>
       <c r="O42" s="2" t="n">
-        <v>449.6754965258203</v>
+        <v>457.3496598375589</v>
       </c>
       <c r="P42" s="2" t="n">
-        <v>459.4315267237035</v>
+        <v>467.5723728126169</v>
       </c>
       <c r="Q42" s="2" t="n">
-        <v>468.9278472826187</v>
+        <v>477.4855413613454</v>
       </c>
       <c r="R42" s="2" t="n">
-        <v>478.1524868271428</v>
-      </c>
-      <c r="S42" s="2" t="n">
-        <v>487.1270825678299</v>
-      </c>
-      <c r="T42" s="1" t="inlineStr"/>
+        <v>487.112205135101</v>
+      </c>
+      <c r="S42" s="1" t="inlineStr"/>
     </row>
     <row r="43" ht="30" customHeight="1">
       <c r="A43" s="1" t="inlineStr">
@@ -2416,51 +2333,48 @@
         <v>0.7697077367416805</v>
       </c>
       <c r="E43" s="2" t="n">
-        <v>0.7790684943630035</v>
+        <v>0.779758718400195</v>
       </c>
       <c r="F43" s="2" t="n">
-        <v>0.7889872801066945</v>
+        <v>0.7904485926897359</v>
       </c>
       <c r="G43" s="2" t="n">
-        <v>0.7994433236842792</v>
+        <v>0.8017518046703783</v>
       </c>
       <c r="H43" s="2" t="n">
-        <v>0.8104158301444142</v>
+        <v>0.8136427930868606</v>
       </c>
       <c r="I43" s="2" t="n">
-        <v>0.8218841147424848</v>
+        <v>0.826096176625411</v>
       </c>
       <c r="J43" s="2" t="n">
-        <v>0.8338277212563164</v>
+        <v>0.8390869151470612</v>
       </c>
       <c r="K43" s="2" t="n">
-        <v>0.8462265239030562</v>
+        <v>0.8525904463163166</v>
       </c>
       <c r="L43" s="2" t="n">
-        <v>0.8590608134065268</v>
+        <v>0.8665827986820737</v>
       </c>
       <c r="M43" s="2" t="n">
-        <v>0.8723113680655563</v>
+        <v>0.8810406827362796</v>
       </c>
       <c r="N43" s="2" t="n">
-        <v>0.885959510888735</v>
+        <v>0.8959415617907894</v>
       </c>
       <c r="O43" s="2" t="n">
-        <v>0.8999871539994868</v>
+        <v>0.9112637046951794</v>
       </c>
       <c r="P43" s="2" t="n">
-        <v>0.9143768315886349</v>
+        <v>0.9269862224911449</v>
       </c>
       <c r="Q43" s="2" t="n">
-        <v>0.9291117227116072</v>
+        <v>0.9430890910857662</v>
       </c>
       <c r="R43" s="2" t="n">
-        <v>0.9441756652055144</v>
-      </c>
-      <c r="S43" s="2" t="n">
         <v>0.9595531619480527</v>
       </c>
-      <c r="T43" s="1" t="inlineStr"/>
+      <c r="S43" s="1" t="inlineStr"/>
     </row>
     <row r="44" ht="30" customHeight="1">
       <c r="A44" s="1" t="inlineStr">
@@ -2478,51 +2392,48 @@
         <v>0.2675658145409672</v>
       </c>
       <c r="E44" s="2" t="n">
-        <v>0.2630332328337259</v>
+        <v>0.2627510762416364</v>
       </c>
       <c r="F44" s="2" t="n">
-        <v>0.2595454831984348</v>
+        <v>0.2591274840795844</v>
       </c>
       <c r="G44" s="2" t="n">
-        <v>0.2570032853991994</v>
+        <v>0.256576799401226</v>
       </c>
       <c r="H44" s="2" t="n">
-        <v>0.2553424548291788</v>
+        <v>0.2550220951838035</v>
       </c>
       <c r="I44" s="2" t="n">
-        <v>0.2545035381647927</v>
+        <v>0.254393016919423</v>
       </c>
       <c r="J44" s="2" t="n">
-        <v>0.254446895246222</v>
+        <v>0.2546621015587227</v>
       </c>
       <c r="K44" s="2" t="n">
-        <v>0.2551637253988659</v>
+        <v>0.2558078397057248</v>
       </c>
       <c r="L44" s="2" t="n">
-        <v>0.2566492233119093</v>
+        <v>0.2578470068353897</v>
       </c>
       <c r="M44" s="2" t="n">
-        <v>0.2589189552819218</v>
+        <v>0.2608045797416076</v>
       </c>
       <c r="N44" s="2" t="n">
-        <v>0.2620001380804975</v>
+        <v>0.2647254322067381</v>
       </c>
       <c r="O44" s="2" t="n">
-        <v>0.2659437917155251</v>
+        <v>0.2696810959896801</v>
       </c>
       <c r="P44" s="2" t="n">
-        <v>0.2708033748788066</v>
+        <v>0.2757469847403645</v>
       </c>
       <c r="Q44" s="2" t="n">
-        <v>0.2766454189831242</v>
+        <v>0.2830232632486962</v>
       </c>
       <c r="R44" s="2" t="n">
-        <v>0.2835539839765567</v>
-      </c>
-      <c r="S44" s="2" t="n">
         <v>0.2916156103246133</v>
       </c>
-      <c r="T44" s="1" t="inlineStr"/>
+      <c r="S44" s="1" t="inlineStr"/>
     </row>
     <row r="45" ht="15" customHeight="1">
       <c r="A45" s="1" t="inlineStr">
@@ -2540,51 +2451,48 @@
         <v>1.180296158977294</v>
       </c>
       <c r="E45" s="2" t="n">
-        <v>1.175660120614364</v>
+        <v>1.175262487903347</v>
       </c>
       <c r="F45" s="2" t="n">
-        <v>1.169301466996413</v>
+        <v>1.168251369555617</v>
       </c>
       <c r="G45" s="2" t="n">
-        <v>1.161220352668794</v>
+        <v>1.15925817796077</v>
       </c>
       <c r="H45" s="2" t="n">
-        <v>1.151371190875526</v>
+        <v>1.148224245120433</v>
       </c>
       <c r="I45" s="2" t="n">
-        <v>1.139702029614363</v>
+        <v>1.135081723832521</v>
       </c>
       <c r="J45" s="2" t="n">
-        <v>1.126131101140586</v>
+        <v>1.119697021419855</v>
       </c>
       <c r="K45" s="2" t="n">
-        <v>1.110526848816953</v>
+        <v>1.101922316939652</v>
       </c>
       <c r="L45" s="2" t="n">
-        <v>1.09274669556362</v>
+        <v>1.081544540058967</v>
       </c>
       <c r="M45" s="2" t="n">
-        <v>1.072611910495834</v>
+        <v>1.058332062101629</v>
       </c>
       <c r="N45" s="2" t="n">
-        <v>1.049922328542544</v>
+        <v>1.032020278583349</v>
       </c>
       <c r="O45" s="2" t="n">
-        <v>1.024439898388269</v>
+        <v>1.0023075858643</v>
       </c>
       <c r="P45" s="2" t="n">
-        <v>0.9959305185620582</v>
+        <v>0.9689068762009189</v>
       </c>
       <c r="Q45" s="2" t="n">
-        <v>0.9641580860903053</v>
+        <v>0.9315321714560333</v>
       </c>
       <c r="R45" s="2" t="n">
-        <v>0.9288932198626439</v>
-      </c>
-      <c r="S45" s="2" t="n">
         <v>0.8899613152251319</v>
       </c>
-      <c r="T45" s="1" t="inlineStr"/>
+      <c r="S45" s="1" t="inlineStr"/>
     </row>
     <row r="46" ht="15" customHeight="1">
       <c r="A46" s="1" t="inlineStr">
@@ -2602,51 +2510,48 @@
         <v>199.2565864072191</v>
       </c>
       <c r="E46" s="2" t="n">
-        <v>193.3299802474146</v>
+        <v>192.906651236</v>
       </c>
       <c r="F46" s="2" t="n">
-        <v>187.4033740876102</v>
+        <v>186.5567160647809</v>
       </c>
       <c r="G46" s="2" t="n">
-        <v>181.4767679278057</v>
+        <v>180.2067808935618</v>
       </c>
       <c r="H46" s="2" t="n">
-        <v>175.5501617680012</v>
+        <v>173.8568457223428</v>
       </c>
       <c r="I46" s="2" t="n">
-        <v>169.6235556081967</v>
+        <v>167.5069105511237</v>
       </c>
       <c r="J46" s="2" t="n">
-        <v>163.6969494483923</v>
+        <v>161.1569753799047</v>
       </c>
       <c r="K46" s="2" t="n">
-        <v>157.7703432885878</v>
+        <v>154.8070402086856</v>
       </c>
       <c r="L46" s="2" t="n">
-        <v>151.8437371287833</v>
+        <v>148.4571050374665</v>
       </c>
       <c r="M46" s="2" t="n">
-        <v>145.9171309689789</v>
+        <v>142.1071698662474</v>
       </c>
       <c r="N46" s="2" t="n">
-        <v>139.9905248091744</v>
+        <v>135.7572346950284</v>
       </c>
       <c r="O46" s="2" t="n">
-        <v>134.06391864937</v>
+        <v>129.4072995238093</v>
       </c>
       <c r="P46" s="2" t="n">
-        <v>128.1373124895655</v>
+        <v>123.0573643525902</v>
       </c>
       <c r="Q46" s="2" t="n">
-        <v>122.210706329761</v>
+        <v>116.7074291813712</v>
       </c>
       <c r="R46" s="2" t="n">
-        <v>116.2841001699566</v>
-      </c>
-      <c r="S46" s="2" t="n">
         <v>110.3574940101521</v>
       </c>
-      <c r="T46" s="1" t="inlineStr"/>
+      <c r="S46" s="1" t="inlineStr"/>
     </row>
     <row r="47" ht="15" customHeight="1">
       <c r="A47" s="1" t="inlineStr">
@@ -2664,51 +2569,48 @@
         <v>0.6934155588636786</v>
       </c>
       <c r="E47" s="2" t="n">
-        <v>0.6451834489675361</v>
+        <v>0.6419546944869913</v>
       </c>
       <c r="F47" s="2" t="n">
-        <v>0.6022559501154908</v>
+        <v>0.5966106211168183</v>
       </c>
       <c r="G47" s="2" t="n">
-        <v>0.5638685802055692</v>
+        <v>0.5561238216798053</v>
       </c>
       <c r="H47" s="2" t="n">
-        <v>0.5291695030894039</v>
+        <v>0.5198537807125588</v>
       </c>
       <c r="I47" s="2" t="n">
-        <v>0.4976467391118254</v>
+        <v>0.4871134947236217</v>
       </c>
       <c r="J47" s="2" t="n">
-        <v>0.4689105164395919</v>
+        <v>0.4573452836046674</v>
       </c>
       <c r="K47" s="2" t="n">
-        <v>0.4426124944584192</v>
+        <v>0.4302607947475137</v>
       </c>
       <c r="L47" s="2" t="n">
-        <v>0.4184202956554766</v>
+        <v>0.4054971202086974</v>
       </c>
       <c r="M47" s="2" t="n">
-        <v>0.3962015376671923</v>
+        <v>0.382866877454614</v>
       </c>
       <c r="N47" s="2" t="n">
-        <v>0.3758216201394586</v>
+        <v>0.3622495702925325</v>
       </c>
       <c r="O47" s="2" t="n">
-        <v>0.3570527093257961</v>
+        <v>0.3434267211217917</v>
       </c>
       <c r="P47" s="2" t="n">
-        <v>0.339880761221536</v>
+        <v>0.3264013915200195</v>
       </c>
       <c r="Q47" s="2" t="n">
-        <v>0.324264400412908</v>
+        <v>0.3111320861419942</v>
       </c>
       <c r="R47" s="2" t="n">
-        <v>0.3101765261475119</v>
-      </c>
-      <c r="S47" s="2" t="n">
         <v>0.2976385445704193</v>
       </c>
-      <c r="T47" s="1" t="inlineStr"/>
+      <c r="S47" s="1" t="inlineStr"/>
     </row>
     <row r="48" ht="15" customHeight="1">
       <c r="A48" s="1" t="inlineStr">
@@ -2726,51 +2628,48 @@
         <v>0.8876763917513479</v>
       </c>
       <c r="E48" s="2" t="n">
-        <v>0.8503589546990444</v>
+        <v>0.8476827557110529</v>
       </c>
       <c r="F48" s="2" t="n">
-        <v>0.8129909497908511</v>
+        <v>0.807838102390409</v>
       </c>
       <c r="G48" s="2" t="n">
-        <v>0.7764600076873178</v>
+        <v>0.7687303178641441</v>
       </c>
       <c r="H48" s="2" t="n">
-        <v>0.7409792133386249</v>
+        <v>0.7310690251477328</v>
       </c>
       <c r="I48" s="2" t="n">
-        <v>0.7068253360544405</v>
+        <v>0.6950438015492818</v>
       </c>
       <c r="J48" s="2" t="n">
-        <v>0.6741948941545413</v>
+        <v>0.6606666216532919</v>
       </c>
       <c r="K48" s="2" t="n">
-        <v>0.643142168620027</v>
+        <v>0.6281613417983278</v>
       </c>
       <c r="L48" s="2" t="n">
-        <v>0.6135779019910447</v>
+        <v>0.5974295303378844</v>
       </c>
       <c r="M48" s="2" t="n">
-        <v>0.5856601694094432</v>
+        <v>0.5685574328276755</v>
       </c>
       <c r="N48" s="2" t="n">
-        <v>0.5594616026793855</v>
+        <v>0.5416626339362809</v>
       </c>
       <c r="O48" s="2" t="n">
-        <v>0.5347809281701855</v>
+        <v>0.5165679427658935</v>
       </c>
       <c r="P48" s="2" t="n">
-        <v>0.5117909068001266</v>
+        <v>0.4934870266617923</v>
       </c>
       <c r="Q48" s="2" t="n">
-        <v>0.4905645083415359</v>
+        <v>0.4724845076896956</v>
       </c>
       <c r="R48" s="2" t="n">
-        <v>0.4711609998268694</v>
-      </c>
-      <c r="S48" s="2" t="n">
         <v>0.4537118711400231</v>
       </c>
-      <c r="T48" s="1" t="inlineStr"/>
+      <c r="S48" s="1" t="inlineStr"/>
     </row>
     <row r="49" ht="15" customHeight="1">
       <c r="A49" s="1" t="inlineStr">
@@ -2788,51 +2687,48 @@
         <v>0.3009117955899137</v>
       </c>
       <c r="E49" s="2" t="n">
-        <v>0.1519633006435085</v>
+        <v>0.1472682986886746</v>
       </c>
       <c r="F49" s="2" t="n">
-        <v>0.1079113763941087</v>
+        <v>0.1040512028785386</v>
       </c>
       <c r="G49" s="2" t="n">
-        <v>0.08720732714641261</v>
+        <v>0.08416531485429166</v>
       </c>
       <c r="H49" s="2" t="n">
-        <v>0.07547728055219156</v>
+        <v>0.07304667532585596</v>
       </c>
       <c r="I49" s="2" t="n">
-        <v>0.06815267638391176</v>
+        <v>0.06619932070733821</v>
       </c>
       <c r="J49" s="2" t="n">
-        <v>0.06333153040060037</v>
+        <v>0.0617872384426807</v>
       </c>
       <c r="K49" s="2" t="n">
-        <v>0.06009085172263932</v>
+        <v>0.05890202559086238</v>
       </c>
       <c r="L49" s="2" t="n">
-        <v>0.05794046605351349</v>
+        <v>0.05707687219159215</v>
       </c>
       <c r="M49" s="2" t="n">
-        <v>0.05657548897759065</v>
+        <v>0.05602993268923052</v>
       </c>
       <c r="N49" s="2" t="n">
-        <v>0.05581207055463994</v>
+        <v>0.05558691697384634</v>
       </c>
       <c r="O49" s="2" t="n">
-        <v>0.05556200340151933</v>
+        <v>0.0556712005930268</v>
       </c>
       <c r="P49" s="2" t="n">
-        <v>0.05574366225286662</v>
+        <v>0.05621043688048771</v>
       </c>
       <c r="Q49" s="2" t="n">
-        <v>0.05631517545884135</v>
+        <v>0.05718010096659844</v>
       </c>
       <c r="R49" s="2" t="n">
-        <v>0.05725981928560088</v>
-      </c>
-      <c r="S49" s="2" t="n">
         <v>0.05857117009930012</v>
       </c>
-      <c r="T49" s="1" t="inlineStr"/>
+      <c r="S49" s="1" t="inlineStr"/>
     </row>
     <row r="50" ht="15" customHeight="1">
       <c r="A50" s="1" t="inlineStr">
@@ -2847,54 +2743,51 @@
       </c>
       <c r="C50" s="1" t="inlineStr"/>
       <c r="D50" s="2" t="n">
-        <v>0.6306666666666667</v>
+        <v>0.6292857142857143</v>
       </c>
       <c r="E50" s="2" t="n">
-        <v>0.6113333333333334</v>
+        <v>0.6085714285714285</v>
       </c>
       <c r="F50" s="2" t="n">
-        <v>0.592</v>
+        <v>0.5878571428571429</v>
       </c>
       <c r="G50" s="2" t="n">
-        <v>0.5726666666666667</v>
+        <v>0.5671428571428572</v>
       </c>
       <c r="H50" s="2" t="n">
-        <v>0.5533333333333333</v>
+        <v>0.5464285714285715</v>
       </c>
       <c r="I50" s="2" t="n">
-        <v>0.534</v>
+        <v>0.5257142857142857</v>
       </c>
       <c r="J50" s="2" t="n">
-        <v>0.5146666666666667</v>
+        <v>0.505</v>
       </c>
       <c r="K50" s="2" t="n">
-        <v>0.4953333333333333</v>
+        <v>0.4842857142857143</v>
       </c>
       <c r="L50" s="2" t="n">
-        <v>0.476</v>
+        <v>0.4635714285714286</v>
       </c>
       <c r="M50" s="2" t="n">
-        <v>0.4566666666666667</v>
+        <v>0.4428571428571428</v>
       </c>
       <c r="N50" s="2" t="n">
-        <v>0.4373333333333334</v>
+        <v>0.4221428571428572</v>
       </c>
       <c r="O50" s="2" t="n">
-        <v>0.418</v>
+        <v>0.4014285714285714</v>
       </c>
       <c r="P50" s="2" t="n">
-        <v>0.3986666666666667</v>
+        <v>0.3807142857142857</v>
       </c>
       <c r="Q50" s="2" t="n">
-        <v>0.3793333333333334</v>
+        <v>0.36</v>
       </c>
       <c r="R50" s="2" t="n">
-        <v>0.36</v>
-      </c>
-      <c r="S50" s="2" t="n">
-        <v>0.3406666666666666</v>
-      </c>
-      <c r="T50" s="1" t="inlineStr"/>
+        <v>0.3392857142857142</v>
+      </c>
+      <c r="S50" s="1" t="inlineStr"/>
     </row>
     <row r="51" ht="15" customHeight="1">
       <c r="A51" s="1" t="inlineStr">
@@ -2909,54 +2802,51 @@
       </c>
       <c r="C51" s="1" t="inlineStr"/>
       <c r="D51" s="2" t="n">
-        <v>193.3299802474146</v>
+        <v>192.906651236</v>
       </c>
       <c r="E51" s="2" t="n">
-        <v>187.4033740876102</v>
+        <v>186.5567160647809</v>
       </c>
       <c r="F51" s="2" t="n">
-        <v>181.4767679278057</v>
+        <v>180.2067808935618</v>
       </c>
       <c r="G51" s="2" t="n">
-        <v>175.5501617680012</v>
+        <v>173.8568457223428</v>
       </c>
       <c r="H51" s="2" t="n">
-        <v>169.6235556081967</v>
+        <v>167.5069105511237</v>
       </c>
       <c r="I51" s="2" t="n">
-        <v>163.6969494483923</v>
+        <v>161.1569753799047</v>
       </c>
       <c r="J51" s="2" t="n">
-        <v>157.7703432885878</v>
+        <v>154.8070402086856</v>
       </c>
       <c r="K51" s="2" t="n">
-        <v>151.8437371287833</v>
+        <v>148.4571050374665</v>
       </c>
       <c r="L51" s="2" t="n">
-        <v>145.9171309689789</v>
+        <v>142.1071698662474</v>
       </c>
       <c r="M51" s="2" t="n">
-        <v>139.9905248091744</v>
+        <v>135.7572346950284</v>
       </c>
       <c r="N51" s="2" t="n">
-        <v>134.06391864937</v>
+        <v>129.4072995238093</v>
       </c>
       <c r="O51" s="2" t="n">
-        <v>128.1373124895655</v>
+        <v>123.0573643525902</v>
       </c>
       <c r="P51" s="2" t="n">
-        <v>122.210706329761</v>
+        <v>116.7074291813712</v>
       </c>
       <c r="Q51" s="2" t="n">
-        <v>116.2841001699566</v>
+        <v>110.3574940101521</v>
       </c>
       <c r="R51" s="2" t="n">
-        <v>110.3574940101521</v>
-      </c>
-      <c r="S51" s="2" t="n">
-        <v>104.4308878503476</v>
-      </c>
-      <c r="T51" s="1" t="inlineStr"/>
+        <v>104.007558838933</v>
+      </c>
+      <c r="S51" s="1" t="inlineStr"/>
     </row>
     <row r="52" ht="30" customHeight="1">
       <c r="A52" s="1" t="inlineStr">
@@ -2971,54 +2861,51 @@
       </c>
       <c r="C52" s="1" t="inlineStr"/>
       <c r="D52" s="2" t="n">
-        <v>0.6542834231611319</v>
+        <v>0.6528609381672205</v>
       </c>
       <c r="E52" s="2" t="n">
-        <v>0.6083435839546485</v>
+        <v>0.6040008906918644</v>
       </c>
       <c r="F52" s="2" t="n">
-        <v>0.5676271902575042</v>
+        <v>0.5608528404519376</v>
       </c>
       <c r="G52" s="2" t="n">
-        <v>0.5311229686801958</v>
+        <v>0.5224733005942056</v>
       </c>
       <c r="H52" s="2" t="n">
-        <v>0.498139622561141</v>
+        <v>0.4880639358485558</v>
       </c>
       <c r="I52" s="2" t="n">
-        <v>0.4681964345049069</v>
+        <v>0.4569203160469202</v>
       </c>
       <c r="J52" s="2" t="n">
-        <v>0.4407596410267861</v>
+        <v>0.4285352724020985</v>
       </c>
       <c r="K52" s="2" t="n">
-        <v>0.4155715601725339</v>
+        <v>0.4026243969644493</v>
       </c>
       <c r="L52" s="2" t="n">
-        <v>0.3924301121422687</v>
+        <v>0.3789240751115422</v>
       </c>
       <c r="M52" s="2" t="n">
-        <v>0.371181142194238</v>
+        <v>0.3572719824747077</v>
       </c>
       <c r="N52" s="2" t="n">
-        <v>0.3515648108563043</v>
+        <v>0.3374139715597593</v>
       </c>
       <c r="O52" s="2" t="n">
-        <v>0.3335057311090038</v>
+        <v>0.3192848027412507</v>
       </c>
       <c r="P52" s="2" t="n">
-        <v>0.3169488695787482</v>
+        <v>0.3028179399616254</v>
       </c>
       <c r="Q52" s="2" t="n">
-        <v>0.3018353833969528</v>
+        <v>0.2879901483751846</v>
       </c>
       <c r="R52" s="2" t="n">
-        <v>0.2881547528997792</v>
-      </c>
-      <c r="S52" s="2" t="n">
-        <v>0.2758920486866353</v>
-      </c>
-      <c r="T52" s="1" t="inlineStr"/>
+        <v>0.2747820638038408</v>
+      </c>
+      <c r="S52" s="1" t="inlineStr"/>
     </row>
     <row r="53" ht="15" customHeight="1">
       <c r="A53" s="1" t="inlineStr">
@@ -3033,54 +2920,51 @@
       </c>
       <c r="C53" s="1" t="inlineStr"/>
       <c r="D53" s="2" t="n">
-        <v>0.857792072117288</v>
+        <v>0.8566449408652137</v>
       </c>
       <c r="E53" s="2" t="n">
-        <v>0.8185252274697533</v>
+        <v>0.8146305802312926</v>
       </c>
       <c r="F53" s="2" t="n">
-        <v>0.7801718219804457</v>
+        <v>0.7734667621979159</v>
       </c>
       <c r="G53" s="2" t="n">
-        <v>0.7430401602428608</v>
+        <v>0.7338759548743808</v>
       </c>
       <c r="H53" s="2" t="n">
-        <v>0.7073740915602904</v>
+        <v>0.6961191242501733</v>
       </c>
       <c r="I53" s="2" t="n">
-        <v>0.6733637173071654</v>
+        <v>0.6601638683567802</v>
       </c>
       <c r="J53" s="2" t="n">
-        <v>0.6409035082100051</v>
+        <v>0.6260427988521639</v>
       </c>
       <c r="K53" s="2" t="n">
-        <v>0.610025403696271</v>
+        <v>0.5937907596548805</v>
       </c>
       <c r="L53" s="2" t="n">
-        <v>0.5808285652718341</v>
+        <v>0.5634296976475788</v>
       </c>
       <c r="M53" s="2" t="n">
-        <v>0.5533778161398634</v>
+        <v>0.5350423151502405</v>
       </c>
       <c r="N53" s="2" t="n">
-        <v>0.5274414228456362</v>
+        <v>0.5084161145598954</v>
       </c>
       <c r="O53" s="2" t="n">
-        <v>0.5031171631548509</v>
+        <v>0.4836795065578707</v>
       </c>
       <c r="P53" s="2" t="n">
-        <v>0.4804625280747954</v>
+        <v>0.4608658406019039</v>
       </c>
       <c r="Q53" s="2" t="n">
-        <v>0.4594949713057526</v>
+        <v>0.4400685175575864</v>
       </c>
       <c r="R53" s="2" t="n">
-        <v>0.4403021559506097</v>
-      </c>
-      <c r="S53" s="2" t="n">
-        <v>0.4229272680516111</v>
-      </c>
-      <c r="T53" s="1" t="inlineStr"/>
+        <v>0.4213432296968064</v>
+      </c>
+      <c r="S53" s="1" t="inlineStr"/>
     </row>
     <row r="54" ht="30" customHeight="1">
       <c r="A54" s="1" t="inlineStr">
@@ -3095,54 +2979,51 @@
       </c>
       <c r="C54" s="1" t="inlineStr"/>
       <c r="D54" s="2" t="n">
-        <v>0.2724616335565606</v>
+        <v>0.2728264862976837</v>
       </c>
       <c r="E54" s="2" t="n">
-        <v>0.1379177624098988</v>
+        <v>0.1338497572918128</v>
       </c>
       <c r="F54" s="2" t="n">
-        <v>0.09816555592580541</v>
+        <v>0.09484023765812551</v>
       </c>
       <c r="G54" s="2" t="n">
-        <v>0.07954151364221926</v>
+        <v>0.07693362720631663</v>
       </c>
       <c r="H54" s="2" t="n">
-        <v>0.06903924748959318</v>
+        <v>0.0669762425432088</v>
       </c>
       <c r="I54" s="2" t="n">
-        <v>0.06252706844095968</v>
+        <v>0.06091105339602894</v>
       </c>
       <c r="J54" s="2" t="n">
-        <v>0.05822474737954209</v>
+        <v>0.05699304098048162</v>
       </c>
       <c r="K54" s="2" t="n">
-        <v>0.05538843076547833</v>
+        <v>0.05449766392638357</v>
       </c>
       <c r="L54" s="2" t="n">
-        <v>0.0535578893703248</v>
+        <v>0.05299351220560669</v>
       </c>
       <c r="M54" s="2" t="n">
-        <v>0.05246103075803894</v>
+        <v>0.05222397695379562</v>
       </c>
       <c r="N54" s="2" t="n">
-        <v>0.05196040341182012</v>
+        <v>0.05206385535377919</v>
       </c>
       <c r="O54" s="2" t="n">
-        <v>0.05195847081933057</v>
+        <v>0.05242649001453024</v>
       </c>
       <c r="P54" s="2" t="n">
-        <v>0.05239292757930168</v>
+        <v>0.05326713372110947</v>
       </c>
       <c r="Q54" s="2" t="n">
-        <v>0.05323751027373903</v>
+        <v>0.05457087868506504</v>
       </c>
       <c r="R54" s="2" t="n">
-        <v>0.05448237155483682</v>
-      </c>
-      <c r="S54" s="2" t="n">
-        <v>0.05614055729666342</v>
-      </c>
-      <c r="T54" s="1" t="inlineStr"/>
+        <v>0.05635161751966029</v>
+      </c>
+      <c r="S54" s="1" t="inlineStr"/>
     </row>
     <row r="55" ht="30" customHeight="1">
       <c r="A55" s="1" t="inlineStr">
@@ -3157,54 +3038,51 @@
       </c>
       <c r="C55" s="1" t="inlineStr"/>
       <c r="D55" s="2" t="n">
-        <v>0.5014648337358059</v>
+        <v>0.5004644049712301</v>
       </c>
       <c r="E55" s="2" t="n">
-        <v>0.7880983118324816</v>
+        <v>0.7951571965663656</v>
       </c>
       <c r="F55" s="2" t="n">
-        <v>0.8545818074176159</v>
+        <v>0.8599102873979747</v>
       </c>
       <c r="G55" s="2" t="n">
-        <v>0.8840112219416179</v>
+        <v>0.8880543221133667</v>
       </c>
       <c r="H55" s="2" t="n">
-        <v>0.9001825839829652</v>
+        <v>0.9033251749764167</v>
       </c>
       <c r="I55" s="2" t="n">
-        <v>0.9100656977821977</v>
+        <v>0.9125016424738571</v>
       </c>
       <c r="J55" s="2" t="n">
-        <v>0.9165365938680218</v>
+        <v>0.9183807441133749</v>
       </c>
       <c r="K55" s="2" t="n">
-        <v>0.9207776778035037</v>
+        <v>0.9221055975212045</v>
       </c>
       <c r="L55" s="2" t="n">
-        <v>0.923504506091347</v>
+        <v>0.9243435965300111</v>
       </c>
       <c r="M55" s="2" t="n">
-        <v>0.9251345681110075</v>
+        <v>0.9254864808911322</v>
       </c>
       <c r="N55" s="2" t="n">
-        <v>0.9258776058992364</v>
+        <v>0.9257241100343748</v>
       </c>
       <c r="O55" s="2" t="n">
-        <v>0.9258804731233909</v>
+        <v>0.9251858531094985</v>
       </c>
       <c r="P55" s="2" t="n">
-        <v>0.925235682823888</v>
+        <v>0.9239368836048013</v>
       </c>
       <c r="Q55" s="2" t="n">
-        <v>0.9239809247449741</v>
+        <v>0.921996524014703</v>
       </c>
       <c r="R55" s="2" t="n">
-        <v>0.9221283780829891</v>
-      </c>
-      <c r="S55" s="2" t="n">
-        <v>0.9196549445310657</v>
-      </c>
-      <c r="T55" s="1" t="inlineStr"/>
+        <v>0.9193396390285498</v>
+      </c>
+      <c r="S55" s="1" t="inlineStr"/>
     </row>
     <row r="56" ht="30" customHeight="1">
       <c r="A56" s="1" t="inlineStr">
@@ -3219,54 +3097,51 @@
       </c>
       <c r="C56" s="1" t="inlineStr"/>
       <c r="D56" s="2" t="n">
-        <v>0.7928308206805679</v>
+        <v>0.7925571175792675</v>
       </c>
       <c r="E56" s="2" t="n">
-        <v>0.9040007107409713</v>
+        <v>0.9071180477959627</v>
       </c>
       <c r="F56" s="2" t="n">
-        <v>0.9334492683903225</v>
+        <v>0.9358895185677403</v>
       </c>
       <c r="G56" s="2" t="n">
-        <v>0.9468052533979796</v>
+        <v>0.948685461697101</v>
       </c>
       <c r="H56" s="2" t="n">
-        <v>0.9542146537324381</v>
+        <v>0.9556884738180345</v>
       </c>
       <c r="I56" s="2" t="n">
-        <v>0.9587578860438596</v>
+        <v>0.9599063667841907</v>
       </c>
       <c r="J56" s="2" t="n">
-        <v>0.9617271470303008</v>
+        <v>0.9625977918536026</v>
       </c>
       <c r="K56" s="2" t="n">
-        <v>0.9636562672173354</v>
+        <v>0.964278961015491</v>
       </c>
       <c r="L56" s="2" t="n">
-        <v>0.9648679757288272</v>
+        <v>0.9652498884133429</v>
       </c>
       <c r="M56" s="2" t="n">
-        <v>0.9655488057857011</v>
+        <v>0.965683442559767</v>
       </c>
       <c r="N56" s="2" t="n">
-        <v>0.9657893502438822</v>
+        <v>0.965658328898274</v>
       </c>
       <c r="O56" s="2" t="n">
-        <v>0.965648737702872</v>
+        <v>0.9652218941086499</v>
       </c>
       <c r="P56" s="2" t="n">
-        <v>0.965158885640413</v>
+        <v>0.9643884025523056</v>
       </c>
       <c r="Q56" s="2" t="n">
-        <v>0.9643233907451992</v>
+        <v>0.9631461936180357</v>
       </c>
       <c r="R56" s="2" t="n">
-        <v>0.9631302347305716</v>
-      </c>
-      <c r="S56" s="2" t="n">
-        <v>0.9615464092563861</v>
-      </c>
-      <c r="T56" s="1" t="inlineStr"/>
+        <v>0.9614571633309685</v>
+      </c>
+      <c r="S56" s="1" t="inlineStr"/>
     </row>
     <row r="57" ht="30" customHeight="1">
       <c r="A57" s="1" t="inlineStr">
@@ -3281,54 +3156,51 @@
       </c>
       <c r="C57" s="1" t="inlineStr"/>
       <c r="D57" s="2" t="n">
-        <v>0.2813905009471096</v>
+        <v>0.2811863433358084</v>
       </c>
       <c r="E57" s="2" t="n">
-        <v>0.3406864454900046</v>
+        <v>0.3419728067953003</v>
       </c>
       <c r="F57" s="2" t="n">
-        <v>0.3505989984212221</v>
+        <v>0.3509410655936228</v>
       </c>
       <c r="G57" s="2" t="n">
-        <v>0.3510039443043173</v>
+        <v>0.3505057511486546</v>
       </c>
       <c r="H57" s="2" t="n">
-        <v>0.3480432983113403</v>
+        <v>0.3468279629635574</v>
       </c>
       <c r="I57" s="2" t="n">
-        <v>0.3435662483967508</v>
+        <v>0.3417081181479366</v>
       </c>
       <c r="J57" s="2" t="n">
-        <v>0.3383531120609656</v>
+        <v>0.3359234221056464</v>
       </c>
       <c r="K57" s="2" t="n">
-        <v>0.3327431785133318</v>
+        <v>0.3297983277471504</v>
       </c>
       <c r="L57" s="2" t="n">
-        <v>0.3269564786201302</v>
+        <v>0.3235650470477323</v>
       </c>
       <c r="M57" s="2" t="n">
-        <v>0.3211507631297974</v>
+        <v>0.31739063742177</v>
       </c>
       <c r="N57" s="2" t="n">
-        <v>0.3154373206322919</v>
+        <v>0.3114061941828092</v>
       </c>
       <c r="O57" s="2" t="n">
-        <v>0.3099364446129152</v>
+        <v>0.3057573784837125</v>
       </c>
       <c r="P57" s="2" t="n">
-        <v>0.3047605865011777</v>
+        <v>0.3005825024172691</v>
       </c>
       <c r="Q57" s="2" t="n">
-        <v>0.3000239632844169</v>
+        <v>0.2960388638501384</v>
       </c>
       <c r="R57" s="2" t="n">
-        <v>0.2958573094930009</v>
-      </c>
-      <c r="S57" s="2" t="n">
-        <v>0.2923912427959964</v>
-      </c>
-      <c r="T57" s="1" t="inlineStr"/>
+        <v>0.2922862607409257</v>
+      </c>
+      <c r="S57" s="1" t="inlineStr"/>
     </row>
     <row r="58" ht="30" customHeight="1">
       <c r="A58" s="1" t="inlineStr">
@@ -3343,54 +3215,51 @@
       </c>
       <c r="C58" s="1" t="inlineStr"/>
       <c r="D58" s="2" t="n">
-        <v>1.151124118776815</v>
+        <v>1.150578245989658</v>
       </c>
       <c r="E58" s="2" t="n">
-        <v>1.062377799270185</v>
+        <v>1.058842137058633</v>
       </c>
       <c r="F58" s="2" t="n">
-        <v>1.036111103650193</v>
+        <v>1.03259772936633</v>
       </c>
       <c r="G58" s="2" t="n">
-        <v>1.020924488333052</v>
+        <v>1.017231933919797</v>
       </c>
       <c r="H58" s="2" t="n">
-        <v>1.00933013835935</v>
+        <v>1.005239401872601</v>
       </c>
       <c r="I58" s="2" t="n">
-        <v>0.9990872116840966</v>
+        <v>0.9944293535476197</v>
       </c>
       <c r="J58" s="2" t="n">
-        <v>0.9892213184073614</v>
+        <v>0.9838133341616834</v>
       </c>
       <c r="K58" s="2" t="n">
-        <v>0.9792785544438508</v>
+        <v>0.9729365229403433</v>
       </c>
       <c r="L58" s="2" t="n">
-        <v>0.9689278286328695</v>
+        <v>0.9614252343707766</v>
       </c>
       <c r="M58" s="2" t="n">
-        <v>0.9578925859460624</v>
+        <v>0.9489575905895593</v>
       </c>
       <c r="N58" s="2" t="n">
-        <v>0.9459345018896737</v>
+        <v>0.9352269846819268</v>
       </c>
       <c r="O58" s="2" t="n">
-        <v>0.9327737435617988</v>
+        <v>0.9198661432115165</v>
       </c>
       <c r="P58" s="2" t="n">
-        <v>0.9181114109748046</v>
+        <v>0.9024768235733482</v>
       </c>
       <c r="Q58" s="2" t="n">
-        <v>0.9016138797803057</v>
+        <v>0.8825869545836461</v>
       </c>
       <c r="R58" s="2" t="n">
-        <v>0.8828878938189587</v>
-      </c>
-      <c r="S58" s="2" t="n">
-        <v>0.861508375559446</v>
-      </c>
-      <c r="T58" s="1" t="inlineStr"/>
+        <v>0.8596778720441994</v>
+      </c>
+      <c r="S58" s="1" t="inlineStr"/>
     </row>
     <row r="59" ht="15" customHeight="1">
       <c r="A59" s="1" t="inlineStr">
@@ -3405,54 +3274,51 @@
       </c>
       <c r="C59" s="1" t="inlineStr"/>
       <c r="D59" s="2" t="n">
-        <v>0.6625199647544942</v>
+        <v>0.6612407210601744</v>
       </c>
       <c r="E59" s="2" t="n">
-        <v>0.6427672737493952</v>
+        <v>0.6393366808686474</v>
       </c>
       <c r="F59" s="2" t="n">
-        <v>0.6072415102197469</v>
+        <v>0.6009807379947486</v>
       </c>
       <c r="G59" s="2" t="n">
-        <v>0.5714268310718572</v>
+        <v>0.5629187482016862</v>
       </c>
       <c r="H59" s="2" t="n">
-        <v>0.5374786818095514</v>
+        <v>0.5272267598629743</v>
       </c>
       <c r="I59" s="2" t="n">
-        <v>0.5057932110432251</v>
+        <v>0.4940432659250179</v>
       </c>
       <c r="J59" s="2" t="n">
-        <v>0.47618307218868</v>
+        <v>0.4632008778470891</v>
       </c>
       <c r="K59" s="2" t="n">
-        <v>0.4485318823583244</v>
+        <v>0.434547983835321</v>
       </c>
       <c r="L59" s="2" t="n">
-        <v>0.4227163777367752</v>
+        <v>0.4078868049211564</v>
       </c>
       <c r="M59" s="2" t="n">
-        <v>0.398621249447761</v>
+        <v>0.3830869581536965</v>
       </c>
       <c r="N59" s="2" t="n">
-        <v>0.3759868888716454</v>
+        <v>0.3598891790707875</v>
       </c>
       <c r="O59" s="2" t="n">
-        <v>0.3547415725698023</v>
+        <v>0.3382266797622753</v>
       </c>
       <c r="P59" s="2" t="n">
-        <v>0.3348255417836918</v>
+        <v>0.3180205486364964</v>
       </c>
       <c r="Q59" s="2" t="n">
-        <v>0.3161665993594145</v>
+        <v>0.2992319827470267</v>
       </c>
       <c r="R59" s="2" t="n">
-        <v>0.2987406862253892</v>
-      </c>
-      <c r="S59" s="2" t="n">
-        <v>0.2825170054424779</v>
-      </c>
-      <c r="T59" s="1" t="inlineStr"/>
+        <v>0.2818236131273244</v>
+      </c>
+      <c r="S59" s="1" t="inlineStr"/>
     </row>
     <row r="60" ht="30" customHeight="1">
       <c r="A60" s="1" t="inlineStr">
@@ -3467,54 +3333,51 @@
       </c>
       <c r="C60" s="1" t="inlineStr"/>
       <c r="D60" s="2" t="n">
-        <v>0.2703888904097833</v>
+        <v>0.2707047831582408</v>
       </c>
       <c r="E60" s="2" t="n">
-        <v>0.1330636745304504</v>
+        <v>0.1289535490674906</v>
       </c>
       <c r="F60" s="2" t="n">
-        <v>0.09367204543933282</v>
+        <v>0.09035121456081503</v>
       </c>
       <c r="G60" s="2" t="n">
-        <v>0.07539032965061968</v>
+        <v>0.07279583956722309</v>
       </c>
       <c r="H60" s="2" t="n">
-        <v>0.06513631074733642</v>
+        <v>0.0630871303195517</v>
       </c>
       <c r="I60" s="2" t="n">
-        <v>0.0588093073356333</v>
+        <v>0.0572051495289134</v>
       </c>
       <c r="J60" s="2" t="n">
-        <v>0.05465801146599711</v>
+        <v>0.05343833731776829</v>
       </c>
       <c r="K60" s="2" t="n">
-        <v>0.05195404749581219</v>
+        <v>0.05108008787467855</v>
       </c>
       <c r="L60" s="2" t="n">
-        <v>0.05025287775359496</v>
+        <v>0.04971625102356635</v>
       </c>
       <c r="M60" s="2" t="n">
-        <v>0.04929609311682435</v>
+        <v>0.04910680533129995</v>
       </c>
       <c r="N60" s="2" t="n">
-        <v>0.04895788964246673</v>
+        <v>0.04914211499311783</v>
       </c>
       <c r="O60" s="2" t="n">
-        <v>0.0491555999156828</v>
+        <v>0.04975559312298664</v>
       </c>
       <c r="P60" s="2" t="n">
-        <v>0.04984413858227942</v>
+        <v>0.0509264267870588</v>
       </c>
       <c r="Q60" s="2" t="n">
-        <v>0.05101770853810567</v>
+        <v>0.05266952243484315</v>
       </c>
       <c r="R60" s="2" t="n">
-        <v>0.05269190168912224</v>
-      </c>
-      <c r="S60" s="2" t="n">
-        <v>0.05491106614839087</v>
-      </c>
-      <c r="T60" s="1" t="inlineStr"/>
+        <v>0.05503600366715333</v>
+      </c>
+      <c r="S60" s="1" t="inlineStr"/>
     </row>
     <row r="61" ht="30" customHeight="1">
       <c r="A61" s="1" t="inlineStr">
@@ -3529,54 +3392,51 @@
       </c>
       <c r="C61" s="1" t="inlineStr"/>
       <c r="D61" s="2" t="n">
-        <v>0.1330636745304504</v>
+        <v>0.1289535490674906</v>
       </c>
       <c r="E61" s="2" t="n">
-        <v>0.09367204543933282</v>
+        <v>0.09035121456081503</v>
       </c>
       <c r="F61" s="2" t="n">
-        <v>0.07539032965061968</v>
+        <v>0.07279583956722309</v>
       </c>
       <c r="G61" s="2" t="n">
-        <v>0.06513631074733642</v>
+        <v>0.0630871303195517</v>
       </c>
       <c r="H61" s="2" t="n">
-        <v>0.0588093073356333</v>
+        <v>0.0572051495289134</v>
       </c>
       <c r="I61" s="2" t="n">
-        <v>0.05465801146599711</v>
+        <v>0.05343833731776829</v>
       </c>
       <c r="J61" s="2" t="n">
-        <v>0.05195404749581219</v>
+        <v>0.05108008787467855</v>
       </c>
       <c r="K61" s="2" t="n">
-        <v>0.05025287775359496</v>
+        <v>0.04971625102356635</v>
       </c>
       <c r="L61" s="2" t="n">
-        <v>0.04929609311682435</v>
+        <v>0.04910680533129995</v>
       </c>
       <c r="M61" s="2" t="n">
-        <v>0.04895788964246673</v>
+        <v>0.04914211499311783</v>
       </c>
       <c r="N61" s="2" t="n">
-        <v>0.0491555999156828</v>
+        <v>0.04975559312298664</v>
       </c>
       <c r="O61" s="2" t="n">
-        <v>0.04984413858227942</v>
+        <v>0.0509264267870588</v>
       </c>
       <c r="P61" s="2" t="n">
-        <v>0.05101770853810567</v>
+        <v>0.05266952243484315</v>
       </c>
       <c r="Q61" s="2" t="n">
-        <v>0.05269190168912224</v>
+        <v>0.05503600366715333</v>
       </c>
       <c r="R61" s="2" t="n">
-        <v>0.05491106614839087</v>
-      </c>
-      <c r="S61" s="2" t="n">
-        <v>0.0571302306076595</v>
-      </c>
-      <c r="T61" s="1" t="inlineStr"/>
+        <v>0.05740248489946351</v>
+      </c>
+      <c r="S61" s="1" t="inlineStr"/>
     </row>
     <row r="62" ht="30" customHeight="1">
       <c r="A62" s="1" t="inlineStr">
@@ -3591,54 +3451,51 @@
       </c>
       <c r="C62" s="1" t="inlineStr"/>
       <c r="D62" s="2" t="n">
-        <v>0.5071108561666231</v>
+        <v>0.5062544510926434</v>
       </c>
       <c r="E62" s="2" t="n">
-        <v>0.7965140112015372</v>
+        <v>0.8035709709007146</v>
       </c>
       <c r="F62" s="2" t="n">
-        <v>0.8617743749479074</v>
+        <v>0.8670515451401452</v>
       </c>
       <c r="G62" s="2" t="n">
-        <v>0.8904383054002251</v>
+        <v>0.8944317807808952</v>
       </c>
       <c r="H62" s="2" t="n">
-        <v>0.9061187619707659</v>
+        <v>0.9092199502745679</v>
       </c>
       <c r="I62" s="2" t="n">
-        <v>0.9156600723535896</v>
+        <v>0.9180634324411635</v>
       </c>
       <c r="J62" s="2" t="n">
-        <v>0.9218666989701296</v>
+        <v>0.9236823143066361</v>
       </c>
       <c r="K62" s="2" t="n">
-        <v>0.9258870356012644</v>
+        <v>0.9271827378215309</v>
       </c>
       <c r="L62" s="2" t="n">
-        <v>0.9284074650572826</v>
+        <v>0.9292011053393887</v>
       </c>
       <c r="M62" s="2" t="n">
-        <v>0.9298220220603441</v>
+        <v>0.9301016194309984</v>
       </c>
       <c r="N62" s="2" t="n">
-        <v>0.9303215240383296</v>
+        <v>0.9300494698354567</v>
       </c>
       <c r="O62" s="2" t="n">
-        <v>0.9300295528929712</v>
+        <v>0.9291429436493502</v>
       </c>
       <c r="P62" s="2" t="n">
-        <v>0.9290120284804108</v>
+        <v>0.9274103632992117</v>
       </c>
       <c r="Q62" s="2" t="n">
-        <v>0.9272751500372671</v>
+        <v>0.9248249459015589</v>
       </c>
       <c r="R62" s="2" t="n">
-        <v>0.924791705252773</v>
-      </c>
-      <c r="S62" s="2" t="n">
-        <v>0.9214895519254134</v>
-      </c>
-      <c r="T62" s="1" t="inlineStr"/>
+        <v>0.9213032909096034</v>
+      </c>
+      <c r="S62" s="1" t="inlineStr"/>
     </row>
     <row r="63" ht="15" customHeight="1">
       <c r="A63" s="1" t="inlineStr">
@@ -3653,54 +3510,51 @@
       </c>
       <c r="C63" s="1" t="inlineStr"/>
       <c r="D63" s="2" t="n">
-        <v>0.7812692787111242</v>
+        <v>0.781132427160474</v>
       </c>
       <c r="E63" s="2" t="n">
-        <v>0.8415346025519874</v>
+        <v>0.8434383830980788</v>
       </c>
       <c r="F63" s="2" t="n">
-        <v>0.8612182742485085</v>
+        <v>0.8631690556287381</v>
       </c>
       <c r="G63" s="2" t="n">
-        <v>0.8731242885411294</v>
+        <v>0.8752186331837397</v>
       </c>
       <c r="H63" s="2" t="n">
-        <v>0.8823152419384261</v>
+        <v>0.8846656334524475</v>
       </c>
       <c r="I63" s="2" t="n">
-        <v>0.8903210003931722</v>
+        <v>0.8930012717048008</v>
       </c>
       <c r="J63" s="2" t="n">
-        <v>0.8977774341433087</v>
+        <v>0.9008423535003319</v>
       </c>
       <c r="K63" s="2" t="n">
-        <v>0.9049413955601958</v>
+        <v>0.9084347036659038</v>
       </c>
       <c r="L63" s="2" t="n">
-        <v>0.911964394567677</v>
+        <v>0.9159163435477082</v>
       </c>
       <c r="M63" s="2" t="n">
-        <v>0.9189300869256287</v>
+        <v>0.9233620626480232</v>
       </c>
       <c r="N63" s="2" t="n">
-        <v>0.9258744305663087</v>
+        <v>0.9307999453445317</v>
       </c>
       <c r="O63" s="2" t="n">
-        <v>0.9328179458511794</v>
+        <v>0.9382427994019147</v>
       </c>
       <c r="P63" s="2" t="n">
-        <v>0.9397678586145239</v>
+        <v>0.9456873125217253</v>
       </c>
       <c r="Q63" s="2" t="n">
-        <v>0.9467175567284032</v>
+        <v>0.953117642351901</v>
       </c>
       <c r="R63" s="2" t="n">
-        <v>0.9536529499680431</v>
-      </c>
-      <c r="S63" s="2" t="n">
-        <v>0.9605497856022194</v>
-      </c>
-      <c r="T63" s="1" t="inlineStr"/>
+        <v>0.9605051626395107</v>
+      </c>
+      <c r="S63" s="1" t="inlineStr"/>
     </row>
     <row r="64" ht="30" customHeight="1">
       <c r="A64" s="1" t="inlineStr">
@@ -3715,54 +3569,51 @@
       </c>
       <c r="C64" s="1" t="inlineStr"/>
       <c r="D64" s="2" t="n">
-        <v>0.4947110208887889</v>
+        <v>0.4947976924542986</v>
       </c>
       <c r="E64" s="2" t="n">
-        <v>0.4777305805592196</v>
+        <v>0.4779735242447286</v>
       </c>
       <c r="F64" s="2" t="n">
-        <v>0.4850371337997327</v>
+        <v>0.4865582469952273</v>
       </c>
       <c r="G64" s="2" t="n">
-        <v>0.4966647621618928</v>
+        <v>0.4994124070984718</v>
       </c>
       <c r="H64" s="2" t="n">
-        <v>0.5098407336349193</v>
+        <v>0.5137734390610369</v>
       </c>
       <c r="I64" s="2" t="n">
-        <v>0.5237673633405326</v>
+        <v>0.5288702372127254</v>
       </c>
       <c r="J64" s="2" t="n">
-        <v>0.5381108674808632</v>
+        <v>0.5443607442121166</v>
       </c>
       <c r="K64" s="2" t="n">
-        <v>0.5527131589300166</v>
+        <v>0.5600965560548041</v>
       </c>
       <c r="L64" s="2" t="n">
-        <v>0.5674653458784754</v>
+        <v>0.5759477597191387</v>
       </c>
       <c r="M64" s="2" t="n">
-        <v>0.5822740841432794</v>
+        <v>0.5918081993459784</v>
       </c>
       <c r="N64" s="2" t="n">
-        <v>0.5970601655016087</v>
+        <v>0.6075771359846209</v>
       </c>
       <c r="O64" s="2" t="n">
-        <v>0.6117280265373947</v>
+        <v>0.6231339534389799</v>
       </c>
       <c r="P64" s="2" t="n">
-        <v>0.6261851294940463</v>
+        <v>0.6383608968284006</v>
       </c>
       <c r="Q64" s="2" t="n">
-        <v>0.6403325756029661</v>
+        <v>0.6531207208541026</v>
       </c>
       <c r="R64" s="2" t="n">
-        <v>0.654056504878885</v>
-      </c>
-      <c r="S64" s="2" t="n">
-        <v>0.6672445293840594</v>
-      </c>
-      <c r="T64" s="1" t="inlineStr"/>
+        <v>0.6672755281010996</v>
+      </c>
+      <c r="S64" s="1" t="inlineStr"/>
     </row>
     <row r="65" ht="15" customHeight="1">
       <c r="A65" s="1" t="inlineStr">
@@ -3780,51 +3631,48 @@
         <v>0.9130337357818</v>
       </c>
       <c r="E65" s="2" t="n">
-        <v>0.8850333252548149</v>
+        <v>0.8830355266498334</v>
       </c>
       <c r="F65" s="2" t="n">
-        <v>0.8570611050841739</v>
+        <v>0.8530645253444216</v>
       </c>
       <c r="G65" s="2" t="n">
-        <v>0.8290571204324678</v>
+        <v>0.8230510799514991</v>
       </c>
       <c r="H65" s="2" t="n">
-        <v>0.8009973827639962</v>
+        <v>0.7929681334991677</v>
       </c>
       <c r="I65" s="2" t="n">
-        <v>0.7728646278053329</v>
+        <v>0.7627977092904863</v>
       </c>
       <c r="J65" s="2" t="n">
-        <v>0.7446612304027046</v>
+        <v>0.7325616461288711</v>
       </c>
       <c r="K65" s="2" t="n">
-        <v>0.7164166267770026</v>
+        <v>0.7022863254977531</v>
       </c>
       <c r="L65" s="2" t="n">
-        <v>0.6881619377878848</v>
+        <v>0.6720276223556498</v>
       </c>
       <c r="M65" s="2" t="n">
-        <v>0.6599421408215783</v>
+        <v>0.6418422361217935</v>
       </c>
       <c r="N65" s="2" t="n">
-        <v>0.6318065171944226</v>
+        <v>0.611794636858556</v>
       </c>
       <c r="O65" s="2" t="n">
-        <v>0.6038156496800842</v>
+        <v>0.5819584578441279</v>
       </c>
       <c r="P65" s="2" t="n">
-        <v>0.5760225971805022</v>
+        <v>0.552396365214525</v>
       </c>
       <c r="Q65" s="2" t="n">
-        <v>0.5484793863228254</v>
+        <v>0.5231726932408487</v>
       </c>
       <c r="R65" s="2" t="n">
-        <v>0.521237818635248</v>
-      </c>
-      <c r="S65" s="2" t="n">
         <v>0.4943374292495647</v>
       </c>
-      <c r="T65" s="1" t="inlineStr"/>
+      <c r="S65" s="1" t="inlineStr"/>
     </row>
     <row r="66" ht="30" customHeight="1">
       <c r="A66" s="1" t="inlineStr">
@@ -3839,54 +3687,51 @@
       </c>
       <c r="C66" s="1" t="inlineStr"/>
       <c r="D66" s="2" t="n">
-        <v>0.6403333333333334</v>
+        <v>0.6396428571428572</v>
       </c>
       <c r="E66" s="2" t="n">
-        <v>0.621</v>
+        <v>0.6189285714285715</v>
       </c>
       <c r="F66" s="2" t="n">
-        <v>0.6016666666666667</v>
+        <v>0.5982142857142857</v>
       </c>
       <c r="G66" s="2" t="n">
-        <v>0.5823333333333334</v>
+        <v>0.5775</v>
       </c>
       <c r="H66" s="2" t="n">
-        <v>0.5629999999999999</v>
+        <v>0.5567857142857143</v>
       </c>
       <c r="I66" s="2" t="n">
-        <v>0.5436666666666667</v>
+        <v>0.5360714285714285</v>
       </c>
       <c r="J66" s="2" t="n">
-        <v>0.5243333333333333</v>
+        <v>0.5153571428571428</v>
       </c>
       <c r="K66" s="2" t="n">
-        <v>0.505</v>
+        <v>0.4946428571428572</v>
       </c>
       <c r="L66" s="2" t="n">
-        <v>0.4856666666666667</v>
+        <v>0.4739285714285715</v>
       </c>
       <c r="M66" s="2" t="n">
-        <v>0.4663333333333333</v>
+        <v>0.4532142857142857</v>
       </c>
       <c r="N66" s="2" t="n">
-        <v>0.447</v>
+        <v>0.4325</v>
       </c>
       <c r="O66" s="2" t="n">
-        <v>0.4276666666666667</v>
+        <v>0.4117857142857143</v>
       </c>
       <c r="P66" s="2" t="n">
-        <v>0.4083333333333333</v>
+        <v>0.3910714285714286</v>
       </c>
       <c r="Q66" s="2" t="n">
-        <v>0.389</v>
+        <v>0.3703571428571428</v>
       </c>
       <c r="R66" s="2" t="n">
-        <v>0.3696666666666667</v>
-      </c>
-      <c r="S66" s="2" t="n">
-        <v>0.3503333333333333</v>
-      </c>
-      <c r="T66" s="1" t="inlineStr"/>
+        <v>0.3496428571428571</v>
+      </c>
+      <c r="S66" s="1" t="inlineStr"/>
     </row>
     <row r="67" ht="15" customHeight="1">
       <c r="A67" s="1" t="inlineStr">
@@ -3901,54 +3746,51 @@
       </c>
       <c r="C67" s="1" t="inlineStr"/>
       <c r="D67" s="2" t="n">
-        <v>1.150011517879318</v>
+        <v>1.149900190948778</v>
       </c>
       <c r="E67" s="2" t="n">
-        <v>1.040856798279222</v>
+        <v>1.037406335378524</v>
       </c>
       <c r="F67" s="2" t="n">
-        <v>1.012030332275313</v>
+        <v>1.008925798296564</v>
       </c>
       <c r="G67" s="2" t="n">
-        <v>0.9969084778913009</v>
+        <v>0.9938963560643232</v>
       </c>
       <c r="H67" s="2" t="n">
-        <v>0.9863173959023402</v>
+        <v>0.9831646987246834</v>
       </c>
       <c r="I67" s="2" t="n">
-        <v>0.9775792957002311</v>
+        <v>0.9741269377820952</v>
       </c>
       <c r="J67" s="2" t="n">
-        <v>0.9695621110230351</v>
+        <v>0.9656506714457721</v>
       </c>
       <c r="K67" s="2" t="n">
-        <v>0.9617625261085604</v>
+        <v>0.9572427390595025</v>
       </c>
       <c r="L67" s="2" t="n">
-        <v>0.9538345017902922</v>
+        <v>0.9485264056880329</v>
       </c>
       <c r="M67" s="2" t="n">
-        <v>0.9455090296099077</v>
+        <v>0.9392010422085477</v>
       </c>
       <c r="N67" s="2" t="n">
-        <v>0.9365735498767322</v>
+        <v>0.9290023750862315</v>
       </c>
       <c r="O67" s="2" t="n">
-        <v>0.9267867253069327</v>
+        <v>0.9176220242343975</v>
       </c>
       <c r="P67" s="2" t="n">
-        <v>0.9159009995558133</v>
+        <v>0.9047385458666748</v>
       </c>
       <c r="Q67" s="2" t="n">
-        <v>0.9036486123004409</v>
+        <v>0.8899750486647011</v>
       </c>
       <c r="R67" s="2" t="n">
-        <v>0.889715679701415</v>
-      </c>
-      <c r="S67" s="2" t="n">
-        <v>0.8737700314689053</v>
-      </c>
-      <c r="T67" s="1" t="inlineStr"/>
+        <v>0.8729257643027138</v>
+      </c>
+      <c r="S67" s="1" t="inlineStr"/>
     </row>
     <row r="68" ht="15" customHeight="1">
       <c r="A68" s="1" t="inlineStr">
@@ -3963,54 +3805,51 @@
       </c>
       <c r="C68" s="1" t="inlineStr"/>
       <c r="D68" s="2" t="n">
-        <v>0.9129976966874244</v>
+        <v>0.9123908734224122</v>
       </c>
       <c r="E68" s="2" t="n">
-        <v>0.9150619818429163</v>
+        <v>0.9132006195531562</v>
       </c>
       <c r="F68" s="2" t="n">
-        <v>0.8923130416932181</v>
+        <v>0.887967323159673</v>
       </c>
       <c r="G68" s="2" t="n">
-        <v>0.8646283651232153</v>
+        <v>0.8577821070040713</v>
       </c>
       <c r="H68" s="2" t="n">
-        <v>0.834907678720365</v>
+        <v>0.8255539583207618</v>
       </c>
       <c r="I68" s="2" t="n">
-        <v>0.8040381898895175</v>
+        <v>0.792160112745544</v>
       </c>
       <c r="J68" s="2" t="n">
-        <v>0.7724311182350889</v>
+        <v>0.7580358219315676</v>
       </c>
       <c r="K68" s="2" t="n">
-        <v>0.740318990147195</v>
+        <v>0.72342089195214</v>
       </c>
       <c r="L68" s="2" t="n">
-        <v>0.7078819770274036</v>
+        <v>0.6885297165190225</v>
       </c>
       <c r="M68" s="2" t="n">
-        <v>0.675279039199588</v>
+        <v>0.6535447189435526</v>
       </c>
       <c r="N68" s="2" t="n">
-        <v>0.6426482553515347</v>
+        <v>0.6186306556226798</v>
       </c>
       <c r="O68" s="2" t="n">
-        <v>0.6101300308937273</v>
+        <v>0.5839510578580409</v>
       </c>
       <c r="P68" s="2" t="n">
-        <v>0.5778478490882533</v>
+        <v>0.5496458774495508</v>
       </c>
       <c r="Q68" s="2" t="n">
-        <v>0.5459136371160284</v>
+        <v>0.5158449565439994</v>
       </c>
       <c r="R68" s="2" t="n">
-        <v>0.5144310989034653</v>
-      </c>
-      <c r="S68" s="2" t="n">
-        <v>0.4834821947991647</v>
-      </c>
-      <c r="T68" s="1" t="inlineStr"/>
+        <v>0.4826515564353129</v>
+      </c>
+      <c r="S68" s="1" t="inlineStr"/>
     </row>
     <row r="69" ht="15" customHeight="1">
       <c r="A69" s="1" t="inlineStr">
@@ -4025,54 +3864,51 @@
       </c>
       <c r="C69" s="1" t="inlineStr"/>
       <c r="D69" s="2" t="n">
-        <v>0.2369777820975177</v>
+        <v>0.236866455166978</v>
       </c>
       <c r="E69" s="2" t="n">
-        <v>0.1558234730244067</v>
+        <v>0.1543708087286905</v>
       </c>
       <c r="F69" s="2" t="n">
-        <v>0.1549692271911389</v>
+        <v>0.1558612729521429</v>
       </c>
       <c r="G69" s="2" t="n">
-        <v>0.1678513574588331</v>
+        <v>0.1708452761128242</v>
       </c>
       <c r="H69" s="2" t="n">
-        <v>0.185320013138344</v>
+        <v>0.1901965652255156</v>
       </c>
       <c r="I69" s="2" t="n">
-        <v>0.2047146678948981</v>
+        <v>0.211329228491609</v>
       </c>
       <c r="J69" s="2" t="n">
-        <v>0.2249008806203305</v>
+        <v>0.233089025316901</v>
       </c>
       <c r="K69" s="2" t="n">
-        <v>0.2453458993315578</v>
+        <v>0.2549564135617495</v>
       </c>
       <c r="L69" s="2" t="n">
-        <v>0.2656725640024074</v>
+        <v>0.2764987833323831</v>
       </c>
       <c r="M69" s="2" t="n">
-        <v>0.2855668887883294</v>
+        <v>0.2973588060867542</v>
       </c>
       <c r="N69" s="2" t="n">
-        <v>0.3047670326823096</v>
+        <v>0.3172077382276756</v>
       </c>
       <c r="O69" s="2" t="n">
-        <v>0.3229710756268486</v>
+        <v>0.3356635663902696</v>
       </c>
       <c r="P69" s="2" t="n">
-        <v>0.3398784023753111</v>
+        <v>0.3523421806521498</v>
       </c>
       <c r="Q69" s="2" t="n">
-        <v>0.3551692259776155</v>
+        <v>0.3668023554238524</v>
       </c>
       <c r="R69" s="2" t="n">
-        <v>0.368477861066167</v>
-      </c>
-      <c r="S69" s="2" t="n">
-        <v>0.3794326022193406</v>
-      </c>
-      <c r="T69" s="1" t="inlineStr"/>
+        <v>0.3785883350531491</v>
+      </c>
+      <c r="S69" s="1" t="inlineStr"/>
     </row>
     <row r="70" ht="15" customHeight="1">
       <c r="A70" s="1" t="inlineStr">
@@ -4087,54 +3923,51 @@
       </c>
       <c r="C70" s="1" t="inlineStr"/>
       <c r="D70" s="2" t="n">
-        <v>0.2381264220893905</v>
+        <v>0.2381873725672461</v>
       </c>
       <c r="E70" s="2" t="n">
-        <v>0.1473158174272687</v>
+        <v>0.1456415175054772</v>
       </c>
       <c r="F70" s="2" t="n">
-        <v>0.1437980619569752</v>
+        <v>0.1446304062066568</v>
       </c>
       <c r="G70" s="2" t="n">
-        <v>0.1562961232098367</v>
+        <v>0.1594498269157253</v>
       </c>
       <c r="H70" s="2" t="n">
-        <v>0.1744224596389855</v>
+        <v>0.1796854435518387</v>
       </c>
       <c r="I70" s="2" t="n">
-        <v>0.1950490217945792</v>
+        <v>0.2022692408020758</v>
       </c>
       <c r="J70" s="2" t="n">
-        <v>0.2167902001722725</v>
+        <v>0.2257775122301158</v>
       </c>
       <c r="K70" s="2" t="n">
-        <v>0.2389595642966558</v>
+        <v>0.2495156309882033</v>
       </c>
       <c r="L70" s="2" t="n">
-        <v>0.2610458516054659</v>
+        <v>0.2728955178517541</v>
       </c>
       <c r="M70" s="2" t="n">
-        <v>0.2826135467464744</v>
+        <v>0.2954128716460067</v>
       </c>
       <c r="N70" s="2" t="n">
-        <v>0.303286246538139</v>
+        <v>0.316596329059247</v>
       </c>
       <c r="O70" s="2" t="n">
-        <v>0.3226437126680715</v>
+        <v>0.3359150853534756</v>
       </c>
       <c r="P70" s="2" t="n">
-        <v>0.3402635618865514</v>
+        <v>0.3528309461237974</v>
       </c>
       <c r="Q70" s="2" t="n">
-        <v>0.3557002426642774</v>
+        <v>0.3667419980396467</v>
       </c>
       <c r="R70" s="2" t="n">
-        <v>0.3684567949154934</v>
-      </c>
-      <c r="S70" s="2" t="n">
-        <v>0.3780261807602814</v>
-      </c>
-      <c r="T70" s="1" t="inlineStr"/>
+        <v>0.3770263156088866</v>
+      </c>
+      <c r="S70" s="1" t="inlineStr"/>
     </row>
     <row r="71" ht="15" customHeight="1">
       <c r="A71" s="1" t="inlineStr">
@@ -4152,51 +3985,48 @@
         <v>251.7894146864385</v>
       </c>
       <c r="E71" s="2" t="n">
-        <v>249.8009621686911</v>
+        <v>249.6625952542775</v>
       </c>
       <c r="F71" s="2" t="n">
-        <v>247.9136892966872</v>
+        <v>247.6528107706313</v>
       </c>
       <c r="G71" s="2" t="n">
-        <v>246.1387065941966</v>
+        <v>245.7731838000793</v>
       </c>
       <c r="H71" s="2" t="n">
-        <v>244.4815971910143</v>
+        <v>244.0304158041251</v>
       </c>
       <c r="I71" s="2" t="n">
-        <v>242.9479317023808</v>
+        <v>242.4310417988148</v>
       </c>
       <c r="J71" s="2" t="n">
-        <v>241.539700983277</v>
+        <v>240.972909827971</v>
       </c>
       <c r="K71" s="2" t="n">
-        <v>240.2521702422908</v>
+        <v>239.6524840515102</v>
       </c>
       <c r="L71" s="2" t="n">
-        <v>239.0793762629544</v>
+        <v>238.4569611637397</v>
       </c>
       <c r="M71" s="2" t="n">
-        <v>238.0101114191572</v>
+        <v>237.3706330162411</v>
       </c>
       <c r="N71" s="2" t="n">
-        <v>237.0296181915506</v>
+        <v>236.3718770966746</v>
       </c>
       <c r="O71" s="2" t="n">
-        <v>236.116342046438</v>
+        <v>235.4310839272837</v>
       </c>
       <c r="P71" s="2" t="n">
-        <v>235.2469960755472</v>
+        <v>234.5161748631908</v>
       </c>
       <c r="Q71" s="2" t="n">
-        <v>234.3939168165112</v>
+        <v>233.5872660970408</v>
       </c>
       <c r="R71" s="2" t="n">
-        <v>233.5237985627082</v>
-      </c>
-      <c r="S71" s="2" t="n">
         <v>232.6016263665796</v>
       </c>
-      <c r="T71" s="1" t="inlineStr"/>
+      <c r="S71" s="1" t="inlineStr"/>
     </row>
     <row r="72" ht="15" customHeight="1">
       <c r="A72" s="1" t="inlineStr">
@@ -4211,54 +4041,51 @@
       </c>
       <c r="C72" s="1" t="inlineStr"/>
       <c r="D72" s="2" t="n">
-        <v>196.2932833273169</v>
+        <v>196.0816188216095</v>
       </c>
       <c r="E72" s="2" t="n">
-        <v>190.3666771675124</v>
+        <v>189.7316836503905</v>
       </c>
       <c r="F72" s="2" t="n">
-        <v>184.4400710077079</v>
+        <v>183.3817484791714</v>
       </c>
       <c r="G72" s="2" t="n">
-        <v>178.5134648479034</v>
+        <v>177.0318133079523</v>
       </c>
       <c r="H72" s="2" t="n">
-        <v>172.5868586880989</v>
+        <v>170.6818781367333</v>
       </c>
       <c r="I72" s="2" t="n">
-        <v>166.6602525282945</v>
+        <v>164.3319429655142</v>
       </c>
       <c r="J72" s="2" t="n">
-        <v>160.73364636849</v>
+        <v>157.9820077942951</v>
       </c>
       <c r="K72" s="2" t="n">
-        <v>154.8070402086856</v>
+        <v>151.6320726230761</v>
       </c>
       <c r="L72" s="2" t="n">
-        <v>148.8804340488811</v>
+        <v>145.282137451857</v>
       </c>
       <c r="M72" s="2" t="n">
-        <v>142.9538278890766</v>
+        <v>138.9322022806379</v>
       </c>
       <c r="N72" s="2" t="n">
-        <v>137.0272217292722</v>
+        <v>132.5822671094188</v>
       </c>
       <c r="O72" s="2" t="n">
-        <v>131.1006155694677</v>
+        <v>126.2323319381998</v>
       </c>
       <c r="P72" s="2" t="n">
-        <v>125.1740094096633</v>
+        <v>119.8823967669807</v>
       </c>
       <c r="Q72" s="2" t="n">
-        <v>119.2474032498588</v>
+        <v>113.5324615957616</v>
       </c>
       <c r="R72" s="2" t="n">
-        <v>113.3207970900543</v>
-      </c>
-      <c r="S72" s="2" t="n">
-        <v>107.3941909302498</v>
-      </c>
-      <c r="T72" s="1" t="inlineStr"/>
+        <v>107.1825264245426</v>
+      </c>
+      <c r="S72" s="1" t="inlineStr"/>
     </row>
     <row r="73" ht="15" customHeight="1">
       <c r="A73" s="1" t="inlineStr">
@@ -4273,54 +4100,51 @@
       </c>
       <c r="C73" s="1" t="inlineStr"/>
       <c r="D73" s="2" t="n">
-        <v>248.0517603648712</v>
+        <v>247.9005511003574</v>
       </c>
       <c r="E73" s="2" t="n">
-        <v>240.1798960230389</v>
+        <v>239.722425110993</v>
       </c>
       <c r="F73" s="2" t="n">
-        <v>236.9094723022859</v>
+        <v>236.3804261005702</v>
       </c>
       <c r="G73" s="2" t="n">
-        <v>234.6224489396598</v>
+        <v>234.0471923727898</v>
       </c>
       <c r="H73" s="2" t="n">
-        <v>232.837041863052</v>
+        <v>232.2443952114634</v>
       </c>
       <c r="I73" s="2" t="n">
-        <v>231.4199672453222</v>
+        <v>230.8447911323391</v>
       </c>
       <c r="J73" s="2" t="n">
-        <v>230.3175196216195</v>
+        <v>229.7932112410973</v>
       </c>
       <c r="K73" s="2" t="n">
-        <v>229.5057972508388</v>
+        <v>229.0678517566361</v>
       </c>
       <c r="L73" s="2" t="n">
-        <v>228.967182502565</v>
+        <v>228.6458226289366</v>
       </c>
       <c r="M73" s="2" t="n">
-        <v>228.68399545452</v>
+        <v>228.5052237669685</v>
       </c>
       <c r="N73" s="2" t="n">
-        <v>228.6387798288928</v>
+        <v>228.6215960141323</v>
       </c>
       <c r="O73" s="2" t="n">
-        <v>228.8072540849443</v>
+        <v>228.9619226465695</v>
       </c>
       <c r="P73" s="2" t="n">
-        <v>229.1630518688698</v>
+        <v>229.4903727663425</v>
       </c>
       <c r="Q73" s="2" t="n">
-        <v>229.6756518894332</v>
+        <v>230.1629008037089</v>
       </c>
       <c r="R73" s="2" t="n">
-        <v>230.3082587879495</v>
-      </c>
-      <c r="S73" s="2" t="n">
-        <v>231.0222911287899</v>
-      </c>
-      <c r="T73" s="1" t="inlineStr"/>
+        <v>230.932388801264</v>
+      </c>
+      <c r="S73" s="1" t="inlineStr"/>
     </row>
     <row r="74" ht="15" customHeight="1">
       <c r="A74" s="1" t="inlineStr">
@@ -4338,51 +4162,48 @@
         <v>0.9198717705829682</v>
       </c>
       <c r="E74" s="2" t="n">
-        <v>0.930908005417769</v>
+        <v>0.9316127880691234</v>
       </c>
       <c r="F74" s="2" t="n">
-        <v>0.9399111885257418</v>
+        <v>0.9411937231993717</v>
       </c>
       <c r="G74" s="2" t="n">
-        <v>0.9475445209109083</v>
+        <v>0.9489889140291673</v>
       </c>
       <c r="H74" s="2" t="n">
-        <v>0.9539515543452253</v>
+        <v>0.9555931563290563</v>
       </c>
       <c r="I74" s="2" t="n">
-        <v>0.9594117104066201</v>
+        <v>0.961206325603477</v>
       </c>
       <c r="J74" s="2" t="n">
-        <v>0.9641351229571883</v>
+        <v>0.9659487560133837</v>
       </c>
       <c r="K74" s="2" t="n">
-        <v>0.9682321979656086</v>
+        <v>0.9700508464641263</v>
       </c>
       <c r="L74" s="2" t="n">
-        <v>0.9717447196250987</v>
+        <v>0.9735532872138978</v>
       </c>
       <c r="M74" s="2" t="n">
-        <v>0.9748160838275998</v>
+        <v>0.9765720654514889</v>
       </c>
       <c r="N74" s="2" t="n">
-        <v>0.9775237620338982</v>
+        <v>0.9792051916840198</v>
       </c>
       <c r="O74" s="2" t="n">
-        <v>0.9798313148293836</v>
+        <v>0.9814270687200961</v>
       </c>
       <c r="P74" s="2" t="n">
-        <v>0.9818335545120593</v>
+        <v>0.9833372387193101</v>
       </c>
       <c r="Q74" s="2" t="n">
-        <v>0.9835696379292527</v>
+        <v>0.9849622306534793</v>
       </c>
       <c r="R74" s="2" t="n">
-        <v>0.985061197937973</v>
-      </c>
-      <c r="S74" s="2" t="n">
         <v>0.9863414798135992</v>
       </c>
-      <c r="T74" s="1" t="inlineStr"/>
+      <c r="S74" s="1" t="inlineStr"/>
     </row>
     <row r="75" ht="15" customHeight="1">
       <c r="A75" s="1" t="inlineStr">
@@ -4400,51 +4221,48 @@
         <v>264.9230699278949</v>
       </c>
       <c r="E75" s="2" t="n">
-        <v>292.8257431134205</v>
+        <v>294.8147930348406</v>
       </c>
       <c r="F75" s="2" t="n">
-        <v>320.6211333531855</v>
+        <v>324.62968952623</v>
       </c>
       <c r="G75" s="2" t="n">
-        <v>348.3910958285558</v>
+        <v>354.3231214071286</v>
       </c>
       <c r="H75" s="2" t="n">
-        <v>376.0830772634475</v>
+        <v>383.9816453978873</v>
       </c>
       <c r="I75" s="2" t="n">
-        <v>403.716948421949</v>
+        <v>413.5895941067111</v>
       </c>
       <c r="J75" s="2" t="n">
-        <v>431.3112687519726</v>
+        <v>443.117562409901</v>
       </c>
       <c r="K75" s="2" t="n">
-        <v>458.8596591757861</v>
+        <v>472.6034652144938</v>
       </c>
       <c r="L75" s="2" t="n">
-        <v>486.3331263978957</v>
+        <v>502.0136192526899</v>
       </c>
       <c r="M75" s="2" t="n">
-        <v>513.7606689161634</v>
+        <v>531.3599424493966</v>
       </c>
       <c r="N75" s="2" t="n">
-        <v>541.1500239054108</v>
+        <v>560.65726222911</v>
       </c>
       <c r="O75" s="2" t="n">
-        <v>568.451073262972</v>
+        <v>589.8572714101675</v>
       </c>
       <c r="P75" s="2" t="n">
-        <v>595.6894595592446</v>
+        <v>618.9875214592724</v>
       </c>
       <c r="Q75" s="2" t="n">
-        <v>622.8656529904968</v>
+        <v>648.0388565102273</v>
       </c>
       <c r="R75" s="2" t="n">
-        <v>649.9727208113966</v>
-      </c>
-      <c r="S75" s="2" t="n">
         <v>677.0139991251236</v>
       </c>
-      <c r="T75" s="1" t="inlineStr"/>
+      <c r="S75" s="1" t="inlineStr"/>
     </row>
     <row r="76" ht="15" customHeight="1">
       <c r="A76" s="1" t="inlineStr">
@@ -4462,51 +4280,48 @@
         <v>298.0389802067385</v>
       </c>
       <c r="E76" s="2" t="n">
-        <v>313.2520727793622</v>
+        <v>314.3092699735009</v>
       </c>
       <c r="F76" s="2" t="n">
-        <v>327.7376828837337</v>
+        <v>329.7159706916777</v>
       </c>
       <c r="G76" s="2" t="n">
-        <v>341.5359363918575</v>
+        <v>344.4249425018446</v>
       </c>
       <c r="H76" s="2" t="n">
-        <v>354.7685386161718</v>
+        <v>358.4549534872339</v>
       </c>
       <c r="I76" s="2" t="n">
-        <v>367.4838532828871</v>
+        <v>371.8862930918287</v>
       </c>
       <c r="J76" s="2" t="n">
-        <v>379.7080435764382</v>
+        <v>384.8173876481858</v>
       </c>
       <c r="K76" s="2" t="n">
-        <v>391.4857966451933</v>
+        <v>397.2404946796239</v>
       </c>
       <c r="L76" s="2" t="n">
-        <v>402.9017712038968</v>
+        <v>409.2488411885599</v>
       </c>
       <c r="M76" s="2" t="n">
-        <v>413.9364337923426</v>
+        <v>420.8560609516754</v>
       </c>
       <c r="N76" s="2" t="n">
-        <v>424.589106731691</v>
+        <v>432.0499545452333</v>
       </c>
       <c r="O76" s="2" t="n">
-        <v>434.9928791022549</v>
+        <v>442.9683589780464</v>
       </c>
       <c r="P76" s="2" t="n">
-        <v>445.1113929581084</v>
+        <v>453.5642238185459</v>
       </c>
       <c r="Q76" s="2" t="n">
-        <v>454.9549308573855</v>
+        <v>463.8734511232522</v>
       </c>
       <c r="R76" s="2" t="n">
-        <v>464.550991329953</v>
-      </c>
-      <c r="S76" s="2" t="n">
         <v>473.8913655885228</v>
       </c>
-      <c r="T76" s="1" t="inlineStr"/>
+      <c r="S76" s="1" t="inlineStr"/>
     </row>
     <row r="77" ht="30" customHeight="1">
       <c r="A77" s="1" t="inlineStr">
@@ -4524,51 +4339,48 @@
         <v>0.8448204141343578</v>
       </c>
       <c r="E77" s="2" t="n">
-        <v>0.7974439241608384</v>
+        <v>0.7943214505742267</v>
       </c>
       <c r="F77" s="2" t="n">
-        <v>0.7564393789426883</v>
+        <v>0.7511095390711756</v>
       </c>
       <c r="G77" s="2" t="n">
-        <v>0.7206817215035083</v>
+        <v>0.7135754513445642</v>
       </c>
       <c r="H77" s="2" t="n">
-        <v>0.6891298708297292</v>
+        <v>0.6807840523057973</v>
       </c>
       <c r="I77" s="2" t="n">
-        <v>0.6611118543904044</v>
+        <v>0.651895609766268</v>
       </c>
       <c r="J77" s="2" t="n">
-        <v>0.6361195267506974</v>
+        <v>0.6262006800178096</v>
       </c>
       <c r="K77" s="2" t="n">
-        <v>0.6136931973039962</v>
+        <v>0.6032931870271456</v>
       </c>
       <c r="L77" s="2" t="n">
-        <v>0.5933937087160716</v>
+        <v>0.582669850624871</v>
       </c>
       <c r="M77" s="2" t="n">
-        <v>0.5749919359322656</v>
+        <v>0.5640185684375758</v>
       </c>
       <c r="N77" s="2" t="n">
-        <v>0.5582564753394292</v>
+        <v>0.5470938594252941</v>
       </c>
       <c r="O77" s="2" t="n">
-        <v>0.5428050742663618</v>
+        <v>0.5314851030679409</v>
       </c>
       <c r="P77" s="2" t="n">
-        <v>0.5285126370550741</v>
+        <v>0.5170517482371183</v>
       </c>
       <c r="Q77" s="2" t="n">
-        <v>0.515202497915088</v>
+        <v>0.5035581698659797</v>
       </c>
       <c r="R77" s="2" t="n">
-        <v>0.5026871170679411</v>
-      </c>
-      <c r="S77" s="2" t="n">
         <v>0.4908332230905137</v>
       </c>
-      <c r="T77" s="1" t="inlineStr"/>
+      <c r="S77" s="1" t="inlineStr"/>
     </row>
     <row r="78" ht="30" customHeight="1">
       <c r="A78" s="1" t="inlineStr">
@@ -4583,54 +4395,51 @@
       </c>
       <c r="C78" s="1" t="inlineStr"/>
       <c r="D78" s="2" t="n">
-        <v>0.7762805497595007</v>
+        <v>0.7758194364498247</v>
       </c>
       <c r="E78" s="2" t="n">
-        <v>0.7195874767764773</v>
+        <v>0.7162072399490459</v>
       </c>
       <c r="F78" s="2" t="n">
-        <v>0.6820840866459945</v>
+        <v>0.6768754162864432</v>
       </c>
       <c r="G78" s="2" t="n">
-        <v>0.6511333780898241</v>
+        <v>0.6446312378490995</v>
       </c>
       <c r="H78" s="2" t="n">
-        <v>0.6245130036369227</v>
+        <v>0.6171656544030198</v>
       </c>
       <c r="I78" s="2" t="n">
-        <v>0.6013365331651109</v>
+        <v>0.5933516387160817</v>
       </c>
       <c r="J78" s="2" t="n">
-        <v>0.5808623041953515</v>
+        <v>0.5724800026430085</v>
       </c>
       <c r="K78" s="2" t="n">
-        <v>0.5627532946453329</v>
+        <v>0.5541992204938717</v>
       </c>
       <c r="L78" s="2" t="n">
-        <v>0.5467519525118658</v>
+        <v>0.5381521735211686</v>
       </c>
       <c r="M78" s="2" t="n">
-        <v>0.5326486714454499</v>
+        <v>0.5241056797248543</v>
       </c>
       <c r="N78" s="2" t="n">
-        <v>0.5200619476864727</v>
+        <v>0.5116577227873375</v>
       </c>
       <c r="O78" s="2" t="n">
-        <v>0.5088274897180355</v>
+        <v>0.5006277313683627</v>
       </c>
       <c r="P78" s="2" t="n">
-        <v>0.4987969665535941</v>
+        <v>0.4908125161156869</v>
       </c>
       <c r="Q78" s="2" t="n">
-        <v>0.4897888944330698</v>
+        <v>0.4820311420268309</v>
       </c>
       <c r="R78" s="2" t="n">
-        <v>0.4816627856862081</v>
-      </c>
-      <c r="S78" s="2" t="n">
-        <v>0.4742546645343235</v>
-      </c>
-      <c r="T78" s="1" t="inlineStr"/>
+        <v>0.474084587425221</v>
+      </c>
+      <c r="S78" s="1" t="inlineStr"/>
     </row>
     <row r="79" ht="15" customHeight="1">
       <c r="A79" s="1" t="inlineStr">
@@ -4648,51 +4457,48 @@
         <v>304.6972711556989</v>
       </c>
       <c r="E79" s="2" t="n">
-        <v>332.5412301095225</v>
+        <v>334.5400980960846</v>
       </c>
       <c r="F79" s="2" t="n">
-        <v>360.3157523649842</v>
+        <v>364.2636577736324</v>
       </c>
       <c r="G79" s="2" t="n">
-        <v>387.9652287313608</v>
+        <v>393.9358180901934</v>
       </c>
       <c r="H79" s="2" t="n">
-        <v>415.5484181640575</v>
+        <v>423.4832578774369</v>
       </c>
       <c r="I79" s="2" t="n">
-        <v>443.0550461864155</v>
+        <v>452.9241266519992</v>
       </c>
       <c r="J79" s="2" t="n">
-        <v>470.7121634428254</v>
+        <v>482.5514447276188</v>
       </c>
       <c r="K79" s="2" t="n">
-        <v>498.295226716079</v>
+        <v>512.0790958565088</v>
       </c>
       <c r="L79" s="2" t="n">
-        <v>525.8469279503316</v>
+        <v>541.5492817938723</v>
       </c>
       <c r="M79" s="2" t="n">
-        <v>553.3116738158444</v>
+        <v>570.9315691201923</v>
       </c>
       <c r="N79" s="2" t="n">
-        <v>580.6553434530979</v>
+        <v>600.1737035863282</v>
       </c>
       <c r="O79" s="2" t="n">
-        <v>607.9683068286746</v>
+        <v>629.3627469314156</v>
       </c>
       <c r="P79" s="2" t="n">
-        <v>635.1835141618287</v>
+        <v>658.4149708618947</v>
       </c>
       <c r="Q79" s="2" t="n">
-        <v>662.2781021930996</v>
+        <v>687.3224160481872</v>
       </c>
       <c r="R79" s="2" t="n">
-        <v>689.2438426770293</v>
-      </c>
-      <c r="S79" s="2" t="n">
         <v>716.0408161885885</v>
       </c>
-      <c r="T79" s="1" t="inlineStr"/>
+      <c r="S79" s="1" t="inlineStr"/>
     </row>
     <row r="80" ht="15" customHeight="1">
       <c r="A80" s="1" t="inlineStr">
@@ -4707,54 +4513,51 @@
       </c>
       <c r="C80" s="1" t="inlineStr"/>
       <c r="D80" s="2" t="n">
-        <v>0.899977269938159</v>
+        <v>0.9001179490256411</v>
       </c>
       <c r="E80" s="2" t="n">
-        <v>0.9142175178994719</v>
+        <v>0.9152540141204015</v>
       </c>
       <c r="F80" s="2" t="n">
-        <v>0.9232442532169893</v>
+        <v>0.9244318040653919</v>
       </c>
       <c r="G80" s="2" t="n">
-        <v>0.9302787318018001</v>
+        <v>0.9317173785273669</v>
       </c>
       <c r="H80" s="2" t="n">
-        <v>0.9360793185234136</v>
+        <v>0.937726382807626</v>
       </c>
       <c r="I80" s="2" t="n">
-        <v>0.9410173094649702</v>
+        <v>0.9426849249698401</v>
       </c>
       <c r="J80" s="2" t="n">
-        <v>0.9452875433583487</v>
+        <v>0.946979765540149</v>
       </c>
       <c r="K80" s="2" t="n">
-        <v>0.9488894882232354</v>
+        <v>0.9505998836898391</v>
       </c>
       <c r="L80" s="2" t="n">
-        <v>0.9520408323758175</v>
+        <v>0.9537141112961338</v>
       </c>
       <c r="M80" s="2" t="n">
-        <v>0.9548516589638915</v>
+        <v>0.9564711798415051</v>
       </c>
       <c r="N80" s="2" t="n">
-        <v>0.9572118925929692</v>
+        <v>0.9587739854529909</v>
       </c>
       <c r="O80" s="2" t="n">
-        <v>0.9592846729101582</v>
+        <v>0.9608011997304212</v>
       </c>
       <c r="P80" s="2" t="n">
-        <v>0.9611226909214362</v>
+        <v>0.9625781653535936</v>
       </c>
       <c r="Q80" s="2" t="n">
-        <v>0.9627508999351054</v>
+        <v>0.9641758826673019</v>
       </c>
       <c r="R80" s="2" t="n">
-        <v>0.9642306135656683</v>
-      </c>
-      <c r="S80" s="2" t="n">
-        <v>0.9655692914167171</v>
-      </c>
-      <c r="T80" s="1" t="inlineStr"/>
+        <v>0.9656098120502704</v>
+      </c>
+      <c r="S80" s="1" t="inlineStr"/>
     </row>
     <row r="81" ht="15" customHeight="1">
       <c r="A81" s="1" t="inlineStr">
@@ -4769,54 +4572,51 @@
       </c>
       <c r="C81" s="1" t="inlineStr"/>
       <c r="D81" s="2" t="n">
-        <v>617.7345504699753</v>
+        <v>617.8311110563023</v>
       </c>
       <c r="E81" s="2" t="n">
-        <v>627.50890085281</v>
+        <v>628.2203405174404</v>
       </c>
       <c r="F81" s="2" t="n">
-        <v>633.7047532035713</v>
+        <v>634.5198751116486</v>
       </c>
       <c r="G81" s="2" t="n">
-        <v>638.5331423324183</v>
+        <v>639.5206137030721</v>
       </c>
       <c r="H81" s="2" t="n">
-        <v>642.5146015876995</v>
+        <v>643.6451284900878</v>
       </c>
       <c r="I81" s="2" t="n">
-        <v>645.9039845381343</v>
+        <v>647.0486175735091</v>
       </c>
       <c r="J81" s="2" t="n">
-        <v>648.835026357345</v>
+        <v>649.9965491465167</v>
       </c>
       <c r="K81" s="2" t="n">
-        <v>651.3073618998652</v>
+        <v>652.4813586328726</v>
       </c>
       <c r="L81" s="2" t="n">
-        <v>653.4704100439648</v>
+        <v>654.6189303857324</v>
       </c>
       <c r="M81" s="2" t="n">
-        <v>655.3997306577534</v>
+        <v>656.5113520672343</v>
       </c>
       <c r="N81" s="2" t="n">
-        <v>657.0197691949074</v>
+        <v>658.0919726414946</v>
       </c>
       <c r="O81" s="2" t="n">
-        <v>658.4425029241156</v>
+        <v>659.4834303395994</v>
       </c>
       <c r="P81" s="2" t="n">
-        <v>659.7040983753325</v>
+        <v>660.7031200996602</v>
       </c>
       <c r="Q81" s="2" t="n">
-        <v>660.8216832263357</v>
+        <v>661.7997757814525</v>
       </c>
       <c r="R81" s="2" t="n">
-        <v>661.8373424712217</v>
-      </c>
-      <c r="S81" s="2" t="n">
-        <v>662.756196300273</v>
-      </c>
-      <c r="T81" s="1" t="inlineStr"/>
+        <v>662.7840092197644</v>
+      </c>
+      <c r="S81" s="1" t="inlineStr"/>
     </row>
     <row r="82" ht="15" customHeight="1">
       <c r="A82" s="1" t="inlineStr">
@@ -4831,54 +4631,51 @@
       </c>
       <c r="C82" s="1" t="inlineStr"/>
       <c r="D82" s="2" t="n">
-        <v>455.0427848274916</v>
+        <v>455.0748040551998</v>
       </c>
       <c r="E82" s="2" t="n">
-        <v>458.53212630562</v>
+        <v>458.7438421848687</v>
       </c>
       <c r="F82" s="2" t="n">
-        <v>460.6914080781864</v>
+        <v>460.9384929530079</v>
       </c>
       <c r="G82" s="2" t="n">
-        <v>462.3222412482408</v>
+        <v>462.6626102681121</v>
       </c>
       <c r="H82" s="2" t="n">
-        <v>463.6529326277467</v>
+        <v>464.0082012350092</v>
       </c>
       <c r="I82" s="2" t="n">
-        <v>464.7411309225139</v>
+        <v>465.0811967823042</v>
       </c>
       <c r="J82" s="2" t="n">
-        <v>465.6208778462529</v>
+        <v>465.9676196840014</v>
       </c>
       <c r="K82" s="2" t="n">
-        <v>466.3341273542305</v>
+        <v>466.6609994820503</v>
       </c>
       <c r="L82" s="2" t="n">
-        <v>466.9342937553715</v>
+        <v>467.2279376337091</v>
       </c>
       <c r="M82" s="2" t="n">
-        <v>467.3958738720804</v>
+        <v>467.6634924923767</v>
       </c>
       <c r="N82" s="2" t="n">
-        <v>467.7481611448815</v>
+        <v>467.9889608220808</v>
       </c>
       <c r="O82" s="2" t="n">
-        <v>468.0650064081697</v>
+        <v>468.2745682991455</v>
       </c>
       <c r="P82" s="2" t="n">
-        <v>468.3166901067456</v>
+        <v>468.4914645249083</v>
       </c>
       <c r="Q82" s="2" t="n">
-        <v>468.51200318471</v>
+        <v>468.6546100479192</v>
       </c>
       <c r="R82" s="2" t="n">
-        <v>468.660793575957</v>
-      </c>
-      <c r="S82" s="2" t="n">
-        <v>468.7633708704671</v>
-      </c>
-      <c r="T82" s="1" t="inlineStr"/>
+        <v>468.7660613130769</v>
+      </c>
+      <c r="S82" s="1" t="inlineStr"/>
     </row>
     <row r="83" ht="15" customHeight="1">
       <c r="A83" s="1" t="inlineStr">
@@ -4893,54 +4690,51 @@
       </c>
       <c r="C83" s="1" t="inlineStr"/>
       <c r="D83" s="2" t="n">
-        <v>0.545117445294531</v>
+        <v>0.5447468172074134</v>
       </c>
       <c r="E83" s="2" t="n">
-        <v>0.5238016754859934</v>
+        <v>0.5225627094398959</v>
       </c>
       <c r="F83" s="2" t="n">
-        <v>0.5142476463595752</v>
+        <v>0.5128242264736803</v>
       </c>
       <c r="G83" s="2" t="n">
-        <v>0.5074868306274732</v>
+        <v>0.5058701247484856</v>
       </c>
       <c r="H83" s="2" t="n">
-        <v>0.5021795948608611</v>
+        <v>0.500517867126743</v>
       </c>
       <c r="I83" s="2" t="n">
-        <v>0.4979545640515015</v>
+        <v>0.4963537393673502</v>
       </c>
       <c r="J83" s="2" t="n">
-        <v>0.4946460319540695</v>
+        <v>0.4931527461005401</v>
       </c>
       <c r="K83" s="2" t="n">
-        <v>0.4921488344697206</v>
+        <v>0.4908656433918407</v>
       </c>
       <c r="L83" s="2" t="n">
-        <v>0.490362746032361</v>
+        <v>0.4893667613005351</v>
       </c>
       <c r="M83" s="2" t="n">
-        <v>0.4892726021734364</v>
+        <v>0.4886103521768771</v>
       </c>
       <c r="N83" s="2" t="n">
-        <v>0.4888074370389106</v>
+        <v>0.4885192069755876</v>
       </c>
       <c r="O83" s="2" t="n">
-        <v>0.4888364884201919</v>
+        <v>0.4889480192746724</v>
       </c>
       <c r="P83" s="2" t="n">
-        <v>0.4893335144998476</v>
+        <v>0.4898496347186731</v>
       </c>
       <c r="Q83" s="2" t="n">
-        <v>0.4902236235746643</v>
+        <v>0.4911141294015546</v>
       </c>
       <c r="R83" s="2" t="n">
-        <v>0.4914178056812916</v>
-      </c>
-      <c r="S83" s="2" t="n">
-        <v>0.4928334965673503</v>
-      </c>
-      <c r="T83" s="1" t="inlineStr"/>
+        <v>0.4926388829310537</v>
+      </c>
+      <c r="S83" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
added fixed nums of dots in export of dots of airfoil
</commit_message>
<xml_diff>
--- a/results/Поступенчатый_расчет_ступеней.xlsx
+++ b/results/Поступенчатый_расчет_ступеней.xlsx
@@ -431,7 +431,7 @@
     <col width="21" customWidth="1" min="5" max="5"/>
     <col width="21" customWidth="1" min="6" max="6"/>
     <col width="21" customWidth="1" min="7" max="7"/>
-    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="21" customWidth="1" min="8" max="8"/>
     <col width="22" customWidth="1" min="9" max="9"/>
     <col width="21" customWidth="1" min="10" max="10"/>
     <col width="22" customWidth="1" min="11" max="11"/>
@@ -439,8 +439,8 @@
     <col width="22" customWidth="1" min="13" max="13"/>
     <col width="22" customWidth="1" min="14" max="14"/>
     <col width="22" customWidth="1" min="15" max="15"/>
-    <col width="22" customWidth="1" min="16" max="16"/>
-    <col width="22" customWidth="1" min="17" max="17"/>
+    <col width="21" customWidth="1" min="16" max="16"/>
+    <col width="21" customWidth="1" min="17" max="17"/>
     <col width="22" customWidth="1" min="18" max="18"/>
     <col width="21" customWidth="1" min="19" max="19"/>
   </cols>
@@ -849,7 +849,7 @@
       <c r="Q11" s="1" t="inlineStr"/>
       <c r="R11" s="1" t="inlineStr"/>
       <c r="S11" s="2" t="n">
-        <v>0.4537118711400231</v>
+        <v>0.4537118711400233</v>
       </c>
     </row>
     <row r="12" ht="15" customHeight="1">
@@ -880,7 +880,7 @@
       <c r="Q12" s="1" t="inlineStr"/>
       <c r="R12" s="1" t="inlineStr"/>
       <c r="S12" s="2" t="n">
-        <v>0.05503600366715333</v>
+        <v>0.05503600366715335</v>
       </c>
     </row>
     <row r="13" ht="15" customHeight="1">
@@ -942,7 +942,7 @@
       <c r="Q14" s="1" t="inlineStr"/>
       <c r="R14" s="1" t="inlineStr"/>
       <c r="S14" s="2" t="n">
-        <v>0.05503600366715333</v>
+        <v>0.05503600366715335</v>
       </c>
     </row>
     <row r="15" ht="15" customHeight="1">
@@ -973,7 +973,7 @@
       <c r="Q15" s="1" t="inlineStr"/>
       <c r="R15" s="1" t="inlineStr"/>
       <c r="S15" s="2" t="n">
-        <v>0.3446443080405253</v>
+        <v>0.3446443080405244</v>
       </c>
     </row>
     <row r="16" ht="15" customHeight="1">
@@ -1004,7 +1004,7 @@
       <c r="Q16" s="1" t="inlineStr"/>
       <c r="R16" s="1" t="inlineStr"/>
       <c r="S16" s="2" t="n">
-        <v>0.5062544510926434</v>
+        <v>0.5062544510926422</v>
       </c>
     </row>
     <row r="17" ht="15" customHeight="1">
@@ -1035,7 +1035,7 @@
       <c r="Q17" s="1" t="inlineStr"/>
       <c r="R17" s="1" t="inlineStr"/>
       <c r="S17" s="2" t="n">
-        <v>0.7925571175792675</v>
+        <v>0.7925571175792671</v>
       </c>
     </row>
     <row r="18" ht="15" customHeight="1">
@@ -1066,7 +1066,7 @@
       <c r="Q18" s="1" t="inlineStr"/>
       <c r="R18" s="1" t="inlineStr"/>
       <c r="S18" s="2" t="n">
-        <v>0.8596778720441994</v>
+        <v>0.8596778720441987</v>
       </c>
     </row>
     <row r="19" ht="15" customHeight="1">
@@ -1097,7 +1097,7 @@
       <c r="Q19" s="1" t="inlineStr"/>
       <c r="R19" s="1" t="inlineStr"/>
       <c r="S19" s="2" t="n">
-        <v>0.7111184547506971</v>
+        <v>0.7111184547506979</v>
       </c>
     </row>
     <row r="20" ht="15" customHeight="1">
@@ -1128,7 +1128,7 @@
       <c r="Q20" s="1" t="inlineStr"/>
       <c r="R20" s="1" t="inlineStr"/>
       <c r="S20" s="2" t="n">
-        <v>141.4703657841591</v>
+        <v>141.4703657841592</v>
       </c>
     </row>
     <row r="21" ht="30" customHeight="1">
@@ -1252,7 +1252,7 @@
       <c r="Q24" s="1" t="inlineStr"/>
       <c r="R24" s="1" t="inlineStr"/>
       <c r="S24" s="2" t="n">
-        <v>0.168064293246209</v>
+        <v>0.1680642932462094</v>
       </c>
     </row>
     <row r="25" ht="30" customHeight="1">
@@ -1681,49 +1681,49 @@
       </c>
       <c r="C32" s="1" t="inlineStr"/>
       <c r="D32" s="2" t="n">
-        <v>16967.12604306373</v>
+        <v>16967.12604306353</v>
       </c>
       <c r="E32" s="2" t="n">
-        <v>18630.78159248007</v>
+        <v>18630.78159247993</v>
       </c>
       <c r="F32" s="2" t="n">
-        <v>20218.5607708968</v>
+        <v>20218.56077089675</v>
       </c>
       <c r="G32" s="2" t="n">
-        <v>21743.63912220311</v>
+        <v>21743.63912220303</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>23213.0501078087</v>
+        <v>23213.05010780867</v>
       </c>
       <c r="I32" s="2" t="n">
-        <v>24632.76848581418</v>
+        <v>24632.76848581409</v>
       </c>
       <c r="J32" s="2" t="n">
-        <v>26002.0239099061</v>
+        <v>26002.02390990612</v>
       </c>
       <c r="K32" s="2" t="n">
         <v>27318.78381964874</v>
       </c>
       <c r="L32" s="2" t="n">
-        <v>28574.47174295057</v>
+        <v>28574.47174295066</v>
       </c>
       <c r="M32" s="2" t="n">
-        <v>29758.48274205851</v>
+        <v>29758.48274205857</v>
       </c>
       <c r="N32" s="2" t="n">
-        <v>30856.11876136259</v>
+        <v>30856.11876136265</v>
       </c>
       <c r="O32" s="2" t="n">
-        <v>31847.15753258983</v>
+        <v>31847.15753258981</v>
       </c>
       <c r="P32" s="2" t="n">
-        <v>32709.42570822144</v>
+        <v>32709.42570822141</v>
       </c>
       <c r="Q32" s="2" t="n">
-        <v>33415.02270248366</v>
+        <v>33415.02270248363</v>
       </c>
       <c r="R32" s="2" t="n">
-        <v>33933.38931404932</v>
+        <v>33933.38931404923</v>
       </c>
       <c r="S32" s="1" t="inlineStr"/>
     </row>
@@ -1740,49 +1740,49 @@
       </c>
       <c r="C33" s="1" t="inlineStr"/>
       <c r="D33" s="2" t="n">
-        <v>16797.45478263309</v>
+        <v>16797.4547826329</v>
       </c>
       <c r="E33" s="2" t="n">
-        <v>18258.16596063047</v>
+        <v>18258.16596063033</v>
       </c>
       <c r="F33" s="2" t="n">
-        <v>19612.0039477699</v>
+        <v>19612.00394776985</v>
       </c>
       <c r="G33" s="2" t="n">
-        <v>20873.89355731498</v>
+        <v>20873.89355731491</v>
       </c>
       <c r="H33" s="2" t="n">
-        <v>22052.39760241826</v>
+        <v>22052.39760241824</v>
       </c>
       <c r="I33" s="2" t="n">
-        <v>23154.80237666533</v>
+        <v>23154.80237666525</v>
       </c>
       <c r="J33" s="2" t="n">
-        <v>24441.90247531174</v>
+        <v>24441.90247531175</v>
       </c>
       <c r="K33" s="2" t="n">
-        <v>25679.65679046981</v>
+        <v>25679.65679046982</v>
       </c>
       <c r="L33" s="2" t="n">
-        <v>26860.00343837353</v>
+        <v>26860.00343837362</v>
       </c>
       <c r="M33" s="2" t="n">
-        <v>27972.97377753499</v>
+        <v>27972.97377753505</v>
       </c>
       <c r="N33" s="2" t="n">
-        <v>29004.75163568083</v>
+        <v>29004.75163568088</v>
       </c>
       <c r="O33" s="2" t="n">
-        <v>29936.32808063443</v>
+        <v>29936.32808063442</v>
       </c>
       <c r="P33" s="2" t="n">
-        <v>30746.86016572815</v>
+        <v>30746.86016572812</v>
       </c>
       <c r="Q33" s="2" t="n">
-        <v>31410.12134033464</v>
+        <v>31410.12134033461</v>
       </c>
       <c r="R33" s="2" t="n">
-        <v>31897.38595520635</v>
+        <v>31897.38595520627</v>
       </c>
       <c r="S33" s="1" t="inlineStr"/>
     </row>
@@ -1799,49 +1799,49 @@
       </c>
       <c r="C34" s="1" t="inlineStr"/>
       <c r="D34" s="2" t="n">
-        <v>13701.87693398603</v>
+        <v>13701.87693398587</v>
       </c>
       <c r="E34" s="2" t="n">
-        <v>15183.18715242576</v>
+        <v>15183.18715242563</v>
       </c>
       <c r="F34" s="2" t="n">
-        <v>16585.02366398544</v>
+        <v>16585.02366398539</v>
       </c>
       <c r="G34" s="2" t="n">
-        <v>17906.52312846286</v>
+        <v>17906.5231284628</v>
       </c>
       <c r="H34" s="2" t="n">
-        <v>19142.33211474175</v>
+        <v>19142.33211474172</v>
       </c>
       <c r="I34" s="2" t="n">
-        <v>20287.40656738138</v>
+        <v>20287.4065673813</v>
       </c>
       <c r="J34" s="2" t="n">
         <v>21560.80915145568</v>
       </c>
       <c r="K34" s="2" t="n">
-        <v>22748.12080720581</v>
+        <v>22748.1208072058</v>
       </c>
       <c r="L34" s="2" t="n">
-        <v>23831.00891765521</v>
+        <v>23831.00891765527</v>
       </c>
       <c r="M34" s="2" t="n">
-        <v>24789.99333265435</v>
+        <v>24789.99333265438</v>
       </c>
       <c r="N34" s="2" t="n">
-        <v>25602.7462639698</v>
+        <v>25602.74626396982</v>
       </c>
       <c r="O34" s="2" t="n">
-        <v>26243.62718943152</v>
+        <v>26243.62718943147</v>
       </c>
       <c r="P34" s="2" t="n">
-        <v>26686.81663025726</v>
+        <v>26686.8166302572</v>
       </c>
       <c r="Q34" s="2" t="n">
-        <v>26904.66888708492</v>
+        <v>26904.66888708486</v>
       </c>
       <c r="R34" s="2" t="n">
-        <v>26870.38869889748</v>
+        <v>26870.38869889738</v>
       </c>
       <c r="S34" s="1" t="inlineStr"/>
     </row>
@@ -1858,49 +1858,49 @@
       </c>
       <c r="C35" s="1" t="inlineStr"/>
       <c r="D35" s="2" t="n">
-        <v>16.6972711556989</v>
+        <v>16.69727115569871</v>
       </c>
       <c r="E35" s="2" t="n">
-        <v>18.08373681547279</v>
+        <v>18.08373681547265</v>
       </c>
       <c r="F35" s="2" t="n">
-        <v>19.35093521240871</v>
+        <v>19.35093521240866</v>
       </c>
       <c r="G35" s="2" t="n">
-        <v>20.56673424835787</v>
+        <v>20.5667342483578</v>
       </c>
       <c r="H35" s="2" t="n">
-        <v>21.65781275498967</v>
+        <v>21.65781275498965</v>
       </c>
       <c r="I35" s="2" t="n">
-        <v>22.64232024894013</v>
+        <v>22.64232024894005</v>
       </c>
       <c r="J35" s="2" t="n">
-        <v>23.81327704394781</v>
+        <v>23.81327704394782</v>
       </c>
       <c r="K35" s="2" t="n">
         <v>24.88456689222609</v>
       </c>
       <c r="L35" s="2" t="n">
-        <v>25.89839154897781</v>
+        <v>25.8983915489779</v>
       </c>
       <c r="M35" s="2" t="n">
-        <v>26.82431759468589</v>
+        <v>26.82431759468595</v>
       </c>
       <c r="N35" s="2" t="n">
-        <v>27.61009078020989</v>
+        <v>27.61009078020994</v>
       </c>
       <c r="O35" s="2" t="n">
-        <v>28.34277284468556</v>
+        <v>28.34277284468554</v>
       </c>
       <c r="P35" s="2" t="n">
-        <v>28.93863549455284</v>
+        <v>28.93863549455281</v>
       </c>
       <c r="Q35" s="2" t="n">
-        <v>29.38971940023348</v>
+        <v>29.38971940023345</v>
       </c>
       <c r="R35" s="2" t="n">
-        <v>29.65175826002295</v>
+        <v>29.65175826002287</v>
       </c>
       <c r="S35" s="1" t="inlineStr"/>
     </row>
@@ -1917,16 +1917,16 @@
       </c>
       <c r="C36" s="1" t="inlineStr"/>
       <c r="D36" s="2" t="n">
-        <v>304.6972711556989</v>
+        <v>304.6972711556987</v>
       </c>
       <c r="E36" s="2" t="n">
-        <v>334.5400980960846</v>
+        <v>334.5400980960845</v>
       </c>
       <c r="F36" s="2" t="n">
-        <v>364.2636577736324</v>
+        <v>364.2636577736323</v>
       </c>
       <c r="G36" s="2" t="n">
-        <v>393.9358180901934</v>
+        <v>393.9358180901933</v>
       </c>
       <c r="H36" s="2" t="n">
         <v>423.4832578774369</v>
@@ -1941,7 +1941,7 @@
         <v>512.0790958565088</v>
       </c>
       <c r="L36" s="2" t="n">
-        <v>541.5492817938723</v>
+        <v>541.5492817938724</v>
       </c>
       <c r="M36" s="2" t="n">
         <v>570.9315691201923</v>
@@ -1976,16 +1976,16 @@
       </c>
       <c r="C37" s="1" t="inlineStr"/>
       <c r="D37" s="2" t="n">
-        <v>304.6972711556989</v>
+        <v>304.6972711556987</v>
       </c>
       <c r="E37" s="2" t="n">
-        <v>334.5400980960846</v>
+        <v>334.5400980960845</v>
       </c>
       <c r="F37" s="2" t="n">
-        <v>364.2636577736324</v>
+        <v>364.2636577736323</v>
       </c>
       <c r="G37" s="2" t="n">
-        <v>393.9358180901934</v>
+        <v>393.9358180901933</v>
       </c>
       <c r="H37" s="2" t="n">
         <v>423.4832578774369</v>
@@ -2000,7 +2000,7 @@
         <v>512.0790958565088</v>
       </c>
       <c r="L37" s="2" t="n">
-        <v>541.5492817938723</v>
+        <v>541.5492817938724</v>
       </c>
       <c r="M37" s="2" t="n">
         <v>570.9315691201923</v>
@@ -2035,22 +2035,22 @@
       </c>
       <c r="C38" s="1" t="inlineStr"/>
       <c r="D38" s="2" t="n">
-        <v>1.175559285399187</v>
+        <v>1.175559285399185</v>
       </c>
       <c r="E38" s="2" t="n">
-        <v>1.177149157361195</v>
+        <v>1.177149157361193</v>
       </c>
       <c r="F38" s="2" t="n">
         <v>1.177580116958397</v>
       </c>
       <c r="G38" s="2" t="n">
-        <v>1.177095915781244</v>
+        <v>1.177095915781243</v>
       </c>
       <c r="H38" s="2" t="n">
-        <v>1.175855347567406</v>
+        <v>1.175855347567405</v>
       </c>
       <c r="I38" s="2" t="n">
-        <v>1.173962116210552</v>
+        <v>1.173962116210551</v>
       </c>
       <c r="J38" s="2" t="n">
         <v>1.173396175963183</v>
@@ -2059,10 +2059,10 @@
         <v>1.172215437821457</v>
       </c>
       <c r="L38" s="2" t="n">
-        <v>1.170376301404517</v>
+        <v>1.170376301404518</v>
       </c>
       <c r="M38" s="2" t="n">
-        <v>1.167847518639031</v>
+        <v>1.167847518639032</v>
       </c>
       <c r="N38" s="2" t="n">
         <v>1.164588351389238</v>
@@ -2074,7 +2074,7 @@
         <v>1.155630506097777</v>
       </c>
       <c r="Q38" s="2" t="n">
-        <v>1.149848870725617</v>
+        <v>1.149848870725616</v>
       </c>
       <c r="R38" s="2" t="n">
         <v>1.143155604508661</v>
@@ -2094,22 +2094,22 @@
       </c>
       <c r="C39" s="1" t="inlineStr"/>
       <c r="D39" s="2" t="n">
-        <v>117900.225235523</v>
+        <v>117900.2252355229</v>
       </c>
       <c r="E39" s="2" t="n">
-        <v>265350.4672140714</v>
+        <v>265350.467214071</v>
       </c>
       <c r="F39" s="2" t="n">
         <v>412792.3261747835</v>
       </c>
       <c r="G39" s="2" t="n">
-        <v>559906.7201888376</v>
+        <v>559906.720188837</v>
       </c>
       <c r="H39" s="2" t="n">
-        <v>706445.5229259076</v>
+        <v>706445.5229259072</v>
       </c>
       <c r="I39" s="2" t="n">
-        <v>852200.0936189106</v>
+        <v>852200.0936189099</v>
       </c>
       <c r="J39" s="2" t="n">
         <v>998610.46481496</v>
@@ -2118,10 +2118,10 @@
         <v>1144279.063503702</v>
       </c>
       <c r="L39" s="2" t="n">
-        <v>1288927.093135038</v>
+        <v>1288927.093135039</v>
       </c>
       <c r="M39" s="2" t="n">
-        <v>1432269.084259004</v>
+        <v>1432269.084259005</v>
       </c>
       <c r="N39" s="2" t="n">
         <v>1573991.10153848</v>
@@ -2130,10 +2130,10 @@
         <v>1713714.468054943</v>
       </c>
       <c r="P39" s="2" t="n">
-        <v>1851080.725235523</v>
+        <v>1851080.725235522</v>
       </c>
       <c r="Q39" s="2" t="n">
-        <v>1985694.583576011</v>
+        <v>1985694.583576009</v>
       </c>
       <c r="R39" s="2" t="n">
         <v>2117173.208233083</v>
@@ -2153,22 +2153,22 @@
       </c>
       <c r="C40" s="1" t="inlineStr"/>
       <c r="D40" s="2" t="n">
-        <v>117900.225235523</v>
+        <v>117900.2252355229</v>
       </c>
       <c r="E40" s="2" t="n">
-        <v>265350.4672140714</v>
+        <v>265350.467214071</v>
       </c>
       <c r="F40" s="2" t="n">
         <v>412792.3261747835</v>
       </c>
       <c r="G40" s="2" t="n">
-        <v>559906.7201888376</v>
+        <v>559906.720188837</v>
       </c>
       <c r="H40" s="2" t="n">
-        <v>706445.5229259076</v>
+        <v>706445.5229259072</v>
       </c>
       <c r="I40" s="2" t="n">
-        <v>852200.0936189106</v>
+        <v>852200.0936189099</v>
       </c>
       <c r="J40" s="2" t="n">
         <v>998610.46481496</v>
@@ -2177,10 +2177,10 @@
         <v>1144279.063503702</v>
       </c>
       <c r="L40" s="2" t="n">
-        <v>1288927.093135038</v>
+        <v>1288927.093135039</v>
       </c>
       <c r="M40" s="2" t="n">
-        <v>1432269.084259004</v>
+        <v>1432269.084259005</v>
       </c>
       <c r="N40" s="2" t="n">
         <v>1573991.10153848</v>
@@ -2189,10 +2189,10 @@
         <v>1713714.468054943</v>
       </c>
       <c r="P40" s="2" t="n">
-        <v>1851080.725235523</v>
+        <v>1851080.725235522</v>
       </c>
       <c r="Q40" s="2" t="n">
-        <v>1985694.583576011</v>
+        <v>1985694.583576009</v>
       </c>
       <c r="R40" s="2" t="n">
         <v>2117173.208233083</v>
@@ -2271,10 +2271,10 @@
       </c>
       <c r="C42" s="1" t="inlineStr"/>
       <c r="D42" s="2" t="n">
-        <v>319.5338237912142</v>
+        <v>319.5338237912141</v>
       </c>
       <c r="E42" s="2" t="n">
-        <v>334.7109771300942</v>
+        <v>334.7109771300941</v>
       </c>
       <c r="F42" s="2" t="n">
         <v>349.222944744292</v>
@@ -2295,7 +2295,7 @@
         <v>413.3312413404398</v>
       </c>
       <c r="L42" s="2" t="n">
-        <v>424.8720601328997</v>
+        <v>424.8720601328998</v>
       </c>
       <c r="M42" s="2" t="n">
         <v>435.9907411935118</v>
@@ -2389,49 +2389,49 @@
       </c>
       <c r="C44" s="1" t="inlineStr"/>
       <c r="D44" s="2" t="n">
-        <v>0.2675658145409672</v>
+        <v>0.2675658145409686</v>
       </c>
       <c r="E44" s="2" t="n">
-        <v>0.2627510762416364</v>
+        <v>0.2627510762416373</v>
       </c>
       <c r="F44" s="2" t="n">
-        <v>0.2591274840795844</v>
+        <v>0.2591274840795847</v>
       </c>
       <c r="G44" s="2" t="n">
-        <v>0.256576799401226</v>
+        <v>0.2565767994012265</v>
       </c>
       <c r="H44" s="2" t="n">
-        <v>0.2550220951838035</v>
+        <v>0.2550220951838037</v>
       </c>
       <c r="I44" s="2" t="n">
-        <v>0.254393016919423</v>
+        <v>0.2543930169194235</v>
       </c>
       <c r="J44" s="2" t="n">
         <v>0.2546621015587227</v>
       </c>
       <c r="K44" s="2" t="n">
-        <v>0.2558078397057248</v>
+        <v>0.2558078397057247</v>
       </c>
       <c r="L44" s="2" t="n">
-        <v>0.2578470068353897</v>
+        <v>0.2578470068353892</v>
       </c>
       <c r="M44" s="2" t="n">
-        <v>0.2608045797416076</v>
+        <v>0.2608045797416072</v>
       </c>
       <c r="N44" s="2" t="n">
-        <v>0.2647254322067381</v>
+        <v>0.2647254322067377</v>
       </c>
       <c r="O44" s="2" t="n">
-        <v>0.2696810959896801</v>
+        <v>0.2696810959896802</v>
       </c>
       <c r="P44" s="2" t="n">
-        <v>0.2757469847403645</v>
+        <v>0.2757469847403647</v>
       </c>
       <c r="Q44" s="2" t="n">
-        <v>0.2830232632486962</v>
+        <v>0.2830232632486964</v>
       </c>
       <c r="R44" s="2" t="n">
-        <v>0.2916156103246133</v>
+        <v>0.2916156103246137</v>
       </c>
       <c r="S44" s="1" t="inlineStr"/>
     </row>
@@ -2448,13 +2448,13 @@
       </c>
       <c r="C45" s="1" t="inlineStr"/>
       <c r="D45" s="2" t="n">
-        <v>1.180296158977294</v>
+        <v>1.180296158977292</v>
       </c>
       <c r="E45" s="2" t="n">
-        <v>1.175262487903347</v>
+        <v>1.175262487903346</v>
       </c>
       <c r="F45" s="2" t="n">
-        <v>1.168251369555617</v>
+        <v>1.168251369555616</v>
       </c>
       <c r="G45" s="2" t="n">
         <v>1.15925817796077</v>
@@ -2463,7 +2463,7 @@
         <v>1.148224245120433</v>
       </c>
       <c r="I45" s="2" t="n">
-        <v>1.135081723832521</v>
+        <v>1.13508172383252</v>
       </c>
       <c r="J45" s="2" t="n">
         <v>1.119697021419855</v>
@@ -2472,10 +2472,10 @@
         <v>1.101922316939652</v>
       </c>
       <c r="L45" s="2" t="n">
-        <v>1.081544540058967</v>
+        <v>1.081544540058968</v>
       </c>
       <c r="M45" s="2" t="n">
-        <v>1.058332062101629</v>
+        <v>1.05833206210163</v>
       </c>
       <c r="N45" s="2" t="n">
         <v>1.032020278583349</v>
@@ -2484,13 +2484,13 @@
         <v>1.0023075858643</v>
       </c>
       <c r="P45" s="2" t="n">
-        <v>0.9689068762009189</v>
+        <v>0.9689068762009185</v>
       </c>
       <c r="Q45" s="2" t="n">
-        <v>0.9315321714560333</v>
+        <v>0.9315321714560331</v>
       </c>
       <c r="R45" s="2" t="n">
-        <v>0.8899613152251319</v>
+        <v>0.8899613152251311</v>
       </c>
       <c r="S45" s="1" t="inlineStr"/>
     </row>
@@ -2566,22 +2566,22 @@
       </c>
       <c r="C47" s="1" t="inlineStr"/>
       <c r="D47" s="2" t="n">
-        <v>0.6934155588636786</v>
+        <v>0.6934155588636791</v>
       </c>
       <c r="E47" s="2" t="n">
-        <v>0.6419546944869913</v>
+        <v>0.6419546944869916</v>
       </c>
       <c r="F47" s="2" t="n">
-        <v>0.5966106211168183</v>
+        <v>0.5966106211168185</v>
       </c>
       <c r="G47" s="2" t="n">
-        <v>0.5561238216798053</v>
+        <v>0.5561238216798055</v>
       </c>
       <c r="H47" s="2" t="n">
         <v>0.5198537807125588</v>
       </c>
       <c r="I47" s="2" t="n">
-        <v>0.4871134947236217</v>
+        <v>0.4871134947236219</v>
       </c>
       <c r="J47" s="2" t="n">
         <v>0.4573452836046674</v>
@@ -2590,13 +2590,13 @@
         <v>0.4302607947475137</v>
       </c>
       <c r="L47" s="2" t="n">
-        <v>0.4054971202086974</v>
+        <v>0.4054971202086972</v>
       </c>
       <c r="M47" s="2" t="n">
-        <v>0.382866877454614</v>
+        <v>0.3828668774546138</v>
       </c>
       <c r="N47" s="2" t="n">
-        <v>0.3622495702925325</v>
+        <v>0.3622495702925324</v>
       </c>
       <c r="O47" s="2" t="n">
         <v>0.3434267211217917</v>
@@ -2605,10 +2605,10 @@
         <v>0.3264013915200195</v>
       </c>
       <c r="Q47" s="2" t="n">
-        <v>0.3111320861419942</v>
+        <v>0.3111320861419943</v>
       </c>
       <c r="R47" s="2" t="n">
-        <v>0.2976385445704193</v>
+        <v>0.2976385445704194</v>
       </c>
       <c r="S47" s="1" t="inlineStr"/>
     </row>
@@ -2625,22 +2625,22 @@
       </c>
       <c r="C48" s="1" t="inlineStr"/>
       <c r="D48" s="2" t="n">
-        <v>0.8876763917513479</v>
+        <v>0.8876763917513484</v>
       </c>
       <c r="E48" s="2" t="n">
-        <v>0.8476827557110529</v>
+        <v>0.8476827557110533</v>
       </c>
       <c r="F48" s="2" t="n">
-        <v>0.807838102390409</v>
+        <v>0.8078381023904093</v>
       </c>
       <c r="G48" s="2" t="n">
-        <v>0.7687303178641441</v>
+        <v>0.7687303178641439</v>
       </c>
       <c r="H48" s="2" t="n">
-        <v>0.7310690251477328</v>
+        <v>0.7310690251477326</v>
       </c>
       <c r="I48" s="2" t="n">
-        <v>0.6950438015492818</v>
+        <v>0.695043801549282</v>
       </c>
       <c r="J48" s="2" t="n">
         <v>0.6606666216532919</v>
@@ -2649,25 +2649,25 @@
         <v>0.6281613417983278</v>
       </c>
       <c r="L48" s="2" t="n">
-        <v>0.5974295303378844</v>
+        <v>0.5974295303378842</v>
       </c>
       <c r="M48" s="2" t="n">
-        <v>0.5685574328276755</v>
+        <v>0.5685574328276751</v>
       </c>
       <c r="N48" s="2" t="n">
-        <v>0.5416626339362809</v>
+        <v>0.5416626339362808</v>
       </c>
       <c r="O48" s="2" t="n">
         <v>0.5165679427658935</v>
       </c>
       <c r="P48" s="2" t="n">
-        <v>0.4934870266617923</v>
+        <v>0.4934870266617922</v>
       </c>
       <c r="Q48" s="2" t="n">
-        <v>0.4724845076896956</v>
+        <v>0.4724845076896957</v>
       </c>
       <c r="R48" s="2" t="n">
-        <v>0.4537118711400231</v>
+        <v>0.4537118711400232</v>
       </c>
       <c r="S48" s="1" t="inlineStr"/>
     </row>
@@ -2684,7 +2684,7 @@
       </c>
       <c r="C49" s="1" t="inlineStr"/>
       <c r="D49" s="2" t="n">
-        <v>0.3009117955899137</v>
+        <v>0.3009117955899138</v>
       </c>
       <c r="E49" s="2" t="n">
         <v>0.1472682986886746</v>
@@ -2693,10 +2693,10 @@
         <v>0.1040512028785386</v>
       </c>
       <c r="G49" s="2" t="n">
-        <v>0.08416531485429166</v>
+        <v>0.08416531485429168</v>
       </c>
       <c r="H49" s="2" t="n">
-        <v>0.07304667532585596</v>
+        <v>0.07304667532585597</v>
       </c>
       <c r="I49" s="2" t="n">
         <v>0.06619932070733821</v>
@@ -2708,7 +2708,7 @@
         <v>0.05890202559086238</v>
       </c>
       <c r="L49" s="2" t="n">
-        <v>0.05707687219159215</v>
+        <v>0.05707687219159214</v>
       </c>
       <c r="M49" s="2" t="n">
         <v>0.05602993268923052</v>
@@ -2720,13 +2720,13 @@
         <v>0.0556712005930268</v>
       </c>
       <c r="P49" s="2" t="n">
-        <v>0.05621043688048771</v>
+        <v>0.05621043688048773</v>
       </c>
       <c r="Q49" s="2" t="n">
         <v>0.05718010096659844</v>
       </c>
       <c r="R49" s="2" t="n">
-        <v>0.05857117009930012</v>
+        <v>0.05857117009930016</v>
       </c>
       <c r="S49" s="1" t="inlineStr"/>
     </row>
@@ -2861,22 +2861,22 @@
       </c>
       <c r="C52" s="1" t="inlineStr"/>
       <c r="D52" s="2" t="n">
-        <v>0.6528609381672205</v>
+        <v>0.652860938167221</v>
       </c>
       <c r="E52" s="2" t="n">
-        <v>0.6040008906918644</v>
+        <v>0.6040008906918648</v>
       </c>
       <c r="F52" s="2" t="n">
-        <v>0.5608528404519376</v>
+        <v>0.5608528404519377</v>
       </c>
       <c r="G52" s="2" t="n">
-        <v>0.5224733005942056</v>
+        <v>0.5224733005942057</v>
       </c>
       <c r="H52" s="2" t="n">
         <v>0.4880639358485558</v>
       </c>
       <c r="I52" s="2" t="n">
-        <v>0.4569203160469202</v>
+        <v>0.4569203160469203</v>
       </c>
       <c r="J52" s="2" t="n">
         <v>0.4285352724020985</v>
@@ -2885,25 +2885,25 @@
         <v>0.4026243969644493</v>
       </c>
       <c r="L52" s="2" t="n">
-        <v>0.3789240751115422</v>
+        <v>0.378924075111542</v>
       </c>
       <c r="M52" s="2" t="n">
-        <v>0.3572719824747077</v>
+        <v>0.3572719824747075</v>
       </c>
       <c r="N52" s="2" t="n">
-        <v>0.3374139715597593</v>
+        <v>0.3374139715597592</v>
       </c>
       <c r="O52" s="2" t="n">
         <v>0.3192848027412507</v>
       </c>
       <c r="P52" s="2" t="n">
-        <v>0.3028179399616254</v>
+        <v>0.3028179399616255</v>
       </c>
       <c r="Q52" s="2" t="n">
-        <v>0.2879901483751846</v>
+        <v>0.2879901483751847</v>
       </c>
       <c r="R52" s="2" t="n">
-        <v>0.2747820638038408</v>
+        <v>0.2747820638038409</v>
       </c>
       <c r="S52" s="1" t="inlineStr"/>
     </row>
@@ -2920,22 +2920,22 @@
       </c>
       <c r="C53" s="1" t="inlineStr"/>
       <c r="D53" s="2" t="n">
-        <v>0.8566449408652137</v>
+        <v>0.856644940865214</v>
       </c>
       <c r="E53" s="2" t="n">
-        <v>0.8146305802312926</v>
+        <v>0.814630580231293</v>
       </c>
       <c r="F53" s="2" t="n">
-        <v>0.7734667621979159</v>
+        <v>0.773466762197916</v>
       </c>
       <c r="G53" s="2" t="n">
-        <v>0.7338759548743808</v>
+        <v>0.733875954874381</v>
       </c>
       <c r="H53" s="2" t="n">
         <v>0.6961191242501733</v>
       </c>
       <c r="I53" s="2" t="n">
-        <v>0.6601638683567802</v>
+        <v>0.6601638683567803</v>
       </c>
       <c r="J53" s="2" t="n">
         <v>0.6260427988521639</v>
@@ -2944,25 +2944,25 @@
         <v>0.5937907596548805</v>
       </c>
       <c r="L53" s="2" t="n">
-        <v>0.5634296976475788</v>
+        <v>0.5634296976475786</v>
       </c>
       <c r="M53" s="2" t="n">
-        <v>0.5350423151502405</v>
+        <v>0.5350423151502401</v>
       </c>
       <c r="N53" s="2" t="n">
-        <v>0.5084161145598954</v>
+        <v>0.5084161145598953</v>
       </c>
       <c r="O53" s="2" t="n">
         <v>0.4836795065578707</v>
       </c>
       <c r="P53" s="2" t="n">
-        <v>0.4608658406019039</v>
+        <v>0.460865840601904</v>
       </c>
       <c r="Q53" s="2" t="n">
-        <v>0.4400685175575864</v>
+        <v>0.4400685175575865</v>
       </c>
       <c r="R53" s="2" t="n">
-        <v>0.4213432296968064</v>
+        <v>0.4213432296968065</v>
       </c>
       <c r="S53" s="1" t="inlineStr"/>
     </row>
@@ -2979,22 +2979,22 @@
       </c>
       <c r="C54" s="1" t="inlineStr"/>
       <c r="D54" s="2" t="n">
-        <v>0.2728264862976837</v>
+        <v>0.2728264862976842</v>
       </c>
       <c r="E54" s="2" t="n">
-        <v>0.1338497572918128</v>
+        <v>0.1338497572918129</v>
       </c>
       <c r="F54" s="2" t="n">
         <v>0.09484023765812551</v>
       </c>
       <c r="G54" s="2" t="n">
-        <v>0.07693362720631663</v>
+        <v>0.07693362720631673</v>
       </c>
       <c r="H54" s="2" t="n">
-        <v>0.0669762425432088</v>
+        <v>0.06697624254320884</v>
       </c>
       <c r="I54" s="2" t="n">
-        <v>0.06091105339602894</v>
+        <v>0.06091105339602899</v>
       </c>
       <c r="J54" s="2" t="n">
         <v>0.05699304098048162</v>
@@ -3003,10 +3003,10 @@
         <v>0.05449766392638357</v>
       </c>
       <c r="L54" s="2" t="n">
-        <v>0.05299351220560669</v>
+        <v>0.05299351220560665</v>
       </c>
       <c r="M54" s="2" t="n">
-        <v>0.05222397695379562</v>
+        <v>0.05222397695379559</v>
       </c>
       <c r="N54" s="2" t="n">
         <v>0.05206385535377919</v>
@@ -3018,10 +3018,10 @@
         <v>0.05326713372110947</v>
       </c>
       <c r="Q54" s="2" t="n">
-        <v>0.05457087868506504</v>
+        <v>0.05457087868506506</v>
       </c>
       <c r="R54" s="2" t="n">
-        <v>0.05635161751966029</v>
+        <v>0.05635161751966031</v>
       </c>
       <c r="S54" s="1" t="inlineStr"/>
     </row>
@@ -3038,16 +3038,16 @@
       </c>
       <c r="C55" s="1" t="inlineStr"/>
       <c r="D55" s="2" t="n">
-        <v>0.5004644049712301</v>
+        <v>0.5004644049712288</v>
       </c>
       <c r="E55" s="2" t="n">
-        <v>0.7951571965663656</v>
+        <v>0.7951571965663653</v>
       </c>
       <c r="F55" s="2" t="n">
         <v>0.8599102873979747</v>
       </c>
       <c r="G55" s="2" t="n">
-        <v>0.8880543221133667</v>
+        <v>0.8880543221133665</v>
       </c>
       <c r="H55" s="2" t="n">
         <v>0.9033251749764167</v>
@@ -3065,7 +3065,7 @@
         <v>0.9243435965300111</v>
       </c>
       <c r="M55" s="2" t="n">
-        <v>0.9254864808911322</v>
+        <v>0.9254864808911323</v>
       </c>
       <c r="N55" s="2" t="n">
         <v>0.9257241100343748</v>
@@ -3080,7 +3080,7 @@
         <v>0.921996524014703</v>
       </c>
       <c r="R55" s="2" t="n">
-        <v>0.9193396390285498</v>
+        <v>0.9193396390285495</v>
       </c>
       <c r="S55" s="1" t="inlineStr"/>
     </row>
@@ -3097,13 +3097,13 @@
       </c>
       <c r="C56" s="1" t="inlineStr"/>
       <c r="D56" s="2" t="n">
-        <v>0.7925571175792675</v>
+        <v>0.7925571175792671</v>
       </c>
       <c r="E56" s="2" t="n">
-        <v>0.9071180477959627</v>
+        <v>0.9071180477959626</v>
       </c>
       <c r="F56" s="2" t="n">
-        <v>0.9358895185677403</v>
+        <v>0.9358895185677402</v>
       </c>
       <c r="G56" s="2" t="n">
         <v>0.948685461697101</v>
@@ -3156,49 +3156,49 @@
       </c>
       <c r="C57" s="1" t="inlineStr"/>
       <c r="D57" s="2" t="n">
-        <v>0.2811863433358084</v>
+        <v>0.2811863433358094</v>
       </c>
       <c r="E57" s="2" t="n">
-        <v>0.3419728067953003</v>
+        <v>0.341972806795301</v>
       </c>
       <c r="F57" s="2" t="n">
-        <v>0.3509410655936228</v>
+        <v>0.350941065593623</v>
       </c>
       <c r="G57" s="2" t="n">
-        <v>0.3505057511486546</v>
+        <v>0.350505751148655</v>
       </c>
       <c r="H57" s="2" t="n">
-        <v>0.3468279629635574</v>
+        <v>0.3468279629635576</v>
       </c>
       <c r="I57" s="2" t="n">
-        <v>0.3417081181479366</v>
+        <v>0.3417081181479371</v>
       </c>
       <c r="J57" s="2" t="n">
         <v>0.3359234221056464</v>
       </c>
       <c r="K57" s="2" t="n">
-        <v>0.3297983277471504</v>
+        <v>0.3297983277471503</v>
       </c>
       <c r="L57" s="2" t="n">
-        <v>0.3235650470477323</v>
+        <v>0.3235650470477318</v>
       </c>
       <c r="M57" s="2" t="n">
-        <v>0.31739063742177</v>
+        <v>0.3173906374217697</v>
       </c>
       <c r="N57" s="2" t="n">
-        <v>0.3114061941828092</v>
+        <v>0.3114061941828089</v>
       </c>
       <c r="O57" s="2" t="n">
-        <v>0.3057573784837125</v>
+        <v>0.3057573784837126</v>
       </c>
       <c r="P57" s="2" t="n">
-        <v>0.3005825024172691</v>
+        <v>0.3005825024172694</v>
       </c>
       <c r="Q57" s="2" t="n">
-        <v>0.2960388638501384</v>
+        <v>0.2960388638501387</v>
       </c>
       <c r="R57" s="2" t="n">
-        <v>0.2922862607409257</v>
+        <v>0.2922862607409261</v>
       </c>
       <c r="S57" s="1" t="inlineStr"/>
     </row>
@@ -3215,7 +3215,7 @@
       </c>
       <c r="C58" s="1" t="inlineStr"/>
       <c r="D58" s="2" t="n">
-        <v>1.150578245989658</v>
+        <v>1.150578245989657</v>
       </c>
       <c r="E58" s="2" t="n">
         <v>1.058842137058633</v>
@@ -3224,13 +3224,13 @@
         <v>1.03259772936633</v>
       </c>
       <c r="G58" s="2" t="n">
-        <v>1.017231933919797</v>
+        <v>1.017231933919796</v>
       </c>
       <c r="H58" s="2" t="n">
-        <v>1.005239401872601</v>
+        <v>1.0052394018726</v>
       </c>
       <c r="I58" s="2" t="n">
-        <v>0.9944293535476197</v>
+        <v>0.9944293535476192</v>
       </c>
       <c r="J58" s="2" t="n">
         <v>0.9838133341616834</v>
@@ -3239,25 +3239,25 @@
         <v>0.9729365229403433</v>
       </c>
       <c r="L58" s="2" t="n">
-        <v>0.9614252343707766</v>
+        <v>0.9614252343707773</v>
       </c>
       <c r="M58" s="2" t="n">
-        <v>0.9489575905895593</v>
+        <v>0.9489575905895599</v>
       </c>
       <c r="N58" s="2" t="n">
-        <v>0.9352269846819268</v>
+        <v>0.9352269846819273</v>
       </c>
       <c r="O58" s="2" t="n">
-        <v>0.9198661432115165</v>
+        <v>0.9198661432115164</v>
       </c>
       <c r="P58" s="2" t="n">
-        <v>0.9024768235733482</v>
+        <v>0.9024768235733479</v>
       </c>
       <c r="Q58" s="2" t="n">
-        <v>0.8825869545836461</v>
+        <v>0.8825869545836458</v>
       </c>
       <c r="R58" s="2" t="n">
-        <v>0.8596778720441994</v>
+        <v>0.8596778720441987</v>
       </c>
       <c r="S58" s="1" t="inlineStr"/>
     </row>
@@ -3274,22 +3274,22 @@
       </c>
       <c r="C59" s="1" t="inlineStr"/>
       <c r="D59" s="2" t="n">
-        <v>0.6612407210601744</v>
+        <v>0.6612407210601751</v>
       </c>
       <c r="E59" s="2" t="n">
-        <v>0.6393366808686474</v>
+        <v>0.6393366808686478</v>
       </c>
       <c r="F59" s="2" t="n">
-        <v>0.6009807379947486</v>
+        <v>0.6009807379947487</v>
       </c>
       <c r="G59" s="2" t="n">
-        <v>0.5629187482016862</v>
+        <v>0.5629187482016864</v>
       </c>
       <c r="H59" s="2" t="n">
-        <v>0.5272267598629743</v>
+        <v>0.5272267598629744</v>
       </c>
       <c r="I59" s="2" t="n">
-        <v>0.4940432659250179</v>
+        <v>0.4940432659250182</v>
       </c>
       <c r="J59" s="2" t="n">
         <v>0.4632008778470891</v>
@@ -3298,13 +3298,13 @@
         <v>0.434547983835321</v>
       </c>
       <c r="L59" s="2" t="n">
-        <v>0.4078868049211564</v>
+        <v>0.4078868049211561</v>
       </c>
       <c r="M59" s="2" t="n">
-        <v>0.3830869581536965</v>
+        <v>0.3830869581536963</v>
       </c>
       <c r="N59" s="2" t="n">
-        <v>0.3598891790707875</v>
+        <v>0.3598891790707873</v>
       </c>
       <c r="O59" s="2" t="n">
         <v>0.3382266797622753</v>
@@ -3313,10 +3313,10 @@
         <v>0.3180205486364964</v>
       </c>
       <c r="Q59" s="2" t="n">
-        <v>0.2992319827470267</v>
+        <v>0.2992319827470268</v>
       </c>
       <c r="R59" s="2" t="n">
-        <v>0.2818236131273244</v>
+        <v>0.2818236131273246</v>
       </c>
       <c r="S59" s="1" t="inlineStr"/>
     </row>
@@ -3333,22 +3333,22 @@
       </c>
       <c r="C60" s="1" t="inlineStr"/>
       <c r="D60" s="2" t="n">
-        <v>0.2707047831582408</v>
+        <v>0.2707047831582413</v>
       </c>
       <c r="E60" s="2" t="n">
-        <v>0.1289535490674906</v>
+        <v>0.1289535490674907</v>
       </c>
       <c r="F60" s="2" t="n">
-        <v>0.09035121456081503</v>
+        <v>0.09035121456081506</v>
       </c>
       <c r="G60" s="2" t="n">
-        <v>0.07279583956722309</v>
+        <v>0.07279583956722319</v>
       </c>
       <c r="H60" s="2" t="n">
-        <v>0.0630871303195517</v>
+        <v>0.06308713031955175</v>
       </c>
       <c r="I60" s="2" t="n">
-        <v>0.0572051495289134</v>
+        <v>0.05720514952891342</v>
       </c>
       <c r="J60" s="2" t="n">
         <v>0.05343833731776829</v>
@@ -3357,13 +3357,13 @@
         <v>0.05108008787467855</v>
       </c>
       <c r="L60" s="2" t="n">
-        <v>0.04971625102356635</v>
+        <v>0.04971625102356633</v>
       </c>
       <c r="M60" s="2" t="n">
-        <v>0.04910680533129995</v>
+        <v>0.04910680533129991</v>
       </c>
       <c r="N60" s="2" t="n">
-        <v>0.04914211499311783</v>
+        <v>0.04914211499311785</v>
       </c>
       <c r="O60" s="2" t="n">
         <v>0.04975559312298664</v>
@@ -3372,10 +3372,10 @@
         <v>0.0509264267870588</v>
       </c>
       <c r="Q60" s="2" t="n">
-        <v>0.05266952243484315</v>
+        <v>0.05266952243484317</v>
       </c>
       <c r="R60" s="2" t="n">
-        <v>0.05503600366715333</v>
+        <v>0.05503600366715335</v>
       </c>
       <c r="S60" s="1" t="inlineStr"/>
     </row>
@@ -3392,19 +3392,19 @@
       </c>
       <c r="C61" s="1" t="inlineStr"/>
       <c r="D61" s="2" t="n">
-        <v>0.1289535490674906</v>
+        <v>0.1289535490674907</v>
       </c>
       <c r="E61" s="2" t="n">
-        <v>0.09035121456081503</v>
+        <v>0.09035121456081506</v>
       </c>
       <c r="F61" s="2" t="n">
-        <v>0.07279583956722309</v>
+        <v>0.07279583956722319</v>
       </c>
       <c r="G61" s="2" t="n">
-        <v>0.0630871303195517</v>
+        <v>0.06308713031955175</v>
       </c>
       <c r="H61" s="2" t="n">
-        <v>0.0572051495289134</v>
+        <v>0.05720514952891342</v>
       </c>
       <c r="I61" s="2" t="n">
         <v>0.05343833731776829</v>
@@ -3413,13 +3413,13 @@
         <v>0.05108008787467855</v>
       </c>
       <c r="K61" s="2" t="n">
-        <v>0.04971625102356635</v>
+        <v>0.04971625102356633</v>
       </c>
       <c r="L61" s="2" t="n">
-        <v>0.04910680533129995</v>
+        <v>0.04910680533129991</v>
       </c>
       <c r="M61" s="2" t="n">
-        <v>0.04914211499311783</v>
+        <v>0.04914211499311785</v>
       </c>
       <c r="N61" s="2" t="n">
         <v>0.04975559312298664</v>
@@ -3428,13 +3428,13 @@
         <v>0.0509264267870588</v>
       </c>
       <c r="P61" s="2" t="n">
-        <v>0.05266952243484315</v>
+        <v>0.05266952243484317</v>
       </c>
       <c r="Q61" s="2" t="n">
-        <v>0.05503600366715333</v>
+        <v>0.05503600366715335</v>
       </c>
       <c r="R61" s="2" t="n">
-        <v>0.05740248489946351</v>
+        <v>0.05740248489946354</v>
       </c>
       <c r="S61" s="1" t="inlineStr"/>
     </row>
@@ -3451,16 +3451,16 @@
       </c>
       <c r="C62" s="1" t="inlineStr"/>
       <c r="D62" s="2" t="n">
-        <v>0.5062544510926434</v>
+        <v>0.5062544510926422</v>
       </c>
       <c r="E62" s="2" t="n">
-        <v>0.8035709709007146</v>
+        <v>0.8035709709007143</v>
       </c>
       <c r="F62" s="2" t="n">
-        <v>0.8670515451401452</v>
+        <v>0.8670515451401449</v>
       </c>
       <c r="G62" s="2" t="n">
-        <v>0.8944317807808952</v>
+        <v>0.8944317807808951</v>
       </c>
       <c r="H62" s="2" t="n">
         <v>0.9092199502745679</v>
@@ -3510,13 +3510,13 @@
       </c>
       <c r="C63" s="1" t="inlineStr"/>
       <c r="D63" s="2" t="n">
-        <v>0.781132427160474</v>
+        <v>0.7811324271604738</v>
       </c>
       <c r="E63" s="2" t="n">
-        <v>0.8434383830980788</v>
+        <v>0.8434383830980787</v>
       </c>
       <c r="F63" s="2" t="n">
-        <v>0.8631690556287381</v>
+        <v>0.863169055628738</v>
       </c>
       <c r="G63" s="2" t="n">
         <v>0.8752186331837397</v>
@@ -3569,49 +3569,49 @@
       </c>
       <c r="C64" s="1" t="inlineStr"/>
       <c r="D64" s="2" t="n">
-        <v>0.4947976924542986</v>
+        <v>0.4947976924542974</v>
       </c>
       <c r="E64" s="2" t="n">
-        <v>0.4779735242447286</v>
+        <v>0.4779735242447278</v>
       </c>
       <c r="F64" s="2" t="n">
-        <v>0.4865582469952273</v>
+        <v>0.486558246995227</v>
       </c>
       <c r="G64" s="2" t="n">
-        <v>0.4994124070984718</v>
+        <v>0.4994124070984713</v>
       </c>
       <c r="H64" s="2" t="n">
         <v>0.5137734390610369</v>
       </c>
       <c r="I64" s="2" t="n">
-        <v>0.5288702372127254</v>
+        <v>0.5288702372127249</v>
       </c>
       <c r="J64" s="2" t="n">
-        <v>0.5443607442121166</v>
+        <v>0.5443607442121167</v>
       </c>
       <c r="K64" s="2" t="n">
         <v>0.5600965560548041</v>
       </c>
       <c r="L64" s="2" t="n">
-        <v>0.5759477597191387</v>
+        <v>0.5759477597191393</v>
       </c>
       <c r="M64" s="2" t="n">
-        <v>0.5918081993459784</v>
+        <v>0.5918081993459788</v>
       </c>
       <c r="N64" s="2" t="n">
-        <v>0.6075771359846209</v>
+        <v>0.6075771359846212</v>
       </c>
       <c r="O64" s="2" t="n">
-        <v>0.6231339534389799</v>
+        <v>0.6231339534389797</v>
       </c>
       <c r="P64" s="2" t="n">
-        <v>0.6383608968284006</v>
+        <v>0.6383608968284005</v>
       </c>
       <c r="Q64" s="2" t="n">
-        <v>0.6531207208541026</v>
+        <v>0.6531207208541023</v>
       </c>
       <c r="R64" s="2" t="n">
-        <v>0.6672755281010996</v>
+        <v>0.6672755281010991</v>
       </c>
       <c r="S64" s="1" t="inlineStr"/>
     </row>
@@ -3628,22 +3628,22 @@
       </c>
       <c r="C65" s="1" t="inlineStr"/>
       <c r="D65" s="2" t="n">
-        <v>0.9130337357818</v>
+        <v>0.9130337357818012</v>
       </c>
       <c r="E65" s="2" t="n">
-        <v>0.8830355266498334</v>
+        <v>0.8830355266498343</v>
       </c>
       <c r="F65" s="2" t="n">
-        <v>0.8530645253444216</v>
+        <v>0.8530645253444218</v>
       </c>
       <c r="G65" s="2" t="n">
-        <v>0.8230510799514991</v>
+        <v>0.8230510799514995</v>
       </c>
       <c r="H65" s="2" t="n">
-        <v>0.7929681334991677</v>
+        <v>0.7929681334991679</v>
       </c>
       <c r="I65" s="2" t="n">
-        <v>0.7627977092904863</v>
+        <v>0.7627977092904867</v>
       </c>
       <c r="J65" s="2" t="n">
         <v>0.7325616461288711</v>
@@ -3652,25 +3652,25 @@
         <v>0.7022863254977531</v>
       </c>
       <c r="L65" s="2" t="n">
-        <v>0.6720276223556498</v>
+        <v>0.6720276223556494</v>
       </c>
       <c r="M65" s="2" t="n">
-        <v>0.6418422361217935</v>
+        <v>0.6418422361217931</v>
       </c>
       <c r="N65" s="2" t="n">
-        <v>0.611794636858556</v>
+        <v>0.6117946368585556</v>
       </c>
       <c r="O65" s="2" t="n">
         <v>0.5819584578441279</v>
       </c>
       <c r="P65" s="2" t="n">
-        <v>0.552396365214525</v>
+        <v>0.5523963652145252</v>
       </c>
       <c r="Q65" s="2" t="n">
-        <v>0.5231726932408487</v>
+        <v>0.5231726932408488</v>
       </c>
       <c r="R65" s="2" t="n">
-        <v>0.4943374292495647</v>
+        <v>0.494337429249565</v>
       </c>
       <c r="S65" s="1" t="inlineStr"/>
     </row>
@@ -3746,49 +3746,49 @@
       </c>
       <c r="C67" s="1" t="inlineStr"/>
       <c r="D67" s="2" t="n">
-        <v>1.149900190948778</v>
+        <v>1.149900190948777</v>
       </c>
       <c r="E67" s="2" t="n">
-        <v>1.037406335378524</v>
+        <v>1.037406335378523</v>
       </c>
       <c r="F67" s="2" t="n">
         <v>1.008925798296564</v>
       </c>
       <c r="G67" s="2" t="n">
-        <v>0.9938963560643232</v>
+        <v>0.9938963560643226</v>
       </c>
       <c r="H67" s="2" t="n">
         <v>0.9831646987246834</v>
       </c>
       <c r="I67" s="2" t="n">
-        <v>0.9741269377820952</v>
+        <v>0.9741269377820945</v>
       </c>
       <c r="J67" s="2" t="n">
-        <v>0.9656506714457721</v>
+        <v>0.9656506714457722</v>
       </c>
       <c r="K67" s="2" t="n">
         <v>0.9572427390595025</v>
       </c>
       <c r="L67" s="2" t="n">
-        <v>0.9485264056880329</v>
+        <v>0.9485264056880337</v>
       </c>
       <c r="M67" s="2" t="n">
-        <v>0.9392010422085477</v>
+        <v>0.9392010422085484</v>
       </c>
       <c r="N67" s="2" t="n">
-        <v>0.9290023750862315</v>
+        <v>0.9290023750862318</v>
       </c>
       <c r="O67" s="2" t="n">
-        <v>0.9176220242343975</v>
+        <v>0.9176220242343971</v>
       </c>
       <c r="P67" s="2" t="n">
-        <v>0.9047385458666748</v>
+        <v>0.9047385458666746</v>
       </c>
       <c r="Q67" s="2" t="n">
-        <v>0.8899750486647011</v>
+        <v>0.8899750486647007</v>
       </c>
       <c r="R67" s="2" t="n">
-        <v>0.8729257643027138</v>
+        <v>0.872925764302713</v>
       </c>
       <c r="S67" s="1" t="inlineStr"/>
     </row>
@@ -3805,22 +3805,22 @@
       </c>
       <c r="C68" s="1" t="inlineStr"/>
       <c r="D68" s="2" t="n">
-        <v>0.9123908734224122</v>
+        <v>0.9123908734224133</v>
       </c>
       <c r="E68" s="2" t="n">
-        <v>0.9132006195531562</v>
+        <v>0.9132006195531571</v>
       </c>
       <c r="F68" s="2" t="n">
-        <v>0.887967323159673</v>
+        <v>0.8879673231596732</v>
       </c>
       <c r="G68" s="2" t="n">
-        <v>0.8577821070040713</v>
+        <v>0.8577821070040718</v>
       </c>
       <c r="H68" s="2" t="n">
         <v>0.8255539583207618</v>
       </c>
       <c r="I68" s="2" t="n">
-        <v>0.792160112745544</v>
+        <v>0.7921601127455445</v>
       </c>
       <c r="J68" s="2" t="n">
         <v>0.7580358219315676</v>
@@ -3829,25 +3829,25 @@
         <v>0.72342089195214</v>
       </c>
       <c r="L68" s="2" t="n">
-        <v>0.6885297165190225</v>
+        <v>0.6885297165190221</v>
       </c>
       <c r="M68" s="2" t="n">
-        <v>0.6535447189435526</v>
+        <v>0.6535447189435523</v>
       </c>
       <c r="N68" s="2" t="n">
-        <v>0.6186306556226798</v>
+        <v>0.6186306556226797</v>
       </c>
       <c r="O68" s="2" t="n">
-        <v>0.5839510578580409</v>
+        <v>0.583951057858041</v>
       </c>
       <c r="P68" s="2" t="n">
-        <v>0.5496458774495508</v>
+        <v>0.549645877449551</v>
       </c>
       <c r="Q68" s="2" t="n">
-        <v>0.5158449565439994</v>
+        <v>0.5158449565439995</v>
       </c>
       <c r="R68" s="2" t="n">
-        <v>0.4826515564353129</v>
+        <v>0.4826515564353131</v>
       </c>
       <c r="S68" s="1" t="inlineStr"/>
     </row>
@@ -3864,49 +3864,49 @@
       </c>
       <c r="C69" s="1" t="inlineStr"/>
       <c r="D69" s="2" t="n">
-        <v>0.236866455166978</v>
+        <v>0.2368664551669755</v>
       </c>
       <c r="E69" s="2" t="n">
-        <v>0.1543708087286905</v>
+        <v>0.1543708087286889</v>
       </c>
       <c r="F69" s="2" t="n">
-        <v>0.1558612729521429</v>
+        <v>0.1558612729521425</v>
       </c>
       <c r="G69" s="2" t="n">
-        <v>0.1708452761128242</v>
+        <v>0.1708452761128231</v>
       </c>
       <c r="H69" s="2" t="n">
-        <v>0.1901965652255156</v>
+        <v>0.1901965652255154</v>
       </c>
       <c r="I69" s="2" t="n">
-        <v>0.211329228491609</v>
+        <v>0.2113292284916077</v>
       </c>
       <c r="J69" s="2" t="n">
-        <v>0.233089025316901</v>
+        <v>0.2330890253169011</v>
       </c>
       <c r="K69" s="2" t="n">
         <v>0.2549564135617495</v>
       </c>
       <c r="L69" s="2" t="n">
-        <v>0.2764987833323831</v>
+        <v>0.2764987833323843</v>
       </c>
       <c r="M69" s="2" t="n">
-        <v>0.2973588060867542</v>
+        <v>0.2973588060867552</v>
       </c>
       <c r="N69" s="2" t="n">
-        <v>0.3172077382276756</v>
+        <v>0.3172077382276762</v>
       </c>
       <c r="O69" s="2" t="n">
-        <v>0.3356635663902696</v>
+        <v>0.3356635663902692</v>
       </c>
       <c r="P69" s="2" t="n">
-        <v>0.3523421806521498</v>
+        <v>0.3523421806521494</v>
       </c>
       <c r="Q69" s="2" t="n">
-        <v>0.3668023554238524</v>
+        <v>0.3668023554238519</v>
       </c>
       <c r="R69" s="2" t="n">
-        <v>0.3785883350531491</v>
+        <v>0.3785883350531479</v>
       </c>
       <c r="S69" s="1" t="inlineStr"/>
     </row>
@@ -3923,22 +3923,22 @@
       </c>
       <c r="C70" s="1" t="inlineStr"/>
       <c r="D70" s="2" t="n">
-        <v>0.2381873725672461</v>
+        <v>0.2381873725672434</v>
       </c>
       <c r="E70" s="2" t="n">
-        <v>0.1456415175054772</v>
+        <v>0.1456415175054754</v>
       </c>
       <c r="F70" s="2" t="n">
-        <v>0.1446304062066568</v>
+        <v>0.1446304062066563</v>
       </c>
       <c r="G70" s="2" t="n">
-        <v>0.1594498269157253</v>
+        <v>0.1594498269157244</v>
       </c>
       <c r="H70" s="2" t="n">
-        <v>0.1796854435518387</v>
+        <v>0.1796854435518385</v>
       </c>
       <c r="I70" s="2" t="n">
-        <v>0.2022692408020758</v>
+        <v>0.2022692408020746</v>
       </c>
       <c r="J70" s="2" t="n">
         <v>0.2257775122301158</v>
@@ -3947,25 +3947,25 @@
         <v>0.2495156309882033</v>
       </c>
       <c r="L70" s="2" t="n">
-        <v>0.2728955178517541</v>
+        <v>0.2728955178517553</v>
       </c>
       <c r="M70" s="2" t="n">
-        <v>0.2954128716460067</v>
+        <v>0.2954128716460076</v>
       </c>
       <c r="N70" s="2" t="n">
-        <v>0.316596329059247</v>
+        <v>0.3165963290592476</v>
       </c>
       <c r="O70" s="2" t="n">
-        <v>0.3359150853534756</v>
+        <v>0.3359150853534754</v>
       </c>
       <c r="P70" s="2" t="n">
-        <v>0.3528309461237974</v>
+        <v>0.352830946123797</v>
       </c>
       <c r="Q70" s="2" t="n">
-        <v>0.3667419980396467</v>
+        <v>0.3667419980396462</v>
       </c>
       <c r="R70" s="2" t="n">
-        <v>0.3770263156088866</v>
+        <v>0.3770263156088856</v>
       </c>
       <c r="S70" s="1" t="inlineStr"/>
     </row>
@@ -3982,22 +3982,22 @@
       </c>
       <c r="C71" s="1" t="inlineStr"/>
       <c r="D71" s="2" t="n">
-        <v>251.7894146864385</v>
+        <v>251.7894146864383</v>
       </c>
       <c r="E71" s="2" t="n">
-        <v>249.6625952542775</v>
+        <v>249.6625952542773</v>
       </c>
       <c r="F71" s="2" t="n">
-        <v>247.6528107706313</v>
+        <v>247.6528107706312</v>
       </c>
       <c r="G71" s="2" t="n">
-        <v>245.7731838000793</v>
+        <v>245.7731838000792</v>
       </c>
       <c r="H71" s="2" t="n">
         <v>244.0304158041251</v>
       </c>
       <c r="I71" s="2" t="n">
-        <v>242.4310417988148</v>
+        <v>242.4310417988147</v>
       </c>
       <c r="J71" s="2" t="n">
         <v>240.972909827971</v>
@@ -4006,25 +4006,25 @@
         <v>239.6524840515102</v>
       </c>
       <c r="L71" s="2" t="n">
-        <v>238.4569611637397</v>
+        <v>238.4569611637399</v>
       </c>
       <c r="M71" s="2" t="n">
-        <v>237.3706330162411</v>
+        <v>237.3706330162412</v>
       </c>
       <c r="N71" s="2" t="n">
-        <v>236.3718770966746</v>
+        <v>236.3718770966747</v>
       </c>
       <c r="O71" s="2" t="n">
         <v>235.4310839272837</v>
       </c>
       <c r="P71" s="2" t="n">
-        <v>234.5161748631908</v>
+        <v>234.5161748631907</v>
       </c>
       <c r="Q71" s="2" t="n">
         <v>233.5872660970408</v>
       </c>
       <c r="R71" s="2" t="n">
-        <v>232.6016263665796</v>
+        <v>232.6016263665795</v>
       </c>
       <c r="S71" s="1" t="inlineStr"/>
     </row>
@@ -4100,22 +4100,22 @@
       </c>
       <c r="C73" s="1" t="inlineStr"/>
       <c r="D73" s="2" t="n">
-        <v>247.9005511003574</v>
+        <v>247.9005511003572</v>
       </c>
       <c r="E73" s="2" t="n">
-        <v>239.722425110993</v>
+        <v>239.7224251109928</v>
       </c>
       <c r="F73" s="2" t="n">
         <v>236.3804261005702</v>
       </c>
       <c r="G73" s="2" t="n">
-        <v>234.0471923727898</v>
+        <v>234.0471923727897</v>
       </c>
       <c r="H73" s="2" t="n">
         <v>232.2443952114634</v>
       </c>
       <c r="I73" s="2" t="n">
-        <v>230.8447911323391</v>
+        <v>230.844791132339</v>
       </c>
       <c r="J73" s="2" t="n">
         <v>229.7932112410973</v>
@@ -4124,10 +4124,10 @@
         <v>229.0678517566361</v>
       </c>
       <c r="L73" s="2" t="n">
-        <v>228.6458226289366</v>
+        <v>228.6458226289367</v>
       </c>
       <c r="M73" s="2" t="n">
-        <v>228.5052237669685</v>
+        <v>228.5052237669686</v>
       </c>
       <c r="N73" s="2" t="n">
         <v>228.6215960141323</v>
@@ -4142,7 +4142,7 @@
         <v>230.1629008037089</v>
       </c>
       <c r="R73" s="2" t="n">
-        <v>230.932388801264</v>
+        <v>230.9323888012639</v>
       </c>
       <c r="S73" s="1" t="inlineStr"/>
     </row>
@@ -4159,7 +4159,7 @@
       </c>
       <c r="C74" s="1" t="inlineStr"/>
       <c r="D74" s="2" t="n">
-        <v>0.9198717705829682</v>
+        <v>0.9198717705829681</v>
       </c>
       <c r="E74" s="2" t="n">
         <v>0.9316127880691234</v>
@@ -4168,7 +4168,7 @@
         <v>0.9411937231993717</v>
       </c>
       <c r="G74" s="2" t="n">
-        <v>0.9489889140291673</v>
+        <v>0.9489889140291672</v>
       </c>
       <c r="H74" s="2" t="n">
         <v>0.9555931563290563</v>
@@ -4183,25 +4183,25 @@
         <v>0.9700508464641263</v>
       </c>
       <c r="L74" s="2" t="n">
-        <v>0.9735532872138978</v>
+        <v>0.9735532872138979</v>
       </c>
       <c r="M74" s="2" t="n">
         <v>0.9765720654514889</v>
       </c>
       <c r="N74" s="2" t="n">
-        <v>0.9792051916840198</v>
+        <v>0.9792051916840199</v>
       </c>
       <c r="O74" s="2" t="n">
         <v>0.9814270687200961</v>
       </c>
       <c r="P74" s="2" t="n">
-        <v>0.9833372387193101</v>
+        <v>0.98333723871931</v>
       </c>
       <c r="Q74" s="2" t="n">
         <v>0.9849622306534793</v>
       </c>
       <c r="R74" s="2" t="n">
-        <v>0.9863414798135992</v>
+        <v>0.9863414798135991</v>
       </c>
       <c r="S74" s="1" t="inlineStr"/>
     </row>
@@ -4218,7 +4218,7 @@
       </c>
       <c r="C75" s="1" t="inlineStr"/>
       <c r="D75" s="2" t="n">
-        <v>264.9230699278949</v>
+        <v>264.9230699278948</v>
       </c>
       <c r="E75" s="2" t="n">
         <v>294.8147930348406</v>
@@ -4254,13 +4254,13 @@
         <v>589.8572714101675</v>
       </c>
       <c r="P75" s="2" t="n">
-        <v>618.9875214592724</v>
+        <v>618.9875214592723</v>
       </c>
       <c r="Q75" s="2" t="n">
         <v>648.0388565102273</v>
       </c>
       <c r="R75" s="2" t="n">
-        <v>677.0139991251236</v>
+        <v>677.0139991251235</v>
       </c>
       <c r="S75" s="1" t="inlineStr"/>
     </row>
@@ -4336,22 +4336,22 @@
       </c>
       <c r="C77" s="1" t="inlineStr"/>
       <c r="D77" s="2" t="n">
-        <v>0.8448204141343578</v>
+        <v>0.8448204141343573</v>
       </c>
       <c r="E77" s="2" t="n">
-        <v>0.7943214505742267</v>
+        <v>0.7943214505742261</v>
       </c>
       <c r="F77" s="2" t="n">
-        <v>0.7511095390711756</v>
+        <v>0.7511095390711755</v>
       </c>
       <c r="G77" s="2" t="n">
-        <v>0.7135754513445642</v>
+        <v>0.7135754513445639</v>
       </c>
       <c r="H77" s="2" t="n">
-        <v>0.6807840523057973</v>
+        <v>0.6807840523057971</v>
       </c>
       <c r="I77" s="2" t="n">
-        <v>0.651895609766268</v>
+        <v>0.6518956097662678</v>
       </c>
       <c r="J77" s="2" t="n">
         <v>0.6262006800178096</v>
@@ -4360,25 +4360,25 @@
         <v>0.6032931870271456</v>
       </c>
       <c r="L77" s="2" t="n">
-        <v>0.582669850624871</v>
+        <v>0.5826698506248713</v>
       </c>
       <c r="M77" s="2" t="n">
-        <v>0.5640185684375758</v>
+        <v>0.5640185684375761</v>
       </c>
       <c r="N77" s="2" t="n">
-        <v>0.5470938594252941</v>
+        <v>0.5470938594252943</v>
       </c>
       <c r="O77" s="2" t="n">
-        <v>0.5314851030679409</v>
+        <v>0.5314851030679412</v>
       </c>
       <c r="P77" s="2" t="n">
-        <v>0.5170517482371183</v>
+        <v>0.5170517482371181</v>
       </c>
       <c r="Q77" s="2" t="n">
-        <v>0.5035581698659797</v>
+        <v>0.5035581698659796</v>
       </c>
       <c r="R77" s="2" t="n">
-        <v>0.4908332230905137</v>
+        <v>0.4908332230905135</v>
       </c>
       <c r="S77" s="1" t="inlineStr"/>
     </row>
@@ -4395,22 +4395,22 @@
       </c>
       <c r="C78" s="1" t="inlineStr"/>
       <c r="D78" s="2" t="n">
-        <v>0.7758194364498247</v>
+        <v>0.7758194364498243</v>
       </c>
       <c r="E78" s="2" t="n">
-        <v>0.7162072399490459</v>
+        <v>0.7162072399490456</v>
       </c>
       <c r="F78" s="2" t="n">
-        <v>0.6768754162864432</v>
+        <v>0.6768754162864431</v>
       </c>
       <c r="G78" s="2" t="n">
-        <v>0.6446312378490995</v>
+        <v>0.6446312378490993</v>
       </c>
       <c r="H78" s="2" t="n">
         <v>0.6171656544030198</v>
       </c>
       <c r="I78" s="2" t="n">
-        <v>0.5933516387160817</v>
+        <v>0.5933516387160813</v>
       </c>
       <c r="J78" s="2" t="n">
         <v>0.5724800026430085</v>
@@ -4419,13 +4419,13 @@
         <v>0.5541992204938717</v>
       </c>
       <c r="L78" s="2" t="n">
-        <v>0.5381521735211686</v>
+        <v>0.5381521735211688</v>
       </c>
       <c r="M78" s="2" t="n">
-        <v>0.5241056797248543</v>
+        <v>0.5241056797248544</v>
       </c>
       <c r="N78" s="2" t="n">
-        <v>0.5116577227873375</v>
+        <v>0.5116577227873376</v>
       </c>
       <c r="O78" s="2" t="n">
         <v>0.5006277313683627</v>
@@ -4434,10 +4434,10 @@
         <v>0.4908125161156869</v>
       </c>
       <c r="Q78" s="2" t="n">
-        <v>0.4820311420268309</v>
+        <v>0.4820311420268308</v>
       </c>
       <c r="R78" s="2" t="n">
-        <v>0.474084587425221</v>
+        <v>0.4740845874252208</v>
       </c>
       <c r="S78" s="1" t="inlineStr"/>
     </row>
@@ -4454,16 +4454,16 @@
       </c>
       <c r="C79" s="1" t="inlineStr"/>
       <c r="D79" s="2" t="n">
-        <v>304.6972711556989</v>
+        <v>304.6972711556987</v>
       </c>
       <c r="E79" s="2" t="n">
-        <v>334.5400980960846</v>
+        <v>334.5400980960845</v>
       </c>
       <c r="F79" s="2" t="n">
-        <v>364.2636577736324</v>
+        <v>364.2636577736323</v>
       </c>
       <c r="G79" s="2" t="n">
-        <v>393.9358180901934</v>
+        <v>393.9358180901933</v>
       </c>
       <c r="H79" s="2" t="n">
         <v>423.4832578774369</v>
@@ -4478,7 +4478,7 @@
         <v>512.0790958565088</v>
       </c>
       <c r="L79" s="2" t="n">
-        <v>541.5492817938723</v>
+        <v>541.5492817938724</v>
       </c>
       <c r="M79" s="2" t="n">
         <v>570.9315691201923</v>
@@ -4513,16 +4513,16 @@
       </c>
       <c r="C80" s="1" t="inlineStr"/>
       <c r="D80" s="2" t="n">
-        <v>0.9001179490256411</v>
+        <v>0.9001179490256412</v>
       </c>
       <c r="E80" s="2" t="n">
-        <v>0.9152540141204015</v>
+        <v>0.9152540141204016</v>
       </c>
       <c r="F80" s="2" t="n">
         <v>0.9244318040653919</v>
       </c>
       <c r="G80" s="2" t="n">
-        <v>0.9317173785273669</v>
+        <v>0.931717378527367</v>
       </c>
       <c r="H80" s="2" t="n">
         <v>0.937726382807626</v>
@@ -4543,7 +4543,7 @@
         <v>0.9564711798415051</v>
       </c>
       <c r="N80" s="2" t="n">
-        <v>0.9587739854529909</v>
+        <v>0.9587739854529908</v>
       </c>
       <c r="O80" s="2" t="n">
         <v>0.9608011997304212</v>
@@ -4572,16 +4572,16 @@
       </c>
       <c r="C81" s="1" t="inlineStr"/>
       <c r="D81" s="2" t="n">
-        <v>617.8311110563023</v>
+        <v>617.8311110563025</v>
       </c>
       <c r="E81" s="2" t="n">
-        <v>628.2203405174404</v>
+        <v>628.2203405174405</v>
       </c>
       <c r="F81" s="2" t="n">
         <v>634.5198751116486</v>
       </c>
       <c r="G81" s="2" t="n">
-        <v>639.5206137030721</v>
+        <v>639.5206137030722</v>
       </c>
       <c r="H81" s="2" t="n">
         <v>643.6451284900878</v>
@@ -4602,7 +4602,7 @@
         <v>656.5113520672343</v>
       </c>
       <c r="N81" s="2" t="n">
-        <v>658.0919726414946</v>
+        <v>658.0919726414945</v>
       </c>
       <c r="O81" s="2" t="n">
         <v>659.4834303395994</v>
@@ -4634,7 +4634,7 @@
         <v>455.0748040551998</v>
       </c>
       <c r="E82" s="2" t="n">
-        <v>458.7438421848687</v>
+        <v>458.7438421848688</v>
       </c>
       <c r="F82" s="2" t="n">
         <v>460.9384929530079</v>
@@ -4661,7 +4661,7 @@
         <v>467.6634924923767</v>
       </c>
       <c r="N82" s="2" t="n">
-        <v>467.9889608220808</v>
+        <v>467.9889608220807</v>
       </c>
       <c r="O82" s="2" t="n">
         <v>468.2745682991455</v>
@@ -4690,22 +4690,22 @@
       </c>
       <c r="C83" s="1" t="inlineStr"/>
       <c r="D83" s="2" t="n">
-        <v>0.5447468172074134</v>
+        <v>0.5447468172074129</v>
       </c>
       <c r="E83" s="2" t="n">
-        <v>0.5225627094398959</v>
+        <v>0.5225627094398955</v>
       </c>
       <c r="F83" s="2" t="n">
         <v>0.5128242264736803</v>
       </c>
       <c r="G83" s="2" t="n">
-        <v>0.5058701247484856</v>
+        <v>0.5058701247484854</v>
       </c>
       <c r="H83" s="2" t="n">
         <v>0.500517867126743</v>
       </c>
       <c r="I83" s="2" t="n">
-        <v>0.4963537393673502</v>
+        <v>0.4963537393673499</v>
       </c>
       <c r="J83" s="2" t="n">
         <v>0.4931527461005401</v>
@@ -4714,13 +4714,13 @@
         <v>0.4908656433918407</v>
       </c>
       <c r="L83" s="2" t="n">
-        <v>0.4893667613005351</v>
+        <v>0.4893667613005354</v>
       </c>
       <c r="M83" s="2" t="n">
-        <v>0.4886103521768771</v>
+        <v>0.4886103521768774</v>
       </c>
       <c r="N83" s="2" t="n">
-        <v>0.4885192069755876</v>
+        <v>0.4885192069755879</v>
       </c>
       <c r="O83" s="2" t="n">
         <v>0.4889480192746724</v>
@@ -4729,10 +4729,10 @@
         <v>0.4898496347186731</v>
       </c>
       <c r="Q83" s="2" t="n">
-        <v>0.4911141294015546</v>
+        <v>0.4911141294015545</v>
       </c>
       <c r="R83" s="2" t="n">
-        <v>0.4926388829310537</v>
+        <v>0.4926388829310535</v>
       </c>
       <c r="S83" s="1" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
changes in deg and rad dimentions
</commit_message>
<xml_diff>
--- a/results/Поступенчатый_расчет_ступеней.xlsx
+++ b/results/Поступенчатый_расчет_ступеней.xlsx
@@ -431,7 +431,7 @@
     <col width="21" customWidth="1" min="5" max="5"/>
     <col width="21" customWidth="1" min="6" max="6"/>
     <col width="21" customWidth="1" min="7" max="7"/>
-    <col width="21" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
     <col width="22" customWidth="1" min="9" max="9"/>
     <col width="21" customWidth="1" min="10" max="10"/>
     <col width="22" customWidth="1" min="11" max="11"/>
@@ -439,8 +439,8 @@
     <col width="22" customWidth="1" min="13" max="13"/>
     <col width="22" customWidth="1" min="14" max="14"/>
     <col width="22" customWidth="1" min="15" max="15"/>
-    <col width="21" customWidth="1" min="16" max="16"/>
-    <col width="21" customWidth="1" min="17" max="17"/>
+    <col width="22" customWidth="1" min="16" max="16"/>
+    <col width="22" customWidth="1" min="17" max="17"/>
     <col width="22" customWidth="1" min="18" max="18"/>
     <col width="21" customWidth="1" min="19" max="19"/>
   </cols>
@@ -849,7 +849,7 @@
       <c r="Q11" s="1" t="inlineStr"/>
       <c r="R11" s="1" t="inlineStr"/>
       <c r="S11" s="2" t="n">
-        <v>0.4537118711400233</v>
+        <v>0.4537118711400231</v>
       </c>
     </row>
     <row r="12" ht="15" customHeight="1">
@@ -880,7 +880,7 @@
       <c r="Q12" s="1" t="inlineStr"/>
       <c r="R12" s="1" t="inlineStr"/>
       <c r="S12" s="2" t="n">
-        <v>0.05503600366715335</v>
+        <v>0.05503600366715333</v>
       </c>
     </row>
     <row r="13" ht="15" customHeight="1">
@@ -942,7 +942,7 @@
       <c r="Q14" s="1" t="inlineStr"/>
       <c r="R14" s="1" t="inlineStr"/>
       <c r="S14" s="2" t="n">
-        <v>0.05503600366715335</v>
+        <v>0.05503600366715333</v>
       </c>
     </row>
     <row r="15" ht="15" customHeight="1">
@@ -973,7 +973,7 @@
       <c r="Q15" s="1" t="inlineStr"/>
       <c r="R15" s="1" t="inlineStr"/>
       <c r="S15" s="2" t="n">
-        <v>0.3446443080405244</v>
+        <v>0.3446443080405253</v>
       </c>
     </row>
     <row r="16" ht="15" customHeight="1">
@@ -1004,7 +1004,7 @@
       <c r="Q16" s="1" t="inlineStr"/>
       <c r="R16" s="1" t="inlineStr"/>
       <c r="S16" s="2" t="n">
-        <v>0.5062544510926422</v>
+        <v>0.5062544510926434</v>
       </c>
     </row>
     <row r="17" ht="15" customHeight="1">
@@ -1035,7 +1035,7 @@
       <c r="Q17" s="1" t="inlineStr"/>
       <c r="R17" s="1" t="inlineStr"/>
       <c r="S17" s="2" t="n">
-        <v>0.7925571175792671</v>
+        <v>0.7925571175792675</v>
       </c>
     </row>
     <row r="18" ht="15" customHeight="1">
@@ -1066,7 +1066,7 @@
       <c r="Q18" s="1" t="inlineStr"/>
       <c r="R18" s="1" t="inlineStr"/>
       <c r="S18" s="2" t="n">
-        <v>0.8596778720441987</v>
+        <v>0.8596778720441994</v>
       </c>
     </row>
     <row r="19" ht="15" customHeight="1">
@@ -1097,7 +1097,7 @@
       <c r="Q19" s="1" t="inlineStr"/>
       <c r="R19" s="1" t="inlineStr"/>
       <c r="S19" s="2" t="n">
-        <v>0.7111184547506979</v>
+        <v>0.7111184547506971</v>
       </c>
     </row>
     <row r="20" ht="15" customHeight="1">
@@ -1128,7 +1128,7 @@
       <c r="Q20" s="1" t="inlineStr"/>
       <c r="R20" s="1" t="inlineStr"/>
       <c r="S20" s="2" t="n">
-        <v>141.4703657841592</v>
+        <v>141.4703657841591</v>
       </c>
     </row>
     <row r="21" ht="30" customHeight="1">
@@ -1252,7 +1252,7 @@
       <c r="Q24" s="1" t="inlineStr"/>
       <c r="R24" s="1" t="inlineStr"/>
       <c r="S24" s="2" t="n">
-        <v>0.1680642932462094</v>
+        <v>0.168064293246209</v>
       </c>
     </row>
     <row r="25" ht="30" customHeight="1">
@@ -1681,49 +1681,49 @@
       </c>
       <c r="C32" s="1" t="inlineStr"/>
       <c r="D32" s="2" t="n">
-        <v>16967.12604306353</v>
+        <v>16967.12604306373</v>
       </c>
       <c r="E32" s="2" t="n">
-        <v>18630.78159247993</v>
+        <v>18630.78159248007</v>
       </c>
       <c r="F32" s="2" t="n">
-        <v>20218.56077089675</v>
+        <v>20218.5607708968</v>
       </c>
       <c r="G32" s="2" t="n">
-        <v>21743.63912220303</v>
+        <v>21743.63912220311</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>23213.05010780867</v>
+        <v>23213.0501078087</v>
       </c>
       <c r="I32" s="2" t="n">
-        <v>24632.76848581409</v>
+        <v>24632.76848581418</v>
       </c>
       <c r="J32" s="2" t="n">
-        <v>26002.02390990612</v>
+        <v>26002.0239099061</v>
       </c>
       <c r="K32" s="2" t="n">
         <v>27318.78381964874</v>
       </c>
       <c r="L32" s="2" t="n">
-        <v>28574.47174295066</v>
+        <v>28574.47174295057</v>
       </c>
       <c r="M32" s="2" t="n">
-        <v>29758.48274205857</v>
+        <v>29758.48274205851</v>
       </c>
       <c r="N32" s="2" t="n">
-        <v>30856.11876136265</v>
+        <v>30856.11876136259</v>
       </c>
       <c r="O32" s="2" t="n">
-        <v>31847.15753258981</v>
+        <v>31847.15753258983</v>
       </c>
       <c r="P32" s="2" t="n">
-        <v>32709.42570822141</v>
+        <v>32709.42570822144</v>
       </c>
       <c r="Q32" s="2" t="n">
-        <v>33415.02270248363</v>
+        <v>33415.02270248366</v>
       </c>
       <c r="R32" s="2" t="n">
-        <v>33933.38931404923</v>
+        <v>33933.38931404932</v>
       </c>
       <c r="S32" s="1" t="inlineStr"/>
     </row>
@@ -1740,49 +1740,49 @@
       </c>
       <c r="C33" s="1" t="inlineStr"/>
       <c r="D33" s="2" t="n">
-        <v>16797.4547826329</v>
+        <v>16797.45478263309</v>
       </c>
       <c r="E33" s="2" t="n">
-        <v>18258.16596063033</v>
+        <v>18258.16596063047</v>
       </c>
       <c r="F33" s="2" t="n">
-        <v>19612.00394776985</v>
+        <v>19612.0039477699</v>
       </c>
       <c r="G33" s="2" t="n">
-        <v>20873.89355731491</v>
+        <v>20873.89355731498</v>
       </c>
       <c r="H33" s="2" t="n">
-        <v>22052.39760241824</v>
+        <v>22052.39760241826</v>
       </c>
       <c r="I33" s="2" t="n">
-        <v>23154.80237666525</v>
+        <v>23154.80237666533</v>
       </c>
       <c r="J33" s="2" t="n">
-        <v>24441.90247531175</v>
+        <v>24441.90247531174</v>
       </c>
       <c r="K33" s="2" t="n">
-        <v>25679.65679046982</v>
+        <v>25679.65679046981</v>
       </c>
       <c r="L33" s="2" t="n">
-        <v>26860.00343837362</v>
+        <v>26860.00343837353</v>
       </c>
       <c r="M33" s="2" t="n">
-        <v>27972.97377753505</v>
+        <v>27972.97377753499</v>
       </c>
       <c r="N33" s="2" t="n">
-        <v>29004.75163568088</v>
+        <v>29004.75163568083</v>
       </c>
       <c r="O33" s="2" t="n">
-        <v>29936.32808063442</v>
+        <v>29936.32808063443</v>
       </c>
       <c r="P33" s="2" t="n">
-        <v>30746.86016572812</v>
+        <v>30746.86016572815</v>
       </c>
       <c r="Q33" s="2" t="n">
-        <v>31410.12134033461</v>
+        <v>31410.12134033464</v>
       </c>
       <c r="R33" s="2" t="n">
-        <v>31897.38595520627</v>
+        <v>31897.38595520635</v>
       </c>
       <c r="S33" s="1" t="inlineStr"/>
     </row>
@@ -1799,49 +1799,49 @@
       </c>
       <c r="C34" s="1" t="inlineStr"/>
       <c r="D34" s="2" t="n">
-        <v>13701.87693398587</v>
+        <v>13701.87693398603</v>
       </c>
       <c r="E34" s="2" t="n">
-        <v>15183.18715242563</v>
+        <v>15183.18715242576</v>
       </c>
       <c r="F34" s="2" t="n">
-        <v>16585.02366398539</v>
+        <v>16585.02366398544</v>
       </c>
       <c r="G34" s="2" t="n">
-        <v>17906.5231284628</v>
+        <v>17906.52312846286</v>
       </c>
       <c r="H34" s="2" t="n">
-        <v>19142.33211474172</v>
+        <v>19142.33211474175</v>
       </c>
       <c r="I34" s="2" t="n">
-        <v>20287.4065673813</v>
+        <v>20287.40656738138</v>
       </c>
       <c r="J34" s="2" t="n">
         <v>21560.80915145568</v>
       </c>
       <c r="K34" s="2" t="n">
-        <v>22748.1208072058</v>
+        <v>22748.12080720581</v>
       </c>
       <c r="L34" s="2" t="n">
-        <v>23831.00891765527</v>
+        <v>23831.00891765521</v>
       </c>
       <c r="M34" s="2" t="n">
-        <v>24789.99333265438</v>
+        <v>24789.99333265435</v>
       </c>
       <c r="N34" s="2" t="n">
-        <v>25602.74626396982</v>
+        <v>25602.7462639698</v>
       </c>
       <c r="O34" s="2" t="n">
-        <v>26243.62718943147</v>
+        <v>26243.62718943152</v>
       </c>
       <c r="P34" s="2" t="n">
-        <v>26686.8166302572</v>
+        <v>26686.81663025726</v>
       </c>
       <c r="Q34" s="2" t="n">
-        <v>26904.66888708486</v>
+        <v>26904.66888708492</v>
       </c>
       <c r="R34" s="2" t="n">
-        <v>26870.38869889738</v>
+        <v>26870.38869889748</v>
       </c>
       <c r="S34" s="1" t="inlineStr"/>
     </row>
@@ -1858,49 +1858,49 @@
       </c>
       <c r="C35" s="1" t="inlineStr"/>
       <c r="D35" s="2" t="n">
-        <v>16.69727115569871</v>
+        <v>16.6972711556989</v>
       </c>
       <c r="E35" s="2" t="n">
-        <v>18.08373681547265</v>
+        <v>18.08373681547279</v>
       </c>
       <c r="F35" s="2" t="n">
-        <v>19.35093521240866</v>
+        <v>19.35093521240871</v>
       </c>
       <c r="G35" s="2" t="n">
-        <v>20.5667342483578</v>
+        <v>20.56673424835787</v>
       </c>
       <c r="H35" s="2" t="n">
-        <v>21.65781275498965</v>
+        <v>21.65781275498967</v>
       </c>
       <c r="I35" s="2" t="n">
-        <v>22.64232024894005</v>
+        <v>22.64232024894013</v>
       </c>
       <c r="J35" s="2" t="n">
-        <v>23.81327704394782</v>
+        <v>23.81327704394781</v>
       </c>
       <c r="K35" s="2" t="n">
         <v>24.88456689222609</v>
       </c>
       <c r="L35" s="2" t="n">
-        <v>25.8983915489779</v>
+        <v>25.89839154897781</v>
       </c>
       <c r="M35" s="2" t="n">
-        <v>26.82431759468595</v>
+        <v>26.82431759468589</v>
       </c>
       <c r="N35" s="2" t="n">
-        <v>27.61009078020994</v>
+        <v>27.61009078020989</v>
       </c>
       <c r="O35" s="2" t="n">
-        <v>28.34277284468554</v>
+        <v>28.34277284468556</v>
       </c>
       <c r="P35" s="2" t="n">
-        <v>28.93863549455281</v>
+        <v>28.93863549455284</v>
       </c>
       <c r="Q35" s="2" t="n">
-        <v>29.38971940023345</v>
+        <v>29.38971940023348</v>
       </c>
       <c r="R35" s="2" t="n">
-        <v>29.65175826002287</v>
+        <v>29.65175826002295</v>
       </c>
       <c r="S35" s="1" t="inlineStr"/>
     </row>
@@ -1917,16 +1917,16 @@
       </c>
       <c r="C36" s="1" t="inlineStr"/>
       <c r="D36" s="2" t="n">
-        <v>304.6972711556987</v>
+        <v>304.6972711556989</v>
       </c>
       <c r="E36" s="2" t="n">
-        <v>334.5400980960845</v>
+        <v>334.5400980960846</v>
       </c>
       <c r="F36" s="2" t="n">
-        <v>364.2636577736323</v>
+        <v>364.2636577736324</v>
       </c>
       <c r="G36" s="2" t="n">
-        <v>393.9358180901933</v>
+        <v>393.9358180901934</v>
       </c>
       <c r="H36" s="2" t="n">
         <v>423.4832578774369</v>
@@ -1941,7 +1941,7 @@
         <v>512.0790958565088</v>
       </c>
       <c r="L36" s="2" t="n">
-        <v>541.5492817938724</v>
+        <v>541.5492817938723</v>
       </c>
       <c r="M36" s="2" t="n">
         <v>570.9315691201923</v>
@@ -1976,16 +1976,16 @@
       </c>
       <c r="C37" s="1" t="inlineStr"/>
       <c r="D37" s="2" t="n">
-        <v>304.6972711556987</v>
+        <v>304.6972711556989</v>
       </c>
       <c r="E37" s="2" t="n">
-        <v>334.5400980960845</v>
+        <v>334.5400980960846</v>
       </c>
       <c r="F37" s="2" t="n">
-        <v>364.2636577736323</v>
+        <v>364.2636577736324</v>
       </c>
       <c r="G37" s="2" t="n">
-        <v>393.9358180901933</v>
+        <v>393.9358180901934</v>
       </c>
       <c r="H37" s="2" t="n">
         <v>423.4832578774369</v>
@@ -2000,7 +2000,7 @@
         <v>512.0790958565088</v>
       </c>
       <c r="L37" s="2" t="n">
-        <v>541.5492817938724</v>
+        <v>541.5492817938723</v>
       </c>
       <c r="M37" s="2" t="n">
         <v>570.9315691201923</v>
@@ -2035,22 +2035,22 @@
       </c>
       <c r="C38" s="1" t="inlineStr"/>
       <c r="D38" s="2" t="n">
-        <v>1.175559285399185</v>
+        <v>1.175559285399187</v>
       </c>
       <c r="E38" s="2" t="n">
-        <v>1.177149157361193</v>
+        <v>1.177149157361195</v>
       </c>
       <c r="F38" s="2" t="n">
         <v>1.177580116958397</v>
       </c>
       <c r="G38" s="2" t="n">
-        <v>1.177095915781243</v>
+        <v>1.177095915781244</v>
       </c>
       <c r="H38" s="2" t="n">
-        <v>1.175855347567405</v>
+        <v>1.175855347567406</v>
       </c>
       <c r="I38" s="2" t="n">
-        <v>1.173962116210551</v>
+        <v>1.173962116210552</v>
       </c>
       <c r="J38" s="2" t="n">
         <v>1.173396175963183</v>
@@ -2059,10 +2059,10 @@
         <v>1.172215437821457</v>
       </c>
       <c r="L38" s="2" t="n">
-        <v>1.170376301404518</v>
+        <v>1.170376301404517</v>
       </c>
       <c r="M38" s="2" t="n">
-        <v>1.167847518639032</v>
+        <v>1.167847518639031</v>
       </c>
       <c r="N38" s="2" t="n">
         <v>1.164588351389238</v>
@@ -2074,7 +2074,7 @@
         <v>1.155630506097777</v>
       </c>
       <c r="Q38" s="2" t="n">
-        <v>1.149848870725616</v>
+        <v>1.149848870725617</v>
       </c>
       <c r="R38" s="2" t="n">
         <v>1.143155604508661</v>
@@ -2094,22 +2094,22 @@
       </c>
       <c r="C39" s="1" t="inlineStr"/>
       <c r="D39" s="2" t="n">
-        <v>117900.2252355229</v>
+        <v>117900.225235523</v>
       </c>
       <c r="E39" s="2" t="n">
-        <v>265350.467214071</v>
+        <v>265350.4672140714</v>
       </c>
       <c r="F39" s="2" t="n">
         <v>412792.3261747835</v>
       </c>
       <c r="G39" s="2" t="n">
-        <v>559906.720188837</v>
+        <v>559906.7201888376</v>
       </c>
       <c r="H39" s="2" t="n">
-        <v>706445.5229259072</v>
+        <v>706445.5229259076</v>
       </c>
       <c r="I39" s="2" t="n">
-        <v>852200.0936189099</v>
+        <v>852200.0936189106</v>
       </c>
       <c r="J39" s="2" t="n">
         <v>998610.46481496</v>
@@ -2118,10 +2118,10 @@
         <v>1144279.063503702</v>
       </c>
       <c r="L39" s="2" t="n">
-        <v>1288927.093135039</v>
+        <v>1288927.093135038</v>
       </c>
       <c r="M39" s="2" t="n">
-        <v>1432269.084259005</v>
+        <v>1432269.084259004</v>
       </c>
       <c r="N39" s="2" t="n">
         <v>1573991.10153848</v>
@@ -2130,10 +2130,10 @@
         <v>1713714.468054943</v>
       </c>
       <c r="P39" s="2" t="n">
-        <v>1851080.725235522</v>
+        <v>1851080.725235523</v>
       </c>
       <c r="Q39" s="2" t="n">
-        <v>1985694.583576009</v>
+        <v>1985694.583576011</v>
       </c>
       <c r="R39" s="2" t="n">
         <v>2117173.208233083</v>
@@ -2153,22 +2153,22 @@
       </c>
       <c r="C40" s="1" t="inlineStr"/>
       <c r="D40" s="2" t="n">
-        <v>117900.2252355229</v>
+        <v>117900.225235523</v>
       </c>
       <c r="E40" s="2" t="n">
-        <v>265350.467214071</v>
+        <v>265350.4672140714</v>
       </c>
       <c r="F40" s="2" t="n">
         <v>412792.3261747835</v>
       </c>
       <c r="G40" s="2" t="n">
-        <v>559906.720188837</v>
+        <v>559906.7201888376</v>
       </c>
       <c r="H40" s="2" t="n">
-        <v>706445.5229259072</v>
+        <v>706445.5229259076</v>
       </c>
       <c r="I40" s="2" t="n">
-        <v>852200.0936189099</v>
+        <v>852200.0936189106</v>
       </c>
       <c r="J40" s="2" t="n">
         <v>998610.46481496</v>
@@ -2177,10 +2177,10 @@
         <v>1144279.063503702</v>
       </c>
       <c r="L40" s="2" t="n">
-        <v>1288927.093135039</v>
+        <v>1288927.093135038</v>
       </c>
       <c r="M40" s="2" t="n">
-        <v>1432269.084259005</v>
+        <v>1432269.084259004</v>
       </c>
       <c r="N40" s="2" t="n">
         <v>1573991.10153848</v>
@@ -2189,10 +2189,10 @@
         <v>1713714.468054943</v>
       </c>
       <c r="P40" s="2" t="n">
-        <v>1851080.725235522</v>
+        <v>1851080.725235523</v>
       </c>
       <c r="Q40" s="2" t="n">
-        <v>1985694.583576009</v>
+        <v>1985694.583576011</v>
       </c>
       <c r="R40" s="2" t="n">
         <v>2117173.208233083</v>
@@ -2271,10 +2271,10 @@
       </c>
       <c r="C42" s="1" t="inlineStr"/>
       <c r="D42" s="2" t="n">
-        <v>319.5338237912141</v>
+        <v>319.5338237912142</v>
       </c>
       <c r="E42" s="2" t="n">
-        <v>334.7109771300941</v>
+        <v>334.7109771300942</v>
       </c>
       <c r="F42" s="2" t="n">
         <v>349.222944744292</v>
@@ -2295,7 +2295,7 @@
         <v>413.3312413404398</v>
       </c>
       <c r="L42" s="2" t="n">
-        <v>424.8720601328998</v>
+        <v>424.8720601328997</v>
       </c>
       <c r="M42" s="2" t="n">
         <v>435.9907411935118</v>
@@ -2389,49 +2389,49 @@
       </c>
       <c r="C44" s="1" t="inlineStr"/>
       <c r="D44" s="2" t="n">
-        <v>0.2675658145409686</v>
+        <v>0.2675658145409672</v>
       </c>
       <c r="E44" s="2" t="n">
-        <v>0.2627510762416373</v>
+        <v>0.2627510762416364</v>
       </c>
       <c r="F44" s="2" t="n">
-        <v>0.2591274840795847</v>
+        <v>0.2591274840795844</v>
       </c>
       <c r="G44" s="2" t="n">
-        <v>0.2565767994012265</v>
+        <v>0.256576799401226</v>
       </c>
       <c r="H44" s="2" t="n">
-        <v>0.2550220951838037</v>
+        <v>0.2550220951838035</v>
       </c>
       <c r="I44" s="2" t="n">
-        <v>0.2543930169194235</v>
+        <v>0.254393016919423</v>
       </c>
       <c r="J44" s="2" t="n">
         <v>0.2546621015587227</v>
       </c>
       <c r="K44" s="2" t="n">
-        <v>0.2558078397057247</v>
+        <v>0.2558078397057248</v>
       </c>
       <c r="L44" s="2" t="n">
-        <v>0.2578470068353892</v>
+        <v>0.2578470068353897</v>
       </c>
       <c r="M44" s="2" t="n">
-        <v>0.2608045797416072</v>
+        <v>0.2608045797416076</v>
       </c>
       <c r="N44" s="2" t="n">
-        <v>0.2647254322067377</v>
+        <v>0.2647254322067381</v>
       </c>
       <c r="O44" s="2" t="n">
-        <v>0.2696810959896802</v>
+        <v>0.2696810959896801</v>
       </c>
       <c r="P44" s="2" t="n">
-        <v>0.2757469847403647</v>
+        <v>0.2757469847403645</v>
       </c>
       <c r="Q44" s="2" t="n">
-        <v>0.2830232632486964</v>
+        <v>0.2830232632486962</v>
       </c>
       <c r="R44" s="2" t="n">
-        <v>0.2916156103246137</v>
+        <v>0.2916156103246133</v>
       </c>
       <c r="S44" s="1" t="inlineStr"/>
     </row>
@@ -2448,13 +2448,13 @@
       </c>
       <c r="C45" s="1" t="inlineStr"/>
       <c r="D45" s="2" t="n">
-        <v>1.180296158977292</v>
+        <v>1.180296158977294</v>
       </c>
       <c r="E45" s="2" t="n">
-        <v>1.175262487903346</v>
+        <v>1.175262487903347</v>
       </c>
       <c r="F45" s="2" t="n">
-        <v>1.168251369555616</v>
+        <v>1.168251369555617</v>
       </c>
       <c r="G45" s="2" t="n">
         <v>1.15925817796077</v>
@@ -2463,7 +2463,7 @@
         <v>1.148224245120433</v>
       </c>
       <c r="I45" s="2" t="n">
-        <v>1.13508172383252</v>
+        <v>1.135081723832521</v>
       </c>
       <c r="J45" s="2" t="n">
         <v>1.119697021419855</v>
@@ -2472,10 +2472,10 @@
         <v>1.101922316939652</v>
       </c>
       <c r="L45" s="2" t="n">
-        <v>1.081544540058968</v>
+        <v>1.081544540058967</v>
       </c>
       <c r="M45" s="2" t="n">
-        <v>1.05833206210163</v>
+        <v>1.058332062101629</v>
       </c>
       <c r="N45" s="2" t="n">
         <v>1.032020278583349</v>
@@ -2484,13 +2484,13 @@
         <v>1.0023075858643</v>
       </c>
       <c r="P45" s="2" t="n">
-        <v>0.9689068762009185</v>
+        <v>0.9689068762009189</v>
       </c>
       <c r="Q45" s="2" t="n">
-        <v>0.9315321714560331</v>
+        <v>0.9315321714560333</v>
       </c>
       <c r="R45" s="2" t="n">
-        <v>0.8899613152251311</v>
+        <v>0.8899613152251319</v>
       </c>
       <c r="S45" s="1" t="inlineStr"/>
     </row>
@@ -2566,22 +2566,22 @@
       </c>
       <c r="C47" s="1" t="inlineStr"/>
       <c r="D47" s="2" t="n">
-        <v>0.6934155588636791</v>
+        <v>0.6934155588636786</v>
       </c>
       <c r="E47" s="2" t="n">
-        <v>0.6419546944869916</v>
+        <v>0.6419546944869913</v>
       </c>
       <c r="F47" s="2" t="n">
-        <v>0.5966106211168185</v>
+        <v>0.5966106211168183</v>
       </c>
       <c r="G47" s="2" t="n">
-        <v>0.5561238216798055</v>
+        <v>0.5561238216798053</v>
       </c>
       <c r="H47" s="2" t="n">
         <v>0.5198537807125588</v>
       </c>
       <c r="I47" s="2" t="n">
-        <v>0.4871134947236219</v>
+        <v>0.4871134947236217</v>
       </c>
       <c r="J47" s="2" t="n">
         <v>0.4573452836046674</v>
@@ -2590,13 +2590,13 @@
         <v>0.4302607947475137</v>
       </c>
       <c r="L47" s="2" t="n">
-        <v>0.4054971202086972</v>
+        <v>0.4054971202086974</v>
       </c>
       <c r="M47" s="2" t="n">
-        <v>0.3828668774546138</v>
+        <v>0.382866877454614</v>
       </c>
       <c r="N47" s="2" t="n">
-        <v>0.3622495702925324</v>
+        <v>0.3622495702925325</v>
       </c>
       <c r="O47" s="2" t="n">
         <v>0.3434267211217917</v>
@@ -2605,10 +2605,10 @@
         <v>0.3264013915200195</v>
       </c>
       <c r="Q47" s="2" t="n">
-        <v>0.3111320861419943</v>
+        <v>0.3111320861419942</v>
       </c>
       <c r="R47" s="2" t="n">
-        <v>0.2976385445704194</v>
+        <v>0.2976385445704193</v>
       </c>
       <c r="S47" s="1" t="inlineStr"/>
     </row>
@@ -2625,22 +2625,22 @@
       </c>
       <c r="C48" s="1" t="inlineStr"/>
       <c r="D48" s="2" t="n">
-        <v>0.8876763917513484</v>
+        <v>0.8876763917513479</v>
       </c>
       <c r="E48" s="2" t="n">
-        <v>0.8476827557110533</v>
+        <v>0.8476827557110529</v>
       </c>
       <c r="F48" s="2" t="n">
-        <v>0.8078381023904093</v>
+        <v>0.807838102390409</v>
       </c>
       <c r="G48" s="2" t="n">
-        <v>0.7687303178641439</v>
+        <v>0.7687303178641441</v>
       </c>
       <c r="H48" s="2" t="n">
-        <v>0.7310690251477326</v>
+        <v>0.7310690251477328</v>
       </c>
       <c r="I48" s="2" t="n">
-        <v>0.695043801549282</v>
+        <v>0.6950438015492818</v>
       </c>
       <c r="J48" s="2" t="n">
         <v>0.6606666216532919</v>
@@ -2649,25 +2649,25 @@
         <v>0.6281613417983278</v>
       </c>
       <c r="L48" s="2" t="n">
-        <v>0.5974295303378842</v>
+        <v>0.5974295303378844</v>
       </c>
       <c r="M48" s="2" t="n">
-        <v>0.5685574328276751</v>
+        <v>0.5685574328276755</v>
       </c>
       <c r="N48" s="2" t="n">
-        <v>0.5416626339362808</v>
+        <v>0.5416626339362809</v>
       </c>
       <c r="O48" s="2" t="n">
         <v>0.5165679427658935</v>
       </c>
       <c r="P48" s="2" t="n">
-        <v>0.4934870266617922</v>
+        <v>0.4934870266617923</v>
       </c>
       <c r="Q48" s="2" t="n">
-        <v>0.4724845076896957</v>
+        <v>0.4724845076896956</v>
       </c>
       <c r="R48" s="2" t="n">
-        <v>0.4537118711400232</v>
+        <v>0.4537118711400231</v>
       </c>
       <c r="S48" s="1" t="inlineStr"/>
     </row>
@@ -2684,7 +2684,7 @@
       </c>
       <c r="C49" s="1" t="inlineStr"/>
       <c r="D49" s="2" t="n">
-        <v>0.3009117955899138</v>
+        <v>0.3009117955899137</v>
       </c>
       <c r="E49" s="2" t="n">
         <v>0.1472682986886746</v>
@@ -2693,10 +2693,10 @@
         <v>0.1040512028785386</v>
       </c>
       <c r="G49" s="2" t="n">
-        <v>0.08416531485429168</v>
+        <v>0.08416531485429166</v>
       </c>
       <c r="H49" s="2" t="n">
-        <v>0.07304667532585597</v>
+        <v>0.07304667532585596</v>
       </c>
       <c r="I49" s="2" t="n">
         <v>0.06619932070733821</v>
@@ -2708,7 +2708,7 @@
         <v>0.05890202559086238</v>
       </c>
       <c r="L49" s="2" t="n">
-        <v>0.05707687219159214</v>
+        <v>0.05707687219159215</v>
       </c>
       <c r="M49" s="2" t="n">
         <v>0.05602993268923052</v>
@@ -2720,13 +2720,13 @@
         <v>0.0556712005930268</v>
       </c>
       <c r="P49" s="2" t="n">
-        <v>0.05621043688048773</v>
+        <v>0.05621043688048771</v>
       </c>
       <c r="Q49" s="2" t="n">
         <v>0.05718010096659844</v>
       </c>
       <c r="R49" s="2" t="n">
-        <v>0.05857117009930016</v>
+        <v>0.05857117009930012</v>
       </c>
       <c r="S49" s="1" t="inlineStr"/>
     </row>
@@ -2861,22 +2861,22 @@
       </c>
       <c r="C52" s="1" t="inlineStr"/>
       <c r="D52" s="2" t="n">
-        <v>0.652860938167221</v>
+        <v>0.6528609381672205</v>
       </c>
       <c r="E52" s="2" t="n">
-        <v>0.6040008906918648</v>
+        <v>0.6040008906918644</v>
       </c>
       <c r="F52" s="2" t="n">
-        <v>0.5608528404519377</v>
+        <v>0.5608528404519376</v>
       </c>
       <c r="G52" s="2" t="n">
-        <v>0.5224733005942057</v>
+        <v>0.5224733005942056</v>
       </c>
       <c r="H52" s="2" t="n">
         <v>0.4880639358485558</v>
       </c>
       <c r="I52" s="2" t="n">
-        <v>0.4569203160469203</v>
+        <v>0.4569203160469202</v>
       </c>
       <c r="J52" s="2" t="n">
         <v>0.4285352724020985</v>
@@ -2885,25 +2885,25 @@
         <v>0.4026243969644493</v>
       </c>
       <c r="L52" s="2" t="n">
-        <v>0.378924075111542</v>
+        <v>0.3789240751115422</v>
       </c>
       <c r="M52" s="2" t="n">
-        <v>0.3572719824747075</v>
+        <v>0.3572719824747077</v>
       </c>
       <c r="N52" s="2" t="n">
-        <v>0.3374139715597592</v>
+        <v>0.3374139715597593</v>
       </c>
       <c r="O52" s="2" t="n">
         <v>0.3192848027412507</v>
       </c>
       <c r="P52" s="2" t="n">
-        <v>0.3028179399616255</v>
+        <v>0.3028179399616254</v>
       </c>
       <c r="Q52" s="2" t="n">
-        <v>0.2879901483751847</v>
+        <v>0.2879901483751846</v>
       </c>
       <c r="R52" s="2" t="n">
-        <v>0.2747820638038409</v>
+        <v>0.2747820638038408</v>
       </c>
       <c r="S52" s="1" t="inlineStr"/>
     </row>
@@ -2920,22 +2920,22 @@
       </c>
       <c r="C53" s="1" t="inlineStr"/>
       <c r="D53" s="2" t="n">
-        <v>0.856644940865214</v>
+        <v>0.8566449408652137</v>
       </c>
       <c r="E53" s="2" t="n">
-        <v>0.814630580231293</v>
+        <v>0.8146305802312926</v>
       </c>
       <c r="F53" s="2" t="n">
-        <v>0.773466762197916</v>
+        <v>0.7734667621979159</v>
       </c>
       <c r="G53" s="2" t="n">
-        <v>0.733875954874381</v>
+        <v>0.7338759548743808</v>
       </c>
       <c r="H53" s="2" t="n">
         <v>0.6961191242501733</v>
       </c>
       <c r="I53" s="2" t="n">
-        <v>0.6601638683567803</v>
+        <v>0.6601638683567802</v>
       </c>
       <c r="J53" s="2" t="n">
         <v>0.6260427988521639</v>
@@ -2944,25 +2944,25 @@
         <v>0.5937907596548805</v>
       </c>
       <c r="L53" s="2" t="n">
-        <v>0.5634296976475786</v>
+        <v>0.5634296976475788</v>
       </c>
       <c r="M53" s="2" t="n">
-        <v>0.5350423151502401</v>
+        <v>0.5350423151502405</v>
       </c>
       <c r="N53" s="2" t="n">
-        <v>0.5084161145598953</v>
+        <v>0.5084161145598954</v>
       </c>
       <c r="O53" s="2" t="n">
         <v>0.4836795065578707</v>
       </c>
       <c r="P53" s="2" t="n">
-        <v>0.460865840601904</v>
+        <v>0.4608658406019039</v>
       </c>
       <c r="Q53" s="2" t="n">
-        <v>0.4400685175575865</v>
+        <v>0.4400685175575864</v>
       </c>
       <c r="R53" s="2" t="n">
-        <v>0.4213432296968065</v>
+        <v>0.4213432296968064</v>
       </c>
       <c r="S53" s="1" t="inlineStr"/>
     </row>
@@ -2979,22 +2979,22 @@
       </c>
       <c r="C54" s="1" t="inlineStr"/>
       <c r="D54" s="2" t="n">
-        <v>0.2728264862976842</v>
+        <v>0.2728264862976837</v>
       </c>
       <c r="E54" s="2" t="n">
-        <v>0.1338497572918129</v>
+        <v>0.1338497572918128</v>
       </c>
       <c r="F54" s="2" t="n">
         <v>0.09484023765812551</v>
       </c>
       <c r="G54" s="2" t="n">
-        <v>0.07693362720631673</v>
+        <v>0.07693362720631663</v>
       </c>
       <c r="H54" s="2" t="n">
-        <v>0.06697624254320884</v>
+        <v>0.0669762425432088</v>
       </c>
       <c r="I54" s="2" t="n">
-        <v>0.06091105339602899</v>
+        <v>0.06091105339602894</v>
       </c>
       <c r="J54" s="2" t="n">
         <v>0.05699304098048162</v>
@@ -3003,10 +3003,10 @@
         <v>0.05449766392638357</v>
       </c>
       <c r="L54" s="2" t="n">
-        <v>0.05299351220560665</v>
+        <v>0.05299351220560669</v>
       </c>
       <c r="M54" s="2" t="n">
-        <v>0.05222397695379559</v>
+        <v>0.05222397695379562</v>
       </c>
       <c r="N54" s="2" t="n">
         <v>0.05206385535377919</v>
@@ -3018,10 +3018,10 @@
         <v>0.05326713372110947</v>
       </c>
       <c r="Q54" s="2" t="n">
-        <v>0.05457087868506506</v>
+        <v>0.05457087868506504</v>
       </c>
       <c r="R54" s="2" t="n">
-        <v>0.05635161751966031</v>
+        <v>0.05635161751966029</v>
       </c>
       <c r="S54" s="1" t="inlineStr"/>
     </row>
@@ -3038,16 +3038,16 @@
       </c>
       <c r="C55" s="1" t="inlineStr"/>
       <c r="D55" s="2" t="n">
-        <v>0.5004644049712288</v>
+        <v>0.5004644049712301</v>
       </c>
       <c r="E55" s="2" t="n">
-        <v>0.7951571965663653</v>
+        <v>0.7951571965663656</v>
       </c>
       <c r="F55" s="2" t="n">
         <v>0.8599102873979747</v>
       </c>
       <c r="G55" s="2" t="n">
-        <v>0.8880543221133665</v>
+        <v>0.8880543221133667</v>
       </c>
       <c r="H55" s="2" t="n">
         <v>0.9033251749764167</v>
@@ -3065,7 +3065,7 @@
         <v>0.9243435965300111</v>
       </c>
       <c r="M55" s="2" t="n">
-        <v>0.9254864808911323</v>
+        <v>0.9254864808911322</v>
       </c>
       <c r="N55" s="2" t="n">
         <v>0.9257241100343748</v>
@@ -3080,7 +3080,7 @@
         <v>0.921996524014703</v>
       </c>
       <c r="R55" s="2" t="n">
-        <v>0.9193396390285495</v>
+        <v>0.9193396390285498</v>
       </c>
       <c r="S55" s="1" t="inlineStr"/>
     </row>
@@ -3097,13 +3097,13 @@
       </c>
       <c r="C56" s="1" t="inlineStr"/>
       <c r="D56" s="2" t="n">
-        <v>0.7925571175792671</v>
+        <v>0.7925571175792675</v>
       </c>
       <c r="E56" s="2" t="n">
-        <v>0.9071180477959626</v>
+        <v>0.9071180477959627</v>
       </c>
       <c r="F56" s="2" t="n">
-        <v>0.9358895185677402</v>
+        <v>0.9358895185677403</v>
       </c>
       <c r="G56" s="2" t="n">
         <v>0.948685461697101</v>
@@ -3156,49 +3156,49 @@
       </c>
       <c r="C57" s="1" t="inlineStr"/>
       <c r="D57" s="2" t="n">
-        <v>0.2811863433358094</v>
+        <v>0.2811863433358084</v>
       </c>
       <c r="E57" s="2" t="n">
-        <v>0.341972806795301</v>
+        <v>0.3419728067953003</v>
       </c>
       <c r="F57" s="2" t="n">
-        <v>0.350941065593623</v>
+        <v>0.3509410655936228</v>
       </c>
       <c r="G57" s="2" t="n">
-        <v>0.350505751148655</v>
+        <v>0.3505057511486546</v>
       </c>
       <c r="H57" s="2" t="n">
-        <v>0.3468279629635576</v>
+        <v>0.3468279629635574</v>
       </c>
       <c r="I57" s="2" t="n">
-        <v>0.3417081181479371</v>
+        <v>0.3417081181479366</v>
       </c>
       <c r="J57" s="2" t="n">
         <v>0.3359234221056464</v>
       </c>
       <c r="K57" s="2" t="n">
-        <v>0.3297983277471503</v>
+        <v>0.3297983277471504</v>
       </c>
       <c r="L57" s="2" t="n">
-        <v>0.3235650470477318</v>
+        <v>0.3235650470477323</v>
       </c>
       <c r="M57" s="2" t="n">
-        <v>0.3173906374217697</v>
+        <v>0.31739063742177</v>
       </c>
       <c r="N57" s="2" t="n">
-        <v>0.3114061941828089</v>
+        <v>0.3114061941828092</v>
       </c>
       <c r="O57" s="2" t="n">
-        <v>0.3057573784837126</v>
+        <v>0.3057573784837125</v>
       </c>
       <c r="P57" s="2" t="n">
-        <v>0.3005825024172694</v>
+        <v>0.3005825024172691</v>
       </c>
       <c r="Q57" s="2" t="n">
-        <v>0.2960388638501387</v>
+        <v>0.2960388638501384</v>
       </c>
       <c r="R57" s="2" t="n">
-        <v>0.2922862607409261</v>
+        <v>0.2922862607409257</v>
       </c>
       <c r="S57" s="1" t="inlineStr"/>
     </row>
@@ -3215,7 +3215,7 @@
       </c>
       <c r="C58" s="1" t="inlineStr"/>
       <c r="D58" s="2" t="n">
-        <v>1.150578245989657</v>
+        <v>1.150578245989658</v>
       </c>
       <c r="E58" s="2" t="n">
         <v>1.058842137058633</v>
@@ -3224,13 +3224,13 @@
         <v>1.03259772936633</v>
       </c>
       <c r="G58" s="2" t="n">
-        <v>1.017231933919796</v>
+        <v>1.017231933919797</v>
       </c>
       <c r="H58" s="2" t="n">
-        <v>1.0052394018726</v>
+        <v>1.005239401872601</v>
       </c>
       <c r="I58" s="2" t="n">
-        <v>0.9944293535476192</v>
+        <v>0.9944293535476197</v>
       </c>
       <c r="J58" s="2" t="n">
         <v>0.9838133341616834</v>
@@ -3239,25 +3239,25 @@
         <v>0.9729365229403433</v>
       </c>
       <c r="L58" s="2" t="n">
-        <v>0.9614252343707773</v>
+        <v>0.9614252343707766</v>
       </c>
       <c r="M58" s="2" t="n">
-        <v>0.9489575905895599</v>
+        <v>0.9489575905895593</v>
       </c>
       <c r="N58" s="2" t="n">
-        <v>0.9352269846819273</v>
+        <v>0.9352269846819268</v>
       </c>
       <c r="O58" s="2" t="n">
-        <v>0.9198661432115164</v>
+        <v>0.9198661432115165</v>
       </c>
       <c r="P58" s="2" t="n">
-        <v>0.9024768235733479</v>
+        <v>0.9024768235733482</v>
       </c>
       <c r="Q58" s="2" t="n">
-        <v>0.8825869545836458</v>
+        <v>0.8825869545836461</v>
       </c>
       <c r="R58" s="2" t="n">
-        <v>0.8596778720441987</v>
+        <v>0.8596778720441994</v>
       </c>
       <c r="S58" s="1" t="inlineStr"/>
     </row>
@@ -3274,22 +3274,22 @@
       </c>
       <c r="C59" s="1" t="inlineStr"/>
       <c r="D59" s="2" t="n">
-        <v>0.6612407210601751</v>
+        <v>0.6612407210601744</v>
       </c>
       <c r="E59" s="2" t="n">
-        <v>0.6393366808686478</v>
+        <v>0.6393366808686474</v>
       </c>
       <c r="F59" s="2" t="n">
-        <v>0.6009807379947487</v>
+        <v>0.6009807379947486</v>
       </c>
       <c r="G59" s="2" t="n">
-        <v>0.5629187482016864</v>
+        <v>0.5629187482016862</v>
       </c>
       <c r="H59" s="2" t="n">
-        <v>0.5272267598629744</v>
+        <v>0.5272267598629743</v>
       </c>
       <c r="I59" s="2" t="n">
-        <v>0.4940432659250182</v>
+        <v>0.4940432659250179</v>
       </c>
       <c r="J59" s="2" t="n">
         <v>0.4632008778470891</v>
@@ -3298,13 +3298,13 @@
         <v>0.434547983835321</v>
       </c>
       <c r="L59" s="2" t="n">
-        <v>0.4078868049211561</v>
+        <v>0.4078868049211564</v>
       </c>
       <c r="M59" s="2" t="n">
-        <v>0.3830869581536963</v>
+        <v>0.3830869581536965</v>
       </c>
       <c r="N59" s="2" t="n">
-        <v>0.3598891790707873</v>
+        <v>0.3598891790707875</v>
       </c>
       <c r="O59" s="2" t="n">
         <v>0.3382266797622753</v>
@@ -3313,10 +3313,10 @@
         <v>0.3180205486364964</v>
       </c>
       <c r="Q59" s="2" t="n">
-        <v>0.2992319827470268</v>
+        <v>0.2992319827470267</v>
       </c>
       <c r="R59" s="2" t="n">
-        <v>0.2818236131273246</v>
+        <v>0.2818236131273244</v>
       </c>
       <c r="S59" s="1" t="inlineStr"/>
     </row>
@@ -3333,22 +3333,22 @@
       </c>
       <c r="C60" s="1" t="inlineStr"/>
       <c r="D60" s="2" t="n">
-        <v>0.2707047831582413</v>
+        <v>0.2707047831582408</v>
       </c>
       <c r="E60" s="2" t="n">
-        <v>0.1289535490674907</v>
+        <v>0.1289535490674906</v>
       </c>
       <c r="F60" s="2" t="n">
-        <v>0.09035121456081506</v>
+        <v>0.09035121456081503</v>
       </c>
       <c r="G60" s="2" t="n">
-        <v>0.07279583956722319</v>
+        <v>0.07279583956722309</v>
       </c>
       <c r="H60" s="2" t="n">
-        <v>0.06308713031955175</v>
+        <v>0.0630871303195517</v>
       </c>
       <c r="I60" s="2" t="n">
-        <v>0.05720514952891342</v>
+        <v>0.0572051495289134</v>
       </c>
       <c r="J60" s="2" t="n">
         <v>0.05343833731776829</v>
@@ -3357,13 +3357,13 @@
         <v>0.05108008787467855</v>
       </c>
       <c r="L60" s="2" t="n">
-        <v>0.04971625102356633</v>
+        <v>0.04971625102356635</v>
       </c>
       <c r="M60" s="2" t="n">
-        <v>0.04910680533129991</v>
+        <v>0.04910680533129995</v>
       </c>
       <c r="N60" s="2" t="n">
-        <v>0.04914211499311785</v>
+        <v>0.04914211499311783</v>
       </c>
       <c r="O60" s="2" t="n">
         <v>0.04975559312298664</v>
@@ -3372,10 +3372,10 @@
         <v>0.0509264267870588</v>
       </c>
       <c r="Q60" s="2" t="n">
-        <v>0.05266952243484317</v>
+        <v>0.05266952243484315</v>
       </c>
       <c r="R60" s="2" t="n">
-        <v>0.05503600366715335</v>
+        <v>0.05503600366715333</v>
       </c>
       <c r="S60" s="1" t="inlineStr"/>
     </row>
@@ -3392,19 +3392,19 @@
       </c>
       <c r="C61" s="1" t="inlineStr"/>
       <c r="D61" s="2" t="n">
-        <v>0.1289535490674907</v>
+        <v>0.1289535490674906</v>
       </c>
       <c r="E61" s="2" t="n">
-        <v>0.09035121456081506</v>
+        <v>0.09035121456081503</v>
       </c>
       <c r="F61" s="2" t="n">
-        <v>0.07279583956722319</v>
+        <v>0.07279583956722309</v>
       </c>
       <c r="G61" s="2" t="n">
-        <v>0.06308713031955175</v>
+        <v>0.0630871303195517</v>
       </c>
       <c r="H61" s="2" t="n">
-        <v>0.05720514952891342</v>
+        <v>0.0572051495289134</v>
       </c>
       <c r="I61" s="2" t="n">
         <v>0.05343833731776829</v>
@@ -3413,13 +3413,13 @@
         <v>0.05108008787467855</v>
       </c>
       <c r="K61" s="2" t="n">
-        <v>0.04971625102356633</v>
+        <v>0.04971625102356635</v>
       </c>
       <c r="L61" s="2" t="n">
-        <v>0.04910680533129991</v>
+        <v>0.04910680533129995</v>
       </c>
       <c r="M61" s="2" t="n">
-        <v>0.04914211499311785</v>
+        <v>0.04914211499311783</v>
       </c>
       <c r="N61" s="2" t="n">
         <v>0.04975559312298664</v>
@@ -3428,13 +3428,13 @@
         <v>0.0509264267870588</v>
       </c>
       <c r="P61" s="2" t="n">
-        <v>0.05266952243484317</v>
+        <v>0.05266952243484315</v>
       </c>
       <c r="Q61" s="2" t="n">
-        <v>0.05503600366715335</v>
+        <v>0.05503600366715333</v>
       </c>
       <c r="R61" s="2" t="n">
-        <v>0.05740248489946354</v>
+        <v>0.05740248489946351</v>
       </c>
       <c r="S61" s="1" t="inlineStr"/>
     </row>
@@ -3451,16 +3451,16 @@
       </c>
       <c r="C62" s="1" t="inlineStr"/>
       <c r="D62" s="2" t="n">
-        <v>0.5062544510926422</v>
+        <v>0.5062544510926434</v>
       </c>
       <c r="E62" s="2" t="n">
-        <v>0.8035709709007143</v>
+        <v>0.8035709709007146</v>
       </c>
       <c r="F62" s="2" t="n">
-        <v>0.8670515451401449</v>
+        <v>0.8670515451401452</v>
       </c>
       <c r="G62" s="2" t="n">
-        <v>0.8944317807808951</v>
+        <v>0.8944317807808952</v>
       </c>
       <c r="H62" s="2" t="n">
         <v>0.9092199502745679</v>
@@ -3510,13 +3510,13 @@
       </c>
       <c r="C63" s="1" t="inlineStr"/>
       <c r="D63" s="2" t="n">
-        <v>0.7811324271604738</v>
+        <v>0.781132427160474</v>
       </c>
       <c r="E63" s="2" t="n">
-        <v>0.8434383830980787</v>
+        <v>0.8434383830980788</v>
       </c>
       <c r="F63" s="2" t="n">
-        <v>0.863169055628738</v>
+        <v>0.8631690556287381</v>
       </c>
       <c r="G63" s="2" t="n">
         <v>0.8752186331837397</v>
@@ -3569,49 +3569,49 @@
       </c>
       <c r="C64" s="1" t="inlineStr"/>
       <c r="D64" s="2" t="n">
-        <v>0.4947976924542974</v>
+        <v>0.4947976924542986</v>
       </c>
       <c r="E64" s="2" t="n">
-        <v>0.4779735242447278</v>
+        <v>0.4779735242447286</v>
       </c>
       <c r="F64" s="2" t="n">
-        <v>0.486558246995227</v>
+        <v>0.4865582469952273</v>
       </c>
       <c r="G64" s="2" t="n">
-        <v>0.4994124070984713</v>
+        <v>0.4994124070984718</v>
       </c>
       <c r="H64" s="2" t="n">
         <v>0.5137734390610369</v>
       </c>
       <c r="I64" s="2" t="n">
-        <v>0.5288702372127249</v>
+        <v>0.5288702372127254</v>
       </c>
       <c r="J64" s="2" t="n">
-        <v>0.5443607442121167</v>
+        <v>0.5443607442121166</v>
       </c>
       <c r="K64" s="2" t="n">
         <v>0.5600965560548041</v>
       </c>
       <c r="L64" s="2" t="n">
-        <v>0.5759477597191393</v>
+        <v>0.5759477597191387</v>
       </c>
       <c r="M64" s="2" t="n">
-        <v>0.5918081993459788</v>
+        <v>0.5918081993459784</v>
       </c>
       <c r="N64" s="2" t="n">
-        <v>0.6075771359846212</v>
+        <v>0.6075771359846209</v>
       </c>
       <c r="O64" s="2" t="n">
-        <v>0.6231339534389797</v>
+        <v>0.6231339534389799</v>
       </c>
       <c r="P64" s="2" t="n">
-        <v>0.6383608968284005</v>
+        <v>0.6383608968284006</v>
       </c>
       <c r="Q64" s="2" t="n">
-        <v>0.6531207208541023</v>
+        <v>0.6531207208541026</v>
       </c>
       <c r="R64" s="2" t="n">
-        <v>0.6672755281010991</v>
+        <v>0.6672755281010996</v>
       </c>
       <c r="S64" s="1" t="inlineStr"/>
     </row>
@@ -3628,22 +3628,22 @@
       </c>
       <c r="C65" s="1" t="inlineStr"/>
       <c r="D65" s="2" t="n">
-        <v>0.9130337357818012</v>
+        <v>0.9130337357818</v>
       </c>
       <c r="E65" s="2" t="n">
-        <v>0.8830355266498343</v>
+        <v>0.8830355266498334</v>
       </c>
       <c r="F65" s="2" t="n">
-        <v>0.8530645253444218</v>
+        <v>0.8530645253444216</v>
       </c>
       <c r="G65" s="2" t="n">
-        <v>0.8230510799514995</v>
+        <v>0.8230510799514991</v>
       </c>
       <c r="H65" s="2" t="n">
-        <v>0.7929681334991679</v>
+        <v>0.7929681334991677</v>
       </c>
       <c r="I65" s="2" t="n">
-        <v>0.7627977092904867</v>
+        <v>0.7627977092904863</v>
       </c>
       <c r="J65" s="2" t="n">
         <v>0.7325616461288711</v>
@@ -3652,25 +3652,25 @@
         <v>0.7022863254977531</v>
       </c>
       <c r="L65" s="2" t="n">
-        <v>0.6720276223556494</v>
+        <v>0.6720276223556498</v>
       </c>
       <c r="M65" s="2" t="n">
-        <v>0.6418422361217931</v>
+        <v>0.6418422361217935</v>
       </c>
       <c r="N65" s="2" t="n">
-        <v>0.6117946368585556</v>
+        <v>0.611794636858556</v>
       </c>
       <c r="O65" s="2" t="n">
         <v>0.5819584578441279</v>
       </c>
       <c r="P65" s="2" t="n">
-        <v>0.5523963652145252</v>
+        <v>0.552396365214525</v>
       </c>
       <c r="Q65" s="2" t="n">
-        <v>0.5231726932408488</v>
+        <v>0.5231726932408487</v>
       </c>
       <c r="R65" s="2" t="n">
-        <v>0.494337429249565</v>
+        <v>0.4943374292495647</v>
       </c>
       <c r="S65" s="1" t="inlineStr"/>
     </row>
@@ -3746,49 +3746,49 @@
       </c>
       <c r="C67" s="1" t="inlineStr"/>
       <c r="D67" s="2" t="n">
-        <v>1.149900190948777</v>
+        <v>1.149900190948778</v>
       </c>
       <c r="E67" s="2" t="n">
-        <v>1.037406335378523</v>
+        <v>1.037406335378524</v>
       </c>
       <c r="F67" s="2" t="n">
         <v>1.008925798296564</v>
       </c>
       <c r="G67" s="2" t="n">
-        <v>0.9938963560643226</v>
+        <v>0.9938963560643232</v>
       </c>
       <c r="H67" s="2" t="n">
         <v>0.9831646987246834</v>
       </c>
       <c r="I67" s="2" t="n">
-        <v>0.9741269377820945</v>
+        <v>0.9741269377820952</v>
       </c>
       <c r="J67" s="2" t="n">
-        <v>0.9656506714457722</v>
+        <v>0.9656506714457721</v>
       </c>
       <c r="K67" s="2" t="n">
         <v>0.9572427390595025</v>
       </c>
       <c r="L67" s="2" t="n">
-        <v>0.9485264056880337</v>
+        <v>0.9485264056880329</v>
       </c>
       <c r="M67" s="2" t="n">
-        <v>0.9392010422085484</v>
+        <v>0.9392010422085477</v>
       </c>
       <c r="N67" s="2" t="n">
-        <v>0.9290023750862318</v>
+        <v>0.9290023750862315</v>
       </c>
       <c r="O67" s="2" t="n">
-        <v>0.9176220242343971</v>
+        <v>0.9176220242343975</v>
       </c>
       <c r="P67" s="2" t="n">
-        <v>0.9047385458666746</v>
+        <v>0.9047385458666748</v>
       </c>
       <c r="Q67" s="2" t="n">
-        <v>0.8899750486647007</v>
+        <v>0.8899750486647011</v>
       </c>
       <c r="R67" s="2" t="n">
-        <v>0.872925764302713</v>
+        <v>0.8729257643027138</v>
       </c>
       <c r="S67" s="1" t="inlineStr"/>
     </row>
@@ -3805,22 +3805,22 @@
       </c>
       <c r="C68" s="1" t="inlineStr"/>
       <c r="D68" s="2" t="n">
-        <v>0.9123908734224133</v>
+        <v>0.9123908734224122</v>
       </c>
       <c r="E68" s="2" t="n">
-        <v>0.9132006195531571</v>
+        <v>0.9132006195531562</v>
       </c>
       <c r="F68" s="2" t="n">
-        <v>0.8879673231596732</v>
+        <v>0.887967323159673</v>
       </c>
       <c r="G68" s="2" t="n">
-        <v>0.8577821070040718</v>
+        <v>0.8577821070040713</v>
       </c>
       <c r="H68" s="2" t="n">
         <v>0.8255539583207618</v>
       </c>
       <c r="I68" s="2" t="n">
-        <v>0.7921601127455445</v>
+        <v>0.792160112745544</v>
       </c>
       <c r="J68" s="2" t="n">
         <v>0.7580358219315676</v>
@@ -3829,25 +3829,25 @@
         <v>0.72342089195214</v>
       </c>
       <c r="L68" s="2" t="n">
-        <v>0.6885297165190221</v>
+        <v>0.6885297165190225</v>
       </c>
       <c r="M68" s="2" t="n">
-        <v>0.6535447189435523</v>
+        <v>0.6535447189435526</v>
       </c>
       <c r="N68" s="2" t="n">
-        <v>0.6186306556226797</v>
+        <v>0.6186306556226798</v>
       </c>
       <c r="O68" s="2" t="n">
-        <v>0.583951057858041</v>
+        <v>0.5839510578580409</v>
       </c>
       <c r="P68" s="2" t="n">
-        <v>0.549645877449551</v>
+        <v>0.5496458774495508</v>
       </c>
       <c r="Q68" s="2" t="n">
-        <v>0.5158449565439995</v>
+        <v>0.5158449565439994</v>
       </c>
       <c r="R68" s="2" t="n">
-        <v>0.4826515564353131</v>
+        <v>0.4826515564353129</v>
       </c>
       <c r="S68" s="1" t="inlineStr"/>
     </row>
@@ -3864,49 +3864,49 @@
       </c>
       <c r="C69" s="1" t="inlineStr"/>
       <c r="D69" s="2" t="n">
-        <v>0.2368664551669755</v>
+        <v>0.236866455166978</v>
       </c>
       <c r="E69" s="2" t="n">
-        <v>0.1543708087286889</v>
+        <v>0.1543708087286905</v>
       </c>
       <c r="F69" s="2" t="n">
-        <v>0.1558612729521425</v>
+        <v>0.1558612729521429</v>
       </c>
       <c r="G69" s="2" t="n">
-        <v>0.1708452761128231</v>
+        <v>0.1708452761128242</v>
       </c>
       <c r="H69" s="2" t="n">
-        <v>0.1901965652255154</v>
+        <v>0.1901965652255156</v>
       </c>
       <c r="I69" s="2" t="n">
-        <v>0.2113292284916077</v>
+        <v>0.211329228491609</v>
       </c>
       <c r="J69" s="2" t="n">
-        <v>0.2330890253169011</v>
+        <v>0.233089025316901</v>
       </c>
       <c r="K69" s="2" t="n">
         <v>0.2549564135617495</v>
       </c>
       <c r="L69" s="2" t="n">
-        <v>0.2764987833323843</v>
+        <v>0.2764987833323831</v>
       </c>
       <c r="M69" s="2" t="n">
-        <v>0.2973588060867552</v>
+        <v>0.2973588060867542</v>
       </c>
       <c r="N69" s="2" t="n">
-        <v>0.3172077382276762</v>
+        <v>0.3172077382276756</v>
       </c>
       <c r="O69" s="2" t="n">
-        <v>0.3356635663902692</v>
+        <v>0.3356635663902696</v>
       </c>
       <c r="P69" s="2" t="n">
-        <v>0.3523421806521494</v>
+        <v>0.3523421806521498</v>
       </c>
       <c r="Q69" s="2" t="n">
-        <v>0.3668023554238519</v>
+        <v>0.3668023554238524</v>
       </c>
       <c r="R69" s="2" t="n">
-        <v>0.3785883350531479</v>
+        <v>0.3785883350531491</v>
       </c>
       <c r="S69" s="1" t="inlineStr"/>
     </row>
@@ -3923,22 +3923,22 @@
       </c>
       <c r="C70" s="1" t="inlineStr"/>
       <c r="D70" s="2" t="n">
-        <v>0.2381873725672434</v>
+        <v>0.2381873725672461</v>
       </c>
       <c r="E70" s="2" t="n">
-        <v>0.1456415175054754</v>
+        <v>0.1456415175054772</v>
       </c>
       <c r="F70" s="2" t="n">
-        <v>0.1446304062066563</v>
+        <v>0.1446304062066568</v>
       </c>
       <c r="G70" s="2" t="n">
-        <v>0.1594498269157244</v>
+        <v>0.1594498269157253</v>
       </c>
       <c r="H70" s="2" t="n">
-        <v>0.1796854435518385</v>
+        <v>0.1796854435518387</v>
       </c>
       <c r="I70" s="2" t="n">
-        <v>0.2022692408020746</v>
+        <v>0.2022692408020758</v>
       </c>
       <c r="J70" s="2" t="n">
         <v>0.2257775122301158</v>
@@ -3947,25 +3947,25 @@
         <v>0.2495156309882033</v>
       </c>
       <c r="L70" s="2" t="n">
-        <v>0.2728955178517553</v>
+        <v>0.2728955178517541</v>
       </c>
       <c r="M70" s="2" t="n">
-        <v>0.2954128716460076</v>
+        <v>0.2954128716460067</v>
       </c>
       <c r="N70" s="2" t="n">
-        <v>0.3165963290592476</v>
+        <v>0.316596329059247</v>
       </c>
       <c r="O70" s="2" t="n">
-        <v>0.3359150853534754</v>
+        <v>0.3359150853534756</v>
       </c>
       <c r="P70" s="2" t="n">
-        <v>0.352830946123797</v>
+        <v>0.3528309461237974</v>
       </c>
       <c r="Q70" s="2" t="n">
-        <v>0.3667419980396462</v>
+        <v>0.3667419980396467</v>
       </c>
       <c r="R70" s="2" t="n">
-        <v>0.3770263156088856</v>
+        <v>0.3770263156088866</v>
       </c>
       <c r="S70" s="1" t="inlineStr"/>
     </row>
@@ -3982,22 +3982,22 @@
       </c>
       <c r="C71" s="1" t="inlineStr"/>
       <c r="D71" s="2" t="n">
-        <v>251.7894146864383</v>
+        <v>251.7894146864385</v>
       </c>
       <c r="E71" s="2" t="n">
-        <v>249.6625952542773</v>
+        <v>249.6625952542775</v>
       </c>
       <c r="F71" s="2" t="n">
-        <v>247.6528107706312</v>
+        <v>247.6528107706313</v>
       </c>
       <c r="G71" s="2" t="n">
-        <v>245.7731838000792</v>
+        <v>245.7731838000793</v>
       </c>
       <c r="H71" s="2" t="n">
         <v>244.0304158041251</v>
       </c>
       <c r="I71" s="2" t="n">
-        <v>242.4310417988147</v>
+        <v>242.4310417988148</v>
       </c>
       <c r="J71" s="2" t="n">
         <v>240.972909827971</v>
@@ -4006,25 +4006,25 @@
         <v>239.6524840515102</v>
       </c>
       <c r="L71" s="2" t="n">
-        <v>238.4569611637399</v>
+        <v>238.4569611637397</v>
       </c>
       <c r="M71" s="2" t="n">
-        <v>237.3706330162412</v>
+        <v>237.3706330162411</v>
       </c>
       <c r="N71" s="2" t="n">
-        <v>236.3718770966747</v>
+        <v>236.3718770966746</v>
       </c>
       <c r="O71" s="2" t="n">
         <v>235.4310839272837</v>
       </c>
       <c r="P71" s="2" t="n">
-        <v>234.5161748631907</v>
+        <v>234.5161748631908</v>
       </c>
       <c r="Q71" s="2" t="n">
         <v>233.5872660970408</v>
       </c>
       <c r="R71" s="2" t="n">
-        <v>232.6016263665795</v>
+        <v>232.6016263665796</v>
       </c>
       <c r="S71" s="1" t="inlineStr"/>
     </row>
@@ -4100,22 +4100,22 @@
       </c>
       <c r="C73" s="1" t="inlineStr"/>
       <c r="D73" s="2" t="n">
-        <v>247.9005511003572</v>
+        <v>247.9005511003574</v>
       </c>
       <c r="E73" s="2" t="n">
-        <v>239.7224251109928</v>
+        <v>239.722425110993</v>
       </c>
       <c r="F73" s="2" t="n">
         <v>236.3804261005702</v>
       </c>
       <c r="G73" s="2" t="n">
-        <v>234.0471923727897</v>
+        <v>234.0471923727898</v>
       </c>
       <c r="H73" s="2" t="n">
         <v>232.2443952114634</v>
       </c>
       <c r="I73" s="2" t="n">
-        <v>230.844791132339</v>
+        <v>230.8447911323391</v>
       </c>
       <c r="J73" s="2" t="n">
         <v>229.7932112410973</v>
@@ -4124,10 +4124,10 @@
         <v>229.0678517566361</v>
       </c>
       <c r="L73" s="2" t="n">
-        <v>228.6458226289367</v>
+        <v>228.6458226289366</v>
       </c>
       <c r="M73" s="2" t="n">
-        <v>228.5052237669686</v>
+        <v>228.5052237669685</v>
       </c>
       <c r="N73" s="2" t="n">
         <v>228.6215960141323</v>
@@ -4142,7 +4142,7 @@
         <v>230.1629008037089</v>
       </c>
       <c r="R73" s="2" t="n">
-        <v>230.9323888012639</v>
+        <v>230.932388801264</v>
       </c>
       <c r="S73" s="1" t="inlineStr"/>
     </row>
@@ -4159,7 +4159,7 @@
       </c>
       <c r="C74" s="1" t="inlineStr"/>
       <c r="D74" s="2" t="n">
-        <v>0.9198717705829681</v>
+        <v>0.9198717705829682</v>
       </c>
       <c r="E74" s="2" t="n">
         <v>0.9316127880691234</v>
@@ -4168,7 +4168,7 @@
         <v>0.9411937231993717</v>
       </c>
       <c r="G74" s="2" t="n">
-        <v>0.9489889140291672</v>
+        <v>0.9489889140291673</v>
       </c>
       <c r="H74" s="2" t="n">
         <v>0.9555931563290563</v>
@@ -4183,25 +4183,25 @@
         <v>0.9700508464641263</v>
       </c>
       <c r="L74" s="2" t="n">
-        <v>0.9735532872138979</v>
+        <v>0.9735532872138978</v>
       </c>
       <c r="M74" s="2" t="n">
         <v>0.9765720654514889</v>
       </c>
       <c r="N74" s="2" t="n">
-        <v>0.9792051916840199</v>
+        <v>0.9792051916840198</v>
       </c>
       <c r="O74" s="2" t="n">
         <v>0.9814270687200961</v>
       </c>
       <c r="P74" s="2" t="n">
-        <v>0.98333723871931</v>
+        <v>0.9833372387193101</v>
       </c>
       <c r="Q74" s="2" t="n">
         <v>0.9849622306534793</v>
       </c>
       <c r="R74" s="2" t="n">
-        <v>0.9863414798135991</v>
+        <v>0.9863414798135992</v>
       </c>
       <c r="S74" s="1" t="inlineStr"/>
     </row>
@@ -4218,7 +4218,7 @@
       </c>
       <c r="C75" s="1" t="inlineStr"/>
       <c r="D75" s="2" t="n">
-        <v>264.9230699278948</v>
+        <v>264.9230699278949</v>
       </c>
       <c r="E75" s="2" t="n">
         <v>294.8147930348406</v>
@@ -4254,13 +4254,13 @@
         <v>589.8572714101675</v>
       </c>
       <c r="P75" s="2" t="n">
-        <v>618.9875214592723</v>
+        <v>618.9875214592724</v>
       </c>
       <c r="Q75" s="2" t="n">
         <v>648.0388565102273</v>
       </c>
       <c r="R75" s="2" t="n">
-        <v>677.0139991251235</v>
+        <v>677.0139991251236</v>
       </c>
       <c r="S75" s="1" t="inlineStr"/>
     </row>
@@ -4336,22 +4336,22 @@
       </c>
       <c r="C77" s="1" t="inlineStr"/>
       <c r="D77" s="2" t="n">
-        <v>0.8448204141343573</v>
+        <v>0.8448204141343578</v>
       </c>
       <c r="E77" s="2" t="n">
-        <v>0.7943214505742261</v>
+        <v>0.7943214505742267</v>
       </c>
       <c r="F77" s="2" t="n">
-        <v>0.7511095390711755</v>
+        <v>0.7511095390711756</v>
       </c>
       <c r="G77" s="2" t="n">
-        <v>0.7135754513445639</v>
+        <v>0.7135754513445642</v>
       </c>
       <c r="H77" s="2" t="n">
-        <v>0.6807840523057971</v>
+        <v>0.6807840523057973</v>
       </c>
       <c r="I77" s="2" t="n">
-        <v>0.6518956097662678</v>
+        <v>0.651895609766268</v>
       </c>
       <c r="J77" s="2" t="n">
         <v>0.6262006800178096</v>
@@ -4360,25 +4360,25 @@
         <v>0.6032931870271456</v>
       </c>
       <c r="L77" s="2" t="n">
-        <v>0.5826698506248713</v>
+        <v>0.582669850624871</v>
       </c>
       <c r="M77" s="2" t="n">
-        <v>0.5640185684375761</v>
+        <v>0.5640185684375758</v>
       </c>
       <c r="N77" s="2" t="n">
-        <v>0.5470938594252943</v>
+        <v>0.5470938594252941</v>
       </c>
       <c r="O77" s="2" t="n">
-        <v>0.5314851030679412</v>
+        <v>0.5314851030679409</v>
       </c>
       <c r="P77" s="2" t="n">
-        <v>0.5170517482371181</v>
+        <v>0.5170517482371183</v>
       </c>
       <c r="Q77" s="2" t="n">
-        <v>0.5035581698659796</v>
+        <v>0.5035581698659797</v>
       </c>
       <c r="R77" s="2" t="n">
-        <v>0.4908332230905135</v>
+        <v>0.4908332230905137</v>
       </c>
       <c r="S77" s="1" t="inlineStr"/>
     </row>
@@ -4395,22 +4395,22 @@
       </c>
       <c r="C78" s="1" t="inlineStr"/>
       <c r="D78" s="2" t="n">
-        <v>0.7758194364498243</v>
+        <v>0.7758194364498247</v>
       </c>
       <c r="E78" s="2" t="n">
-        <v>0.7162072399490456</v>
+        <v>0.7162072399490459</v>
       </c>
       <c r="F78" s="2" t="n">
-        <v>0.6768754162864431</v>
+        <v>0.6768754162864432</v>
       </c>
       <c r="G78" s="2" t="n">
-        <v>0.6446312378490993</v>
+        <v>0.6446312378490995</v>
       </c>
       <c r="H78" s="2" t="n">
         <v>0.6171656544030198</v>
       </c>
       <c r="I78" s="2" t="n">
-        <v>0.5933516387160813</v>
+        <v>0.5933516387160817</v>
       </c>
       <c r="J78" s="2" t="n">
         <v>0.5724800026430085</v>
@@ -4419,13 +4419,13 @@
         <v>0.5541992204938717</v>
       </c>
       <c r="L78" s="2" t="n">
-        <v>0.5381521735211688</v>
+        <v>0.5381521735211686</v>
       </c>
       <c r="M78" s="2" t="n">
-        <v>0.5241056797248544</v>
+        <v>0.5241056797248543</v>
       </c>
       <c r="N78" s="2" t="n">
-        <v>0.5116577227873376</v>
+        <v>0.5116577227873375</v>
       </c>
       <c r="O78" s="2" t="n">
         <v>0.5006277313683627</v>
@@ -4434,10 +4434,10 @@
         <v>0.4908125161156869</v>
       </c>
       <c r="Q78" s="2" t="n">
-        <v>0.4820311420268308</v>
+        <v>0.4820311420268309</v>
       </c>
       <c r="R78" s="2" t="n">
-        <v>0.4740845874252208</v>
+        <v>0.474084587425221</v>
       </c>
       <c r="S78" s="1" t="inlineStr"/>
     </row>
@@ -4454,16 +4454,16 @@
       </c>
       <c r="C79" s="1" t="inlineStr"/>
       <c r="D79" s="2" t="n">
-        <v>304.6972711556987</v>
+        <v>304.6972711556989</v>
       </c>
       <c r="E79" s="2" t="n">
-        <v>334.5400980960845</v>
+        <v>334.5400980960846</v>
       </c>
       <c r="F79" s="2" t="n">
-        <v>364.2636577736323</v>
+        <v>364.2636577736324</v>
       </c>
       <c r="G79" s="2" t="n">
-        <v>393.9358180901933</v>
+        <v>393.9358180901934</v>
       </c>
       <c r="H79" s="2" t="n">
         <v>423.4832578774369</v>
@@ -4478,7 +4478,7 @@
         <v>512.0790958565088</v>
       </c>
       <c r="L79" s="2" t="n">
-        <v>541.5492817938724</v>
+        <v>541.5492817938723</v>
       </c>
       <c r="M79" s="2" t="n">
         <v>570.9315691201923</v>
@@ -4513,16 +4513,16 @@
       </c>
       <c r="C80" s="1" t="inlineStr"/>
       <c r="D80" s="2" t="n">
-        <v>0.9001179490256412</v>
+        <v>0.9001179490256411</v>
       </c>
       <c r="E80" s="2" t="n">
-        <v>0.9152540141204016</v>
+        <v>0.9152540141204015</v>
       </c>
       <c r="F80" s="2" t="n">
         <v>0.9244318040653919</v>
       </c>
       <c r="G80" s="2" t="n">
-        <v>0.931717378527367</v>
+        <v>0.9317173785273669</v>
       </c>
       <c r="H80" s="2" t="n">
         <v>0.937726382807626</v>
@@ -4543,7 +4543,7 @@
         <v>0.9564711798415051</v>
       </c>
       <c r="N80" s="2" t="n">
-        <v>0.9587739854529908</v>
+        <v>0.9587739854529909</v>
       </c>
       <c r="O80" s="2" t="n">
         <v>0.9608011997304212</v>
@@ -4572,16 +4572,16 @@
       </c>
       <c r="C81" s="1" t="inlineStr"/>
       <c r="D81" s="2" t="n">
-        <v>617.8311110563025</v>
+        <v>617.8311110563023</v>
       </c>
       <c r="E81" s="2" t="n">
-        <v>628.2203405174405</v>
+        <v>628.2203405174404</v>
       </c>
       <c r="F81" s="2" t="n">
         <v>634.5198751116486</v>
       </c>
       <c r="G81" s="2" t="n">
-        <v>639.5206137030722</v>
+        <v>639.5206137030721</v>
       </c>
       <c r="H81" s="2" t="n">
         <v>643.6451284900878</v>
@@ -4602,7 +4602,7 @@
         <v>656.5113520672343</v>
       </c>
       <c r="N81" s="2" t="n">
-        <v>658.0919726414945</v>
+        <v>658.0919726414946</v>
       </c>
       <c r="O81" s="2" t="n">
         <v>659.4834303395994</v>
@@ -4634,7 +4634,7 @@
         <v>455.0748040551998</v>
       </c>
       <c r="E82" s="2" t="n">
-        <v>458.7438421848688</v>
+        <v>458.7438421848687</v>
       </c>
       <c r="F82" s="2" t="n">
         <v>460.9384929530079</v>
@@ -4661,7 +4661,7 @@
         <v>467.6634924923767</v>
       </c>
       <c r="N82" s="2" t="n">
-        <v>467.9889608220807</v>
+        <v>467.9889608220808</v>
       </c>
       <c r="O82" s="2" t="n">
         <v>468.2745682991455</v>
@@ -4690,22 +4690,22 @@
       </c>
       <c r="C83" s="1" t="inlineStr"/>
       <c r="D83" s="2" t="n">
-        <v>0.5447468172074129</v>
+        <v>0.5447468172074134</v>
       </c>
       <c r="E83" s="2" t="n">
-        <v>0.5225627094398955</v>
+        <v>0.5225627094398959</v>
       </c>
       <c r="F83" s="2" t="n">
         <v>0.5128242264736803</v>
       </c>
       <c r="G83" s="2" t="n">
-        <v>0.5058701247484854</v>
+        <v>0.5058701247484856</v>
       </c>
       <c r="H83" s="2" t="n">
         <v>0.500517867126743</v>
       </c>
       <c r="I83" s="2" t="n">
-        <v>0.4963537393673499</v>
+        <v>0.4963537393673502</v>
       </c>
       <c r="J83" s="2" t="n">
         <v>0.4931527461005401</v>
@@ -4714,13 +4714,13 @@
         <v>0.4908656433918407</v>
       </c>
       <c r="L83" s="2" t="n">
-        <v>0.4893667613005354</v>
+        <v>0.4893667613005351</v>
       </c>
       <c r="M83" s="2" t="n">
-        <v>0.4886103521768774</v>
+        <v>0.4886103521768771</v>
       </c>
       <c r="N83" s="2" t="n">
-        <v>0.4885192069755879</v>
+        <v>0.4885192069755876</v>
       </c>
       <c r="O83" s="2" t="n">
         <v>0.4889480192746724</v>
@@ -4729,10 +4729,10 @@
         <v>0.4898496347186731</v>
       </c>
       <c r="Q83" s="2" t="n">
-        <v>0.4911141294015545</v>
+        <v>0.4911141294015546</v>
       </c>
       <c r="R83" s="2" t="n">
-        <v>0.4926388829310535</v>
+        <v>0.4926388829310537</v>
       </c>
       <c r="S83" s="1" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
added pdf as a example
</commit_message>
<xml_diff>
--- a/results/Поступенчатый_расчет_ступеней.xlsx
+++ b/results/Поступенчатый_расчет_ступеней.xlsx
@@ -431,7 +431,7 @@
     <col width="21" customWidth="1" min="5" max="5"/>
     <col width="21" customWidth="1" min="6" max="6"/>
     <col width="21" customWidth="1" min="7" max="7"/>
-    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="21" customWidth="1" min="8" max="8"/>
     <col width="22" customWidth="1" min="9" max="9"/>
     <col width="21" customWidth="1" min="10" max="10"/>
     <col width="22" customWidth="1" min="11" max="11"/>
@@ -439,8 +439,8 @@
     <col width="22" customWidth="1" min="13" max="13"/>
     <col width="22" customWidth="1" min="14" max="14"/>
     <col width="22" customWidth="1" min="15" max="15"/>
-    <col width="22" customWidth="1" min="16" max="16"/>
-    <col width="22" customWidth="1" min="17" max="17"/>
+    <col width="21" customWidth="1" min="16" max="16"/>
+    <col width="21" customWidth="1" min="17" max="17"/>
     <col width="22" customWidth="1" min="18" max="18"/>
     <col width="21" customWidth="1" min="19" max="19"/>
   </cols>
@@ -849,7 +849,7 @@
       <c r="Q11" s="1" t="inlineStr"/>
       <c r="R11" s="1" t="inlineStr"/>
       <c r="S11" s="2" t="n">
-        <v>0.4537118711400231</v>
+        <v>0.4537118711400233</v>
       </c>
     </row>
     <row r="12" ht="15" customHeight="1">
@@ -880,7 +880,7 @@
       <c r="Q12" s="1" t="inlineStr"/>
       <c r="R12" s="1" t="inlineStr"/>
       <c r="S12" s="2" t="n">
-        <v>0.05503600366715333</v>
+        <v>0.05503600366715335</v>
       </c>
     </row>
     <row r="13" ht="15" customHeight="1">
@@ -942,7 +942,7 @@
       <c r="Q14" s="1" t="inlineStr"/>
       <c r="R14" s="1" t="inlineStr"/>
       <c r="S14" s="2" t="n">
-        <v>0.05503600366715333</v>
+        <v>0.05503600366715335</v>
       </c>
     </row>
     <row r="15" ht="15" customHeight="1">
@@ -973,7 +973,7 @@
       <c r="Q15" s="1" t="inlineStr"/>
       <c r="R15" s="1" t="inlineStr"/>
       <c r="S15" s="2" t="n">
-        <v>0.3559988181585447</v>
+        <v>0.3446443080405244</v>
       </c>
     </row>
     <row r="16" ht="15" customHeight="1">
@@ -1004,7 +1004,7 @@
       <c r="Q16" s="1" t="inlineStr"/>
       <c r="R16" s="1" t="inlineStr"/>
       <c r="S16" s="2" t="n">
-        <v>0.5229333027467026</v>
+        <v>0.5062544510926422</v>
       </c>
     </row>
     <row r="17" ht="15" customHeight="1">
@@ -1035,7 +1035,7 @@
       <c r="Q17" s="1" t="inlineStr"/>
       <c r="R17" s="1" t="inlineStr"/>
       <c r="S17" s="2" t="n">
-        <v>0.7979533943538226</v>
+        <v>0.7925571175792671</v>
       </c>
     </row>
     <row r="18" ht="15" customHeight="1">
@@ -1066,7 +1066,7 @@
       <c r="Q18" s="1" t="inlineStr"/>
       <c r="R18" s="1" t="inlineStr"/>
       <c r="S18" s="2" t="n">
-        <v>0.8596778720441994</v>
+        <v>0.8596778720441987</v>
       </c>
     </row>
     <row r="19" ht="15" customHeight="1">
@@ -1097,7 +1097,7 @@
       <c r="Q19" s="1" t="inlineStr"/>
       <c r="R19" s="1" t="inlineStr"/>
       <c r="S19" s="2" t="n">
-        <v>0.7111184547506971</v>
+        <v>0.7111184547506979</v>
       </c>
     </row>
     <row r="20" ht="15" customHeight="1">
@@ -1128,7 +1128,7 @@
       <c r="Q20" s="1" t="inlineStr"/>
       <c r="R20" s="1" t="inlineStr"/>
       <c r="S20" s="2" t="n">
-        <v>141.4703657841591</v>
+        <v>141.4703657841592</v>
       </c>
     </row>
     <row r="21" ht="30" customHeight="1">
@@ -1252,7 +1252,7 @@
       <c r="Q24" s="1" t="inlineStr"/>
       <c r="R24" s="1" t="inlineStr"/>
       <c r="S24" s="2" t="n">
-        <v>0.1623870381871993</v>
+        <v>0.1680642932462094</v>
       </c>
     </row>
     <row r="25" ht="30" customHeight="1">
@@ -1681,49 +1681,49 @@
       </c>
       <c r="C32" s="1" t="inlineStr"/>
       <c r="D32" s="2" t="n">
-        <v>16967.12604306373</v>
+        <v>16967.12604306353</v>
       </c>
       <c r="E32" s="2" t="n">
-        <v>18630.78159248007</v>
+        <v>18630.78159247993</v>
       </c>
       <c r="F32" s="2" t="n">
-        <v>20218.5607708968</v>
+        <v>20218.56077089675</v>
       </c>
       <c r="G32" s="2" t="n">
-        <v>21743.63912220311</v>
+        <v>21743.63912220303</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>23213.0501078087</v>
+        <v>23213.05010780867</v>
       </c>
       <c r="I32" s="2" t="n">
-        <v>24632.76848581418</v>
+        <v>24632.76848581409</v>
       </c>
       <c r="J32" s="2" t="n">
-        <v>26002.0239099061</v>
+        <v>26002.02390990612</v>
       </c>
       <c r="K32" s="2" t="n">
         <v>27318.78381964874</v>
       </c>
       <c r="L32" s="2" t="n">
-        <v>28574.47174295057</v>
+        <v>28574.47174295066</v>
       </c>
       <c r="M32" s="2" t="n">
-        <v>29758.48274205851</v>
+        <v>29758.48274205857</v>
       </c>
       <c r="N32" s="2" t="n">
-        <v>30856.11876136259</v>
+        <v>30856.11876136265</v>
       </c>
       <c r="O32" s="2" t="n">
-        <v>31847.15753258983</v>
+        <v>31847.15753258981</v>
       </c>
       <c r="P32" s="2" t="n">
-        <v>32709.42570822144</v>
+        <v>32709.42570822141</v>
       </c>
       <c r="Q32" s="2" t="n">
-        <v>33415.02270248366</v>
+        <v>33415.02270248363</v>
       </c>
       <c r="R32" s="2" t="n">
-        <v>33933.38931404932</v>
+        <v>33933.38931404923</v>
       </c>
       <c r="S32" s="1" t="inlineStr"/>
     </row>
@@ -1740,49 +1740,49 @@
       </c>
       <c r="C33" s="1" t="inlineStr"/>
       <c r="D33" s="2" t="n">
-        <v>16797.45478263309</v>
+        <v>16797.4547826329</v>
       </c>
       <c r="E33" s="2" t="n">
-        <v>18258.16596063047</v>
+        <v>18258.16596063033</v>
       </c>
       <c r="F33" s="2" t="n">
-        <v>19612.0039477699</v>
+        <v>19612.00394776985</v>
       </c>
       <c r="G33" s="2" t="n">
-        <v>20873.89355731498</v>
+        <v>20873.89355731491</v>
       </c>
       <c r="H33" s="2" t="n">
-        <v>22052.39760241826</v>
+        <v>22052.39760241824</v>
       </c>
       <c r="I33" s="2" t="n">
-        <v>23154.80237666533</v>
+        <v>23154.80237666525</v>
       </c>
       <c r="J33" s="2" t="n">
-        <v>24441.90247531174</v>
+        <v>24441.90247531175</v>
       </c>
       <c r="K33" s="2" t="n">
-        <v>25679.65679046981</v>
+        <v>25679.65679046982</v>
       </c>
       <c r="L33" s="2" t="n">
-        <v>26860.00343837353</v>
+        <v>26860.00343837362</v>
       </c>
       <c r="M33" s="2" t="n">
-        <v>27972.97377753499</v>
+        <v>27972.97377753505</v>
       </c>
       <c r="N33" s="2" t="n">
-        <v>29004.75163568083</v>
+        <v>29004.75163568088</v>
       </c>
       <c r="O33" s="2" t="n">
-        <v>29936.32808063443</v>
+        <v>29936.32808063442</v>
       </c>
       <c r="P33" s="2" t="n">
-        <v>30746.86016572815</v>
+        <v>30746.86016572812</v>
       </c>
       <c r="Q33" s="2" t="n">
-        <v>31410.12134033464</v>
+        <v>31410.12134033461</v>
       </c>
       <c r="R33" s="2" t="n">
-        <v>31897.38595520635</v>
+        <v>31897.38595520627</v>
       </c>
       <c r="S33" s="1" t="inlineStr"/>
     </row>
@@ -1799,49 +1799,49 @@
       </c>
       <c r="C34" s="1" t="inlineStr"/>
       <c r="D34" s="2" t="n">
-        <v>13701.87693398603</v>
+        <v>13701.87693398587</v>
       </c>
       <c r="E34" s="2" t="n">
-        <v>15183.18715242576</v>
+        <v>15183.18715242563</v>
       </c>
       <c r="F34" s="2" t="n">
-        <v>16585.02366398544</v>
+        <v>16585.02366398539</v>
       </c>
       <c r="G34" s="2" t="n">
-        <v>17906.52312846286</v>
+        <v>17906.5231284628</v>
       </c>
       <c r="H34" s="2" t="n">
-        <v>19142.33211474175</v>
+        <v>19142.33211474172</v>
       </c>
       <c r="I34" s="2" t="n">
-        <v>20287.40656738138</v>
+        <v>20287.4065673813</v>
       </c>
       <c r="J34" s="2" t="n">
         <v>21560.80915145568</v>
       </c>
       <c r="K34" s="2" t="n">
-        <v>22748.12080720581</v>
+        <v>22748.1208072058</v>
       </c>
       <c r="L34" s="2" t="n">
-        <v>23831.00891765521</v>
+        <v>23831.00891765527</v>
       </c>
       <c r="M34" s="2" t="n">
-        <v>24789.99333265435</v>
+        <v>24789.99333265438</v>
       </c>
       <c r="N34" s="2" t="n">
-        <v>25602.7462639698</v>
+        <v>25602.74626396982</v>
       </c>
       <c r="O34" s="2" t="n">
-        <v>26243.62718943152</v>
+        <v>26243.62718943147</v>
       </c>
       <c r="P34" s="2" t="n">
-        <v>26686.81663025726</v>
+        <v>26686.8166302572</v>
       </c>
       <c r="Q34" s="2" t="n">
-        <v>26904.66888708492</v>
+        <v>26904.66888708486</v>
       </c>
       <c r="R34" s="2" t="n">
-        <v>26870.38869889748</v>
+        <v>26870.38869889738</v>
       </c>
       <c r="S34" s="1" t="inlineStr"/>
     </row>
@@ -1858,49 +1858,49 @@
       </c>
       <c r="C35" s="1" t="inlineStr"/>
       <c r="D35" s="2" t="n">
-        <v>16.6972711556989</v>
+        <v>16.69727115569871</v>
       </c>
       <c r="E35" s="2" t="n">
-        <v>18.08373681547279</v>
+        <v>18.08373681547265</v>
       </c>
       <c r="F35" s="2" t="n">
-        <v>19.35093521240871</v>
+        <v>19.35093521240866</v>
       </c>
       <c r="G35" s="2" t="n">
-        <v>20.56673424835787</v>
+        <v>20.5667342483578</v>
       </c>
       <c r="H35" s="2" t="n">
-        <v>21.65781275498967</v>
+        <v>21.65781275498965</v>
       </c>
       <c r="I35" s="2" t="n">
-        <v>22.64232024894013</v>
+        <v>22.64232024894005</v>
       </c>
       <c r="J35" s="2" t="n">
-        <v>23.81327704394781</v>
+        <v>23.81327704394782</v>
       </c>
       <c r="K35" s="2" t="n">
         <v>24.88456689222609</v>
       </c>
       <c r="L35" s="2" t="n">
-        <v>25.89839154897781</v>
+        <v>25.8983915489779</v>
       </c>
       <c r="M35" s="2" t="n">
-        <v>26.82431759468589</v>
+        <v>26.82431759468595</v>
       </c>
       <c r="N35" s="2" t="n">
-        <v>27.61009078020989</v>
+        <v>27.61009078020994</v>
       </c>
       <c r="O35" s="2" t="n">
-        <v>28.34277284468556</v>
+        <v>28.34277284468554</v>
       </c>
       <c r="P35" s="2" t="n">
-        <v>28.93863549455284</v>
+        <v>28.93863549455281</v>
       </c>
       <c r="Q35" s="2" t="n">
-        <v>29.38971940023348</v>
+        <v>29.38971940023345</v>
       </c>
       <c r="R35" s="2" t="n">
-        <v>29.65175826002295</v>
+        <v>29.65175826002287</v>
       </c>
       <c r="S35" s="1" t="inlineStr"/>
     </row>
@@ -1917,16 +1917,16 @@
       </c>
       <c r="C36" s="1" t="inlineStr"/>
       <c r="D36" s="2" t="n">
-        <v>304.6972711556989</v>
+        <v>304.6972711556987</v>
       </c>
       <c r="E36" s="2" t="n">
-        <v>334.5400980960846</v>
+        <v>334.5400980960845</v>
       </c>
       <c r="F36" s="2" t="n">
-        <v>364.2636577736324</v>
+        <v>364.2636577736323</v>
       </c>
       <c r="G36" s="2" t="n">
-        <v>393.9358180901934</v>
+        <v>393.9358180901933</v>
       </c>
       <c r="H36" s="2" t="n">
         <v>423.4832578774369</v>
@@ -1941,7 +1941,7 @@
         <v>512.0790958565088</v>
       </c>
       <c r="L36" s="2" t="n">
-        <v>541.5492817938723</v>
+        <v>541.5492817938724</v>
       </c>
       <c r="M36" s="2" t="n">
         <v>570.9315691201923</v>
@@ -1976,16 +1976,16 @@
       </c>
       <c r="C37" s="1" t="inlineStr"/>
       <c r="D37" s="2" t="n">
-        <v>304.6972711556989</v>
+        <v>304.6972711556987</v>
       </c>
       <c r="E37" s="2" t="n">
-        <v>334.5400980960846</v>
+        <v>334.5400980960845</v>
       </c>
       <c r="F37" s="2" t="n">
-        <v>364.2636577736324</v>
+        <v>364.2636577736323</v>
       </c>
       <c r="G37" s="2" t="n">
-        <v>393.9358180901934</v>
+        <v>393.9358180901933</v>
       </c>
       <c r="H37" s="2" t="n">
         <v>423.4832578774369</v>
@@ -2000,7 +2000,7 @@
         <v>512.0790958565088</v>
       </c>
       <c r="L37" s="2" t="n">
-        <v>541.5492817938723</v>
+        <v>541.5492817938724</v>
       </c>
       <c r="M37" s="2" t="n">
         <v>570.9315691201923</v>
@@ -2035,22 +2035,22 @@
       </c>
       <c r="C38" s="1" t="inlineStr"/>
       <c r="D38" s="2" t="n">
-        <v>1.175559285399187</v>
+        <v>1.175559285399185</v>
       </c>
       <c r="E38" s="2" t="n">
-        <v>1.177149157361195</v>
+        <v>1.177149157361193</v>
       </c>
       <c r="F38" s="2" t="n">
         <v>1.177580116958397</v>
       </c>
       <c r="G38" s="2" t="n">
-        <v>1.177095915781244</v>
+        <v>1.177095915781243</v>
       </c>
       <c r="H38" s="2" t="n">
-        <v>1.175855347567406</v>
+        <v>1.175855347567405</v>
       </c>
       <c r="I38" s="2" t="n">
-        <v>1.173962116210552</v>
+        <v>1.173962116210551</v>
       </c>
       <c r="J38" s="2" t="n">
         <v>1.173396175963183</v>
@@ -2059,10 +2059,10 @@
         <v>1.172215437821457</v>
       </c>
       <c r="L38" s="2" t="n">
-        <v>1.170376301404517</v>
+        <v>1.170376301404518</v>
       </c>
       <c r="M38" s="2" t="n">
-        <v>1.167847518639031</v>
+        <v>1.167847518639032</v>
       </c>
       <c r="N38" s="2" t="n">
         <v>1.164588351389238</v>
@@ -2074,7 +2074,7 @@
         <v>1.155630506097777</v>
       </c>
       <c r="Q38" s="2" t="n">
-        <v>1.149848870725617</v>
+        <v>1.149848870725616</v>
       </c>
       <c r="R38" s="2" t="n">
         <v>1.143155604508661</v>
@@ -2094,22 +2094,22 @@
       </c>
       <c r="C39" s="1" t="inlineStr"/>
       <c r="D39" s="2" t="n">
-        <v>117900.225235523</v>
+        <v>117900.2252355229</v>
       </c>
       <c r="E39" s="2" t="n">
-        <v>265350.4672140714</v>
+        <v>265350.467214071</v>
       </c>
       <c r="F39" s="2" t="n">
         <v>412792.3261747835</v>
       </c>
       <c r="G39" s="2" t="n">
-        <v>559906.7201888376</v>
+        <v>559906.720188837</v>
       </c>
       <c r="H39" s="2" t="n">
-        <v>706445.5229259076</v>
+        <v>706445.5229259072</v>
       </c>
       <c r="I39" s="2" t="n">
-        <v>852200.0936189106</v>
+        <v>852200.0936189099</v>
       </c>
       <c r="J39" s="2" t="n">
         <v>998610.46481496</v>
@@ -2118,10 +2118,10 @@
         <v>1144279.063503702</v>
       </c>
       <c r="L39" s="2" t="n">
-        <v>1288927.093135038</v>
+        <v>1288927.093135039</v>
       </c>
       <c r="M39" s="2" t="n">
-        <v>1432269.084259004</v>
+        <v>1432269.084259005</v>
       </c>
       <c r="N39" s="2" t="n">
         <v>1573991.10153848</v>
@@ -2130,10 +2130,10 @@
         <v>1713714.468054943</v>
       </c>
       <c r="P39" s="2" t="n">
-        <v>1851080.725235523</v>
+        <v>1851080.725235522</v>
       </c>
       <c r="Q39" s="2" t="n">
-        <v>1985694.583576011</v>
+        <v>1985694.583576009</v>
       </c>
       <c r="R39" s="2" t="n">
         <v>2117173.208233083</v>
@@ -2153,22 +2153,22 @@
       </c>
       <c r="C40" s="1" t="inlineStr"/>
       <c r="D40" s="2" t="n">
-        <v>117900.225235523</v>
+        <v>117900.2252355229</v>
       </c>
       <c r="E40" s="2" t="n">
-        <v>265350.4672140714</v>
+        <v>265350.467214071</v>
       </c>
       <c r="F40" s="2" t="n">
         <v>412792.3261747835</v>
       </c>
       <c r="G40" s="2" t="n">
-        <v>559906.7201888376</v>
+        <v>559906.720188837</v>
       </c>
       <c r="H40" s="2" t="n">
-        <v>706445.5229259076</v>
+        <v>706445.5229259072</v>
       </c>
       <c r="I40" s="2" t="n">
-        <v>852200.0936189106</v>
+        <v>852200.0936189099</v>
       </c>
       <c r="J40" s="2" t="n">
         <v>998610.46481496</v>
@@ -2177,10 +2177,10 @@
         <v>1144279.063503702</v>
       </c>
       <c r="L40" s="2" t="n">
-        <v>1288927.093135038</v>
+        <v>1288927.093135039</v>
       </c>
       <c r="M40" s="2" t="n">
-        <v>1432269.084259004</v>
+        <v>1432269.084259005</v>
       </c>
       <c r="N40" s="2" t="n">
         <v>1573991.10153848</v>
@@ -2189,10 +2189,10 @@
         <v>1713714.468054943</v>
       </c>
       <c r="P40" s="2" t="n">
-        <v>1851080.725235523</v>
+        <v>1851080.725235522</v>
       </c>
       <c r="Q40" s="2" t="n">
-        <v>1985694.583576011</v>
+        <v>1985694.583576009</v>
       </c>
       <c r="R40" s="2" t="n">
         <v>2117173.208233083</v>
@@ -2271,10 +2271,10 @@
       </c>
       <c r="C42" s="1" t="inlineStr"/>
       <c r="D42" s="2" t="n">
-        <v>319.5338237912142</v>
+        <v>319.5338237912141</v>
       </c>
       <c r="E42" s="2" t="n">
-        <v>334.7109771300942</v>
+        <v>334.7109771300941</v>
       </c>
       <c r="F42" s="2" t="n">
         <v>349.222944744292</v>
@@ -2295,7 +2295,7 @@
         <v>413.3312413404398</v>
       </c>
       <c r="L42" s="2" t="n">
-        <v>424.8720601328997</v>
+        <v>424.8720601328998</v>
       </c>
       <c r="M42" s="2" t="n">
         <v>435.9907411935118</v>
@@ -2389,49 +2389,49 @@
       </c>
       <c r="C44" s="1" t="inlineStr"/>
       <c r="D44" s="2" t="n">
-        <v>0.2675658145409672</v>
+        <v>0.2675658145409686</v>
       </c>
       <c r="E44" s="2" t="n">
-        <v>0.2627510762416364</v>
+        <v>0.2627510762416373</v>
       </c>
       <c r="F44" s="2" t="n">
-        <v>0.2591274840795844</v>
+        <v>0.2591274840795847</v>
       </c>
       <c r="G44" s="2" t="n">
-        <v>0.256576799401226</v>
+        <v>0.2565767994012265</v>
       </c>
       <c r="H44" s="2" t="n">
-        <v>0.2550220951838035</v>
+        <v>0.2550220951838037</v>
       </c>
       <c r="I44" s="2" t="n">
-        <v>0.254393016919423</v>
+        <v>0.2543930169194235</v>
       </c>
       <c r="J44" s="2" t="n">
         <v>0.2546621015587227</v>
       </c>
       <c r="K44" s="2" t="n">
-        <v>0.2558078397057248</v>
+        <v>0.2558078397057247</v>
       </c>
       <c r="L44" s="2" t="n">
-        <v>0.2578470068353897</v>
+        <v>0.2578470068353892</v>
       </c>
       <c r="M44" s="2" t="n">
-        <v>0.2608045797416076</v>
+        <v>0.2608045797416072</v>
       </c>
       <c r="N44" s="2" t="n">
-        <v>0.2647254322067381</v>
+        <v>0.2647254322067377</v>
       </c>
       <c r="O44" s="2" t="n">
-        <v>0.2696810959896801</v>
+        <v>0.2696810959896802</v>
       </c>
       <c r="P44" s="2" t="n">
-        <v>0.2757469847403645</v>
+        <v>0.2757469847403647</v>
       </c>
       <c r="Q44" s="2" t="n">
-        <v>0.2830232632486962</v>
+        <v>0.2830232632486964</v>
       </c>
       <c r="R44" s="2" t="n">
-        <v>0.2916156103246133</v>
+        <v>0.2916156103246137</v>
       </c>
       <c r="S44" s="1" t="inlineStr"/>
     </row>
@@ -2448,13 +2448,13 @@
       </c>
       <c r="C45" s="1" t="inlineStr"/>
       <c r="D45" s="2" t="n">
-        <v>1.241053280171341</v>
+        <v>1.180296158977292</v>
       </c>
       <c r="E45" s="2" t="n">
-        <v>1.175262487903347</v>
+        <v>1.175262487903346</v>
       </c>
       <c r="F45" s="2" t="n">
-        <v>1.168251369555617</v>
+        <v>1.168251369555616</v>
       </c>
       <c r="G45" s="2" t="n">
         <v>1.15925817796077</v>
@@ -2463,7 +2463,7 @@
         <v>1.148224245120433</v>
       </c>
       <c r="I45" s="2" t="n">
-        <v>1.135081723832521</v>
+        <v>1.13508172383252</v>
       </c>
       <c r="J45" s="2" t="n">
         <v>1.119697021419855</v>
@@ -2472,10 +2472,10 @@
         <v>1.101922316939652</v>
       </c>
       <c r="L45" s="2" t="n">
-        <v>1.081544540058967</v>
+        <v>1.081544540058968</v>
       </c>
       <c r="M45" s="2" t="n">
-        <v>1.058332062101629</v>
+        <v>1.05833206210163</v>
       </c>
       <c r="N45" s="2" t="n">
         <v>1.032020278583349</v>
@@ -2484,13 +2484,13 @@
         <v>1.0023075858643</v>
       </c>
       <c r="P45" s="2" t="n">
-        <v>0.9689068762009189</v>
+        <v>0.9689068762009185</v>
       </c>
       <c r="Q45" s="2" t="n">
-        <v>0.9315321714560333</v>
+        <v>0.9315321714560331</v>
       </c>
       <c r="R45" s="2" t="n">
-        <v>0.8899613152251319</v>
+        <v>0.8899613152251311</v>
       </c>
       <c r="S45" s="1" t="inlineStr"/>
     </row>
@@ -2566,22 +2566,22 @@
       </c>
       <c r="C47" s="1" t="inlineStr"/>
       <c r="D47" s="2" t="n">
-        <v>0.6777265196059805</v>
+        <v>0.6934155588636791</v>
       </c>
       <c r="E47" s="2" t="n">
-        <v>0.6419546944869913</v>
+        <v>0.6419546944869916</v>
       </c>
       <c r="F47" s="2" t="n">
-        <v>0.5966106211168183</v>
+        <v>0.5966106211168185</v>
       </c>
       <c r="G47" s="2" t="n">
-        <v>0.5561238216798053</v>
+        <v>0.5561238216798055</v>
       </c>
       <c r="H47" s="2" t="n">
         <v>0.5198537807125588</v>
       </c>
       <c r="I47" s="2" t="n">
-        <v>0.4871134947236217</v>
+        <v>0.4871134947236219</v>
       </c>
       <c r="J47" s="2" t="n">
         <v>0.4573452836046674</v>
@@ -2590,13 +2590,13 @@
         <v>0.4302607947475137</v>
       </c>
       <c r="L47" s="2" t="n">
-        <v>0.4054971202086974</v>
+        <v>0.4054971202086972</v>
       </c>
       <c r="M47" s="2" t="n">
-        <v>0.382866877454614</v>
+        <v>0.3828668774546138</v>
       </c>
       <c r="N47" s="2" t="n">
-        <v>0.3622495702925325</v>
+        <v>0.3622495702925324</v>
       </c>
       <c r="O47" s="2" t="n">
         <v>0.3434267211217917</v>
@@ -2605,10 +2605,10 @@
         <v>0.3264013915200195</v>
       </c>
       <c r="Q47" s="2" t="n">
-        <v>0.3111320861419942</v>
+        <v>0.3111320861419943</v>
       </c>
       <c r="R47" s="2" t="n">
-        <v>0.2976385445704193</v>
+        <v>0.2976385445704194</v>
       </c>
       <c r="S47" s="1" t="inlineStr"/>
     </row>
@@ -2625,22 +2625,22 @@
       </c>
       <c r="C48" s="1" t="inlineStr"/>
       <c r="D48" s="2" t="n">
-        <v>0.8760708611733966</v>
+        <v>0.8876763917513484</v>
       </c>
       <c r="E48" s="2" t="n">
-        <v>0.8476827557110529</v>
+        <v>0.8476827557110533</v>
       </c>
       <c r="F48" s="2" t="n">
-        <v>0.807838102390409</v>
+        <v>0.8078381023904093</v>
       </c>
       <c r="G48" s="2" t="n">
-        <v>0.7687303178641441</v>
+        <v>0.7687303178641439</v>
       </c>
       <c r="H48" s="2" t="n">
-        <v>0.7310690251477328</v>
+        <v>0.7310690251477326</v>
       </c>
       <c r="I48" s="2" t="n">
-        <v>0.6950438015492818</v>
+        <v>0.695043801549282</v>
       </c>
       <c r="J48" s="2" t="n">
         <v>0.6606666216532919</v>
@@ -2649,25 +2649,25 @@
         <v>0.6281613417983278</v>
       </c>
       <c r="L48" s="2" t="n">
-        <v>0.5974295303378844</v>
+        <v>0.5974295303378842</v>
       </c>
       <c r="M48" s="2" t="n">
-        <v>0.5685574328276755</v>
+        <v>0.5685574328276751</v>
       </c>
       <c r="N48" s="2" t="n">
-        <v>0.5416626339362809</v>
+        <v>0.5416626339362808</v>
       </c>
       <c r="O48" s="2" t="n">
         <v>0.5165679427658935</v>
       </c>
       <c r="P48" s="2" t="n">
-        <v>0.4934870266617923</v>
+        <v>0.4934870266617922</v>
       </c>
       <c r="Q48" s="2" t="n">
-        <v>0.4724845076896956</v>
+        <v>0.4724845076896957</v>
       </c>
       <c r="R48" s="2" t="n">
-        <v>0.4537118711400231</v>
+        <v>0.4537118711400232</v>
       </c>
       <c r="S48" s="1" t="inlineStr"/>
     </row>
@@ -2684,7 +2684,7 @@
       </c>
       <c r="C49" s="1" t="inlineStr"/>
       <c r="D49" s="2" t="n">
-        <v>0.2979995060628132</v>
+        <v>0.3009117955899138</v>
       </c>
       <c r="E49" s="2" t="n">
         <v>0.1472682986886746</v>
@@ -2693,10 +2693,10 @@
         <v>0.1040512028785386</v>
       </c>
       <c r="G49" s="2" t="n">
-        <v>0.08416531485429166</v>
+        <v>0.08416531485429168</v>
       </c>
       <c r="H49" s="2" t="n">
-        <v>0.07304667532585596</v>
+        <v>0.07304667532585597</v>
       </c>
       <c r="I49" s="2" t="n">
         <v>0.06619932070733821</v>
@@ -2708,7 +2708,7 @@
         <v>0.05890202559086238</v>
       </c>
       <c r="L49" s="2" t="n">
-        <v>0.05707687219159215</v>
+        <v>0.05707687219159214</v>
       </c>
       <c r="M49" s="2" t="n">
         <v>0.05602993268923052</v>
@@ -2720,13 +2720,13 @@
         <v>0.0556712005930268</v>
       </c>
       <c r="P49" s="2" t="n">
-        <v>0.05621043688048771</v>
+        <v>0.05621043688048773</v>
       </c>
       <c r="Q49" s="2" t="n">
         <v>0.05718010096659844</v>
       </c>
       <c r="R49" s="2" t="n">
-        <v>0.05857117009930012</v>
+        <v>0.05857117009930016</v>
       </c>
       <c r="S49" s="1" t="inlineStr"/>
     </row>
@@ -2861,22 +2861,22 @@
       </c>
       <c r="C52" s="1" t="inlineStr"/>
       <c r="D52" s="2" t="n">
-        <v>0.6380894771611995</v>
+        <v>0.652860938167221</v>
       </c>
       <c r="E52" s="2" t="n">
-        <v>0.6040008906918644</v>
+        <v>0.6040008906918648</v>
       </c>
       <c r="F52" s="2" t="n">
-        <v>0.5608528404519376</v>
+        <v>0.5608528404519377</v>
       </c>
       <c r="G52" s="2" t="n">
-        <v>0.5224733005942056</v>
+        <v>0.5224733005942057</v>
       </c>
       <c r="H52" s="2" t="n">
         <v>0.4880639358485558</v>
       </c>
       <c r="I52" s="2" t="n">
-        <v>0.4569203160469202</v>
+        <v>0.4569203160469203</v>
       </c>
       <c r="J52" s="2" t="n">
         <v>0.4285352724020985</v>
@@ -2885,25 +2885,25 @@
         <v>0.4026243969644493</v>
       </c>
       <c r="L52" s="2" t="n">
-        <v>0.3789240751115422</v>
+        <v>0.378924075111542</v>
       </c>
       <c r="M52" s="2" t="n">
-        <v>0.3572719824747077</v>
+        <v>0.3572719824747075</v>
       </c>
       <c r="N52" s="2" t="n">
-        <v>0.3374139715597593</v>
+        <v>0.3374139715597592</v>
       </c>
       <c r="O52" s="2" t="n">
         <v>0.3192848027412507</v>
       </c>
       <c r="P52" s="2" t="n">
-        <v>0.3028179399616254</v>
+        <v>0.3028179399616255</v>
       </c>
       <c r="Q52" s="2" t="n">
-        <v>0.2879901483751846</v>
+        <v>0.2879901483751847</v>
       </c>
       <c r="R52" s="2" t="n">
-        <v>0.2747820638038408</v>
+        <v>0.2747820638038409</v>
       </c>
       <c r="S52" s="1" t="inlineStr"/>
     </row>
@@ -2920,22 +2920,22 @@
       </c>
       <c r="C53" s="1" t="inlineStr"/>
       <c r="D53" s="2" t="n">
-        <v>0.8444462060062202</v>
+        <v>0.856644940865214</v>
       </c>
       <c r="E53" s="2" t="n">
-        <v>0.8146305802312926</v>
+        <v>0.814630580231293</v>
       </c>
       <c r="F53" s="2" t="n">
-        <v>0.7734667621979159</v>
+        <v>0.773466762197916</v>
       </c>
       <c r="G53" s="2" t="n">
-        <v>0.7338759548743808</v>
+        <v>0.733875954874381</v>
       </c>
       <c r="H53" s="2" t="n">
         <v>0.6961191242501733</v>
       </c>
       <c r="I53" s="2" t="n">
-        <v>0.6601638683567802</v>
+        <v>0.6601638683567803</v>
       </c>
       <c r="J53" s="2" t="n">
         <v>0.6260427988521639</v>
@@ -2944,25 +2944,25 @@
         <v>0.5937907596548805</v>
       </c>
       <c r="L53" s="2" t="n">
-        <v>0.5634296976475788</v>
+        <v>0.5634296976475786</v>
       </c>
       <c r="M53" s="2" t="n">
-        <v>0.5350423151502405</v>
+        <v>0.5350423151502401</v>
       </c>
       <c r="N53" s="2" t="n">
-        <v>0.5084161145598954</v>
+        <v>0.5084161145598953</v>
       </c>
       <c r="O53" s="2" t="n">
         <v>0.4836795065578707</v>
       </c>
       <c r="P53" s="2" t="n">
-        <v>0.4608658406019039</v>
+        <v>0.460865840601904</v>
       </c>
       <c r="Q53" s="2" t="n">
-        <v>0.4400685175575864</v>
+        <v>0.4400685175575865</v>
       </c>
       <c r="R53" s="2" t="n">
-        <v>0.4213432296968064</v>
+        <v>0.4213432296968065</v>
       </c>
       <c r="S53" s="1" t="inlineStr"/>
     </row>
@@ -2979,22 +2979,22 @@
       </c>
       <c r="C54" s="1" t="inlineStr"/>
       <c r="D54" s="2" t="n">
-        <v>0.2705056205597923</v>
+        <v>0.2728264862976842</v>
       </c>
       <c r="E54" s="2" t="n">
-        <v>0.1338497572918128</v>
+        <v>0.1338497572918129</v>
       </c>
       <c r="F54" s="2" t="n">
         <v>0.09484023765812551</v>
       </c>
       <c r="G54" s="2" t="n">
-        <v>0.07693362720631663</v>
+        <v>0.07693362720631673</v>
       </c>
       <c r="H54" s="2" t="n">
-        <v>0.0669762425432088</v>
+        <v>0.06697624254320884</v>
       </c>
       <c r="I54" s="2" t="n">
-        <v>0.06091105339602894</v>
+        <v>0.06091105339602899</v>
       </c>
       <c r="J54" s="2" t="n">
         <v>0.05699304098048162</v>
@@ -3003,10 +3003,10 @@
         <v>0.05449766392638357</v>
       </c>
       <c r="L54" s="2" t="n">
-        <v>0.05299351220560669</v>
+        <v>0.05299351220560665</v>
       </c>
       <c r="M54" s="2" t="n">
-        <v>0.05222397695379562</v>
+        <v>0.05222397695379559</v>
       </c>
       <c r="N54" s="2" t="n">
         <v>0.05206385535377919</v>
@@ -3018,10 +3018,10 @@
         <v>0.05326713372110947</v>
       </c>
       <c r="Q54" s="2" t="n">
-        <v>0.05457087868506504</v>
+        <v>0.05457087868506506</v>
       </c>
       <c r="R54" s="2" t="n">
-        <v>0.05635161751966029</v>
+        <v>0.05635161751966031</v>
       </c>
       <c r="S54" s="1" t="inlineStr"/>
     </row>
@@ -3038,16 +3038,16 @@
       </c>
       <c r="C55" s="1" t="inlineStr"/>
       <c r="D55" s="2" t="n">
-        <v>0.5067945619819988</v>
+        <v>0.5004644049712288</v>
       </c>
       <c r="E55" s="2" t="n">
-        <v>0.7951571965663656</v>
+        <v>0.7951571965663653</v>
       </c>
       <c r="F55" s="2" t="n">
         <v>0.8599102873979747</v>
       </c>
       <c r="G55" s="2" t="n">
-        <v>0.8880543221133667</v>
+        <v>0.8880543221133665</v>
       </c>
       <c r="H55" s="2" t="n">
         <v>0.9033251749764167</v>
@@ -3065,7 +3065,7 @@
         <v>0.9243435965300111</v>
       </c>
       <c r="M55" s="2" t="n">
-        <v>0.9254864808911322</v>
+        <v>0.9254864808911323</v>
       </c>
       <c r="N55" s="2" t="n">
         <v>0.9257241100343748</v>
@@ -3080,7 +3080,7 @@
         <v>0.921996524014703</v>
       </c>
       <c r="R55" s="2" t="n">
-        <v>0.9193396390285498</v>
+        <v>0.9193396390285495</v>
       </c>
       <c r="S55" s="1" t="inlineStr"/>
     </row>
@@ -3097,13 +3097,13 @@
       </c>
       <c r="C56" s="1" t="inlineStr"/>
       <c r="D56" s="2" t="n">
-        <v>0.7979533943538226</v>
+        <v>0.7925571175792671</v>
       </c>
       <c r="E56" s="2" t="n">
-        <v>0.9071180477959627</v>
+        <v>0.9071180477959626</v>
       </c>
       <c r="F56" s="2" t="n">
-        <v>0.9358895185677403</v>
+        <v>0.9358895185677402</v>
       </c>
       <c r="G56" s="2" t="n">
         <v>0.948685461697101</v>
@@ -3156,49 +3156,49 @@
       </c>
       <c r="C57" s="1" t="inlineStr"/>
       <c r="D57" s="2" t="n">
-        <v>0.2824829975607913</v>
+        <v>0.2811863433358094</v>
       </c>
       <c r="E57" s="2" t="n">
-        <v>0.3419728067953003</v>
+        <v>0.341972806795301</v>
       </c>
       <c r="F57" s="2" t="n">
-        <v>0.3509410655936228</v>
+        <v>0.350941065593623</v>
       </c>
       <c r="G57" s="2" t="n">
-        <v>0.3505057511486546</v>
+        <v>0.350505751148655</v>
       </c>
       <c r="H57" s="2" t="n">
-        <v>0.3468279629635574</v>
+        <v>0.3468279629635576</v>
       </c>
       <c r="I57" s="2" t="n">
-        <v>0.3417081181479366</v>
+        <v>0.3417081181479371</v>
       </c>
       <c r="J57" s="2" t="n">
         <v>0.3359234221056464</v>
       </c>
       <c r="K57" s="2" t="n">
-        <v>0.3297983277471504</v>
+        <v>0.3297983277471503</v>
       </c>
       <c r="L57" s="2" t="n">
-        <v>0.3235650470477323</v>
+        <v>0.3235650470477318</v>
       </c>
       <c r="M57" s="2" t="n">
-        <v>0.31739063742177</v>
+        <v>0.3173906374217697</v>
       </c>
       <c r="N57" s="2" t="n">
-        <v>0.3114061941828092</v>
+        <v>0.3114061941828089</v>
       </c>
       <c r="O57" s="2" t="n">
-        <v>0.3057573784837125</v>
+        <v>0.3057573784837126</v>
       </c>
       <c r="P57" s="2" t="n">
-        <v>0.3005825024172691</v>
+        <v>0.3005825024172694</v>
       </c>
       <c r="Q57" s="2" t="n">
-        <v>0.2960388638501384</v>
+        <v>0.2960388638501387</v>
       </c>
       <c r="R57" s="2" t="n">
-        <v>0.2922862607409257</v>
+        <v>0.2922862607409261</v>
       </c>
       <c r="S57" s="1" t="inlineStr"/>
     </row>
@@ -3215,7 +3215,7 @@
       </c>
       <c r="C58" s="1" t="inlineStr"/>
       <c r="D58" s="2" t="n">
-        <v>1.148861981379653</v>
+        <v>1.150578245989657</v>
       </c>
       <c r="E58" s="2" t="n">
         <v>1.058842137058633</v>
@@ -3224,13 +3224,13 @@
         <v>1.03259772936633</v>
       </c>
       <c r="G58" s="2" t="n">
-        <v>1.017231933919797</v>
+        <v>1.017231933919796</v>
       </c>
       <c r="H58" s="2" t="n">
-        <v>1.005239401872601</v>
+        <v>1.0052394018726</v>
       </c>
       <c r="I58" s="2" t="n">
-        <v>0.9944293535476197</v>
+        <v>0.9944293535476192</v>
       </c>
       <c r="J58" s="2" t="n">
         <v>0.9838133341616834</v>
@@ -3239,25 +3239,25 @@
         <v>0.9729365229403433</v>
       </c>
       <c r="L58" s="2" t="n">
-        <v>0.9614252343707766</v>
+        <v>0.9614252343707773</v>
       </c>
       <c r="M58" s="2" t="n">
-        <v>0.9489575905895593</v>
+        <v>0.9489575905895599</v>
       </c>
       <c r="N58" s="2" t="n">
-        <v>0.9352269846819268</v>
+        <v>0.9352269846819273</v>
       </c>
       <c r="O58" s="2" t="n">
-        <v>0.9198661432115165</v>
+        <v>0.9198661432115164</v>
       </c>
       <c r="P58" s="2" t="n">
-        <v>0.9024768235733482</v>
+        <v>0.9024768235733479</v>
       </c>
       <c r="Q58" s="2" t="n">
-        <v>0.8825869545836461</v>
+        <v>0.8825869545836458</v>
       </c>
       <c r="R58" s="2" t="n">
-        <v>0.8596778720441994</v>
+        <v>0.8596778720441987</v>
       </c>
       <c r="S58" s="1" t="inlineStr"/>
     </row>
@@ -3274,22 +3274,22 @@
       </c>
       <c r="C59" s="1" t="inlineStr"/>
       <c r="D59" s="2" t="n">
-        <v>0.6617491813593513</v>
+        <v>0.6612407210601751</v>
       </c>
       <c r="E59" s="2" t="n">
-        <v>0.6393366808686474</v>
+        <v>0.6393366808686478</v>
       </c>
       <c r="F59" s="2" t="n">
-        <v>0.6009807379947486</v>
+        <v>0.6009807379947487</v>
       </c>
       <c r="G59" s="2" t="n">
-        <v>0.5629187482016862</v>
+        <v>0.5629187482016864</v>
       </c>
       <c r="H59" s="2" t="n">
-        <v>0.5272267598629743</v>
+        <v>0.5272267598629744</v>
       </c>
       <c r="I59" s="2" t="n">
-        <v>0.4940432659250179</v>
+        <v>0.4940432659250182</v>
       </c>
       <c r="J59" s="2" t="n">
         <v>0.4632008778470891</v>
@@ -3298,13 +3298,13 @@
         <v>0.434547983835321</v>
       </c>
       <c r="L59" s="2" t="n">
-        <v>0.4078868049211564</v>
+        <v>0.4078868049211561</v>
       </c>
       <c r="M59" s="2" t="n">
-        <v>0.3830869581536965</v>
+        <v>0.3830869581536963</v>
       </c>
       <c r="N59" s="2" t="n">
-        <v>0.3598891790707875</v>
+        <v>0.3598891790707873</v>
       </c>
       <c r="O59" s="2" t="n">
         <v>0.3382266797622753</v>
@@ -3313,10 +3313,10 @@
         <v>0.3180205486364964</v>
       </c>
       <c r="Q59" s="2" t="n">
-        <v>0.2992319827470267</v>
+        <v>0.2992319827470268</v>
       </c>
       <c r="R59" s="2" t="n">
-        <v>0.2818236131273244</v>
+        <v>0.2818236131273246</v>
       </c>
       <c r="S59" s="1" t="inlineStr"/>
     </row>
@@ -3333,22 +3333,22 @@
       </c>
       <c r="C60" s="1" t="inlineStr"/>
       <c r="D60" s="2" t="n">
-        <v>0.2644565799050165</v>
+        <v>0.2707047831582413</v>
       </c>
       <c r="E60" s="2" t="n">
-        <v>0.1289535490674906</v>
+        <v>0.1289535490674907</v>
       </c>
       <c r="F60" s="2" t="n">
-        <v>0.09035121456081503</v>
+        <v>0.09035121456081506</v>
       </c>
       <c r="G60" s="2" t="n">
-        <v>0.07279583956722309</v>
+        <v>0.07279583956722319</v>
       </c>
       <c r="H60" s="2" t="n">
-        <v>0.0630871303195517</v>
+        <v>0.06308713031955175</v>
       </c>
       <c r="I60" s="2" t="n">
-        <v>0.0572051495289134</v>
+        <v>0.05720514952891342</v>
       </c>
       <c r="J60" s="2" t="n">
         <v>0.05343833731776829</v>
@@ -3357,13 +3357,13 @@
         <v>0.05108008787467855</v>
       </c>
       <c r="L60" s="2" t="n">
-        <v>0.04971625102356635</v>
+        <v>0.04971625102356633</v>
       </c>
       <c r="M60" s="2" t="n">
-        <v>0.04910680533129995</v>
+        <v>0.04910680533129991</v>
       </c>
       <c r="N60" s="2" t="n">
-        <v>0.04914211499311783</v>
+        <v>0.04914211499311785</v>
       </c>
       <c r="O60" s="2" t="n">
         <v>0.04975559312298664</v>
@@ -3372,10 +3372,10 @@
         <v>0.0509264267870588</v>
       </c>
       <c r="Q60" s="2" t="n">
-        <v>0.05266952243484315</v>
+        <v>0.05266952243484317</v>
       </c>
       <c r="R60" s="2" t="n">
-        <v>0.05503600366715333</v>
+        <v>0.05503600366715335</v>
       </c>
       <c r="S60" s="1" t="inlineStr"/>
     </row>
@@ -3392,19 +3392,19 @@
       </c>
       <c r="C61" s="1" t="inlineStr"/>
       <c r="D61" s="2" t="n">
-        <v>0.1289535490674906</v>
+        <v>0.1289535490674907</v>
       </c>
       <c r="E61" s="2" t="n">
-        <v>0.09035121456081503</v>
+        <v>0.09035121456081506</v>
       </c>
       <c r="F61" s="2" t="n">
-        <v>0.07279583956722309</v>
+        <v>0.07279583956722319</v>
       </c>
       <c r="G61" s="2" t="n">
-        <v>0.0630871303195517</v>
+        <v>0.06308713031955175</v>
       </c>
       <c r="H61" s="2" t="n">
-        <v>0.0572051495289134</v>
+        <v>0.05720514952891342</v>
       </c>
       <c r="I61" s="2" t="n">
         <v>0.05343833731776829</v>
@@ -3413,13 +3413,13 @@
         <v>0.05108008787467855</v>
       </c>
       <c r="K61" s="2" t="n">
-        <v>0.04971625102356635</v>
+        <v>0.04971625102356633</v>
       </c>
       <c r="L61" s="2" t="n">
-        <v>0.04910680533129995</v>
+        <v>0.04910680533129991</v>
       </c>
       <c r="M61" s="2" t="n">
-        <v>0.04914211499311783</v>
+        <v>0.04914211499311785</v>
       </c>
       <c r="N61" s="2" t="n">
         <v>0.04975559312298664</v>
@@ -3428,13 +3428,13 @@
         <v>0.0509264267870588</v>
       </c>
       <c r="P61" s="2" t="n">
-        <v>0.05266952243484315</v>
+        <v>0.05266952243484317</v>
       </c>
       <c r="Q61" s="2" t="n">
-        <v>0.05503600366715333</v>
+        <v>0.05503600366715335</v>
       </c>
       <c r="R61" s="2" t="n">
-        <v>0.05740248489946351</v>
+        <v>0.05740248489946354</v>
       </c>
       <c r="S61" s="1" t="inlineStr"/>
     </row>
@@ -3451,16 +3451,16 @@
       </c>
       <c r="C62" s="1" t="inlineStr"/>
       <c r="D62" s="2" t="n">
-        <v>0.5229333027467026</v>
+        <v>0.5062544510926422</v>
       </c>
       <c r="E62" s="2" t="n">
-        <v>0.8035709709007146</v>
+        <v>0.8035709709007143</v>
       </c>
       <c r="F62" s="2" t="n">
-        <v>0.8670515451401452</v>
+        <v>0.8670515451401449</v>
       </c>
       <c r="G62" s="2" t="n">
-        <v>0.8944317807808952</v>
+        <v>0.8944317807808951</v>
       </c>
       <c r="H62" s="2" t="n">
         <v>0.9092199502745679</v>
@@ -3510,13 +3510,13 @@
       </c>
       <c r="C63" s="1" t="inlineStr"/>
       <c r="D63" s="2" t="n">
-        <v>0.7838305655477515</v>
+        <v>0.7811324271604738</v>
       </c>
       <c r="E63" s="2" t="n">
-        <v>0.8434383830980788</v>
+        <v>0.8434383830980787</v>
       </c>
       <c r="F63" s="2" t="n">
-        <v>0.8631690556287381</v>
+        <v>0.863169055628738</v>
       </c>
       <c r="G63" s="2" t="n">
         <v>0.8752186331837397</v>
@@ -3569,49 +3569,49 @@
       </c>
       <c r="C64" s="1" t="inlineStr"/>
       <c r="D64" s="2" t="n">
-        <v>0.49309447659793</v>
+        <v>0.4947976924542974</v>
       </c>
       <c r="E64" s="2" t="n">
-        <v>0.4779735242447286</v>
+        <v>0.4779735242447278</v>
       </c>
       <c r="F64" s="2" t="n">
-        <v>0.4865582469952273</v>
+        <v>0.486558246995227</v>
       </c>
       <c r="G64" s="2" t="n">
-        <v>0.4994124070984718</v>
+        <v>0.4994124070984713</v>
       </c>
       <c r="H64" s="2" t="n">
         <v>0.5137734390610369</v>
       </c>
       <c r="I64" s="2" t="n">
-        <v>0.5288702372127254</v>
+        <v>0.5288702372127249</v>
       </c>
       <c r="J64" s="2" t="n">
-        <v>0.5443607442121166</v>
+        <v>0.5443607442121167</v>
       </c>
       <c r="K64" s="2" t="n">
         <v>0.5600965560548041</v>
       </c>
       <c r="L64" s="2" t="n">
-        <v>0.5759477597191387</v>
+        <v>0.5759477597191393</v>
       </c>
       <c r="M64" s="2" t="n">
-        <v>0.5918081993459784</v>
+        <v>0.5918081993459788</v>
       </c>
       <c r="N64" s="2" t="n">
-        <v>0.6075771359846209</v>
+        <v>0.6075771359846212</v>
       </c>
       <c r="O64" s="2" t="n">
-        <v>0.6231339534389799</v>
+        <v>0.6231339534389797</v>
       </c>
       <c r="P64" s="2" t="n">
-        <v>0.6383608968284006</v>
+        <v>0.6383608968284005</v>
       </c>
       <c r="Q64" s="2" t="n">
-        <v>0.6531207208541026</v>
+        <v>0.6531207208541023</v>
       </c>
       <c r="R64" s="2" t="n">
-        <v>0.6672755281010996</v>
+        <v>0.6672755281010991</v>
       </c>
       <c r="S64" s="1" t="inlineStr"/>
     </row>
@@ -3628,22 +3628,22 @@
       </c>
       <c r="C65" s="1" t="inlineStr"/>
       <c r="D65" s="2" t="n">
-        <v>0.9130337357818</v>
+        <v>0.9130337357818012</v>
       </c>
       <c r="E65" s="2" t="n">
-        <v>0.8830355266498334</v>
+        <v>0.8830355266498343</v>
       </c>
       <c r="F65" s="2" t="n">
-        <v>0.8530645253444216</v>
+        <v>0.8530645253444218</v>
       </c>
       <c r="G65" s="2" t="n">
-        <v>0.8230510799514991</v>
+        <v>0.8230510799514995</v>
       </c>
       <c r="H65" s="2" t="n">
-        <v>0.7929681334991677</v>
+        <v>0.7929681334991679</v>
       </c>
       <c r="I65" s="2" t="n">
-        <v>0.7627977092904863</v>
+        <v>0.7627977092904867</v>
       </c>
       <c r="J65" s="2" t="n">
         <v>0.7325616461288711</v>
@@ -3652,25 +3652,25 @@
         <v>0.7022863254977531</v>
       </c>
       <c r="L65" s="2" t="n">
-        <v>0.6720276223556498</v>
+        <v>0.6720276223556494</v>
       </c>
       <c r="M65" s="2" t="n">
-        <v>0.6418422361217935</v>
+        <v>0.6418422361217931</v>
       </c>
       <c r="N65" s="2" t="n">
-        <v>0.611794636858556</v>
+        <v>0.6117946368585556</v>
       </c>
       <c r="O65" s="2" t="n">
         <v>0.5819584578441279</v>
       </c>
       <c r="P65" s="2" t="n">
-        <v>0.552396365214525</v>
+        <v>0.5523963652145252</v>
       </c>
       <c r="Q65" s="2" t="n">
-        <v>0.5231726932408487</v>
+        <v>0.5231726932408488</v>
       </c>
       <c r="R65" s="2" t="n">
-        <v>0.4943374292495647</v>
+        <v>0.494337429249565</v>
       </c>
       <c r="S65" s="1" t="inlineStr"/>
     </row>
@@ -3746,49 +3746,49 @@
       </c>
       <c r="C67" s="1" t="inlineStr"/>
       <c r="D67" s="2" t="n">
-        <v>1.144182651182124</v>
+        <v>1.149900190948777</v>
       </c>
       <c r="E67" s="2" t="n">
-        <v>1.037406335378524</v>
+        <v>1.037406335378523</v>
       </c>
       <c r="F67" s="2" t="n">
         <v>1.008925798296564</v>
       </c>
       <c r="G67" s="2" t="n">
-        <v>0.9938963560643232</v>
+        <v>0.9938963560643226</v>
       </c>
       <c r="H67" s="2" t="n">
         <v>0.9831646987246834</v>
       </c>
       <c r="I67" s="2" t="n">
-        <v>0.9741269377820952</v>
+        <v>0.9741269377820945</v>
       </c>
       <c r="J67" s="2" t="n">
-        <v>0.9656506714457721</v>
+        <v>0.9656506714457722</v>
       </c>
       <c r="K67" s="2" t="n">
         <v>0.9572427390595025</v>
       </c>
       <c r="L67" s="2" t="n">
-        <v>0.9485264056880329</v>
+        <v>0.9485264056880337</v>
       </c>
       <c r="M67" s="2" t="n">
-        <v>0.9392010422085477</v>
+        <v>0.9392010422085484</v>
       </c>
       <c r="N67" s="2" t="n">
-        <v>0.9290023750862315</v>
+        <v>0.9290023750862318</v>
       </c>
       <c r="O67" s="2" t="n">
-        <v>0.9176220242343975</v>
+        <v>0.9176220242343971</v>
       </c>
       <c r="P67" s="2" t="n">
-        <v>0.9047385458666748</v>
+        <v>0.9047385458666746</v>
       </c>
       <c r="Q67" s="2" t="n">
-        <v>0.8899750486647011</v>
+        <v>0.8899750486647007</v>
       </c>
       <c r="R67" s="2" t="n">
-        <v>0.8729257643027138</v>
+        <v>0.872925764302713</v>
       </c>
       <c r="S67" s="1" t="inlineStr"/>
     </row>
@@ -3805,22 +3805,22 @@
       </c>
       <c r="C68" s="1" t="inlineStr"/>
       <c r="D68" s="2" t="n">
-        <v>0.9140589290878374</v>
+        <v>0.9123908734224133</v>
       </c>
       <c r="E68" s="2" t="n">
-        <v>0.9132006195531562</v>
+        <v>0.9132006195531571</v>
       </c>
       <c r="F68" s="2" t="n">
-        <v>0.887967323159673</v>
+        <v>0.8879673231596732</v>
       </c>
       <c r="G68" s="2" t="n">
-        <v>0.8577821070040713</v>
+        <v>0.8577821070040718</v>
       </c>
       <c r="H68" s="2" t="n">
         <v>0.8255539583207618</v>
       </c>
       <c r="I68" s="2" t="n">
-        <v>0.792160112745544</v>
+        <v>0.7921601127455445</v>
       </c>
       <c r="J68" s="2" t="n">
         <v>0.7580358219315676</v>
@@ -3829,25 +3829,25 @@
         <v>0.72342089195214</v>
       </c>
       <c r="L68" s="2" t="n">
-        <v>0.6885297165190225</v>
+        <v>0.6885297165190221</v>
       </c>
       <c r="M68" s="2" t="n">
-        <v>0.6535447189435526</v>
+        <v>0.6535447189435523</v>
       </c>
       <c r="N68" s="2" t="n">
-        <v>0.6186306556226798</v>
+        <v>0.6186306556226797</v>
       </c>
       <c r="O68" s="2" t="n">
-        <v>0.5839510578580409</v>
+        <v>0.583951057858041</v>
       </c>
       <c r="P68" s="2" t="n">
-        <v>0.5496458774495508</v>
+        <v>0.549645877449551</v>
       </c>
       <c r="Q68" s="2" t="n">
-        <v>0.5158449565439994</v>
+        <v>0.5158449565439995</v>
       </c>
       <c r="R68" s="2" t="n">
-        <v>0.4826515564353129</v>
+        <v>0.4826515564353131</v>
       </c>
       <c r="S68" s="1" t="inlineStr"/>
     </row>
@@ -3864,49 +3864,49 @@
       </c>
       <c r="C69" s="1" t="inlineStr"/>
       <c r="D69" s="2" t="n">
-        <v>0.2311489154003236</v>
+        <v>0.2368664551669755</v>
       </c>
       <c r="E69" s="2" t="n">
-        <v>0.1543708087286905</v>
+        <v>0.1543708087286889</v>
       </c>
       <c r="F69" s="2" t="n">
-        <v>0.1558612729521429</v>
+        <v>0.1558612729521425</v>
       </c>
       <c r="G69" s="2" t="n">
-        <v>0.1708452761128242</v>
+        <v>0.1708452761128231</v>
       </c>
       <c r="H69" s="2" t="n">
-        <v>0.1901965652255156</v>
+        <v>0.1901965652255154</v>
       </c>
       <c r="I69" s="2" t="n">
-        <v>0.211329228491609</v>
+        <v>0.2113292284916077</v>
       </c>
       <c r="J69" s="2" t="n">
-        <v>0.233089025316901</v>
+        <v>0.2330890253169011</v>
       </c>
       <c r="K69" s="2" t="n">
         <v>0.2549564135617495</v>
       </c>
       <c r="L69" s="2" t="n">
-        <v>0.2764987833323831</v>
+        <v>0.2764987833323843</v>
       </c>
       <c r="M69" s="2" t="n">
-        <v>0.2973588060867542</v>
+        <v>0.2973588060867552</v>
       </c>
       <c r="N69" s="2" t="n">
-        <v>0.3172077382276756</v>
+        <v>0.3172077382276762</v>
       </c>
       <c r="O69" s="2" t="n">
-        <v>0.3356635663902696</v>
+        <v>0.3356635663902692</v>
       </c>
       <c r="P69" s="2" t="n">
-        <v>0.3523421806521498</v>
+        <v>0.3523421806521494</v>
       </c>
       <c r="Q69" s="2" t="n">
-        <v>0.3668023554238524</v>
+        <v>0.3668023554238519</v>
       </c>
       <c r="R69" s="2" t="n">
-        <v>0.3785883350531491</v>
+        <v>0.3785883350531479</v>
       </c>
       <c r="S69" s="1" t="inlineStr"/>
     </row>
@@ -3923,22 +3923,22 @@
       </c>
       <c r="C70" s="1" t="inlineStr"/>
       <c r="D70" s="2" t="n">
-        <v>0.2348030522918152</v>
+        <v>0.2381873725672434</v>
       </c>
       <c r="E70" s="2" t="n">
-        <v>0.1456415175054772</v>
+        <v>0.1456415175054754</v>
       </c>
       <c r="F70" s="2" t="n">
-        <v>0.1446304062066568</v>
+        <v>0.1446304062066563</v>
       </c>
       <c r="G70" s="2" t="n">
-        <v>0.1594498269157253</v>
+        <v>0.1594498269157244</v>
       </c>
       <c r="H70" s="2" t="n">
-        <v>0.1796854435518387</v>
+        <v>0.1796854435518385</v>
       </c>
       <c r="I70" s="2" t="n">
-        <v>0.2022692408020758</v>
+        <v>0.2022692408020746</v>
       </c>
       <c r="J70" s="2" t="n">
         <v>0.2257775122301158</v>
@@ -3947,25 +3947,25 @@
         <v>0.2495156309882033</v>
       </c>
       <c r="L70" s="2" t="n">
-        <v>0.2728955178517541</v>
+        <v>0.2728955178517553</v>
       </c>
       <c r="M70" s="2" t="n">
-        <v>0.2954128716460067</v>
+        <v>0.2954128716460076</v>
       </c>
       <c r="N70" s="2" t="n">
-        <v>0.316596329059247</v>
+        <v>0.3165963290592476</v>
       </c>
       <c r="O70" s="2" t="n">
-        <v>0.3359150853534756</v>
+        <v>0.3359150853534754</v>
       </c>
       <c r="P70" s="2" t="n">
-        <v>0.3528309461237974</v>
+        <v>0.352830946123797</v>
       </c>
       <c r="Q70" s="2" t="n">
-        <v>0.3667419980396467</v>
+        <v>0.3667419980396462</v>
       </c>
       <c r="R70" s="2" t="n">
-        <v>0.3770263156088866</v>
+        <v>0.3770263156088856</v>
       </c>
       <c r="S70" s="1" t="inlineStr"/>
     </row>
@@ -3982,22 +3982,22 @@
       </c>
       <c r="C71" s="1" t="inlineStr"/>
       <c r="D71" s="2" t="n">
-        <v>251.7894146864385</v>
+        <v>251.7894146864383</v>
       </c>
       <c r="E71" s="2" t="n">
-        <v>249.6625952542775</v>
+        <v>249.6625952542773</v>
       </c>
       <c r="F71" s="2" t="n">
-        <v>247.6528107706313</v>
+        <v>247.6528107706312</v>
       </c>
       <c r="G71" s="2" t="n">
-        <v>245.7731838000793</v>
+        <v>245.7731838000792</v>
       </c>
       <c r="H71" s="2" t="n">
         <v>244.0304158041251</v>
       </c>
       <c r="I71" s="2" t="n">
-        <v>242.4310417988148</v>
+        <v>242.4310417988147</v>
       </c>
       <c r="J71" s="2" t="n">
         <v>240.972909827971</v>
@@ -4006,25 +4006,25 @@
         <v>239.6524840515102</v>
       </c>
       <c r="L71" s="2" t="n">
-        <v>238.4569611637397</v>
+        <v>238.4569611637399</v>
       </c>
       <c r="M71" s="2" t="n">
-        <v>237.3706330162411</v>
+        <v>237.3706330162412</v>
       </c>
       <c r="N71" s="2" t="n">
-        <v>236.3718770966746</v>
+        <v>236.3718770966747</v>
       </c>
       <c r="O71" s="2" t="n">
         <v>235.4310839272837</v>
       </c>
       <c r="P71" s="2" t="n">
-        <v>234.5161748631908</v>
+        <v>234.5161748631907</v>
       </c>
       <c r="Q71" s="2" t="n">
         <v>233.5872660970408</v>
       </c>
       <c r="R71" s="2" t="n">
-        <v>232.6016263665796</v>
+        <v>232.6016263665795</v>
       </c>
       <c r="S71" s="1" t="inlineStr"/>
     </row>
@@ -4100,22 +4100,22 @@
       </c>
       <c r="C73" s="1" t="inlineStr"/>
       <c r="D73" s="2" t="n">
-        <v>247.581434039078</v>
+        <v>247.9005511003572</v>
       </c>
       <c r="E73" s="2" t="n">
-        <v>239.722425110993</v>
+        <v>239.7224251109928</v>
       </c>
       <c r="F73" s="2" t="n">
         <v>236.3804261005702</v>
       </c>
       <c r="G73" s="2" t="n">
-        <v>234.0471923727898</v>
+        <v>234.0471923727897</v>
       </c>
       <c r="H73" s="2" t="n">
         <v>232.2443952114634</v>
       </c>
       <c r="I73" s="2" t="n">
-        <v>230.8447911323391</v>
+        <v>230.844791132339</v>
       </c>
       <c r="J73" s="2" t="n">
         <v>229.7932112410973</v>
@@ -4124,10 +4124,10 @@
         <v>229.0678517566361</v>
       </c>
       <c r="L73" s="2" t="n">
-        <v>228.6458226289366</v>
+        <v>228.6458226289367</v>
       </c>
       <c r="M73" s="2" t="n">
-        <v>228.5052237669685</v>
+        <v>228.5052237669686</v>
       </c>
       <c r="N73" s="2" t="n">
         <v>228.6215960141323</v>
@@ -4142,7 +4142,7 @@
         <v>230.1629008037089</v>
       </c>
       <c r="R73" s="2" t="n">
-        <v>230.932388801264</v>
+        <v>230.9323888012639</v>
       </c>
       <c r="S73" s="1" t="inlineStr"/>
     </row>
@@ -4159,7 +4159,7 @@
       </c>
       <c r="C74" s="1" t="inlineStr"/>
       <c r="D74" s="2" t="n">
-        <v>0.9234566717804606</v>
+        <v>0.9198717705829681</v>
       </c>
       <c r="E74" s="2" t="n">
         <v>0.9316127880691234</v>
@@ -4168,7 +4168,7 @@
         <v>0.9411937231993717</v>
       </c>
       <c r="G74" s="2" t="n">
-        <v>0.9489889140291673</v>
+        <v>0.9489889140291672</v>
       </c>
       <c r="H74" s="2" t="n">
         <v>0.9555931563290563</v>
@@ -4183,25 +4183,25 @@
         <v>0.9700508464641263</v>
       </c>
       <c r="L74" s="2" t="n">
-        <v>0.9735532872138978</v>
+        <v>0.9735532872138979</v>
       </c>
       <c r="M74" s="2" t="n">
         <v>0.9765720654514889</v>
       </c>
       <c r="N74" s="2" t="n">
-        <v>0.9792051916840198</v>
+        <v>0.9792051916840199</v>
       </c>
       <c r="O74" s="2" t="n">
         <v>0.9814270687200961</v>
       </c>
       <c r="P74" s="2" t="n">
-        <v>0.9833372387193101</v>
+        <v>0.98333723871931</v>
       </c>
       <c r="Q74" s="2" t="n">
         <v>0.9849622306534793</v>
       </c>
       <c r="R74" s="2" t="n">
-        <v>0.9863414798135992</v>
+        <v>0.9863414798135991</v>
       </c>
       <c r="S74" s="1" t="inlineStr"/>
     </row>
@@ -4218,7 +4218,7 @@
       </c>
       <c r="C75" s="1" t="inlineStr"/>
       <c r="D75" s="2" t="n">
-        <v>265.9555214727727</v>
+        <v>264.9230699278948</v>
       </c>
       <c r="E75" s="2" t="n">
         <v>294.8147930348406</v>
@@ -4254,13 +4254,13 @@
         <v>589.8572714101675</v>
       </c>
       <c r="P75" s="2" t="n">
-        <v>618.9875214592724</v>
+        <v>618.9875214592723</v>
       </c>
       <c r="Q75" s="2" t="n">
         <v>648.0388565102273</v>
       </c>
       <c r="R75" s="2" t="n">
-        <v>677.0139991251236</v>
+        <v>677.0139991251235</v>
       </c>
       <c r="S75" s="1" t="inlineStr"/>
     </row>
@@ -4277,7 +4277,7 @@
       </c>
       <c r="C76" s="1" t="inlineStr"/>
       <c r="D76" s="2" t="n">
-        <v>298.6191705006453</v>
+        <v>298.0389802067385</v>
       </c>
       <c r="E76" s="2" t="n">
         <v>314.3092699735009</v>
@@ -4336,22 +4336,22 @@
       </c>
       <c r="C77" s="1" t="inlineStr"/>
       <c r="D77" s="2" t="n">
-        <v>0.8431790037602239</v>
+        <v>0.8448204141343573</v>
       </c>
       <c r="E77" s="2" t="n">
-        <v>0.7943214505742267</v>
+        <v>0.7943214505742261</v>
       </c>
       <c r="F77" s="2" t="n">
-        <v>0.7511095390711756</v>
+        <v>0.7511095390711755</v>
       </c>
       <c r="G77" s="2" t="n">
-        <v>0.7135754513445642</v>
+        <v>0.7135754513445639</v>
       </c>
       <c r="H77" s="2" t="n">
-        <v>0.6807840523057973</v>
+        <v>0.6807840523057971</v>
       </c>
       <c r="I77" s="2" t="n">
-        <v>0.651895609766268</v>
+        <v>0.6518956097662678</v>
       </c>
       <c r="J77" s="2" t="n">
         <v>0.6262006800178096</v>
@@ -4360,25 +4360,25 @@
         <v>0.6032931870271456</v>
       </c>
       <c r="L77" s="2" t="n">
-        <v>0.582669850624871</v>
+        <v>0.5826698506248713</v>
       </c>
       <c r="M77" s="2" t="n">
-        <v>0.5640185684375758</v>
+        <v>0.5640185684375761</v>
       </c>
       <c r="N77" s="2" t="n">
-        <v>0.5470938594252941</v>
+        <v>0.5470938594252943</v>
       </c>
       <c r="O77" s="2" t="n">
-        <v>0.5314851030679409</v>
+        <v>0.5314851030679412</v>
       </c>
       <c r="P77" s="2" t="n">
-        <v>0.5170517482371183</v>
+        <v>0.5170517482371181</v>
       </c>
       <c r="Q77" s="2" t="n">
-        <v>0.5035581698659797</v>
+        <v>0.5035581698659796</v>
       </c>
       <c r="R77" s="2" t="n">
-        <v>0.4908332230905137</v>
+        <v>0.4908332230905135</v>
       </c>
       <c r="S77" s="1" t="inlineStr"/>
     </row>
@@ -4395,22 +4395,22 @@
       </c>
       <c r="C78" s="1" t="inlineStr"/>
       <c r="D78" s="2" t="n">
-        <v>0.7748207407327543</v>
+        <v>0.7758194364498243</v>
       </c>
       <c r="E78" s="2" t="n">
-        <v>0.7162072399490459</v>
+        <v>0.7162072399490456</v>
       </c>
       <c r="F78" s="2" t="n">
-        <v>0.6768754162864432</v>
+        <v>0.6768754162864431</v>
       </c>
       <c r="G78" s="2" t="n">
-        <v>0.6446312378490995</v>
+        <v>0.6446312378490993</v>
       </c>
       <c r="H78" s="2" t="n">
         <v>0.6171656544030198</v>
       </c>
       <c r="I78" s="2" t="n">
-        <v>0.5933516387160817</v>
+        <v>0.5933516387160813</v>
       </c>
       <c r="J78" s="2" t="n">
         <v>0.5724800026430085</v>
@@ -4419,13 +4419,13 @@
         <v>0.5541992204938717</v>
       </c>
       <c r="L78" s="2" t="n">
-        <v>0.5381521735211686</v>
+        <v>0.5381521735211688</v>
       </c>
       <c r="M78" s="2" t="n">
-        <v>0.5241056797248543</v>
+        <v>0.5241056797248544</v>
       </c>
       <c r="N78" s="2" t="n">
-        <v>0.5116577227873375</v>
+        <v>0.5116577227873376</v>
       </c>
       <c r="O78" s="2" t="n">
         <v>0.5006277313683627</v>
@@ -4434,10 +4434,10 @@
         <v>0.4908125161156869</v>
       </c>
       <c r="Q78" s="2" t="n">
-        <v>0.4820311420268309</v>
+        <v>0.4820311420268308</v>
       </c>
       <c r="R78" s="2" t="n">
-        <v>0.474084587425221</v>
+        <v>0.4740845874252208</v>
       </c>
       <c r="S78" s="1" t="inlineStr"/>
     </row>
@@ -4454,16 +4454,16 @@
       </c>
       <c r="C79" s="1" t="inlineStr"/>
       <c r="D79" s="2" t="n">
-        <v>304.6972711556989</v>
+        <v>304.6972711556987</v>
       </c>
       <c r="E79" s="2" t="n">
-        <v>334.5400980960846</v>
+        <v>334.5400980960845</v>
       </c>
       <c r="F79" s="2" t="n">
-        <v>364.2636577736324</v>
+        <v>364.2636577736323</v>
       </c>
       <c r="G79" s="2" t="n">
-        <v>393.9358180901934</v>
+        <v>393.9358180901933</v>
       </c>
       <c r="H79" s="2" t="n">
         <v>423.4832578774369</v>
@@ -4478,7 +4478,7 @@
         <v>512.0790958565088</v>
       </c>
       <c r="L79" s="2" t="n">
-        <v>541.5492817938723</v>
+        <v>541.5492817938724</v>
       </c>
       <c r="M79" s="2" t="n">
         <v>570.9315691201923</v>
@@ -4513,16 +4513,16 @@
       </c>
       <c r="C80" s="1" t="inlineStr"/>
       <c r="D80" s="2" t="n">
-        <v>0.9003749355554335</v>
+        <v>0.9001179490256412</v>
       </c>
       <c r="E80" s="2" t="n">
-        <v>0.9152540141204015</v>
+        <v>0.9152540141204016</v>
       </c>
       <c r="F80" s="2" t="n">
         <v>0.9244318040653919</v>
       </c>
       <c r="G80" s="2" t="n">
-        <v>0.9317173785273669</v>
+        <v>0.931717378527367</v>
       </c>
       <c r="H80" s="2" t="n">
         <v>0.937726382807626</v>
@@ -4543,7 +4543,7 @@
         <v>0.9564711798415051</v>
       </c>
       <c r="N80" s="2" t="n">
-        <v>0.9587739854529909</v>
+        <v>0.9587739854529908</v>
       </c>
       <c r="O80" s="2" t="n">
         <v>0.9608011997304212</v>
@@ -4572,16 +4572,16 @@
       </c>
       <c r="C81" s="1" t="inlineStr"/>
       <c r="D81" s="2" t="n">
-        <v>618.0075037983869</v>
+        <v>617.8311110563025</v>
       </c>
       <c r="E81" s="2" t="n">
-        <v>628.2203405174404</v>
+        <v>628.2203405174405</v>
       </c>
       <c r="F81" s="2" t="n">
         <v>634.5198751116486</v>
       </c>
       <c r="G81" s="2" t="n">
-        <v>639.5206137030721</v>
+        <v>639.5206137030722</v>
       </c>
       <c r="H81" s="2" t="n">
         <v>643.6451284900878</v>
@@ -4602,7 +4602,7 @@
         <v>656.5113520672343</v>
       </c>
       <c r="N81" s="2" t="n">
-        <v>658.0919726414946</v>
+        <v>658.0919726414945</v>
       </c>
       <c r="O81" s="2" t="n">
         <v>659.4834303395994</v>
@@ -4631,10 +4631,10 @@
       </c>
       <c r="C82" s="1" t="inlineStr"/>
       <c r="D82" s="2" t="n">
-        <v>455.1397620691718</v>
+        <v>455.0748040551998</v>
       </c>
       <c r="E82" s="2" t="n">
-        <v>458.7438421848687</v>
+        <v>458.7438421848688</v>
       </c>
       <c r="F82" s="2" t="n">
         <v>460.9384929530079</v>
@@ -4661,7 +4661,7 @@
         <v>467.6634924923767</v>
       </c>
       <c r="N82" s="2" t="n">
-        <v>467.9889608220808</v>
+        <v>467.9889608220807</v>
       </c>
       <c r="O82" s="2" t="n">
         <v>468.2745682991455</v>
@@ -4690,22 +4690,22 @@
       </c>
       <c r="C83" s="1" t="inlineStr"/>
       <c r="D83" s="2" t="n">
-        <v>0.5439679295729182</v>
+        <v>0.5447468172074129</v>
       </c>
       <c r="E83" s="2" t="n">
-        <v>0.5225627094398959</v>
+        <v>0.5225627094398955</v>
       </c>
       <c r="F83" s="2" t="n">
         <v>0.5128242264736803</v>
       </c>
       <c r="G83" s="2" t="n">
-        <v>0.5058701247484856</v>
+        <v>0.5058701247484854</v>
       </c>
       <c r="H83" s="2" t="n">
         <v>0.500517867126743</v>
       </c>
       <c r="I83" s="2" t="n">
-        <v>0.4963537393673502</v>
+        <v>0.4963537393673499</v>
       </c>
       <c r="J83" s="2" t="n">
         <v>0.4931527461005401</v>
@@ -4714,13 +4714,13 @@
         <v>0.4908656433918407</v>
       </c>
       <c r="L83" s="2" t="n">
-        <v>0.4893667613005351</v>
+        <v>0.4893667613005354</v>
       </c>
       <c r="M83" s="2" t="n">
-        <v>0.4886103521768771</v>
+        <v>0.4886103521768774</v>
       </c>
       <c r="N83" s="2" t="n">
-        <v>0.4885192069755876</v>
+        <v>0.4885192069755879</v>
       </c>
       <c r="O83" s="2" t="n">
         <v>0.4889480192746724</v>
@@ -4729,10 +4729,10 @@
         <v>0.4898496347186731</v>
       </c>
       <c r="Q83" s="2" t="n">
-        <v>0.4911141294015546</v>
+        <v>0.4911141294015545</v>
       </c>
       <c r="R83" s="2" t="n">
-        <v>0.4926388829310537</v>
+        <v>0.4926388829310535</v>
       </c>
       <c r="S83" s="1" t="inlineStr"/>
     </row>

</xml_diff>